<commit_message>
21th commit: checked all xpaths and verified screenshot in super admin login test
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27A2CB06-2D63-4FE1-AEC6-6990FFD9D7A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862934A6-1612-4AD5-9A8B-5567FCB3FBBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="41">
   <si>
     <t>The Admin login page is accessible. Valid  Super Admin credentials are available.</t>
   </si>
@@ -123,16 +123,6 @@
   </si>
   <si>
     <t>SA_TS_0</t>
-  </si>
-  <si>
-    <t>Verify that an  super admin can login with the provided credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
-2. Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
-3. Click Login,click,,"//button[@type='submit']"
-4. Verify Dashboard,verify,,"//div[contains(text(),'☰ Date Wise Statistics')]"
-</t>
   </si>
   <si>
     <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
@@ -393,12 +383,89 @@
   <si>
     <t>TC_CA_00_super_admin_login</t>
   </si>
+  <si>
+    <t>1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
+2. Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
+3. Click Login,click,,"//button[@type='submit']"
+4. Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"</t>
+  </si>
+  <si>
+    <t>Verify successful authentication of the Super Admin role using valid credentials and Dashboard access validation.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The WE1 Application is deployed and the Login URL is reachable (https://dev.we1.co/#/login)  and configured as base.url in config.properties.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Super Admin credentials (email and password) are configured in the config.properties file.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -410,6 +477,14 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -751,9 +826,9 @@
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
     <col min="2" max="2" width="21.5546875" customWidth="1"/>
     <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="31.6640625" customWidth="1"/>
+    <col min="4" max="4" width="26.6640625" customWidth="1"/>
     <col min="5" max="5" width="53.21875" customWidth="1"/>
-    <col min="6" max="6" width="29" customWidth="1"/>
+    <col min="6" max="6" width="36.88671875" customWidth="1"/>
     <col min="7" max="7" width="16.33203125" customWidth="1"/>
     <col min="8" max="8" width="15.21875" customWidth="1"/>
   </cols>
@@ -784,7 +859,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
@@ -792,16 +867,16 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -868,13 +943,13 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>0</v>
@@ -949,7 +1024,7 @@
         <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>15</v>
@@ -1014,7 +1089,7 @@
         <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>18</v>
@@ -1086,7 +1161,7 @@
         <v>24</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>18</v>
@@ -1158,7 +1233,7 @@
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
22th commit: checked all xpaths and verified screenshot in add city area test
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862934A6-1612-4AD5-9A8B-5567FCB3FBBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7252816A-2999-4E47-8795-D07AA2A0CE83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -32,9 +32,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="41">
   <si>
-    <t>The Admin login page is accessible. Valid  Super Admin credentials are available.</t>
-  </si>
-  <si>
     <t>City Area</t>
   </si>
   <si>
@@ -65,9 +62,6 @@
     <t>SA_TS_2</t>
   </si>
   <si>
-    <t>Super Admin can log in .Validate that an admin can add a new city area by entering the area name, selecting status, mapping the area, and saving. The new area should be listed on the City Area List and displayed in City Wise Manage Services (Ride Service Edit) and City Admin’s select city dropdown</t>
-  </si>
-  <si>
     <t>SA_TS_1</t>
   </si>
   <si>
@@ -123,35 +117,6 @@
   </si>
   <si>
     <t>SA_TS_0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-2. Click City area menu,click,,"//span[normalize-space()='City area']"
-3. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
-4. Click Add City Area button , click ,, "//button[@class='buttonWidget']"
-5. Verify City Area heading,verify,,"//div[@class='ng-star-inserted']//div[contains(text(),'City Area')]"
-6. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
-7. Open Status Dropdown,click,,"//span[@aria-label='select status']"
-8. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-9. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
-10. Click Submit,click,,"//button[normalize-space()='Submit']"
-11. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
-12. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
-13. Verify Transport Page,verify,,"//div[contains(text(),'☰ TRANSPORT SERVICES')]"
-14. Click Add Category,click,,"//button[normalize-space()='Add Category']"
-15. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
-16. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
-17. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
-18. Click close,click,,"//button[normalize-space()='Close']"
-19. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-20. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-21. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
-22. Click Add City Admin button , click ,, "//button[@class='buttonWidget']"
-23. Open Select City Dropdown,click,,"//select[@id='cityId']"
-24. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-25. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
-26. Click back,click,,"//button[@type='button']"
-</t>
   </si>
   <si>
     <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
@@ -458,6 +423,82 @@
         <scheme val="minor"/>
       </rPr>
       <t>Super Admin credentials (email and password) are configured in the config.properties file.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+2. Click City area menu,click,,"//span[normalize-space()='City area']"
+3. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
+4. Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
+5. Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
+6. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
+7. Open Status Dropdown,click,,"//span[@aria-label='select status']"
+8. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+9. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
+10. Click Submit,click,,"//button[normalize-space()='Submit']"
+11. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
+12. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
+13. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
+14. Click Add Category,click,,"//button[normalize-space()='Add Category']"
+15. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
+16. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
+17. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
+18. Click close,click,,"//button[normalize-space()='Close']"
+19. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+20. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+21. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
+22. Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
+23. Open Select City Dropdown,click,,"//select[@id='cityId']"
+24. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
+25. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
+</t>
+  </si>
+  <si>
+    <t>Validate the end-to-end creation of a City Area, including status configuration and polygon mapping. Verify data persistence by ensuring the new area is correctly listed and available for selection in 'City Wise Manage Services' in ' Transport Service ' and 'City Admin' modules.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
     </r>
   </si>
 </sst>
@@ -835,48 +876,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -911,48 +952,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -986,48 +1027,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1051,48 +1092,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C2" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1123,48 +1164,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="C2" s="7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1195,48 +1236,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
23th commit: checked all xpaths and verified screenshot in add city admin test
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7252816A-2999-4E47-8795-D07AA2A0CE83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F421D90A-B2AE-4955-A726-1CC45C5CB90B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -176,51 +176,6 @@
 56.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
 57.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
 58.wait,3000,,</t>
-  </si>
-  <si>
-    <t>1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-4. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
-5. Click Add City Admin button,click,,"//button[@class='buttonWidget']"
-6. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
-7.Click the Name field  "//input[@id='name']"
-8. Enter Admin Name, type, faizal_{timestamp} &gt;&gt; adminName, "//input[@id='name']"
-9.Click the Email field  "//input[@id='email']"
-10. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
-11.Click the password field "//input[@id='password']"
-12.Enter the Password as "faizal@123". "//input[@id='password']"
-13.Click the city field  "//select[@id='cityId']"
-14.Select the City as "triplicane" from the dropdown "//select[@id='cityId']"
-15. Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
-16.Click on the "Customers" → "Add Customers" checkbox. "//label[normalize-space()='Add Customers']"
-17.Click on the "Customers" → "Verified Customers"checkbox. "//div[3]//div[1]//div[1]//label[2]"
-18.Click on the "Customers" → "Non Verified Customers" checkbox. "//label[normalize-space()='Non Verified Customers']"
-19.Click on the "Customers" → "Blocked Customers" checkbox. "//label[normalize-space()='Blocked Customers']"
-20.Click on the "Customers" → "Deleted Customers" checkbox. "//label[normalize-space()='Deleted Customers']"
-21.Click on the "Providers" → "Transport Providers List" checkbox. "//label[normalize-space()='Transport Providers List']"
-22.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
-23.Click on the "Drivers" → "Approved Drivers" checkbox. "//body//app-root//div[3]//div[3]//div[1]//label[2]"
-24.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
-25.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
-26.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
-27.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
-28.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox. "//label[normalize-space()='Driver Subscription Plan']"
-29.Click on the "Cash Out" → "Driver Cash Out" checkbox. "//label[normalize-space()='Driver Cash Out']"
-30.Click on the "Report Issue" → "Customer Report Issues" checkbox. "//label[normalize-space()='Customer Report Issues']"
-31.Click on the "Report Issue" → "Driver Report Issues" checkbox. "//label[normalize-space()='Driver Report Issues']"
-32.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
-33.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
-34.Click on the "Report Issue" → "FAQs" checkbox. "//div[6]//div[1]//label[6]"
-35.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
-36.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
-37.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[7]//div[1]//label[3]"
-38.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[7]//div[1]//label[4]"
-39.Click on the "Website Settings" → "FAQs" checkbox. "//div[7]//div[1]//label[5]"
-40.Click on the "Add City Admin" button. "//button[@type='submit']"
-41. Verify Success Message,verify,,"//div[@aria-label='Info']"
-42.wait,3000,,
-42. Verify that "{adminName}" appears in the City Admin List with the correct details and permissions. "//span[normalize-space()='{adminName}']"</t>
   </si>
   <si>
     <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
@@ -500,6 +455,51 @@
       </rPr>
       <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
     </r>
+  </si>
+  <si>
+    <t>1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+4. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
+5. Click Add City Admin button,click,,"//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
+6. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
+7.Click the Name field  "//input[@id='name']"
+8. Enter Admin Name, type, faizal_{timestamp} &gt;&gt; adminName, "//input[@id='name']"
+9.Click the Email field  "//input[@id='email']"
+10. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
+11.Click the password field "//input[@id='password']"
+12.Enter the Password as "faizal@123". "//input[@id='password']"
+13.Click the city field  "//select[@id='cityId']"
+14.Select the City as "triplicane" from the dropdown "//select[@id='cityId']"
+15. Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
+16.Click on the "Customers" → "Add Customers" checkbox. "//label[normalize-space()='Add Customers']"
+17.Click on the "Customers" → "Verified Customers"checkbox. "//label[normalize-space()='Verified Customers']"
+18.Click on the "Customers" → "Non Verified Customers" checkbox. "//label[normalize-space()='Non Verified Customers']"
+19.Click on the "Customers" → "Blocked Customers" checkbox. "//label[normalize-space()='Blocked Customers']"
+20.Click on the "Customers" → "Deleted Customers" checkbox. "//label[normalize-space()='Deleted Customers']"
+21.Click on the "Providers" → "Transport Providers List" checkbox. "//label[normalize-space()='Transport Providers List']"
+22.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
+23.Click on the "Drivers" → "Approved Drivers" checkbox. "//label[normalize-space()='Approved Drivers']"
+24.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
+25.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
+26.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
+27.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
+28.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox. "//label[normalize-space()='Driver Subscription Plan']"
+29.Click on the "Cash Out" → "Driver Cash Out" checkbox. "//label[normalize-space()='Driver Cash Out']"
+30.Click on the "Report Issue" → "Customer Report Issues" checkbox. "//label[normalize-space()='Customer Report Issues']"
+31.Click on the "Report Issue" → "Driver Report Issues" checkbox. "//label[normalize-space()='Driver Report Issues']"
+32.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
+33.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
+34.Click on the "Report Issue" → "FAQs" checkbox. "(//h3[contains(.,'Report Issue')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
+35.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
+36.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
+37.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[h3[contains(.,'Website Settings')]]//label[contains(.,'Delivery')]"
+38.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[.//h3[contains(text(),'Website Settings')]]//label[contains(.,'Transport')]"
+39.Click on the "Website Settings" → "FAQs" checkbox. "(//h3[contains(.,'Website Settings')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
+40.Click on the "Add City Admin" button. "//button[@type='submit']"
+41. Verify Success Message,verify,,"//div[@aria-label='Info']"
+42.wait,3000,,
+42. Verify that "{adminName}" appears in the City Admin List with the correct details and permissions. "//span[normalize-space()='{adminName}']"</t>
   </si>
 </sst>
 </file>
@@ -908,16 +908,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -984,16 +984,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1065,7 +1065,7 @@
         <v>12</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>13</v>
@@ -1202,7 +1202,7 @@
         <v>22</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>16</v>
@@ -1274,7 +1274,7 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
24th commit: Made add city admin test data independent
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F421D90A-B2AE-4955-A726-1CC45C5CB90B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17DC7603-8BB0-4DBF-8CFA-46FC70C88ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,12 +66,6 @@
   </si>
   <si>
     <t>CityAdmin</t>
-  </si>
-  <si>
-    <t>Validate that the admin can successfully add a new City Admin by entering valid details, selecting city, and assigning multiple service and module permissions.</t>
-  </si>
-  <si>
-    <t>Admin is logged in and has access to the City Admin module and City Area data.</t>
   </si>
   <si>
     <t>TC_CA_02_add_city_admin</t>
@@ -457,6 +451,98 @@
     </r>
   </si>
   <si>
+    <t>To verify that the Super Admin can successfully create a new City Admin account by providing valid personal details, associating them with a specific city, and granting multiple service and module-level permissions.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddCityArea test suite must be always executed before this test. This is critical because the AddCityAdmin process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>System State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
+    </r>
+  </si>
+  <si>
     <t>1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
 2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
 3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
@@ -469,37 +555,38 @@
 10. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
 11.Click the password field "//input[@id='password']"
 12.Enter the Password as "faizal@123". "//input[@id='password']"
-13.Click the city field  "//select[@id='cityId']"
-14.Select the City as "triplicane" from the dropdown "//select[@id='cityId']"
+13.Open Select City Dropdown,click,,"//select[@id='cityId']"
+14.Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
 15. Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
 16.Click on the "Customers" → "Add Customers" checkbox. "//label[normalize-space()='Add Customers']"
 17.Click on the "Customers" → "Verified Customers"checkbox. "//label[normalize-space()='Verified Customers']"
 18.Click on the "Customers" → "Non Verified Customers" checkbox. "//label[normalize-space()='Non Verified Customers']"
 19.Click on the "Customers" → "Blocked Customers" checkbox. "//label[normalize-space()='Blocked Customers']"
 20.Click on the "Customers" → "Deleted Customers" checkbox. "//label[normalize-space()='Deleted Customers']"
-21.Click on the "Providers" → "Transport Providers List" checkbox. "//label[normalize-space()='Transport Providers List']"
-22.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
-23.Click on the "Drivers" → "Approved Drivers" checkbox. "//label[normalize-space()='Approved Drivers']"
-24.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
-25.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
-26.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
-27.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
-28.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox. "//label[normalize-space()='Driver Subscription Plan']"
-29.Click on the "Cash Out" → "Driver Cash Out" checkbox. "//label[normalize-space()='Driver Cash Out']"
-30.Click on the "Report Issue" → "Customer Report Issues" checkbox. "//label[normalize-space()='Customer Report Issues']"
-31.Click on the "Report Issue" → "Driver Report Issues" checkbox. "//label[normalize-space()='Driver Report Issues']"
-32.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
-33.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
-34.Click on the "Report Issue" → "FAQs" checkbox. "(//h3[contains(.,'Report Issue')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
-35.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
-36.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
-37.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[h3[contains(.,'Website Settings')]]//label[contains(.,'Delivery')]"
-38.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[.//h3[contains(text(),'Website Settings')]]//label[contains(.,'Transport')]"
-39.Click on the "Website Settings" → "FAQs" checkbox. "(//h3[contains(.,'Website Settings')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
-40.Click on the "Add City Admin" button. "//button[@type='submit']"
-41. Verify Success Message,verify,,"//div[@aria-label='Info']"
-42.wait,3000,,
-42. Verify that "{adminName}" appears in the City Admin List with the correct details and permissions. "//span[normalize-space()='{adminName}']"</t>
+21.Click on the "Customers" → "Pending Customers" checkbox. "//label[normalize-space()='Pending Customers']"
+22.Click on the "Providers" → "Transport Providers List" checkbox. "//label[normalize-space()='Transport Providers List']"
+23.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
+24.Click on the "Drivers" → "Approved Drivers" checkbox. "//label[normalize-space()='Approved Drivers']"
+25.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
+26.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
+27.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
+28.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
+29.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox. "//label[normalize-space()='Driver Subscription Plan']"
+30.Click on the "Cash Out" → "Driver Cash Out" checkbox. "//label[normalize-space()='Driver Cash Out']"
+31.Click on the "Report Issue" → "Customer Report Issues" checkbox. "//label[normalize-space()='Customer Report Issues']"
+32.Click on the "Report Issue" → "Driver Report Issues" checkbox. "//label[normalize-space()='Driver Report Issues']"
+33.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
+34.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
+35.Click on the "Report Issue" → "FAQs" checkbox. "(//h3[contains(.,'Report Issue')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
+36.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
+37.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
+38.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[h3[contains(.,'Website Settings')]]//label[contains(.,'Delivery')]"
+39.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[.//h3[contains(text(),'Website Settings')]]//label[contains(.,'Transport')]"
+40.Click on the "Website Settings" → "FAQs" checkbox. "(//h3[contains(.,'Website Settings')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
+41.Click on the "Add City Admin" button. "//button[@type='submit']"
+42. Verify Success Message,verify,,"//div[@aria-label='Info']"
+43.wait,3000,,
+44. Verify that "{adminName}" appears in the City Admin List with the correct details and permissions. "//span[normalize-space()='{adminName}']"</t>
   </si>
 </sst>
 </file>
@@ -902,22 +989,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="E2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -984,16 +1071,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1021,7 +1108,7 @@
     <col min="3" max="3" width="25.44140625" customWidth="1"/>
     <col min="4" max="4" width="34.77734375" customWidth="1"/>
     <col min="5" max="5" width="64" customWidth="1"/>
-    <col min="6" max="6" width="23.6640625" customWidth="1"/>
+    <col min="6" max="6" width="32.6640625" customWidth="1"/>
     <col min="7" max="7" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1059,16 +1146,16 @@
         <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1118,22 +1205,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C2" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1190,22 +1277,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="C2" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1262,22 +1349,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
25th commit: Add city admin test verified and completed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17DC7603-8BB0-4DBF-8CFA-46FC70C88ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C77A61C2-BBB0-4E87-A8D6-CCB9A92AE97D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -549,11 +549,11 @@
 4. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
 5. Click Add City Admin button,click,,"//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
 6. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
-7.Click the Name field  "//input[@id='name']"
+7.Select Name field,click ,, "//input[@id='name']"
 8. Enter Admin Name, type, faizal_{timestamp} &gt;&gt; adminName, "//input[@id='name']"
-9.Click the Email field  "//input[@id='email']"
+9.Select Email field,click,, "//input[@id='email']"
 10. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
-11.Click the password field "//input[@id='password']"
+11.select the password field,click,, "//input[@id='password']"
 12.Enter the Password as "faizal@123". "//input[@id='password']"
 13.Open Select City Dropdown,click,,"//select[@id='cityId']"
 14.Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
@@ -586,7 +586,8 @@
 41.Click on the "Add City Admin" button. "//button[@type='submit']"
 42. Verify Success Message,verify,,"//div[@aria-label='Info']"
 43.wait,3000,,
-44. Verify that "{adminName}" appears in the City Admin List with the correct details and permissions. "//span[normalize-space()='{adminName}']"</t>
+44.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
+45.wait,2000,,</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
26th commit: All driver tests verified and completed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C77A61C2-BBB0-4E87-A8D6-CCB9A92AE97D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{979834A0-81AA-42FE-A33E-AF574933EE89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="43">
   <si>
     <t>City Area</t>
   </si>
@@ -72,9 +72,6 @@
   </si>
   <si>
     <t>SA_TS_3</t>
-  </si>
-  <si>
-    <t>Admin is logged in and has access to add driver module.</t>
   </si>
   <si>
     <t>SA_TS_4</t>
@@ -588,6 +585,216 @@
 43.wait,3000,,
 44.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
 45.wait,2000,,</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FileSystem State (Crucial)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
+-&gt; C:\images\autodriver.jpg (For Driver Profile)
+-&gt; C:\images\vehicle.jpg (For Vehicle Image)
+-&gt; C:\images\license.jpg (For Driving License Document)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FileSystem State (Crucial):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
+-&gt; C:\images\bikedriver.jpg (For Driver Profile)
+-&gt; C:\images\bike.jpg (For Vehicle Image)
+-&gt; C:\images\license.jpg (For Driving License Document)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FileSystem State (Crucial)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
+-&gt; C:\images\taxidriver.jpg (For Driver Profile)
+-&gt; C:\images\taxi.jpg (For Vehicle Image)
+-&gt; C:\images\license.jpg (For Driving License Document)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -990,22 +1197,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1072,16 +1279,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1150,13 +1357,13 @@
         <v>12</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1174,7 +1381,7 @@
     <col min="3" max="3" width="30.88671875" customWidth="1"/>
     <col min="4" max="4" width="35.5546875" customWidth="1"/>
     <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="20.77734375" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" customWidth="1"/>
     <col min="7" max="7" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1209,19 +1416,19 @@
         <v>13</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1246,7 +1453,7 @@
     <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="4" width="35.5546875" customWidth="1"/>
     <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="20.77734375" customWidth="1"/>
+    <col min="6" max="6" width="29.5546875" customWidth="1"/>
     <col min="7" max="7" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1278,22 +1485,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1318,7 +1525,7 @@
     <col min="3" max="3" width="29.5546875" customWidth="1"/>
     <col min="4" max="4" width="35.5546875" customWidth="1"/>
     <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="20.77734375" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" customWidth="1"/>
     <col min="7" max="7" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1350,22 +1557,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="C2" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
28th commit: Add store test started
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{979834A0-81AA-42FE-A33E-AF574933EE89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A618674-2B05-40F4-926E-34A8443934EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="AddAutoDriver" sheetId="3" r:id="rId4"/>
     <sheet name="AddBikeDriver" sheetId="4" r:id="rId5"/>
     <sheet name="AddTaxiDriver" sheetId="5" r:id="rId6"/>
+    <sheet name="AddStore" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="48">
   <si>
     <t>City Area</t>
   </si>
@@ -795,6 +796,45 @@
 -&gt; C:\images\taxi.jpg (For Vehicle Image)
 -&gt; C:\images\license.jpg (For Driving License Document)</t>
     </r>
+  </si>
+  <si>
+    <t>SA_TS_6</t>
+  </si>
+  <si>
+    <t>TC_CA_06_add_store</t>
+  </si>
+  <si>
+    <t>Add New Store</t>
+  </si>
+  <si>
+    <t>Validate that the admin can successfully add a new store</t>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
+3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
+4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
+5.wait,2000,,
+6.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
+7.Click  Stores,click,,"//button[contains(., 'Stores')]"
+8.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
+9.Verify Add Store,verify,,"//div[contains(text(),'☰ Add Store')]"
+10.Enter Store Name, type, KFC_{timestamp} &gt;&gt; storeName, "//input[@placeholder='Store Name']"
+11.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
+12.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
+13.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
+14. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
+15.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
+16.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
+17.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
+18.Upload Banner Image, uploadfile, "C:\images\kfcbanner.jpg", "//input[@type='file']"
+19.wait,2000,,
+20.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
+21.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
+22.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
+23.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
+24.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+25.wait,2000,,</t>
   </si>
 </sst>
 </file>
@@ -1585,4 +1625,76 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C456A73-57BC-411E-B40E-DADED30882CB}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
29th commit: In Add store fixed issue of google map synced box implemented up and down navigation
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A618674-2B05-40F4-926E-34A8443934EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC88ED59-3BD4-4F4F-92CB-5950430A24AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -810,7 +810,7 @@
     <t>Validate that the admin can successfully add a new store</t>
   </si>
   <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
+    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
 2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
 3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
 4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
@@ -834,7 +834,12 @@
 22.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
 23.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
 24.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-25.wait,2000,,</t>
+25..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
+26.wait,2000,,
+27.Select First Option,type,\ue015,"//input[@placeholder='Search location']"
+28.Confirm Option,type,\ue007,"//input[@placeholder='Search location']"
+29.wait,2000,,
+</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
30th commit:Introduced keyboard navigation to  fix issue of google map synced box
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC88ED59-3BD4-4F4F-92CB-5950430A24AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F48DE51-96AA-4A80-83AD-1DCFD9170936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -810,7 +810,7 @@
     <t>Validate that the admin can successfully add a new store</t>
   </si>
   <si>
-    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
 2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
 3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
 4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
@@ -836,10 +836,9 @@
 24.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
 25..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
 26.wait,2000,,
-27.Select First Option,type,\ue015,"//input[@placeholder='Search location']"
-28.Confirm Option,type,\ue007,"//input[@placeholder='Search location']"
-29.wait,2000,,
-</t>
+27.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
+28.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
+29.wait,2000,,</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
31th commit:Implemented Browser Overlay Test Status Bar
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F48DE51-96AA-4A80-83AD-1DCFD9170936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BE50711-37D0-48A8-BD40-2D843D8FCD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -838,7 +838,7 @@
 26.wait,2000,,
 27.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
 28.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
-29.wait,2000,,</t>
+29.wait,3000,,</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
32th commit:Add Store Completed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BE50711-37D0-48A8-BD40-2D843D8FCD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B30C9174-BEE4-438C-A670-856382E5CA96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -838,7 +838,31 @@
 26.wait,2000,,
 27.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
 28.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
-29.wait,3000,,</t>
+29.wait,1000,,
+30.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
+31.wait,1000,,
+32..Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
+33.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
+34.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
+35.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
+36.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
+37.Enter Contact Person Full Name, type, storeowner_{timestamp} &gt;&gt; storeOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
+38.Enter Email, type, kfc_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
+39.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
+40.Upload Store Image, uploadfile, "C:\images\kfcstore.jpg", "(//input[@type='file'])[2]"
+41.wait,2000,,
+42.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
+43.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
+44.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
+45.Enter Accont Holder Name, type, {storeOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
+46.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
+47.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
+48.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
+49.Enter From Time, type, 100000, "(//label[contains(.,'From Time')]/following-sibling::input)[1]"
+50.Enter To Time, type, 220000, "(//label[contains(.,'To Time')]/following-sibling::input)[1]"
+51.Submit Add Store,click,,"//button[normalize-space()='Submit']"
+52. Verify Success Message,verify,,"//div[@aria-label='Info']"
+53.wait,3000,,</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
33th commit: grid navigation fixed ussing tab key
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B30C9174-BEE4-438C-A670-856382E5CA96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B995DB3-6A42-49BA-A579-DAEED7636E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -230,7 +230,527 @@
 58.wait,3000,,</t>
   </si>
   <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+    <t>TC_CA_01_add_city_area</t>
+  </si>
+  <si>
+    <t>TC_CA_00_super_admin_login</t>
+  </si>
+  <si>
+    <t>1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
+2. Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
+3. Click Login,click,,"//button[@type='submit']"
+4. Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"</t>
+  </si>
+  <si>
+    <t>Verify successful authentication of the Super Admin role using valid credentials and Dashboard access validation.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The WE1 Application is deployed and the Login URL is reachable (https://dev.we1.co/#/login)  and configured as base.url in config.properties.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Super Admin credentials (email and password) are configured in the config.properties file.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+2. Click City area menu,click,,"//span[normalize-space()='City area']"
+3. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
+4. Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
+5. Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
+6. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
+7. Open Status Dropdown,click,,"//span[@aria-label='select status']"
+8. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+9. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
+10. Click Submit,click,,"//button[normalize-space()='Submit']"
+11. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
+12. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
+13. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
+14. Click Add Category,click,,"//button[normalize-space()='Add Category']"
+15. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
+16. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
+17. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
+18. Click close,click,,"//button[normalize-space()='Close']"
+19. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+20. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+21. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
+22. Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
+23. Open Select City Dropdown,click,,"//select[@id='cityId']"
+24. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
+25. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
+</t>
+  </si>
+  <si>
+    <t>Validate the end-to-end creation of a City Area, including status configuration and polygon mapping. Verify data persistence by ensuring the new area is correctly listed and available for selection in 'City Wise Manage Services' in ' Transport Service ' and 'City Admin' modules.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
+    </r>
+  </si>
+  <si>
+    <t>To verify that the Super Admin can successfully create a new City Admin account by providing valid personal details, associating them with a specific city, and granting multiple service and module-level permissions.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddCityArea test suite must be always executed before this test. This is critical because the AddCityAdmin process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>System State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+4. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
+5. Click Add City Admin button,click,,"//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
+6. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
+7.Select Name field,click ,, "//input[@id='name']"
+8. Enter Admin Name, type, faizal_{timestamp} &gt;&gt; adminName, "//input[@id='name']"
+9.Select Email field,click,, "//input[@id='email']"
+10. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
+11.select the password field,click,, "//input[@id='password']"
+12.Enter the Password as "faizal@123". "//input[@id='password']"
+13.Open Select City Dropdown,click,,"//select[@id='cityId']"
+14.Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
+15. Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
+16.Click on the "Customers" → "Add Customers" checkbox. "//label[normalize-space()='Add Customers']"
+17.Click on the "Customers" → "Verified Customers"checkbox. "//label[normalize-space()='Verified Customers']"
+18.Click on the "Customers" → "Non Verified Customers" checkbox. "//label[normalize-space()='Non Verified Customers']"
+19.Click on the "Customers" → "Blocked Customers" checkbox. "//label[normalize-space()='Blocked Customers']"
+20.Click on the "Customers" → "Deleted Customers" checkbox. "//label[normalize-space()='Deleted Customers']"
+21.Click on the "Customers" → "Pending Customers" checkbox. "//label[normalize-space()='Pending Customers']"
+22.Click on the "Providers" → "Transport Providers List" checkbox. "//label[normalize-space()='Transport Providers List']"
+23.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
+24.Click on the "Drivers" → "Approved Drivers" checkbox. "//label[normalize-space()='Approved Drivers']"
+25.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
+26.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
+27.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
+28.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
+29.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox. "//label[normalize-space()='Driver Subscription Plan']"
+30.Click on the "Cash Out" → "Driver Cash Out" checkbox. "//label[normalize-space()='Driver Cash Out']"
+31.Click on the "Report Issue" → "Customer Report Issues" checkbox. "//label[normalize-space()='Customer Report Issues']"
+32.Click on the "Report Issue" → "Driver Report Issues" checkbox. "//label[normalize-space()='Driver Report Issues']"
+33.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
+34.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
+35.Click on the "Report Issue" → "FAQs" checkbox. "(//h3[contains(.,'Report Issue')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
+36.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
+37.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
+38.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[h3[contains(.,'Website Settings')]]//label[contains(.,'Delivery')]"
+39.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[.//h3[contains(text(),'Website Settings')]]//label[contains(.,'Transport')]"
+40.Click on the "Website Settings" → "FAQs" checkbox. "(//h3[contains(.,'Website Settings')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
+41.Click on the "Add City Admin" button. "//button[@type='submit']"
+42. Verify Success Message,verify,,"//div[@aria-label='Info']"
+43.wait,3000,,
+44.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
+45.wait,2000,,</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FileSystem State (Crucial)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
+-&gt; C:\images\autodriver.jpg (For Driver Profile)
+-&gt; C:\images\vehicle.jpg (For Vehicle Image)
+-&gt; C:\images\license.jpg (For Driving License Document)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FileSystem State (Crucial):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
+-&gt; C:\images\bikedriver.jpg (For Driver Profile)
+-&gt; C:\images\bike.jpg (For Vehicle Image)
+-&gt; C:\images\license.jpg (For Driving License Document)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FileSystem State (Crucial)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
+-&gt; C:\images\taxidriver.jpg (For Driver Profile)
+-&gt; C:\images\taxi.jpg (For Vehicle Image)
+-&gt; C:\images\license.jpg (For Driving License Document)</t>
+    </r>
+  </si>
+  <si>
+    <t>SA_TS_6</t>
+  </si>
+  <si>
+    <t>TC_CA_06_add_store</t>
+  </si>
+  <si>
+    <t>Add New Store</t>
+  </si>
+  <si>
+    <t>Validate that the admin can successfully add a new store</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 2. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 3. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
 4. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
@@ -287,530 +807,11 @@
 55.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
 56.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
 57.Filter Approved Driver,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
-58.wait,3000,,</t>
-  </si>
-  <si>
-    <t>TC_CA_01_add_city_area</t>
-  </si>
-  <si>
-    <t>TC_CA_00_super_admin_login</t>
-  </si>
-  <si>
-    <t>1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
-2. Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
-3. Click Login,click,,"//button[@type='submit']"
-4. Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"</t>
-  </si>
-  <si>
-    <t>Verify successful authentication of the Super Admin role using valid credentials and Dashboard access validation.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">System State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The WE1 Application is deployed and the Login URL is reachable (https://dev.we1.co/#/login)  and configured as base.url in config.properties.
+58.wait,2000,,
 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Access Rights:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A valid Super Admin account exists in the database.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Data Availability: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Super Admin credentials (email and password) are configured in the config.properties file.</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-2. Click City area menu,click,,"//span[normalize-space()='City area']"
-3. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
-4. Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
-5. Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
-6. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
-7. Open Status Dropdown,click,,"//span[@aria-label='select status']"
-8. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-9. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
-10. Click Submit,click,,"//button[normalize-space()='Submit']"
-11. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
-12. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
-13. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
-14. Click Add Category,click,,"//button[normalize-space()='Add Category']"
-15. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
-16. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
-17. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
-18. Click close,click,,"//button[normalize-space()='Close']"
-19. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-20. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-21. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
-22. Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
-23. Open Select City Dropdown,click,,"//select[@id='cityId']"
-24. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-25. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
-</t>
-  </si>
-  <si>
-    <t>Validate the end-to-end creation of a City Area, including status configuration and polygon mapping. Verify data persistence by ensuring the new area is correctly listed and available for selection in 'City Wise Manage Services' in ' Transport Service ' and 'City Admin' modules.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Authentication State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
-    </r>
-  </si>
-  <si>
-    <t>To verify that the Super Admin can successfully create a new City Admin account by providing valid personal details, associating them with a specific city, and granting multiple service and module-level permissions.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The AddCityArea test suite must be always executed before this test. This is critical because the AddCityAdmin process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>System State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
-    </r>
-  </si>
-  <si>
-    <t>1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-4. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
-5. Click Add City Admin button,click,,"//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
-6. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
-7.Select Name field,click ,, "//input[@id='name']"
-8. Enter Admin Name, type, faizal_{timestamp} &gt;&gt; adminName, "//input[@id='name']"
-9.Select Email field,click,, "//input[@id='email']"
-10. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
-11.select the password field,click,, "//input[@id='password']"
-12.Enter the Password as "faizal@123". "//input[@id='password']"
-13.Open Select City Dropdown,click,,"//select[@id='cityId']"
-14.Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-15. Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
-16.Click on the "Customers" → "Add Customers" checkbox. "//label[normalize-space()='Add Customers']"
-17.Click on the "Customers" → "Verified Customers"checkbox. "//label[normalize-space()='Verified Customers']"
-18.Click on the "Customers" → "Non Verified Customers" checkbox. "//label[normalize-space()='Non Verified Customers']"
-19.Click on the "Customers" → "Blocked Customers" checkbox. "//label[normalize-space()='Blocked Customers']"
-20.Click on the "Customers" → "Deleted Customers" checkbox. "//label[normalize-space()='Deleted Customers']"
-21.Click on the "Customers" → "Pending Customers" checkbox. "//label[normalize-space()='Pending Customers']"
-22.Click on the "Providers" → "Transport Providers List" checkbox. "//label[normalize-space()='Transport Providers List']"
-23.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
-24.Click on the "Drivers" → "Approved Drivers" checkbox. "//label[normalize-space()='Approved Drivers']"
-25.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
-26.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
-27.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
-28.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
-29.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox. "//label[normalize-space()='Driver Subscription Plan']"
-30.Click on the "Cash Out" → "Driver Cash Out" checkbox. "//label[normalize-space()='Driver Cash Out']"
-31.Click on the "Report Issue" → "Customer Report Issues" checkbox. "//label[normalize-space()='Customer Report Issues']"
-32.Click on the "Report Issue" → "Driver Report Issues" checkbox. "//label[normalize-space()='Driver Report Issues']"
-33.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
-34.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
-35.Click on the "Report Issue" → "FAQs" checkbox. "(//h3[contains(.,'Report Issue')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
-36.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
-37.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
-38.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[h3[contains(.,'Website Settings')]]//label[contains(.,'Delivery')]"
-39.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[.//h3[contains(text(),'Website Settings')]]//label[contains(.,'Transport')]"
-40.Click on the "Website Settings" → "FAQs" checkbox. "(//h3[contains(.,'Website Settings')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
-41.Click on the "Add City Admin" button. "//button[@type='submit']"
-42. Verify Success Message,verify,,"//div[@aria-label='Info']"
-43.wait,3000,,
-44.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
-45.wait,2000,,</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>FileSystem State (Crucial)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
--&gt; C:\images\autodriver.jpg (For Driver Profile)
--&gt; C:\images\vehicle.jpg (For Vehicle Image)
--&gt; C:\images\license.jpg (For Driving License Document)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>FileSystem State (Crucial):</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
--&gt; C:\images\bikedriver.jpg (For Driver Profile)
--&gt; C:\images\bike.jpg (For Vehicle Image)
--&gt; C:\images\license.jpg (For Driving License Document)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>FileSystem State (Crucial)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
--&gt; C:\images\taxidriver.jpg (For Driver Profile)
--&gt; C:\images\taxi.jpg (For Vehicle Image)
--&gt; C:\images\license.jpg (For Driving License Document)</t>
-    </r>
-  </si>
-  <si>
-    <t>SA_TS_6</t>
-  </si>
-  <si>
-    <t>TC_CA_06_add_store</t>
-  </si>
-  <si>
-    <t>Add New Store</t>
-  </si>
-  <si>
-    <t>Validate that the admin can successfully add a new store</t>
-  </si>
-  <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
+  </si>
+  <si>
+    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
 2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
 3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
 4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
@@ -862,7 +863,21 @@
 50.Enter To Time, type, 220000, "(//label[contains(.,'To Time')]/following-sibling::input)[1]"
 51.Submit Add Store,click,,"//button[normalize-space()='Submit']"
 52. Verify Success Message,verify,,"//div[@aria-label='Info']"
-53.wait,3000,,</t>
+53.wait,3000,,
+54.Click  Stores,click,,"//button[contains(., 'Stores')]"
+55.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+56.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
+57.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+58.wait,2000,,
+59.Click  Stores,click,,"//button[contains(., 'Stores')]"
+60.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
+61.Verify Add Store,verify,,"//div[contains(text(),'☰ Pending Documents Store')]"
+62.Filter Pending Document Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+63.wait,2000,,
+64.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+65.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
+65.wait,3000,,
+</t>
   </si>
 </sst>
 </file>
@@ -1271,16 +1286,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1347,16 +1362,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1425,13 +1440,13 @@
         <v>12</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1496,7 +1511,7 @@
         <v>26</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1568,7 +1583,7 @@
         <v>27</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1637,10 +1652,10 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1697,22 +1712,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>47</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
34th commit: Add Store Creation And Approval Completed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B995DB3-6A42-49BA-A579-DAEED7636E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03815199-E40B-4F94-9418-1BDE14F88AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -877,6 +877,29 @@
 64.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
 65.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
 65.wait,3000,,
+66. Store Required Documents,verify,,"//div[contains(text(),'☰ Documents')]"
+67.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+68.wait,3000,,
+69.Upload Address Proof, uploadfile, "C:\images\addressproof.png", "//input[@type='file']"
+70.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+71.wait,1000,,
+72.Click Submit, click, , "//button[normalize-space()='Submit']"
+73.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+74.wait,2000,,
+75.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+76.wait,2000,,
+77.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+78.wait,3000,,
+79.Click Back, click, , "//button[@class='buttonWidget']"
+80.wait,2000,,
+81.Click  Stores,click,,"//button[contains(., 'Stores')]"
+82.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+83.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
+84.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+85.wait,2000,,
+86.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+87.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
+88.wait,3000,,
 </t>
   </si>
 </sst>

</xml_diff>

<commit_message>
35th commit: Add Store And Add Drivers Completed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03815199-E40B-4F94-9418-1BDE14F88AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C063F592-4BDC-438D-8AE1-76F6F7BACE9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="49">
   <si>
     <t>City Area</t>
   </si>
@@ -109,6 +109,520 @@
   </si>
   <si>
     <t>SA_TS_0</t>
+  </si>
+  <si>
+    <t>TC_CA_01_add_city_area</t>
+  </si>
+  <si>
+    <t>TC_CA_00_super_admin_login</t>
+  </si>
+  <si>
+    <t>1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
+2. Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
+3. Click Login,click,,"//button[@type='submit']"
+4. Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"</t>
+  </si>
+  <si>
+    <t>Verify successful authentication of the Super Admin role using valid credentials and Dashboard access validation.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The WE1 Application is deployed and the Login URL is reachable (https://dev.we1.co/#/login)  and configured as base.url in config.properties.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Super Admin credentials (email and password) are configured in the config.properties file.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+2. Click City area menu,click,,"//span[normalize-space()='City area']"
+3. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
+4. Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
+5. Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
+6. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
+7. Open Status Dropdown,click,,"//span[@aria-label='select status']"
+8. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+9. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
+10. Click Submit,click,,"//button[normalize-space()='Submit']"
+11. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
+12. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
+13. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
+14. Click Add Category,click,,"//button[normalize-space()='Add Category']"
+15. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
+16. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
+17. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
+18. Click close,click,,"//button[normalize-space()='Close']"
+19. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+20. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+21. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
+22. Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
+23. Open Select City Dropdown,click,,"//select[@id='cityId']"
+24. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
+25. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
+</t>
+  </si>
+  <si>
+    <t>Validate the end-to-end creation of a City Area, including status configuration and polygon mapping. Verify data persistence by ensuring the new area is correctly listed and available for selection in 'City Wise Manage Services' in ' Transport Service ' and 'City Admin' modules.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
+    </r>
+  </si>
+  <si>
+    <t>To verify that the Super Admin can successfully create a new City Admin account by providing valid personal details, associating them with a specific city, and granting multiple service and module-level permissions.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddCityArea test suite must be always executed before this test. This is critical because the AddCityAdmin process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>System State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+4. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
+5. Click Add City Admin button,click,,"//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
+6. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
+7.Select Name field,click ,, "//input[@id='name']"
+8. Enter Admin Name, type, faizal_{timestamp} &gt;&gt; adminName, "//input[@id='name']"
+9.Select Email field,click,, "//input[@id='email']"
+10. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
+11.select the password field,click,, "//input[@id='password']"
+12.Enter the Password as "faizal@123". "//input[@id='password']"
+13.Open Select City Dropdown,click,,"//select[@id='cityId']"
+14.Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
+15. Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
+16.Click on the "Customers" → "Add Customers" checkbox. "//label[normalize-space()='Add Customers']"
+17.Click on the "Customers" → "Verified Customers"checkbox. "//label[normalize-space()='Verified Customers']"
+18.Click on the "Customers" → "Non Verified Customers" checkbox. "//label[normalize-space()='Non Verified Customers']"
+19.Click on the "Customers" → "Blocked Customers" checkbox. "//label[normalize-space()='Blocked Customers']"
+20.Click on the "Customers" → "Deleted Customers" checkbox. "//label[normalize-space()='Deleted Customers']"
+21.Click on the "Customers" → "Pending Customers" checkbox. "//label[normalize-space()='Pending Customers']"
+22.Click on the "Providers" → "Transport Providers List" checkbox. "//label[normalize-space()='Transport Providers List']"
+23.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
+24.Click on the "Drivers" → "Approved Drivers" checkbox. "//label[normalize-space()='Approved Drivers']"
+25.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
+26.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
+27.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
+28.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
+29.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox. "//label[normalize-space()='Driver Subscription Plan']"
+30.Click on the "Cash Out" → "Driver Cash Out" checkbox. "//label[normalize-space()='Driver Cash Out']"
+31.Click on the "Report Issue" → "Customer Report Issues" checkbox. "//label[normalize-space()='Customer Report Issues']"
+32.Click on the "Report Issue" → "Driver Report Issues" checkbox. "//label[normalize-space()='Driver Report Issues']"
+33.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
+34.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
+35.Click on the "Report Issue" → "FAQs" checkbox. "(//h3[contains(.,'Report Issue')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
+36.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
+37.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
+38.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[h3[contains(.,'Website Settings')]]//label[contains(.,'Delivery')]"
+39.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[.//h3[contains(text(),'Website Settings')]]//label[contains(.,'Transport')]"
+40.Click on the "Website Settings" → "FAQs" checkbox. "(//h3[contains(.,'Website Settings')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
+41.Click on the "Add City Admin" button. "//button[@type='submit']"
+42. Verify Success Message,verify,,"//div[@aria-label='Info']"
+43.wait,3000,,
+44.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
+45.wait,2000,,</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FileSystem State (Crucial)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
+-&gt; C:\images\autodriver.jpg (For Driver Profile)
+-&gt; C:\images\vehicle.jpg (For Vehicle Image)
+-&gt; C:\images\license.jpg (For Driving License Document)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FileSystem State (Crucial):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
+-&gt; C:\images\bikedriver.jpg (For Driver Profile)
+-&gt; C:\images\bike.jpg (For Vehicle Image)
+-&gt; C:\images\license.jpg (For Driving License Document)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FileSystem State (Crucial)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
+-&gt; C:\images\taxidriver.jpg (For Driver Profile)
+-&gt; C:\images\taxi.jpg (For Vehicle Image)
+-&gt; C:\images\license.jpg (For Driving License Document)</t>
+    </r>
+  </si>
+  <si>
+    <t>SA_TS_6</t>
+  </si>
+  <si>
+    <t>TC_CA_06_add_store</t>
   </si>
   <si>
     <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
@@ -167,7 +681,11 @@
 55.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
 56.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
 57.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-58.wait,3000,,</t>
+58.wait,2000,,
+59.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+60.Click Doc Icon,click,,"//i[@title='Document']"
+61.Click Eye Icon,click,,"//i[@title='View']"
+62.wait,2000,,</t>
   </si>
   <si>
     <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
@@ -227,527 +745,11 @@
 55.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
 56.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
 57.Filter Approved Driver,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
-58.wait,3000,,</t>
-  </si>
-  <si>
-    <t>TC_CA_01_add_city_area</t>
-  </si>
-  <si>
-    <t>TC_CA_00_super_admin_login</t>
-  </si>
-  <si>
-    <t>1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
-2. Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
-3. Click Login,click,,"//button[@type='submit']"
-4. Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"</t>
-  </si>
-  <si>
-    <t>Verify successful authentication of the Super Admin role using valid credentials and Dashboard access validation.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">System State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The WE1 Application is deployed and the Login URL is reachable (https://dev.we1.co/#/login)  and configured as base.url in config.properties.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Access Rights:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A valid Super Admin account exists in the database.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Data Availability: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Super Admin credentials (email and password) are configured in the config.properties file.</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-2. Click City area menu,click,,"//span[normalize-space()='City area']"
-3. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
-4. Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
-5. Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
-6. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
-7. Open Status Dropdown,click,,"//span[@aria-label='select status']"
-8. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-9. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
-10. Click Submit,click,,"//button[normalize-space()='Submit']"
-11. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
-12. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
-13. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
-14. Click Add Category,click,,"//button[normalize-space()='Add Category']"
-15. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
-16. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
-17. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
-18. Click close,click,,"//button[normalize-space()='Close']"
-19. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-20. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-21. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
-22. Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
-23. Open Select City Dropdown,click,,"//select[@id='cityId']"
-24. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-25. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
-</t>
-  </si>
-  <si>
-    <t>Validate the end-to-end creation of a City Area, including status configuration and polygon mapping. Verify data persistence by ensuring the new area is correctly listed and available for selection in 'City Wise Manage Services' in ' Transport Service ' and 'City Admin' modules.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Authentication State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
-    </r>
-  </si>
-  <si>
-    <t>To verify that the Super Admin can successfully create a new City Admin account by providing valid personal details, associating them with a specific city, and granting multiple service and module-level permissions.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The AddCityArea test suite must be always executed before this test. This is critical because the AddCityAdmin process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>System State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
-    </r>
-  </si>
-  <si>
-    <t>1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-4. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
-5. Click Add City Admin button,click,,"//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
-6. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
-7.Select Name field,click ,, "//input[@id='name']"
-8. Enter Admin Name, type, faizal_{timestamp} &gt;&gt; adminName, "//input[@id='name']"
-9.Select Email field,click,, "//input[@id='email']"
-10. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
-11.select the password field,click,, "//input[@id='password']"
-12.Enter the Password as "faizal@123". "//input[@id='password']"
-13.Open Select City Dropdown,click,,"//select[@id='cityId']"
-14.Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-15. Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
-16.Click on the "Customers" → "Add Customers" checkbox. "//label[normalize-space()='Add Customers']"
-17.Click on the "Customers" → "Verified Customers"checkbox. "//label[normalize-space()='Verified Customers']"
-18.Click on the "Customers" → "Non Verified Customers" checkbox. "//label[normalize-space()='Non Verified Customers']"
-19.Click on the "Customers" → "Blocked Customers" checkbox. "//label[normalize-space()='Blocked Customers']"
-20.Click on the "Customers" → "Deleted Customers" checkbox. "//label[normalize-space()='Deleted Customers']"
-21.Click on the "Customers" → "Pending Customers" checkbox. "//label[normalize-space()='Pending Customers']"
-22.Click on the "Providers" → "Transport Providers List" checkbox. "//label[normalize-space()='Transport Providers List']"
-23.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
-24.Click on the "Drivers" → "Approved Drivers" checkbox. "//label[normalize-space()='Approved Drivers']"
-25.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
-26.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
-27.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
-28.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
-29.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox. "//label[normalize-space()='Driver Subscription Plan']"
-30.Click on the "Cash Out" → "Driver Cash Out" checkbox. "//label[normalize-space()='Driver Cash Out']"
-31.Click on the "Report Issue" → "Customer Report Issues" checkbox. "//label[normalize-space()='Customer Report Issues']"
-32.Click on the "Report Issue" → "Driver Report Issues" checkbox. "//label[normalize-space()='Driver Report Issues']"
-33.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
-34.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
-35.Click on the "Report Issue" → "FAQs" checkbox. "(//h3[contains(.,'Report Issue')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
-36.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
-37.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
-38.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[h3[contains(.,'Website Settings')]]//label[contains(.,'Delivery')]"
-39.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[.//h3[contains(text(),'Website Settings')]]//label[contains(.,'Transport')]"
-40.Click on the "Website Settings" → "FAQs" checkbox. "(//h3[contains(.,'Website Settings')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
-41.Click on the "Add City Admin" button. "//button[@type='submit']"
-42. Verify Success Message,verify,,"//div[@aria-label='Info']"
-43.wait,3000,,
-44.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
-45.wait,2000,,</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>FileSystem State (Crucial)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
--&gt; C:\images\autodriver.jpg (For Driver Profile)
--&gt; C:\images\vehicle.jpg (For Vehicle Image)
--&gt; C:\images\license.jpg (For Driving License Document)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>FileSystem State (Crucial):</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
--&gt; C:\images\bikedriver.jpg (For Driver Profile)
--&gt; C:\images\bike.jpg (For Vehicle Image)
--&gt; C:\images\license.jpg (For Driving License Document)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>FileSystem State (Crucial)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
--&gt; C:\images\taxidriver.jpg (For Driver Profile)
--&gt; C:\images\taxi.jpg (For Vehicle Image)
--&gt; C:\images\license.jpg (For Driving License Document)</t>
-    </r>
-  </si>
-  <si>
-    <t>SA_TS_6</t>
-  </si>
-  <si>
-    <t>TC_CA_06_add_store</t>
-  </si>
-  <si>
-    <t>Add New Store</t>
-  </si>
-  <si>
-    <t>Validate that the admin can successfully add a new store</t>
+58.wait,2000,,
+59.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+60.Click Doc Icon,click,,"//i[@title='Document']"
+61.Click Eye Icon,click,,"//i[@title='View']"
+62.wait,2000,,</t>
   </si>
   <si>
     <t xml:space="preserve">1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
@@ -808,7 +810,87 @@
 56.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
 57.Filter Approved Driver,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
 58.wait,2000,,
+59.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+60.Click Doc Icon,click,,"//i[@title='Document']"
+61.Click Eye Icon,click,,"//i[@title='View']"
+62.wait,2000,,
 </t>
+  </si>
+  <si>
+    <t>Add New Store &amp; Approve</t>
+  </si>
+  <si>
+    <t>This test validates the complete administrative workflow for registering and authorizing a new merchant within the food delivery system. The automation navigates to the Add Store module to dynamically create a unique store profile, populating operational data including delivery radius, commission structures, and banking details. Following creation, the script transitions to the Compliance phase, where it filters for the new store in the "Pending Documents" list, automates the upload of regulatory files, and sets document expiry dates. The workflow concludes by triggering the Final Approval and verifying the store’s successful migration to the active Store List, ensuring end-to-end data consistency and functional status transitions.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FileSystem State (Crucial)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
+-&gt; C:\images\kfcbanner.jpg (For Store  Banner Image)
+-&gt; C:\images\kfcstore.jpg (For Store Image)
+-&gt; C:\images\addressproof.png (For Address Proof Document)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
@@ -899,7 +981,8 @@
 85.wait,2000,,
 86.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
 87.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-88.wait,3000,,
+88.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
+89.wait,3000,,
 </t>
   </si>
 </sst>
@@ -1309,16 +1392,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="E2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1385,16 +1468,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1463,13 +1546,13 @@
         <v>12</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1531,10 +1614,10 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1603,10 +1686,10 @@
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1675,10 +1758,10 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1735,22 +1818,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
36th commit: Store Operatiions Test Sheet Started
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C063F592-4BDC-438D-8AE1-76F6F7BACE9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E9E20A-0411-4FC5-B5EB-54062D38253C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="AddBikeDriver" sheetId="4" r:id="rId5"/>
     <sheet name="AddTaxiDriver" sheetId="5" r:id="rId6"/>
     <sheet name="AddStore" sheetId="7" r:id="rId7"/>
+    <sheet name="StoreOperations" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="55">
   <si>
     <t>City Area</t>
   </si>
@@ -984,6 +985,123 @@
 88.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
 89.wait,3000,,
 </t>
+  </si>
+  <si>
+    <t>SA_TS_7</t>
+  </si>
+  <si>
+    <t>Store Operations</t>
+  </si>
+  <si>
+    <t>This test validates the operational readiness of an approved store by managing its digital inventory and verifying financial synchronization. The workflow begins by navigating to the Store Operations module to define product categories and populate the digital menu with diverse items, ensuring attributes such as pricing, descriptions, and tax settings are correctly mapped. Following the catalog setup, the script executes a Wallet Audit to confirm that the merchant's financial dashboard accurately reflects the initial balance and pre-configured commission rules. By successfully linking physical product management with backend financial tracking, the test ensures the store is fully equipped to process live orders and handle automated revenue settlements.</t>
+  </si>
+  <si>
+    <t>TC_CA_07_store_oprerations</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FileSystem State (Crucial)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
+-&gt; C:\images\kfcbanner.jpg (For Store  Banner Image)
+-&gt; C:\images\kfcstore.jpg (For Store Image)
+-&gt; C:\images\addressproof.png (For Address Proof Document)</t>
+    </r>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
+3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
+4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
+5.wait,2000,,
+6.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
+7.Click  Stores,click,,"//button[contains(., 'Stores')]"
+8.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+9.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
+10.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+11.wait,2000,,</t>
   </si>
 </sst>
 </file>
@@ -1846,4 +1964,76 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86A4538F-421E-4B0B-A965-0382A5BEF523}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
39th commit: Store Operations Completed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E9E20A-0411-4FC5-B5EB-54062D38253C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C092330D-6225-4A7D-8970-40F3BD8F6460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -993,10 +993,10 @@
     <t>Store Operations</t>
   </si>
   <si>
-    <t>This test validates the operational readiness of an approved store by managing its digital inventory and verifying financial synchronization. The workflow begins by navigating to the Store Operations module to define product categories and populate the digital menu with diverse items, ensuring attributes such as pricing, descriptions, and tax settings are correctly mapped. Following the catalog setup, the script executes a Wallet Audit to confirm that the merchant's financial dashboard accurately reflects the initial balance and pre-configured commission rules. By successfully linking physical product management with backend financial tracking, the test ensures the store is fully equipped to process live orders and handle automated revenue settlements.</t>
-  </si>
-  <si>
     <t>TC_CA_07_store_oprerations</t>
+  </si>
+  <si>
+    <t>This test validates the end-to-end lifecycle of a delivery store's operational setup, focusing on catalog management, financial provisioning, and logistics readiness. The workflow begins by navigating through the delivery services hierarchy to locate a specific store, where it performs a menu expansion by adding new products with precise attributes including pricing, imagery, and discount logic. Following inventory setup, the script executes a comprehensive financial audit by performing both credit and debit transactions within the store’s wallet to ensure backend accounting synchronization. Finally, the test secures the store's fulfillment capabilities by registering a new private driver, capturing personal and vehicle details alongside document uploads, thereby ensuring the merchant is fully prepared to manage products, finances, and last-mile delivery.</t>
   </si>
   <si>
     <r>
@@ -1085,9 +1085,9 @@
         <scheme val="minor"/>
       </rPr>
       <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
--&gt; C:\images\kfcbanner.jpg (For Store  Banner Image)
--&gt; C:\images\kfcstore.jpg (For Store Image)
--&gt; C:\images\addressproof.png (For Address Proof Document)</t>
+-&gt; C:\images\grillchicken.jpg (For Product Image)
+-&gt; C:\images\bikedriver.jpg (For Private Driver Image)
+-&gt; C:\images\bike.png (For Vehicle Image )</t>
     </r>
   </si>
   <si>
@@ -1101,7 +1101,74 @@
 8.Select Store List,click,,"//div[contains(text(), 'Store List')]"
 9.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
 10.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-11.wait,2000,,</t>
+11.wait,2000,,
+12.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+13.Click Product Icon,click,,"//i[@title='Product View']"
+14.wait,1000,,
+15.Click  Add  Products,click,,"//button[normalize-space()='Add Products']"
+16.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[1]"
+17.Select Grill Chicken,click,,"//li[@role='option'][contains(.,'Grill Chicken')]"
+18.wait,1000,,
+19.Enter Product Name, type, Grill Chicken, "//label[contains(.,'Product Name')]/following-sibling::input"
+20.Enter Product Amount, type, 500, "//label[contains(.,'Product Amount')]/following-sibling::input"
+21.Enter Product Description, type, KFC special grill chicken, "//label[contains(text(),'Product Description')]/following-sibling::textarea"
+22.Upload Product Image, uploadfile, "C:\images\grillchicken.jpg", "//input[@type='file' and @accept='image/*']"
+23.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[2]"
+24.Select Activate,click,,"//li[@role='option'][contains(.,'Activate')]"
+25.Open Discount Type Dropdown,click,,"//label[contains(.,'Discount Type')]/following-sibling::select/option[text()='Discount in Amount']"
+26.Enter Discount Amount, type, 50, "//label[contains(.,'Discount Amount')]/following-sibling::input"
+27.Click Save, click, , "//button[normalize-space()='Save']"
+28.Verify Saved Succesfully, verify, , "//div[@aria-label='Product added successfully']"
+29.wait,3000,,
+30.Verify Store Products,verify,,"//div[contains(text(),'☰ Store Products')]"
+31.Filter Product List,type,Grill Chicken,"//input[@aria-label='Product Name Filter Input']"
+32.wait,2000,,
+33.Click Back, click, , "//button[normalize-space()='Back']"
+34.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+35.wait,2000,,
+36.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+37.Click Wallet Icon,click,,"//i[@title='Wallet']"
+38.wait,2000,,
+39.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
+40.wait,2000,,
+41.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
+42.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+43.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
+44.Click Submit, click, , "//button[normalize-space()='Submit']"
+45.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+46.wait,3000,,
+47.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
+48.wait,2000,,
+49.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
+50.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+51.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
+52.Click Submit, click, , "//button[normalize-space()='Submit']"
+53.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+54.wait,3000,,
+55.Click Back, click, , "//button[normalize-space()='Back']"
+56.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+57.wait,2000,,
+58.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+59.Click Drivers Icon,click,,"//i[@title='Drivers']"
+60.wait,2000,,
+61.Click Add Private Driver, click, , "//button[normalize-space()='Add Private Driver']"
+62.Enter Driver Name, type, kfcdriver_{timestamp} &gt;&gt; kfcdriverName, "//label[contains(., 'Driver Full Name')]/following-sibling::div//input"
+63.Enter Email, type, kfcdriver_{timestamp}@gmail.com, "//label[contains(., 'Email')]/following-sibling::div//input"
+64.Enter Contact Number, type, {randomPhone}, "//label[contains(., 'Contact No')]/following-sibling::div//input"
+65.Upload Profile Image, uploadfile, "C:\images\bikedriver.jpg", "//input[@type='file' and @accept='image/*']"
+66.wait,3000,,
+67. Select Male Gender, click, , "//div[contains(text(), 'Male')]/preceding-sibling::mat-radio-button"
+68.Click Vehicle Type Dropdown,click,,"//label[contains(., 'Vehicle Type')]/following-sibling::p-dropdown"
+69.Select  Scooter Option,click,,"//li[@role='option'][contains(.,'Scooter')]"
+70. Enter Model Year, type, 2013, "//label[span[text()='Model Year']]/following::input[1]"
+71.Enter Vehicle Company, type, honda, "//label[contains(., 'Vehicle Company')]/following-sibling::div//input"
+72. Enter Plate No, type, KL-01-AB-1634, "//label[contains(., 'Plate No')]/following-sibling::div//input"
+73. Enter Model Name, type, activa, "//label[contains(., 'Model Name')]/following-sibling::div//input"
+74. Upload Vehicle Image, uploadfile, "C:\images\bike.jpg", "(//app-image-upload//input[@type='file'])[2]"
+75. Enter Vehicle Color, type, white, "//label[contains(., 'Vehicle Color')]/following::input[1]"
+76. Click Submit, click, , "//button[contains(.,'Submit')]"
+77. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+78. Wait for Toast to hide, wait, 3000,</t>
   </si>
 </sst>
 </file>
@@ -2014,10 +2081,10 @@
         <v>50</v>
       </c>
       <c r="C2" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>54</v>

</xml_diff>

<commit_message>
40th commit: Stores Status Management Test Started
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C092330D-6225-4A7D-8970-40F3BD8F6460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50416155-9BE0-4BA2-9CC0-03CF940C2B80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="AddTaxiDriver" sheetId="5" r:id="rId6"/>
     <sheet name="AddStore" sheetId="7" r:id="rId7"/>
     <sheet name="StoreOperations" sheetId="8" r:id="rId8"/>
+    <sheet name="StoreStatusManagement" sheetId="10" r:id="rId9"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="60">
   <si>
     <t>City Area</t>
   </si>
@@ -1170,6 +1171,79 @@
 77. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
 78. Wait for Toast to hide, wait, 3000,</t>
   </si>
+  <si>
+    <t>SA_TS_8</t>
+  </si>
+  <si>
+    <t>Store Status Mangement</t>
+  </si>
+  <si>
+    <t>TC_CA_08_store_status_management</t>
+  </si>
+  <si>
+    <t>This test validates the complete workflow for registering and authorizing a new merchant within the food delivery system. The automation navigates to the Add Store module to dynamically create a unique store profile verifying it . Rejecting it if doucments are not up to date and also checking the blocking action for already approved stores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
+3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
+4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
+5.wait,2000,,
+6.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
+7.Click  Stores,click,,"//button[contains(., 'Stores')]"
+8.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
+9.Verify Add Store,verify,,"//div[contains(text(),'☰ Add Store')]"
+10.Enter Store Name, type, KFC_{timestamp} &gt;&gt; storeName, "//input[@placeholder='Store Name']"
+11.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
+12.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
+13.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
+14. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
+15.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
+16.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
+17.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
+18.Upload Banner Image, uploadfile, "C:\images\kfcbanner.jpg", "//input[@type='file']"
+19.wait,2000,,
+20.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
+21.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
+22.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
+23.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
+24.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+25..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
+26.wait,2000,,
+27.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
+28.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
+29.wait,1000,,
+30.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
+31.wait,1000,,
+32..Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
+33.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
+34.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
+35.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
+36.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
+37.Enter Contact Person Full Name, type, storeowner_{timestamp} &gt;&gt; storeOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
+38.Enter Email, type, kfc_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
+39.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
+40.Upload Store Image, uploadfile, "C:\images\kfcstore.jpg", "(//input[@type='file'])[2]"
+41.wait,2000,,
+42.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
+43.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
+44.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
+45.Enter Accont Holder Name, type, {storeOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
+46.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
+47.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
+48.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
+49.Enter From Time, type, 100000, "(//label[contains(.,'From Time')]/following-sibling::input)[1]"
+50.Enter To Time, type, 220000, "(//label[contains(.,'To Time')]/following-sibling::input)[1]"
+51.Submit Add Store,click,,"//button[normalize-space()='Submit']"
+52. Verify Success Message,verify,,"//div[@aria-label='Info']"
+53.wait,3000,,
+54.Click  Stores,click,,"//button[contains(., 'Stores')]"
+55.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+56.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
+57.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+58.wait,2000,,
+</t>
+  </si>
 </sst>
 </file>
 
@@ -1226,7 +1300,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1249,6 +1323,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2103,4 +2180,76 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57207608-1AD9-408F-B018-55A141C9A651}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
41th commit: Stores Status Management Test Completed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50416155-9BE0-4BA2-9CC0-03CF940C2B80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AABE84E0-C4CF-47D5-9287-0C2DCC4F87B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1181,10 +1181,7 @@
     <t>TC_CA_08_store_status_management</t>
   </si>
   <si>
-    <t>This test validates the complete workflow for registering and authorizing a new merchant within the food delivery system. The automation navigates to the Add Store module to dynamically create a unique store profile verifying it . Rejecting it if doucments are not up to date and also checking the blocking action for already approved stores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
 2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
 3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
 4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
@@ -1193,7 +1190,7 @@
 7.Click  Stores,click,,"//button[contains(., 'Stores')]"
 8.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
 9.Verify Add Store,verify,,"//div[contains(text(),'☰ Add Store')]"
-10.Enter Store Name, type, KFC_{timestamp} &gt;&gt; storeName, "//input[@placeholder='Store Name']"
+10.Enter Store Name, type, bilal_{timestamp} &gt;&gt; storeName, "//input[@placeholder='Store Name']"
 11.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
 12.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
 13.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
@@ -1242,7 +1239,67 @@
 56.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
 57.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
 58.wait,2000,,
-</t>
+59.Click  Stores,click,,"//button[contains(., 'Stores')]"
+60.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
+61.Verify Add Store,verify,,"//div[contains(text(),'☰ Pending Documents Store')]"
+62.Filter Pending Document Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+63.wait,2000,,
+64.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+65.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
+65.wait,3000,,
+66. Store Required Documents,verify,,"//div[contains(text(),'☰ Documents')]"
+67.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+68.wait,3000,,
+69.Upload Address Proof, uploadfile, "C:\images\addressproof.png", "//input[@type='file']"
+70.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+71.wait,1000,,
+72.Click Submit, click, , "//button[normalize-space()='Submit']"
+73.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+74.wait,2000,,
+75.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+76.wait,2000,,
+77.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+78.wait,3000,,
+79.Click Back, click, , "//button[@class='buttonWidget']"
+80.wait,2000,,
+81.Click  Stores,click,,"//button[contains(., 'Stores')]"
+82.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+83.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
+84.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+85.wait,2000,,
+86.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+87.Click Block Icon,click,,"//i[@title='Blocked']"
+88.wait,2000,,
+89.Click Block  Yes,click,,"//button[normalize-space()='Yes']"
+90.Click  Stores,click,,"//button[contains(., 'Stores')]"
+91.Select Blocked Store,click,,"//div[normalize-space()='Blocked Stores']"
+92.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+93.wait,2000,,
+94.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+95.Click unBlock Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
+96.wait,3000,,
+97.Click  Stores,click,,"//button[contains(., 'Stores')]"
+98.Select Rejected Store,click,,"//div[normalize-space()='Rejected Stores']"
+99.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+100.wait,2000,,
+101.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+102.Click Approve Icon,click,,"//i[@title='Approve']"
+103.Click  Stores,click,,"//button[contains(., 'Stores')]"
+104.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+105.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+106.wait,2000,,
+107.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+108.Click Doc Icon,click,,"//i[@title='Document']"
+109.wait,1000,,
+110.Click UnApprove Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
+111.wait,1000,,
+112.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+113.Rejection Reason,type,document insufficent,"//textarea[@id='swal2-textarea']"
+114.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+115.wait,3000,,</t>
+  </si>
+  <si>
+    <t>This test validates the complete lifecycle of a store within a delivery services platform, beginning with the creation of a new store (using dynamic timestamps for uniqueness) and the configuration of its operational settings, bank details, and timing. It then navigates through various administrative states, including uploading and verifying compliance documents, moving the store from a pending status to approved, and then testing the blocking/unblocking functionality. Finally, the script validates the rejection workflow by moving a store to the rejected list with a specific reason, ensuring that status transitions and data filtering across the "Store List," "Pending," and "Blocked" modules are functioning as expected.</t>
   </si>
 </sst>
 </file>
@@ -2233,10 +2290,10 @@
         <v>57</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>59</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>47</v>

</xml_diff>

<commit_message>
44th commit: Image issue fixed added to project stucture
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AABE84E0-C4CF-47D5-9287-0C2DCC4F87B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9875E29-0092-4CD3-B95A-F64F7240A0D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -411,220 +411,40 @@
 45.wait,2000,,</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>FileSystem State (Crucial)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
--&gt; C:\images\autodriver.jpg (For Driver Profile)
--&gt; C:\images\vehicle.jpg (For Vehicle Image)
--&gt; C:\images\license.jpg (For Driving License Document)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>FileSystem State (Crucial):</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
--&gt; C:\images\bikedriver.jpg (For Driver Profile)
--&gt; C:\images\bike.jpg (For Vehicle Image)
--&gt; C:\images\license.jpg (For Driving License Document)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>FileSystem State (Crucial)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
--&gt; C:\images\taxidriver.jpg (For Driver Profile)
--&gt; C:\images\taxi.jpg (For Vehicle Image)
--&gt; C:\images\license.jpg (For Driving License Document)</t>
-    </r>
-  </si>
-  <si>
     <t>SA_TS_6</t>
   </si>
   <si>
     <t>TC_CA_06_add_store</t>
+  </si>
+  <si>
+    <t>Add New Store &amp; Approve</t>
+  </si>
+  <si>
+    <t>This test validates the complete administrative workflow for registering and authorizing a new merchant within the food delivery system. The automation navigates to the Add Store module to dynamically create a unique store profile, populating operational data including delivery radius, commission structures, and banking details. Following creation, the script transitions to the Compliance phase, where it filters for the new store in the "Pending Documents" list, automates the upload of regulatory files, and sets document expiry dates. The workflow concludes by triggering the Final Approval and verifying the store’s successful migration to the active Store List, ensuring end-to-end data consistency and functional status transitions.</t>
+  </si>
+  <si>
+    <t>SA_TS_7</t>
+  </si>
+  <si>
+    <t>Store Operations</t>
+  </si>
+  <si>
+    <t>TC_CA_07_store_oprerations</t>
+  </si>
+  <si>
+    <t>This test validates the end-to-end lifecycle of a delivery store's operational setup, focusing on catalog management, financial provisioning, and logistics readiness. The workflow begins by navigating through the delivery services hierarchy to locate a specific store, where it performs a menu expansion by adding new products with precise attributes including pricing, imagery, and discount logic. Following inventory setup, the script executes a comprehensive financial audit by performing both credit and debit transactions within the store’s wallet to ensure backend accounting synchronization. Finally, the test secures the store's fulfillment capabilities by registering a new private driver, capturing personal and vehicle details alongside document uploads, thereby ensuring the merchant is fully prepared to manage products, finances, and last-mile delivery.</t>
+  </si>
+  <si>
+    <t>SA_TS_8</t>
+  </si>
+  <si>
+    <t>Store Status Mangement</t>
+  </si>
+  <si>
+    <t>TC_CA_08_store_status_management</t>
+  </si>
+  <si>
+    <t>This test validates the complete lifecycle of a store within a delivery services platform, beginning with the creation of a new store (using dynamic timestamps for uniqueness) and the configuration of its operational settings, bank details, and timing. It then navigates through various administrative states, including uploading and verifying compliance documents, moving the store from a pending status to approved, and then testing the blocking/unblocking functionality. Finally, the script validates the rejection workflow by moving a store to the rejected list with a specific reason, ensuring that status transitions and data filtering across the "Store List," "Pending," and "Blocked" modules are functioning as expected.</t>
   </si>
   <si>
     <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
@@ -638,7 +458,7 @@
 10. Enter Email, type, autodriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
 11. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
 12. wait, 1000,,
-13. Upload Profile Image, uploadfile, "C:\images\autodriver.jpg", "//input[@type='file']"
+13. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
 14. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
 15.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
 16.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
@@ -646,7 +466,7 @@
 18.Enter Vehicle Company, type, bajaj, "//label[contains(.,'Vehicle Company')]/following::input[1]"
 19. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
 20. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-21. Upload Vehicle Image, uploadfile, "C:\images\vehicle.jpg", "(//input[@type='file'])[2]"
+21. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
 22. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
 23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
 24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
@@ -668,7 +488,7 @@
 40. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
 41.Add Driving License,click,,"//i[@title='Edit']"
 42.wait,3000,,
-43.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
+43.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
 44.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
 45.wait,1000,,
 46.Click Submit, click, , "//button[normalize-space()='Submit']"
@@ -702,7 +522,7 @@
 10. Enter Email, type, bikedriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
 11. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
 12. wait, 1000,,
-13. Upload Profile Image, uploadfile, "C:\images\bikedriver.jpg", "//input[@type='file']"
+13. Upload Profile Image, uploadfile, "src/main/resources/test-data/bikedriver.jpg", "//input[@type='file']"
 14. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
 15.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
 16.Select  Scooter Option,click,,"//li[@role='option']//span[text()='Scooter']"
@@ -710,7 +530,7 @@
 18.Enter Vehicle Company, type, honda, "//label[contains(.,'Vehicle Company')]/following::input[1]"
 19. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
 20. Enter Model Name, type, activa, "//label[contains(.,'Model Name')]/following::input[1]"
-21. Upload Vehicle Image, uploadfile, "C:\images\bike.jpg", "(//input[@type='file'])[2]"
+21. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/bike.jpg", "(//input[@type='file'])[2]"
 22. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
 23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
 24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
@@ -732,7 +552,7 @@
 40. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
 41.Add Driving License,click,,"//i[@title='Edit']"
 42.wait,3000,,
-43.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
+43.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
 44.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
 45.wait,1000,,
 46.Click Submit, click, , "//button[normalize-space()='Submit']"
@@ -766,7 +586,7 @@
 10. Enter Email, type, taxidriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
 11. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
 12. wait, 1000,,
-13. Upload Profile Image, uploadfile, "C:\images\taxidriver.jpg", "//input[@type='file']"
+13. Upload Profile Image, uploadfile, "src/main/resources/test-data/taxidriver.jpg", "//input[@type='file']"
 14. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
 15.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
 16.Select  Suv Option,click,,"//li[@role='option']//span[text()='SUV']"
@@ -774,7 +594,7 @@
 18.Enter Vehicle Company, type, toyota, "//label[contains(.,'Vehicle Company')]/following::input[1]"
 19. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
 20. Enter Model Name, type, etios, "//label[contains(.,'Model Name')]/following::input[1]"
-21. Upload Vehicle Image, uploadfile, "C:\images\taxi.jpg", "(//input[@type='file'])[2]"
+21. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/taxi.jpg", "(//input[@type='file'])[2]"
 22. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
 23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
 24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
@@ -796,7 +616,7 @@
 40. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
 41.Add Driving License,click,,"//i[@title='Edit']"
 42.wait,3000,,
-43.Upload Driving Iicense, uploadfile, "C:\images\license.jpg", "//input[@type='file']"
+43.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
 44.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
 45.wait,1000,,
 46.Click Submit, click, , "//button[normalize-space()='Submit']"
@@ -819,82 +639,6 @@
 </t>
   </si>
   <si>
-    <t>Add New Store &amp; Approve</t>
-  </si>
-  <si>
-    <t>This test validates the complete administrative workflow for registering and authorizing a new merchant within the food delivery system. The automation navigates to the Add Store module to dynamically create a unique store profile, populating operational data including delivery radius, commission structures, and banking details. Following creation, the script transitions to the Compliance phase, where it filters for the new store in the "Pending Documents" list, automates the upload of regulatory files, and sets document expiry dates. The workflow concludes by triggering the Final Approval and verifying the store’s successful migration to the active Store List, ensuring end-to-end data consistency and functional status transitions.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>FileSystem State (Crucial)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
--&gt; C:\images\kfcbanner.jpg (For Store  Banner Image)
--&gt; C:\images\kfcstore.jpg (For Store Image)
--&gt; C:\images\addressproof.png (For Address Proof Document)</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
 2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
 3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
@@ -912,7 +656,7 @@
 15.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
 16.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
 17.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
-18.Upload Banner Image, uploadfile, "C:\images\kfcbanner.jpg", "//input[@type='file']"
+18.Upload Banner Image, uploadfile, "src/main/resources/test-data/kfcbanner.jpg", "//input[@type='file']"
 19.wait,2000,,
 20.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
 21.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
@@ -934,7 +678,7 @@
 37.Enter Contact Person Full Name, type, storeowner_{timestamp} &gt;&gt; storeOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
 38.Enter Email, type, kfc_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
 39.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
-40.Upload Store Image, uploadfile, "C:\images\kfcstore.jpg", "(//input[@type='file'])[2]"
+40.Upload Store Image, uploadfile, "src/main/resources/test-data/kfcstore.jpg", "(//input[@type='file'])[2]"
 41.wait,2000,,
 42.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
 43.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
@@ -964,7 +708,7 @@
 66. Store Required Documents,verify,,"//div[contains(text(),'☰ Documents')]"
 67.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
 68.wait,3000,,
-69.Upload Address Proof, uploadfile, "C:\images\addressproof.png", "//input[@type='file']"
+69.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
 70.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
 71.wait,1000,,
 72.Click Submit, click, , "//button[normalize-space()='Submit']"
@@ -988,110 +732,6 @@
 </t>
   </si>
   <si>
-    <t>SA_TS_7</t>
-  </si>
-  <si>
-    <t>Store Operations</t>
-  </si>
-  <si>
-    <t>TC_CA_07_store_oprerations</t>
-  </si>
-  <si>
-    <t>This test validates the end-to-end lifecycle of a delivery store's operational setup, focusing on catalog management, financial provisioning, and logistics readiness. The workflow begins by navigating through the delivery services hierarchy to locate a specific store, where it performs a menu expansion by adding new products with precise attributes including pricing, imagery, and discount logic. Following inventory setup, the script executes a comprehensive financial audit by performing both credit and debit transactions within the store’s wallet to ensure backend accounting synchronization. Finally, the test secures the store's fulfillment capabilities by registering a new private driver, capturing personal and vehicle details alongside document uploads, thereby ensuring the merchant is fully prepared to manage products, finances, and last-mile delivery.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Authentication State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>FileSystem State (Crucial)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: The following local image files must exist at the specified paths on the machine running the automation. If these files are missing, the uploadfile action will fail:
--&gt; C:\images\grillchicken.jpg (For Product Image)
--&gt; C:\images\bikedriver.jpg (For Private Driver Image)
--&gt; C:\images\bike.png (For Vehicle Image )</t>
-    </r>
-  </si>
-  <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
 2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
 3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
@@ -1113,7 +753,7 @@
 19.Enter Product Name, type, Grill Chicken, "//label[contains(.,'Product Name')]/following-sibling::input"
 20.Enter Product Amount, type, 500, "//label[contains(.,'Product Amount')]/following-sibling::input"
 21.Enter Product Description, type, KFC special grill chicken, "//label[contains(text(),'Product Description')]/following-sibling::textarea"
-22.Upload Product Image, uploadfile, "C:\images\grillchicken.jpg", "//input[@type='file' and @accept='image/*']"
+22.Upload Product Image, uploadfile, "src/main/resources/test-data/grillchicken.jpg", "//input[@type='file' and @accept='image/*']"
 23.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[2]"
 24.Select Activate,click,,"//li[@role='option'][contains(.,'Activate')]"
 25.Open Discount Type Dropdown,click,,"//label[contains(.,'Discount Type')]/following-sibling::select/option[text()='Discount in Amount']"
@@ -1156,7 +796,7 @@
 62.Enter Driver Name, type, kfcdriver_{timestamp} &gt;&gt; kfcdriverName, "//label[contains(., 'Driver Full Name')]/following-sibling::div//input"
 63.Enter Email, type, kfcdriver_{timestamp}@gmail.com, "//label[contains(., 'Email')]/following-sibling::div//input"
 64.Enter Contact Number, type, {randomPhone}, "//label[contains(., 'Contact No')]/following-sibling::div//input"
-65.Upload Profile Image, uploadfile, "C:\images\bikedriver.jpg", "//input[@type='file' and @accept='image/*']"
+65.Upload Profile Image, uploadfile, "src/main/resources/test-data/bikedriver.jpg", "//input[@type='file' and @accept='image/*']"
 66.wait,3000,,
 67. Select Male Gender, click, , "//div[contains(text(), 'Male')]/preceding-sibling::mat-radio-button"
 68.Click Vehicle Type Dropdown,click,,"//label[contains(., 'Vehicle Type')]/following-sibling::p-dropdown"
@@ -1165,20 +805,11 @@
 71.Enter Vehicle Company, type, honda, "//label[contains(., 'Vehicle Company')]/following-sibling::div//input"
 72. Enter Plate No, type, KL-01-AB-1634, "//label[contains(., 'Plate No')]/following-sibling::div//input"
 73. Enter Model Name, type, activa, "//label[contains(., 'Model Name')]/following-sibling::div//input"
-74. Upload Vehicle Image, uploadfile, "C:\images\bike.jpg", "(//app-image-upload//input[@type='file'])[2]"
+74. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/bike.jpg", "(//app-image-upload//input[@type='file'])[2]"
 75. Enter Vehicle Color, type, white, "//label[contains(., 'Vehicle Color')]/following::input[1]"
 76. Click Submit, click, , "//button[contains(.,'Submit')]"
 77. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
 78. Wait for Toast to hide, wait, 3000,</t>
-  </si>
-  <si>
-    <t>SA_TS_8</t>
-  </si>
-  <si>
-    <t>Store Status Mangement</t>
-  </si>
-  <si>
-    <t>TC_CA_08_store_status_management</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
@@ -1198,7 +829,7 @@
 15.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
 16.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
 17.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
-18.Upload Banner Image, uploadfile, "C:\images\kfcbanner.jpg", "//input[@type='file']"
+18.Upload Banner Image, uploadfile, "src/main/resources/test-data/kfcbanner.jpg", "//input[@type='file']"
 19.wait,2000,,
 20.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
 21.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
@@ -1220,7 +851,7 @@
 37.Enter Contact Person Full Name, type, storeowner_{timestamp} &gt;&gt; storeOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
 38.Enter Email, type, kfc_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
 39.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
-40.Upload Store Image, uploadfile, "C:\images\kfcstore.jpg", "(//input[@type='file'])[2]"
+40.Upload Store Image, uploadfile, "src/main/resources/test-data/kfcstore.jpg", "(//input[@type='file'])[2]"
 41.wait,2000,,
 42.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
 43.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
@@ -1250,7 +881,7 @@
 66. Store Required Documents,verify,,"//div[contains(text(),'☰ Documents')]"
 67.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
 68.wait,3000,,
-69.Upload Address Proof, uploadfile, "C:\images\addressproof.png", "//input[@type='file']"
+69.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
 70.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
 71.wait,1000,,
 72.Click Submit, click, , "//button[normalize-space()='Submit']"
@@ -1299,7 +930,256 @@
 115.wait,3000,,</t>
   </si>
   <si>
-    <t>This test validates the complete lifecycle of a store within a delivery services platform, beginning with the creation of a new store (using dynamic timestamps for uniqueness) and the configuration of its operational settings, bank details, and timing. It then navigates through various administrative states, including uploading and verifying compliance documents, moving the store from a pending status to approved, and then testing the blocking/unblocking functionality. Finally, the script validates the rejection workflow by moving a store to the rejected list with a specific reason, ensuring that status transitions and data filtering across the "Store List," "Pending," and "Blocked" modules are functioning as expected.</t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1933,10 +1813,10 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2005,10 +1885,10 @@
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2077,10 +1957,10 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>39</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2137,22 +2017,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>46</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2209,22 +2089,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2281,22 +2161,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
45th commit: Add Provider Test Started
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9875E29-0092-4CD3-B95A-F64F7240A0D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D024C09-8E9F-4A08-8C92-9CD2B83CDF4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="AddStore" sheetId="7" r:id="rId7"/>
     <sheet name="StoreOperations" sheetId="8" r:id="rId8"/>
     <sheet name="StoreStatusManagement" sheetId="10" r:id="rId9"/>
+    <sheet name="AddProvider" sheetId="11" r:id="rId10"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="66">
   <si>
     <t>City Area</t>
   </si>
@@ -939,6 +940,74 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
+      <t xml:space="preserve">Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>Authentication State</t>
     </r>
     <r>
@@ -985,17 +1054,17 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Authentication State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+      <t>Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
 </t>
     </r>
     <r>
@@ -1007,39 +1076,17 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
 </t>
     </r>
   </si>
@@ -1075,6 +1122,64 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>SA_TS_9</t>
+  </si>
+  <si>
+    <t>Add New Provider &amp; Approve</t>
+  </si>
+  <si>
+    <t>TC_CA_09_add_provider</t>
+  </si>
+  <si>
+    <t>This test validates the complete administrative workflow for registering and authorizing a new provider within the Plumbers. The automation navigates to the Add Providers module to dynamically create a unique pumbler profile, populating operational data including provider service radius, service time, address and banking details. Following creation, the script transitions to the Compliance phase, where it filters for the new pumbler in the "Pending Documents" list, automates the upload of regulatory files, and sets document expiry dates. The workflow concludes by triggering the Final Approval and verifying the pumbler successful migration to the active provider List, ensuring end-to-end data consistency and functional status transitions.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>Navigation State:</t>
     </r>
     <r>
@@ -1099,17 +1204,17 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Store and Document Management.
 </t>
     </r>
     <r>
@@ -1121,65 +1226,32 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
 </t>
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
+3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ ON-DEMAND SERVICES')]"
+4.Click Home Icon Plumbers,click,,"//div[@role='row'][.//span[text()='Plumbers']]//i[@title='Home']"
+5.wait,2000,,
+6.Verify Plumbers Summary,verify,,"//div[contains(text(),'☰ Plumbers Summary')]"
+7.Click  Providers,click,,"//button[contains(., 'Providers')]"
+8.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
+9.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
+10.Enter Provider Full Name, type, plumber_{timestamp} &gt;&gt; plumberName, "//input[@placeholder='Provider Full Name']"
 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
   </si>
 </sst>
 </file>
@@ -1618,6 +1690,78 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F63FB6C5-854C-4D7D-9CEB-846B4D7D2F52}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="302.39999999999998" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H3"/>
@@ -1816,7 +1960,7 @@
         <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1888,7 +2032,7 @@
         <v>50</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1960,7 +2104,7 @@
         <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2032,7 +2176,7 @@
         <v>52</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2104,7 +2248,7 @@
         <v>53</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2176,7 +2320,7 @@
         <v>54</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
46th commit: Step Parser Updated For Random Alphabat Generation
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D024C09-8E9F-4A08-8C92-9CD2B83CDF4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E9CEDF3-0328-47CB-9FD2-DB2177FD8E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -1250,7 +1250,13 @@
 7.Click  Providers,click,,"//button[contains(., 'Providers')]"
 8.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
 9.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
-10.Enter Provider Full Name, type, plumber_{timestamp} &gt;&gt; plumberName, "//input[@placeholder='Provider Full Name']"
+10.Enter Provider Full Name, type, Plumber{randomAlpha}&gt;&gt; plumberName, "//input[@placeholder='Provider Full Name']"
+11.Upload Plumber Image, uploadfile, "src/main/resources/test-data/plumber.jpg", "//input[@type='file']"
+12.Wait For Image To Load,3000,,
+13.Enter Email, type, Plumber_{timestamp}@gmail.com&gt;&gt;plumberEmail, "//input[@placeholder='Unique Email']"
+14.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
+15.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
+16.wait,2000,,
 </t>
   </si>
 </sst>
@@ -1730,7 +1736,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>59</v>
       </c>

</xml_diff>

<commit_message>
47th commit: Created Plumber Provider in Add Provider Test Suite
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E9CEDF3-0328-47CB-9FD2-DB2177FD8E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31D6680E-D83B-4AB0-9398-3C9BF991F0ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -733,6 +733,361 @@
 </t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>SA_TS_9</t>
+  </si>
+  <si>
+    <t>Add New Provider &amp; Approve</t>
+  </si>
+  <si>
+    <t>TC_CA_09_add_provider</t>
+  </si>
+  <si>
+    <t>This test validates the complete administrative workflow for registering and authorizing a new provider within the Plumbers. The automation navigates to the Add Providers module to dynamically create a unique pumbler profile, populating operational data including provider service radius, service time, address and banking details. Following creation, the script transitions to the Compliance phase, where it filters for the new pumbler in the "Pending Documents" list, automates the upload of regulatory files, and sets document expiry dates. The workflow concludes by triggering the Final Approval and verifying the pumbler successful migration to the active provider List, ensuring end-to-end data consistency and functional status transitions.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Store and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
+3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ ON-DEMAND SERVICES')]"
+4.Click Home Icon Plumbers,click,,"//div[@role='row'][.//span[text()='Plumbers']]//i[@title='Home']"
+5.wait,2000,,
+6.Verify Plumbers Summary,verify,,"//div[contains(text(),'☰ Plumbers Summary')]"
+7.Click  Providers,click,,"//button[contains(., 'Providers')]"
+8.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
+9.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
+10.Enter Provider Full Name, type, Plumber{randomAlpha}&gt;&gt; plumberName, "//input[@placeholder='Provider Full Name']"
+11.Upload Plumber Image, uploadfile, "src/main/resources/test-data/plumber.jpg", "//input[@type='file']"
+12.Wait For Image To Load,3000,,
+13.Enter Email, type, Plumber_{timestamp}@gmail.com&gt;&gt;plumberEmail, "//input[@placeholder='Unique Email']"
+14.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
+15.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
+16.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
+17.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
+18.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
+19..Enter Provider Address, type, plumber chennai, "//input[@placeholder='Enter provider Address']"
+20.wait,2000,,
+21.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
+22.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
+23.wait,2000,,
+24.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
+25.wait,1000,,
+26.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
+27.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
+27.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
+28.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
+29.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
+30.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
+31.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
+32.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
+33.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
+34.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
+35.Enter Accont Holder Name, type, {plumberName}, "//input[@placeholder='Account Holder Name']"
+36.Enter Payment Email Address, type, {plumberEmail}, "//input[@placeholder='Email Address for Payment Notification']"
+37.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
+38.Click Save, click, , "//button[@type='submit']"
+39.Verify Sucess, verify, , "//div[@aria-label='Info']"
+40.wait,3000,,
+41.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+42.wait,2000,,</t>
+  </si>
+  <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
 2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
 3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
@@ -810,7 +1165,11 @@
 75. Enter Vehicle Color, type, white, "//label[contains(., 'Vehicle Color')]/following::input[1]"
 76. Click Submit, click, , "//button[contains(.,'Submit')]"
 77. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-78. Wait for Toast to hide, wait, 3000,</t>
+78. Wait for Toast to hide, wait, 3000,
+79.Filter Driver List,type,{kfcdriverName},"//input[@aria-label='Driver Name Filter Input']"
+80.wait,2000,,
+81.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
+82.wait,1000,,</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
@@ -914,7 +1273,7 @@
 98.Select Rejected Store,click,,"//div[normalize-space()='Rejected Stores']"
 99.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
 100.wait,2000,,
-101.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+101.Scroll Grid, tab, 7, "//input[@aria-label='Store Name Filter Input']"
 102.Click Approve Icon,click,,"//i[@title='Approve']"
 103.Click  Stores,click,,"//button[contains(., 'Stores')]"
 104.Select Store List,click,,"//div[contains(text(), 'Store List')]"
@@ -929,335 +1288,6 @@
 113.Rejection Reason,type,document insufficent,"//textarea[@id='swal2-textarea']"
 114.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
 115.wait,3000,,</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Authentication State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <t>SA_TS_9</t>
-  </si>
-  <si>
-    <t>Add New Provider &amp; Approve</t>
-  </si>
-  <si>
-    <t>TC_CA_09_add_provider</t>
-  </si>
-  <si>
-    <t>This test validates the complete administrative workflow for registering and authorizing a new provider within the Plumbers. The automation navigates to the Add Providers module to dynamically create a unique pumbler profile, populating operational data including provider service radius, service time, address and banking details. Following creation, the script transitions to the Compliance phase, where it filters for the new pumbler in the "Pending Documents" list, automates the upload of regulatory files, and sets document expiry dates. The workflow concludes by triggering the Final Approval and verifying the pumbler successful migration to the active provider List, ensuring end-to-end data consistency and functional status transitions.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Store and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ ON-DEMAND SERVICES')]"
-4.Click Home Icon Plumbers,click,,"//div[@role='row'][.//span[text()='Plumbers']]//i[@title='Home']"
-5.wait,2000,,
-6.Verify Plumbers Summary,verify,,"//div[contains(text(),'☰ Plumbers Summary')]"
-7.Click  Providers,click,,"//button[contains(., 'Providers')]"
-8.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
-9.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
-10.Enter Provider Full Name, type, Plumber{randomAlpha}&gt;&gt; plumberName, "//input[@placeholder='Provider Full Name']"
-11.Upload Plumber Image, uploadfile, "src/main/resources/test-data/plumber.jpg", "//input[@type='file']"
-12.Wait For Image To Load,3000,,
-13.Enter Email, type, Plumber_{timestamp}@gmail.com&gt;&gt;plumberEmail, "//input[@placeholder='Unique Email']"
-14.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
-15.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
-16.wait,2000,,
-</t>
   </si>
 </sst>
 </file>
@@ -1736,24 +1766,24 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="E2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1966,7 +1996,7 @@
         <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2038,7 +2068,7 @@
         <v>50</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2110,7 +2140,7 @@
         <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2182,7 +2212,7 @@
         <v>52</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2251,10 +2281,10 @@
         <v>44</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2323,10 +2353,10 @@
         <v>48</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
49th commit: Add Provider Test Suite Completed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31D6680E-D83B-4AB0-9398-3C9BF991F0ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23FAD1B6-8ED8-4773-9F31-38EF340BB63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1041,51 +1041,6 @@
       <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
 </t>
     </r>
-  </si>
-  <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ ON-DEMAND SERVICES')]"
-4.Click Home Icon Plumbers,click,,"//div[@role='row'][.//span[text()='Plumbers']]//i[@title='Home']"
-5.wait,2000,,
-6.Verify Plumbers Summary,verify,,"//div[contains(text(),'☰ Plumbers Summary')]"
-7.Click  Providers,click,,"//button[contains(., 'Providers')]"
-8.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
-9.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
-10.Enter Provider Full Name, type, Plumber{randomAlpha}&gt;&gt; plumberName, "//input[@placeholder='Provider Full Name']"
-11.Upload Plumber Image, uploadfile, "src/main/resources/test-data/plumber.jpg", "//input[@type='file']"
-12.Wait For Image To Load,3000,,
-13.Enter Email, type, Plumber_{timestamp}@gmail.com&gt;&gt;plumberEmail, "//input[@placeholder='Unique Email']"
-14.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
-15.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
-16.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
-17.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
-18.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
-19..Enter Provider Address, type, plumber chennai, "//input[@placeholder='Enter provider Address']"
-20.wait,2000,,
-21.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
-22.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
-23.wait,2000,,
-24.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
-25.wait,1000,,
-26.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
-27.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
-27.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
-28.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
-29.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
-30.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
-31.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
-32.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
-33.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
-34.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
-35.Enter Accont Holder Name, type, {plumberName}, "//input[@placeholder='Account Holder Name']"
-36.Enter Payment Email Address, type, {plumberEmail}, "//input[@placeholder='Email Address for Payment Notification']"
-37.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
-38.Click Save, click, , "//button[@type='submit']"
-39.Verify Sucess, verify, , "//div[@aria-label='Info']"
-40.wait,3000,,
-41.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-42.wait,2000,,</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
@@ -1288,6 +1243,86 @@
 113.Rejection Reason,type,document insufficent,"//textarea[@id='swal2-textarea']"
 114.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
 115.wait,3000,,</t>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
+3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ ON-DEMAND SERVICES')]"
+4.Click Home Icon Plumbers,click,,"//div[@role='row'][.//span[text()='Plumbers']]//i[@title='Home']"
+5.wait,2000,,
+6.Verify Plumbers Summary,verify,,"//div[contains(text(),'☰ Plumbers Summary')]"
+7.Click  Providers,click,,"//button[contains(., 'Providers')]"
+8.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
+9.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
+10.Enter Provider Full Name, type, Plumber{randomAlpha}&gt;&gt; plumberName, "//input[@placeholder='Provider Full Name']"
+11.Upload Plumber Image, uploadfile, "src/main/resources/test-data/plumber.jpg", "//input[@type='file']"
+12.Wait For Image To Load,3000,,
+13.Enter Email, type, Plumber_{timestamp}@gmail.com&gt;&gt;plumberEmail, "//input[@placeholder='Unique Email']"
+14.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
+15.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
+16.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
+17.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
+18.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
+19..Enter Provider Address, type, plumber chennai, "//input[@placeholder='Enter provider Address']"
+20.wait,2000,,
+21.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
+22.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
+23.wait,2000,,
+24.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
+25.wait,1000,,
+26.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
+27.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
+28.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
+29.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
+30.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
+31.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
+32.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
+33.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
+34.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
+35.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
+36.Enter Accont Holder Name, type, {plumberName}, "//input[@placeholder='Account Holder Name']"
+37.Enter Payment Email Address, type, {plumberEmail}, "//input[@placeholder='Email Address for Payment Notification']"
+38.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
+39.Click Save, click, , "//button[@type='submit']"
+40.Verify Sucess, verify, , "//div[@aria-label='Info']"
+41.wait,3000,,
+42.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+43.wait,2000,,
+44.Click  Providers,click,,"//button[contains(., 'Providers')]"
+45.Select Pending Document Providers,click,,"//div[normalize-space()='Pending Document Providers']"
+46.wait,2000,,
+47.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+48.wait,2000,,
+49.Click Document Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+50.wait,2000,,
+51. Provider Required Documents,verify,,"//div[contains(text(),'☰ Documents')]"
+52.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
+53.wait,2000,,
+54.Add Address Proof,click,,"(//i[contains(@class, 'Edit')])[1]"
+55.wait,3000,,
+54.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
+55.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+56.wait,1000,,
+57.Click Submit, click, , "//button[normalize-space()='Submit']"
+58.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+59.wait,2000,,
+60.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
+61.wait,2000,,
+62.Click Approve Store,click,,"//div[@row-index='0']//i[contains(@class, 'bi-hand-thumbs-up-fill')]"
+63.wait,2000,,
+64.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+65.wait,3000,,
+66.Click Back, click, , "//button[@class='buttonWidget']"
+67.wait,2000,,
+68.Click  Providers,click,,"//button[contains(., 'Providers')]"
+69.Select Provider List,click,,"//div[normalize-space()='Provider List']"
+70.Verify Approved Provider,verify,,"//div[normalize-space()='☰ Approved Plumbers Service Providers']"
+71.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+72.wait,2000,,
+73.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+74.wait,2000,,
+75.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
+76.wait,2000,,</t>
   </si>
 </sst>
 </file>
@@ -1780,7 +1815,7 @@
         <v>60</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>61</v>
@@ -2281,7 +2316,7 @@
         <v>44</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>53</v>
@@ -2353,7 +2388,7 @@
         <v>48</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>62</v>

</xml_diff>

<commit_message>
50th commit: Test Sheets OPtimaized To Increase Test Speed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23FAD1B6-8ED8-4773-9F31-38EF340BB63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30DBC129-B7F6-4D3B-A122-E12094FF71DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -365,7 +365,350 @@
     </r>
   </si>
   <si>
-    <t>1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+    <t>SA_TS_6</t>
+  </si>
+  <si>
+    <t>TC_CA_06_add_store</t>
+  </si>
+  <si>
+    <t>Add New Store &amp; Approve</t>
+  </si>
+  <si>
+    <t>This test validates the complete administrative workflow for registering and authorizing a new merchant within the food delivery system. The automation navigates to the Add Store module to dynamically create a unique store profile, populating operational data including delivery radius, commission structures, and banking details. Following creation, the script transitions to the Compliance phase, where it filters for the new store in the "Pending Documents" list, automates the upload of regulatory files, and sets document expiry dates. The workflow concludes by triggering the Final Approval and verifying the store’s successful migration to the active Store List, ensuring end-to-end data consistency and functional status transitions.</t>
+  </si>
+  <si>
+    <t>SA_TS_7</t>
+  </si>
+  <si>
+    <t>Store Operations</t>
+  </si>
+  <si>
+    <t>TC_CA_07_store_oprerations</t>
+  </si>
+  <si>
+    <t>This test validates the end-to-end lifecycle of a delivery store's operational setup, focusing on catalog management, financial provisioning, and logistics readiness. The workflow begins by navigating through the delivery services hierarchy to locate a specific store, where it performs a menu expansion by adding new products with precise attributes including pricing, imagery, and discount logic. Following inventory setup, the script executes a comprehensive financial audit by performing both credit and debit transactions within the store’s wallet to ensure backend accounting synchronization. Finally, the test secures the store's fulfillment capabilities by registering a new private driver, capturing personal and vehicle details alongside document uploads, thereby ensuring the merchant is fully prepared to manage products, finances, and last-mile delivery.</t>
+  </si>
+  <si>
+    <t>SA_TS_8</t>
+  </si>
+  <si>
+    <t>Store Status Mangement</t>
+  </si>
+  <si>
+    <t>TC_CA_08_store_status_management</t>
+  </si>
+  <si>
+    <t>This test validates the complete lifecycle of a store within a delivery services platform, beginning with the creation of a new store (using dynamic timestamps for uniqueness) and the configuration of its operational settings, bank details, and timing. It then navigates through various administrative states, including uploading and verifying compliance documents, moving the store from a pending status to approved, and then testing the blocking/unblocking functionality. Finally, the script validates the rejection workflow by moving a store to the rejected list with a specific reason, ensuring that status transitions and data filtering across the "Store List," "Pending," and "Blocked" modules are functioning as expected.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>SA_TS_9</t>
+  </si>
+  <si>
+    <t>Add New Provider &amp; Approve</t>
+  </si>
+  <si>
+    <t>TC_CA_09_add_provider</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Store and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
 2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
 3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
 4. Verify City Admin List,verify,,"//div[contains(text(),'☰ City Admin List')]"
@@ -407,108 +750,206 @@
 40.Click on the "Website Settings" → "FAQs" checkbox. "(//h3[contains(.,'Website Settings')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
 41.Click on the "Add City Admin" button. "//button[@type='submit']"
 42. Verify Success Message,verify,,"//div[@aria-label='Info']"
-43.wait,3000,,
-44.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
-45.wait,2000,,</t>
-  </si>
-  <si>
-    <t>SA_TS_6</t>
-  </si>
-  <si>
-    <t>TC_CA_06_add_store</t>
-  </si>
-  <si>
-    <t>Add New Store &amp; Approve</t>
-  </si>
-  <si>
-    <t>This test validates the complete administrative workflow for registering and authorizing a new merchant within the food delivery system. The automation navigates to the Add Store module to dynamically create a unique store profile, populating operational data including delivery radius, commission structures, and banking details. Following creation, the script transitions to the Compliance phase, where it filters for the new store in the "Pending Documents" list, automates the upload of regulatory files, and sets document expiry dates. The workflow concludes by triggering the Final Approval and verifying the store’s successful migration to the active Store List, ensuring end-to-end data consistency and functional status transitions.</t>
-  </si>
-  <si>
-    <t>SA_TS_7</t>
-  </si>
-  <si>
-    <t>Store Operations</t>
-  </si>
-  <si>
-    <t>TC_CA_07_store_oprerations</t>
-  </si>
-  <si>
-    <t>This test validates the end-to-end lifecycle of a delivery store's operational setup, focusing on catalog management, financial provisioning, and logistics readiness. The workflow begins by navigating through the delivery services hierarchy to locate a specific store, where it performs a menu expansion by adding new products with precise attributes including pricing, imagery, and discount logic. Following inventory setup, the script executes a comprehensive financial audit by performing both credit and debit transactions within the store’s wallet to ensure backend accounting synchronization. Finally, the test secures the store's fulfillment capabilities by registering a new private driver, capturing personal and vehicle details alongside document uploads, thereby ensuring the merchant is fully prepared to manage products, finances, and last-mile delivery.</t>
-  </si>
-  <si>
-    <t>SA_TS_8</t>
-  </si>
-  <si>
-    <t>Store Status Mangement</t>
-  </si>
-  <si>
-    <t>TC_CA_08_store_status_management</t>
-  </si>
-  <si>
-    <t>This test validates the complete lifecycle of a store within a delivery services platform, beginning with the creation of a new store (using dynamic timestamps for uniqueness) and the configuration of its operational settings, bank details, and timing. It then navigates through various administrative states, including uploading and verifying compliance documents, moving the store from a pending status to approved, and then testing the blocking/unblocking functionality. Finally, the script validates the rejection workflow by moving a store to the rejected list with a specific reason, ensuring that status transitions and data filtering across the "Store List," "Pending," and "Blocked" modules are functioning as expected.</t>
+43.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
+</t>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
+3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
+4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
+5.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
+6.Click  Stores,click,,"//button[contains(., 'Stores')]"
+7.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+8.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
+9.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+10.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+11.Click Product Icon,click,,"//i[@title='Product View']"
+12.Click  Add  Products,click,,"//button[normalize-space()='Add Products']"
+13.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[1]"
+14.Select Grill Chicken,click,,"//li[@role='option'][contains(.,'Grill Chicken')]"
+15.Enter Product Name, type, Grill Chicken, "//label[contains(.,'Product Name')]/following-sibling::input"
+16.Enter Product Amount, type, 500, "//label[contains(.,'Product Amount')]/following-sibling::input"
+17.Enter Product Description, type, KFC special grill chicken, "//label[contains(text(),'Product Description')]/following-sibling::textarea"
+18.Upload Product Image, uploadfile, "src/main/resources/test-data/grillchicken.jpg", "//input[@type='file' and @accept='image/*']"
+19.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[2]"
+20.Select Activate,click,,"//li[@role='option'][contains(.,'Activate')]"
+21.Open Discount Type Dropdown,click,,"//label[contains(.,'Discount Type')]/following-sibling::select/option[text()='Discount in Amount']"
+22.Enter Discount Amount, type, 50, "//label[contains(.,'Discount Amount')]/following-sibling::input"
+23.Click Save, click, , "//button[normalize-space()='Save']"
+24.Verify Saved Succesfully, verify, , "//div[@aria-label='Product added successfully']"
+25.Verify Store Products,verify,,"//div[contains(text(),'☰ Store Products')]"
+26.Filter Product List,type,Grill Chicken,"//input[@aria-label='Product Name Filter Input']"
+27.Click Back, click, , "//button[normalize-space()='Back']"
+28.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+29.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+30.Click Wallet Icon,click,,"//i[@title='Wallet']"
+31.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
+32.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
+33.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+34.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
+35.Click Submit, click, , "//button[normalize-space()='Submit']"
+36.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+37.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
+38.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
+39.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+40.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
+41.Click Submit, click, , "//button[normalize-space()='Submit']"
+42.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+43.Click Back, click, , "//button[normalize-space()='Back']"
+44.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+45.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+46.Click Drivers Icon,click,,"//i[@title='Drivers']"
+47.Click Add Private Driver, click, , "//button[normalize-space()='Add Private Driver']"
+48.Enter Driver Name, type, kfcdriver_{timestamp} &gt;&gt; kfcdriverName, "//label[contains(., 'Driver Full Name')]/following-sibling::div//input"
+49.Enter Email, type, kfcdriver_{timestamp}@gmail.com, "//label[contains(., 'Email')]/following-sibling::div//input"
+50.Enter Contact Number, type, {randomPhone}, "//label[contains(., 'Contact No')]/following-sibling::div//input"
+51.Upload Profile Image, uploadfile, "src/main/resources/test-data/bikedriver.jpg", "//input[@type='file' and @accept='image/*']"
+52. Select Male Gender, click, , "//div[contains(text(), 'Male')]/preceding-sibling::mat-radio-button"
+53.Click Vehicle Type Dropdown,click,,"//label[contains(., 'Vehicle Type')]/following-sibling::p-dropdown"
+54.Select  Scooter Option,click,,"//li[@role='option'][contains(.,'Scooter')]"
+55. Enter Model Year, type, 2013, "//label[span[text()='Model Year']]/following::input[1]"
+56.Enter Vehicle Company, type, honda, "//label[contains(., 'Vehicle Company')]/following-sibling::div//input"
+57. Enter Plate No, type, KL-01-AB-1634, "//label[contains(., 'Plate No')]/following-sibling::div//input"
+58. Enter Model Name, type, activa, "//label[contains(., 'Model Name')]/following-sibling::div//input"
+59. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/bike.jpg", "(//app-image-upload//input[@type='file'])[2]"
+60. Enter Vehicle Color, type, white, "//label[contains(., 'Vehicle Color')]/following::input[1]"
+61. Click Submit, click, , "//button[contains(.,'Submit')]"
+62. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+63.Filter Driver List,type,{kfcdriverName},"//input[@aria-label='Driver Name Filter Input']"
+64.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
+65.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
+3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
+4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
+5.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
+6.Click  Stores,click,,"//button[contains(., 'Stores')]"
+7.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
+8.Verify Add Store,verify,,"//div[contains(text(),'☰ Add Store')]"
+9.Enter Store Name, type, KFC_{timestamp} &gt;&gt; storeName, "//input[@placeholder='Store Name']"
+10.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
+11.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
+12.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
+13. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
+14.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
+15.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
+16.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
+17.Upload Banner Image, uploadfile, "src/main/resources/test-data/kfcbanner.jpg", "//input[@type='file']"
+18.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
+19.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
+20.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
+21.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
+22.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+23..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
+24.wait,1000,,
+25.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
+26.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
+27.wait,1000,,
+28.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
+29.Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
+30.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
+31.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
+32.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
+33.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
+34.Enter Contact Person Full Name, type, storeowner_{timestamp} &gt;&gt; storeOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
+35.Enter Email, type, kfc_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
+36.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
+37.Upload Store Image, uploadfile, "src/main/resources/test-data/kfcstore.jpg", "(//input[@type='file'])[2]"
+38.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
+39.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
+40.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
+41.Enter Accont Holder Name, type, {storeOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
+42.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
+43.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
+44.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
+45.Enter From Time, type, 100000, "(//label[contains(.,'From Time')]/following-sibling::input)[1]"
+46.Enter To Time, type, 220000, "(//label[contains(.,'To Time')]/following-sibling::input)[1]"
+47.Submit Add Store,click,,"//button[normalize-space()='Submit']"
+48. Verify Success Message,verify,,"//div[@aria-label='Info']"
+49.Click  Stores,click,,"//button[contains(., 'Stores')]"
+50.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+51.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
+52.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+53.Click  Stores,click,,"//button[contains(., 'Stores')]"
+54.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
+55.Verify Add Store,verify,,"//div[contains(text(),'☰ Pending Documents Store')]"
+56.Filter Pending Document Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+57.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+58.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
+59. Store Required Documents,verify,,"//div[contains(text(),'☰ Documents')]"
+60.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+61.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
+62.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+63.Click Submit, click, , "//button[normalize-space()='Submit']"
+64.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+65.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+66.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+67.Click Back, click, , "//button[@class='buttonWidget']"
+68.Click  Stores,click,,"//button[contains(., 'Stores')]"
+69.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+70.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
+71.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+72.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+73.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
+74.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
+75.wait,1000,,</t>
   </si>
   <si>
     <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 3. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
 4. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
 5.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-6.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-7. wait, 1000,,
-8. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-9. Enter Driver Name, type, autodriver_{timestamp} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-10. Enter Email, type, autodriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-11. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-12. wait, 1000,,
-13. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-14. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-15.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-16.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
-17. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-18.Enter Vehicle Company, type, bajaj, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-19. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-20. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-21. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-22. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-25. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-26. Enter Account Holder Name, type, Shafi, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-27. Enter Payment Email Address, type, shabeer_pay@gmail.com, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-29. Click Submit, click, , "//button[contains(.,'Submit')]"
-30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-31. Wait for Toast to hide, wait, 5000,
-32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-34.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-35.wait, 3000,,
-36.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-37.wait,3000,,
-38.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-39.wait,3000,,
-40. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
-41.Add Driving License,click,,"//i[@title='Edit']"
-42.wait,3000,,
-43.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-44.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-45.wait,1000,,
-46.Click Submit, click, , "//button[normalize-space()='Submit']"
-47.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-48.wait,2000,,
-49.Click Approve Driver,click,,"//i[@title='Approve']"
-50.wait,2000,,
-51.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-52.wait,5000,,
-53.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-54.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-55.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-56.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
-57.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-58.wait,2000,,
-59.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-60.Click Doc Icon,click,,"//i[@title='Document']"
-61.Click Eye Icon,click,,"//i[@title='View']"
-62.wait,2000,,</t>
+6.Select Taxi Ride Option,click,,"//span[normalize-space()='Taxi Ride']"
+7. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+8. Enter Driver Name, type, taxidriver_{timestamp} &gt;&gt; taxiName, "//label[contains(.,'Full Name')]/following::input[1]"
+9. Enter Email, type, taxidriver_{timestamp}@gmail.com&gt;&gt;taxiEmail, "//label[contains(.,'Email')]/following::input[1]"
+10. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+11. Upload Profile Image, uploadfile, "src/main/resources/test-data/taxidriver.jpg", "//input[@type='file']"
+12. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+13.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+14.Select  Suv Option,click,,"//li[@role='option']//span[text()='SUV']"
+15. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+16.Enter Vehicle Company, type, toyota, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+17. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+18. Enter Model Name, type, etios, "//label[contains(.,'Model Name')]/following::input[1]"
+19.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/taxi.jpg", "(//input[@type='file'])[2]"
+20. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+21. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+22. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+23. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+24. Enter Account Holder Name, type, {taxiName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+25. Enter Payment Email Address, type, {taxiEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+26. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+27. Click Submit, click, , "//button[contains(.,'Submit')]"
+28. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+29. Wait for Toast to hide, wait, 1000,
+30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+32.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+33.Filter by Name,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
+34.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+35. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
+36.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+37.Add Driving License,click,,"//i[@title='Edit']"
+38.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+39.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+40.Click Submit, click, , "//button[normalize-space()='Submit']"
+41.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+42.Click Approve Driver,click,,"//i[@title='Approve']"
+43.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+44.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+46.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+47.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
+48.Filter Approved Driver,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
+49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+50.Click Doc Icon,click,,"//i[@title='Document']"
+51.Click Eye Icon,click,,"//i[@title='View']"
+52.wait,1000,,</t>
   </si>
   <si>
     <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
@@ -517,812 +958,283 @@
 4. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
 5.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
 6.Select Bike Ride Option,click,,"//span[normalize-space()='Bike Ride']"
-7. wait, 3000,,
-8. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-9. Enter Driver Name, type, bikedriver_{timestamp} &gt;&gt; bikeName, "//label[contains(.,'Full Name')]/following::input[1]"
-10. Enter Email, type, bikedriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-11. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-12. wait, 1000,,
-13. Upload Profile Image, uploadfile, "src/main/resources/test-data/bikedriver.jpg", "//input[@type='file']"
-14. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-15.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-16.Select  Scooter Option,click,,"//li[@role='option']//span[text()='Scooter']"
-17. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-18.Enter Vehicle Company, type, honda, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-19. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
-20. Enter Model Name, type, activa, "//label[contains(.,'Model Name')]/following::input[1]"
-21. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/bike.jpg", "(//input[@type='file'])[2]"
-22. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-25. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-26. Enter Account Holder Name, type, jai, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-27. Enter Payment Email Address, type, jai_pay@gmail.com, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-29. Click Submit, click, , "//button[contains(.,'Submit')]"
-30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-31. Wait for Toast to hide, wait, 5000,
-32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-34.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-35.wait, 3000,,
-36.Filter by Name,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
-37.wait,3000,,
-38.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-39.wait,3000,,
-40. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
-41.Add Driving License,click,,"//i[@title='Edit']"
-42.wait,3000,,
-43.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-44.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-45.wait,1000,,
-46.Click Submit, click, , "//button[normalize-space()='Submit']"
-47.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-48.wait,2000,,
-49.Click Approve Driver,click,,"//i[@title='Approve']"
-50.wait,2000,,
-51.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-52.wait,5000,,
-53.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-54.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-55.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-56.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
-57.Filter Approved Driver,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
-58.wait,2000,,
-59.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-60.Click Doc Icon,click,,"//i[@title='Document']"
-61.Click Eye Icon,click,,"//i[@title='View']"
-62.wait,2000,,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-3. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-4. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
-5.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-6.Select Taxi Ride Option,click,,"//span[normalize-space()='Taxi Ride']"
-7. wait, 3000,,
-8. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-9. Enter Driver Name, type, taxidriver_{timestamp} &gt;&gt; taxiName, "//label[contains(.,'Full Name')]/following::input[1]"
-10. Enter Email, type, taxidriver_{timestamp}@gmail.com, "//label[contains(.,'Email')]/following::input[1]"
-11. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-12. wait, 1000,,
-13. Upload Profile Image, uploadfile, "src/main/resources/test-data/taxidriver.jpg", "//input[@type='file']"
-14. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-15.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-16.Select  Suv Option,click,,"//li[@role='option']//span[text()='SUV']"
-17. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-18.Enter Vehicle Company, type, toyota, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-19. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
-20. Enter Model Name, type, etios, "//label[contains(.,'Model Name')]/following::input[1]"
-21. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/taxi.jpg", "(//input[@type='file'])[2]"
-22. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-25. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-26. Enter Account Holder Name, type, jai, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-27. Enter Payment Email Address, type, jai_pay@gmail.com, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-29. Click Submit, click, , "//button[contains(.,'Submit')]"
-30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-31. Wait for Toast to hide, wait, 5000,
-32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-34.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-35.wait, 3000,,
-36.Filter by Name,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
-37.wait,3000,,
-38.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-39.wait,3000,,
-40. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
-41.Add Driving License,click,,"//i[@title='Edit']"
-42.wait,3000,,
-43.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-44.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-45.wait,1000,,
-46.Click Submit, click, , "//button[normalize-space()='Submit']"
-47.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-48.wait,2000,,
-49.Click Approve Driver,click,,"//i[@title='Approve']"
-50.wait,2000,,
-51.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-52.wait,5000,,
-53.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-54.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-55.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-56.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
-57.Filter Approved Driver,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
-58.wait,2000,,
-59.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-60.Click Doc Icon,click,,"//i[@title='Document']"
-61.Click Eye Icon,click,,"//i[@title='View']"
-62.wait,2000,,
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
-3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
-4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
-5.wait,2000,,
-6.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
-7.Click  Stores,click,,"//button[contains(., 'Stores')]"
-8.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
-9.Verify Add Store,verify,,"//div[contains(text(),'☰ Add Store')]"
-10.Enter Store Name, type, KFC_{timestamp} &gt;&gt; storeName, "//input[@placeholder='Store Name']"
-11.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
-12.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
-13.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
-14. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
-15.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
-16.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
-17.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
-18.Upload Banner Image, uploadfile, "src/main/resources/test-data/kfcbanner.jpg", "//input[@type='file']"
-19.wait,2000,,
-20.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
-21.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
-22.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
-23.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
-24.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-25..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
-26.wait,2000,,
-27.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
-28.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
-29.wait,1000,,
-30.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
-31.wait,1000,,
-32..Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
-33.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
-34.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
-35.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
-36.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
-37.Enter Contact Person Full Name, type, storeowner_{timestamp} &gt;&gt; storeOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
-38.Enter Email, type, kfc_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
-39.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
-40.Upload Store Image, uploadfile, "src/main/resources/test-data/kfcstore.jpg", "(//input[@type='file'])[2]"
-41.wait,2000,,
-42.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
-43.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
-44.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
-45.Enter Accont Holder Name, type, {storeOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
-46.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
-47.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
-48.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
-49.Enter From Time, type, 100000, "(//label[contains(.,'From Time')]/following-sibling::input)[1]"
-50.Enter To Time, type, 220000, "(//label[contains(.,'To Time')]/following-sibling::input)[1]"
-51.Submit Add Store,click,,"//button[normalize-space()='Submit']"
-52. Verify Success Message,verify,,"//div[@aria-label='Info']"
-53.wait,3000,,
-54.Click  Stores,click,,"//button[contains(., 'Stores')]"
-55.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-56.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
-57.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-58.wait,2000,,
-59.Click  Stores,click,,"//button[contains(., 'Stores')]"
-60.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
-61.Verify Add Store,verify,,"//div[contains(text(),'☰ Pending Documents Store')]"
-62.Filter Pending Document Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-63.wait,2000,,
-64.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-65.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-65.wait,3000,,
-66. Store Required Documents,verify,,"//div[contains(text(),'☰ Documents')]"
-67.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-68.wait,3000,,
-69.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-70.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-71.wait,1000,,
-72.Click Submit, click, , "//button[normalize-space()='Submit']"
-73.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-74.wait,2000,,
-75.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-76.wait,2000,,
-77.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-78.wait,3000,,
-79.Click Back, click, , "//button[@class='buttonWidget']"
-80.wait,2000,,
-81.Click  Stores,click,,"//button[contains(., 'Stores')]"
-82.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-83.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
-84.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-85.wait,2000,,
-86.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-87.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-88.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
-89.wait,3000,,
-</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Authentication State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <t>SA_TS_9</t>
-  </si>
-  <si>
-    <t>Add New Provider &amp; Approve</t>
-  </si>
-  <si>
-    <t>TC_CA_09_add_provider</t>
-  </si>
-  <si>
-    <t>This test validates the complete administrative workflow for registering and authorizing a new provider within the Plumbers. The automation navigates to the Add Providers module to dynamically create a unique pumbler profile, populating operational data including provider service radius, service time, address and banking details. Following creation, the script transitions to the Compliance phase, where it filters for the new pumbler in the "Pending Documents" list, automates the upload of regulatory files, and sets document expiry dates. The workflow concludes by triggering the Final Approval and verifying the pumbler successful migration to the active provider List, ensuring end-to-end data consistency and functional status transitions.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Store and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
+7. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+8. Enter Driver Name, type, bikedriver_{timestamp} &gt;&gt; bikeName, "//label[contains(.,'Full Name')]/following::input[1]"
+9. Enter Email, type, bikedriver_{timestamp}@gmail.com&gt;&gt;bikeEmail, "//label[contains(.,'Email')]/following::input[1]"
+10. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+11. Upload Profile Image, uploadfile, "src/main/resources/test-data/bikedriver.jpg", "//input[@type='file']"
+12. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+13.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+14.Select  Scooter Option,click,,"//li[@role='option']//span[text()='Scooter']"
+15. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+16.Enter Vehicle Company, type, honda, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+17. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+18. Enter Model Name, type, activa, "//label[contains(.,'Model Name')]/following::input[1]"
+19. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/bike.jpg", "(//input[@type='file'])[2]"
+20. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+21. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+22. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+23. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+24. Enter Account Holder Name, type, {bikeName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+25. Enter Payment Email Address, type, {bikeEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+26. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+27. Click Submit, click, , "//button[contains(.,'Submit')]"
+28. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+29. Wait for Toast to hide, wait, 1000,
+30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+32.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+33.Filter by Name,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
+34.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+35. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
+36.FilterDocumet List,type,Vehicle Permit Copy,"//input[@aria-label='Document Name Filter Input']"
+37.Add Vehicle Permit Copy,click,,"//i[@title='Edit']"
+38.Upload Vehicle Permit Copy, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+39.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+40.Click Submit, click, , "//button[normalize-space()='Submit']"
+41.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+42.Click Approve Driver,click,,"//i[@title='Approve']"
+43.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+44.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+46.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+47.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
+48.Filter Approved Driver,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
+49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+50.Click Doc Icon,click,,"//i[@title='Document']"
+51.Click Eye Icon,click,,"//i[@title='View']"
+52.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+3. Verify Add Driver,verify,,"//div[contains(text(),'☰ Add Driver')]"
+4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+6. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
+7. Enter Driver Name, type, autodriver_{timestamp} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+8. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+9. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+10. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+11. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+12.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+13.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
+14. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+15.Enter Vehicle Company, type, bajaj, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+16. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+17. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+18. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+19. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+20. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+21. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+22. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+23. Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+24. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+25. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+26. Click Submit, click, , "//button[contains(.,'Submit')]"
+27. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+28. Wait for Toast to hide, wait, 1000,
+29.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+32.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+33.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+34. Driver Required Documents,verify,,"//div[contains(text(),'☰ Driver Required Documents')]"
+35.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+36.Add Driving License,click,,"//i[@title='Edit']"
+37.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+38.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+39.Click Submit, click, , "//button[normalize-space()='Submit']"
+40.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+41.Click Approve Driver,click,,"//i[@title='Approve']"
+42.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+43.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+44.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+45.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+46.Approved Drivers List,verify,,"//div[contains(text(),'☰ Approved Drivers List')]"
+47.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+48.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+49.Click Doc Icon,click,,"//i[@title='Document']"
+50.Click Eye Icon,click,,"//i[@title='View']"
+51.wait,1000,,</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
 2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
 3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
 4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
-5.wait,2000,,
-6.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
-7.Click  Stores,click,,"//button[contains(., 'Stores')]"
-8.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-9.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
-10.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-11.wait,2000,,
-12.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-13.Click Product Icon,click,,"//i[@title='Product View']"
-14.wait,1000,,
-15.Click  Add  Products,click,,"//button[normalize-space()='Add Products']"
-16.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[1]"
-17.Select Grill Chicken,click,,"//li[@role='option'][contains(.,'Grill Chicken')]"
-18.wait,1000,,
-19.Enter Product Name, type, Grill Chicken, "//label[contains(.,'Product Name')]/following-sibling::input"
-20.Enter Product Amount, type, 500, "//label[contains(.,'Product Amount')]/following-sibling::input"
-21.Enter Product Description, type, KFC special grill chicken, "//label[contains(text(),'Product Description')]/following-sibling::textarea"
-22.Upload Product Image, uploadfile, "src/main/resources/test-data/grillchicken.jpg", "//input[@type='file' and @accept='image/*']"
-23.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[2]"
-24.Select Activate,click,,"//li[@role='option'][contains(.,'Activate')]"
-25.Open Discount Type Dropdown,click,,"//label[contains(.,'Discount Type')]/following-sibling::select/option[text()='Discount in Amount']"
-26.Enter Discount Amount, type, 50, "//label[contains(.,'Discount Amount')]/following-sibling::input"
-27.Click Save, click, , "//button[normalize-space()='Save']"
-28.Verify Saved Succesfully, verify, , "//div[@aria-label='Product added successfully']"
-29.wait,3000,,
-30.Verify Store Products,verify,,"//div[contains(text(),'☰ Store Products')]"
-31.Filter Product List,type,Grill Chicken,"//input[@aria-label='Product Name Filter Input']"
-32.wait,2000,,
-33.Click Back, click, , "//button[normalize-space()='Back']"
-34.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-35.wait,2000,,
-36.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-37.Click Wallet Icon,click,,"//i[@title='Wallet']"
-38.wait,2000,,
-39.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
-40.wait,2000,,
-41.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
-42.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-43.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
-44.Click Submit, click, , "//button[normalize-space()='Submit']"
-45.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-46.wait,3000,,
-47.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
-48.wait,2000,,
-49.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
-50.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-51.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
-52.Click Submit, click, , "//button[normalize-space()='Submit']"
-53.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-54.wait,3000,,
-55.Click Back, click, , "//button[normalize-space()='Back']"
-56.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-57.wait,2000,,
-58.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-59.Click Drivers Icon,click,,"//i[@title='Drivers']"
-60.wait,2000,,
-61.Click Add Private Driver, click, , "//button[normalize-space()='Add Private Driver']"
-62.Enter Driver Name, type, kfcdriver_{timestamp} &gt;&gt; kfcdriverName, "//label[contains(., 'Driver Full Name')]/following-sibling::div//input"
-63.Enter Email, type, kfcdriver_{timestamp}@gmail.com, "//label[contains(., 'Email')]/following-sibling::div//input"
-64.Enter Contact Number, type, {randomPhone}, "//label[contains(., 'Contact No')]/following-sibling::div//input"
-65.Upload Profile Image, uploadfile, "src/main/resources/test-data/bikedriver.jpg", "//input[@type='file' and @accept='image/*']"
-66.wait,3000,,
-67. Select Male Gender, click, , "//div[contains(text(), 'Male')]/preceding-sibling::mat-radio-button"
-68.Click Vehicle Type Dropdown,click,,"//label[contains(., 'Vehicle Type')]/following-sibling::p-dropdown"
-69.Select  Scooter Option,click,,"//li[@role='option'][contains(.,'Scooter')]"
-70. Enter Model Year, type, 2013, "//label[span[text()='Model Year']]/following::input[1]"
-71.Enter Vehicle Company, type, honda, "//label[contains(., 'Vehicle Company')]/following-sibling::div//input"
-72. Enter Plate No, type, KL-01-AB-1634, "//label[contains(., 'Plate No')]/following-sibling::div//input"
-73. Enter Model Name, type, activa, "//label[contains(., 'Model Name')]/following-sibling::div//input"
-74. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/bike.jpg", "(//app-image-upload//input[@type='file'])[2]"
-75. Enter Vehicle Color, type, white, "//label[contains(., 'Vehicle Color')]/following::input[1]"
-76. Click Submit, click, , "//button[contains(.,'Submit')]"
-77. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-78. Wait for Toast to hide, wait, 3000,
-79.Filter Driver List,type,{kfcdriverName},"//input[@aria-label='Driver Name Filter Input']"
-80.wait,2000,,
-81.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
-82.wait,1000,,</t>
-  </si>
-  <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
-3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ DELIVERY SERVICES')]"
-4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
-5.wait,2000,,
-6.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
-7.Click  Stores,click,,"//button[contains(., 'Stores')]"
-8.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
-9.Verify Add Store,verify,,"//div[contains(text(),'☰ Add Store')]"
-10.Enter Store Name, type, bilal_{timestamp} &gt;&gt; storeName, "//input[@placeholder='Store Name']"
-11.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
-12.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
-13.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
-14. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
-15.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
-16.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
-17.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
-18.Upload Banner Image, uploadfile, "src/main/resources/test-data/kfcbanner.jpg", "//input[@type='file']"
-19.wait,2000,,
-20.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
-21.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
-22.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
-23.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
-24.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-25..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
-26.wait,2000,,
-27.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
-28.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
-29.wait,1000,,
-30.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
-31.wait,1000,,
-32..Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
-33.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
-34.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
-35.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
-36.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
-37.Enter Contact Person Full Name, type, storeowner_{timestamp} &gt;&gt; storeOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
-38.Enter Email, type, kfc_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
-39.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
-40.Upload Store Image, uploadfile, "src/main/resources/test-data/kfcstore.jpg", "(//input[@type='file'])[2]"
-41.wait,2000,,
-42.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
-43.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
-44.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
-45.Enter Accont Holder Name, type, {storeOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
-46.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
-47.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
-48.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
-49.Enter From Time, type, 100000, "(//label[contains(.,'From Time')]/following-sibling::input)[1]"
-50.Enter To Time, type, 220000, "(//label[contains(.,'To Time')]/following-sibling::input)[1]"
-51.Submit Add Store,click,,"//button[normalize-space()='Submit']"
-52. Verify Success Message,verify,,"//div[@aria-label='Info']"
-53.wait,3000,,
-54.Click  Stores,click,,"//button[contains(., 'Stores')]"
-55.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-56.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
-57.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-58.wait,2000,,
-59.Click  Stores,click,,"//button[contains(., 'Stores')]"
-60.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
-61.Verify Add Store,verify,,"//div[contains(text(),'☰ Pending Documents Store')]"
-62.Filter Pending Document Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-63.wait,2000,,
-64.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-65.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-65.wait,3000,,
-66. Store Required Documents,verify,,"//div[contains(text(),'☰ Documents')]"
-67.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-68.wait,3000,,
-69.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-70.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-71.wait,1000,,
-72.Click Submit, click, , "//button[normalize-space()='Submit']"
-73.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-74.wait,2000,,
-75.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-76.wait,2000,,
-77.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-78.wait,3000,,
-79.Click Back, click, , "//button[@class='buttonWidget']"
-80.wait,2000,,
-81.Click  Stores,click,,"//button[contains(., 'Stores')]"
-82.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-83.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
-84.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-85.wait,2000,,
-86.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-87.Click Block Icon,click,,"//i[@title='Blocked']"
-88.wait,2000,,
-89.Click Block  Yes,click,,"//button[normalize-space()='Yes']"
-90.Click  Stores,click,,"//button[contains(., 'Stores')]"
-91.Select Blocked Store,click,,"//div[normalize-space()='Blocked Stores']"
-92.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-93.wait,2000,,
-94.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-95.Click unBlock Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
-96.wait,3000,,
-97.Click  Stores,click,,"//button[contains(., 'Stores')]"
-98.Select Rejected Store,click,,"//div[normalize-space()='Rejected Stores']"
-99.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-100.wait,2000,,
-101.Scroll Grid, tab, 7, "//input[@aria-label='Store Name Filter Input']"
-102.Click Approve Icon,click,,"//i[@title='Approve']"
-103.Click  Stores,click,,"//button[contains(., 'Stores')]"
-104.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-105.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-106.wait,2000,,
-107.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-108.Click Doc Icon,click,,"//i[@title='Document']"
-109.wait,1000,,
-110.Click UnApprove Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
-111.wait,1000,,
-112.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-113.Rejection Reason,type,document insufficent,"//textarea[@id='swal2-textarea']"
-114.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-115.wait,3000,,</t>
+5.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
+6.Click  Stores,click,,"//button[contains(., 'Stores')]"
+7.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
+8.Verify Add Store,verify,,"//div[contains(text(),'☰ Add Store')]"
+9.Enter Store Name, type, bilal_{timestamp} &gt;&gt; storeName, "//input[@placeholder='Store Name']"
+10.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
+11.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
+12.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
+13. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
+14.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
+15.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
+16.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
+17.Upload Banner Image, uploadfile, "src/main/resources/test-data/kfcbanner.jpg", "//input[@type='file']"
+18.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
+19.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
+20.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
+21.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
+22.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+23..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
+24.wait,1000,,
+25.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
+26.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
+27.wait,1000,,
+28.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
+29.Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
+30.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
+31.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
+32.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
+33.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
+34.Enter Contact Person Full Name, type, storeowner_{timestamp} &gt;&gt; storeOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
+35.Enter Email, type, kfc_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
+36.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
+37.Upload Store Image, uploadfile, "src/main/resources/test-data/kfcstore.jpg", "(//input[@type='file'])[2]"
+38.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
+39.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
+40.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
+41.Enter Accont Holder Name, type, {storeOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
+42.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
+43.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
+44.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
+45.Enter From Time, type, 100000, "(//label[contains(.,'From Time')]/following-sibling::input)[1]"
+46.Enter To Time, type, 220000, "(//label[contains(.,'To Time')]/following-sibling::input)[1]"
+47.Submit Add Store,click,,"//button[normalize-space()='Submit']"
+48. Verify Success Message,verify,,"//div[@aria-label='Info']"
+49.Click  Stores,click,,"//button[contains(., 'Stores')]"
+50.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+51.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
+52.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+53.Click  Stores,click,,"//button[contains(., 'Stores')]"
+54.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
+55.Verify Add Store,verify,,"//div[contains(text(),'☰ Pending Documents Store')]"
+56.Filter Pending Document Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+57.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+58.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
+59. Store Required Documents,verify,,"//div[contains(text(),'☰ Documents')]"
+60.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+61.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
+62.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+63.Click Submit, click, , "//button[normalize-space()='Submit']"
+64.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+65.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+66.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+67.Click Back, click, , "//button[@class='buttonWidget']"
+68.Click  Stores,click,,"//button[contains(., 'Stores')]"
+69.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+70.Verify Add Store,verify,,"//div[contains(text(),'☰ Store List')]"
+71.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+72.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+73.Click Block Icon,click,,"//i[@title='Blocked']"
+74.Click Block  Yes,click,,"//button[normalize-space()='Yes']"
+75.Click  Stores,click,,"//button[contains(., 'Stores')]"
+76.Select Blocked Store,click,,"//div[normalize-space()='Blocked Stores']"
+77.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+78.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+79.Click unBlock Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
+80.Click  Stores,click,,"//button[contains(., 'Stores')]"
+81.Select Rejected Store,click,,"//div[normalize-space()='Rejected Stores']"
+82.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+83.Scroll Grid, tab, 7, "//input[@aria-label='Store Name Filter Input']"
+84.Click Approve Icon,click,,"//i[@title='Approve']"
+85.Click  Stores,click,,"//button[contains(., 'Stores')]"
+86.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+87.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+88.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+89.Click Doc Icon,click,,"//i[@title='Document']"
+90.Click UnApprove Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
+91.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+92.Rejection Reason,type,document insufficent,"//textarea[@id='swal2-textarea']"
+93.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+94.wait,1000,,</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
 2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
 3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ ON-DEMAND SERVICES')]"
 4.Click Home Icon Plumbers,click,,"//div[@role='row'][.//span[text()='Plumbers']]//i[@title='Home']"
-5.wait,2000,,
-6.Verify Plumbers Summary,verify,,"//div[contains(text(),'☰ Plumbers Summary')]"
-7.Click  Providers,click,,"//button[contains(., 'Providers')]"
-8.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
-9.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
-10.Enter Provider Full Name, type, Plumber{randomAlpha}&gt;&gt; plumberName, "//input[@placeholder='Provider Full Name']"
-11.Upload Plumber Image, uploadfile, "src/main/resources/test-data/plumber.jpg", "//input[@type='file']"
-12.Wait For Image To Load,3000,,
-13.Enter Email, type, Plumber_{timestamp}@gmail.com&gt;&gt;plumberEmail, "//input[@placeholder='Unique Email']"
-14.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
-15.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
-16.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
-17.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
-18.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
-19..Enter Provider Address, type, plumber chennai, "//input[@placeholder='Enter provider Address']"
-20.wait,2000,,
-21.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
-22.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
-23.wait,2000,,
-24.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
-25.wait,1000,,
-26.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
-27.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
-28.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
-29.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
-30.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
-31.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
-32.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
-33.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
-34.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
-35.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
-36.Enter Accont Holder Name, type, {plumberName}, "//input[@placeholder='Account Holder Name']"
-37.Enter Payment Email Address, type, {plumberEmail}, "//input[@placeholder='Email Address for Payment Notification']"
-38.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
-39.Click Save, click, , "//button[@type='submit']"
-40.Verify Sucess, verify, , "//div[@aria-label='Info']"
-41.wait,3000,,
-42.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-43.wait,2000,,
-44.Click  Providers,click,,"//button[contains(., 'Providers')]"
-45.Select Pending Document Providers,click,,"//div[normalize-space()='Pending Document Providers']"
-46.wait,2000,,
-47.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-48.wait,2000,,
-49.Click Document Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-50.wait,2000,,
-51. Provider Required Documents,verify,,"//div[contains(text(),'☰ Documents')]"
-52.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
-53.wait,2000,,
-54.Add Address Proof,click,,"(//i[contains(@class, 'Edit')])[1]"
-55.wait,3000,,
-54.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-55.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-56.wait,1000,,
-57.Click Submit, click, , "//button[normalize-space()='Submit']"
-58.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-59.wait,2000,,
-60.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
-61.wait,2000,,
-62.Click Approve Store,click,,"//div[@row-index='0']//i[contains(@class, 'bi-hand-thumbs-up-fill')]"
-63.wait,2000,,
-64.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-65.wait,3000,,
-66.Click Back, click, , "//button[@class='buttonWidget']"
-67.wait,2000,,
-68.Click  Providers,click,,"//button[contains(., 'Providers')]"
-69.Select Provider List,click,,"//div[normalize-space()='Provider List']"
-70.Verify Approved Provider,verify,,"//div[normalize-space()='☰ Approved Plumbers Service Providers']"
-71.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-72.wait,2000,,
-73.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-74.wait,2000,,
-75.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
-76.wait,2000,,</t>
+5.Verify Plumbers Summary,verify,,"//div[contains(text(),'☰ Plumbers Summary')]"
+6.Click  Providers,click,,"//button[contains(., 'Providers')]"
+7.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
+8.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
+9.Enter Provider Full Name, type, Plumber{randomAlpha}&gt;&gt; plumberName, "//input[@placeholder='Provider Full Name']"
+10.Upload Plumber Image, uploadfile, "src/main/resources/test-data/plumber.jpg", "//input[@type='file']"
+11.Enter Email, type, Plumber_{timestamp}@gmail.com&gt;&gt;plumberEmail, "//input[@placeholder='Unique Email']"
+12.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
+13.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
+14.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
+15.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
+16.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
+17..Enter Provider Address, type, plumber chennai, "//input[@placeholder='Enter provider Address']"
+18.wait,1000,,
+19.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
+20.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
+21.wait,1000,,
+22.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
+23.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
+24.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
+25.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
+26.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
+27.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
+28.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
+29.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
+30.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
+31.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
+32.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
+33.Enter Accont Holder Name, type, {plumberName}, "//input[@placeholder='Account Holder Name']"
+34.Enter Payment Email Address, type, {plumberEmail}, "//input[@placeholder='Email Address for Payment Notification']"
+35.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
+36.Click Save, click, , "//button[@type='submit']"
+37.Verify Sucess, verify, , "//div[@aria-label='Info']"
+38.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+39.Click  Providers,click,,"//button[contains(., 'Providers')]"
+40.Select Pending Document Providers,click,,"//div[normalize-space()='Pending Document Providers']"
+41.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+42.Click Document Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+43. Provider Required Documents,verify,,"//div[contains(text(),'☰ Documents')]"
+44.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
+45.Add Address Proof,click,,"(//i[contains(@class, 'Edit')])[1]"
+46.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
+47.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+48.Click Submit, click, , "//button[normalize-space()='Submit']"
+49.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+50.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
+51.Click Approve Store,click,,"//div[@row-index='0']//i[contains(@class, 'bi-hand-thumbs-up-fill')]"
+52.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+53.Click Back, click, , "//button[@class='buttonWidget']"
+54.Click  Providers,click,,"//button[contains(., 'Providers')]"
+55.Select Provider List,click,,"//div[normalize-space()='Provider List']"
+56.Verify Approved Provider,verify,,"//div[normalize-space()='☰ Approved Plumbers Service Providers']"
+57.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+58.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+59.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
+60.Click Back, click, , "//button[@class='buttonWidget']"
+61.Verify Approved Provider,verify,,"//div[normalize-space()='☰ Approved Plumbers Service Providers']"
+62.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+63.Scroll Grid, tab, 11, "//input[@aria-label='Provider Name Filter Input']"
+64.Click Wallet Icon,click,,"//i[@class='bi bi-cash-stack cursor-pointer gridIcon Navigate']"
+65.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
+66.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
+67.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+68.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
+69.Click Submit, click, , "//button[normalize-space()='Submit']"
+70.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+71.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
+72.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
+73.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+74.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
+75.Click Submit, click, , "//button[normalize-space()='Submit']"
+76.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+77.wait,1000,,</t>
+  </si>
+  <si>
+    <t>This test validates the complete administrative workflow for registering and authorizing a new provider within the Plumbers. The automation navigates to the Add Providers module to dynamically create a unique pumbler profile, populating operational data including provider service radius, service time, address and banking details. Following creation, the script transitions to the Compliance phase, where it filters for the new pumbler in the "Pending Documents" list, automates the upload of regulatory files, and sets document expiry dates. The workflow then triggers  the Final Approval and verifying the pumbler successful migration to the active provider List, ensuring end-to-end data consistency and functional status transitions. Following verification, the script executes a comprehensive financial audit by performing both credit and debit transactions within the store’s wallet to ensure backend accounting synchronization.</t>
   </si>
 </sst>
 </file>
@@ -1803,22 +1715,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1963,7 +1875,7 @@
         <v>34</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>35</v>
@@ -2028,10 +1940,10 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2100,10 +2012,10 @@
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2172,10 +2084,10 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2232,22 +2144,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2304,22 +2216,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>44</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2376,22 +2288,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="D2" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>48</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
51th commit: Automatic Running Of Dependent TestSheet Implemented
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30DBC129-B7F6-4D3B-A122-E12094FF71DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4D0B09B-36EC-4CA1-BDCE-5F0F00D72F6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -127,74 +127,6 @@
   </si>
   <si>
     <t>Verify successful authentication of the Super Admin role using valid credentials and Dashboard access validation.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">System State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The WE1 Application is deployed and the Login URL is reachable (https://dev.we1.co/#/login)  and configured as base.url in config.properties.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Access Rights:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A valid Super Admin account exists in the database.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Data Availability: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Super Admin credentials (email and password) are configured in the config.properties file.</t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
@@ -228,143 +160,9 @@
     <t>Validate the end-to-end creation of a City Area, including status configuration and polygon mapping. Verify data persistence by ensuring the new area is correctly listed and available for selection in 'City Wise Manage Services' in ' Transport Service ' and 'City Admin' modules.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Authentication State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
-    </r>
-  </si>
-  <si>
     <t>To verify that the Super Admin can successfully create a new City Admin account by providing valid personal details, associating them with a specific city, and granting multiple service and module-level permissions.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The AddCityArea test suite must be always executed before this test. This is critical because the AddCityAdmin process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>System State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
-    </r>
-  </si>
-  <si>
     <t>SA_TS_6</t>
   </si>
   <si>
@@ -401,212 +199,6 @@
     <t>This test validates the complete lifecycle of a store within a delivery services platform, beginning with the creation of a new store (using dynamic timestamps for uniqueness) and the configuration of its operational settings, bank details, and timing. It then navigates through various administrative states, including uploading and verifying compliance documents, moving the store from a pending status to approved, and then testing the blocking/unblocking functionality. Finally, the script validates the rejection workflow by moving a store to the rejected list with a specific reason, ensuring that status transitions and data filtering across the "Store List," "Pending," and "Blocked" modules are functioning as expected.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Authentication State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
     <t>SA_TS_9</t>
   </si>
   <si>
@@ -614,98 +206,6 @@
   </si>
   <si>
     <t>TC_CA_09_add_provider</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Store and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
@@ -1235,6 +735,663 @@
   </si>
   <si>
     <t>This test validates the complete administrative workflow for registering and authorizing a new provider within the Plumbers. The automation navigates to the Add Providers module to dynamically create a unique pumbler profile, populating operational data including provider service radius, service time, address and banking details. Following creation, the script transitions to the Compliance phase, where it filters for the new pumbler in the "Pending Documents" list, automates the upload of regulatory files, and sets document expiry dates. The workflow then triggers  the Final Approval and verifying the pumbler successful migration to the active provider List, ensuring end-to-end data consistency and functional status transitions. Following verification, the script executes a comprehensive financial audit by performing both credit and debit transactions within the store’s wallet to ensure backend accounting synchronization.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The WE1 Application is deployed and the Login URL is reachable (https://dev.we1.co/#/login)  and configured as base.url in config.properties.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Super Admin credentials (email and password) are configured in the config.properties file.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddCityArea test suite must be always executed before this test. This is critical because the AddCityAdmin process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
+RunSheet: AddCityArea</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>System State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Store and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
+RunSheet: AddStore
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1638,7 +1795,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
@@ -1655,7 +1812,7 @@
         <v>28</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1715,22 +1872,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1797,13 +1954,13 @@
         <v>26</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1872,13 +2029,13 @@
         <v>12</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1940,10 +2097,10 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2012,10 +2169,10 @@
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2084,10 +2241,10 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2144,22 +2301,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>39</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2216,22 +2373,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2288,22 +2445,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>47</v>
-      </c>
       <c r="E2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
52th commit: Add Provider Test Suite Completed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4D0B09B-36EC-4CA1-BDCE-5F0F00D72F6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{953360AA-F7E3-48B8-B20D-72CEB4A510DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -655,7 +655,667 @@
 94.wait,1000,,</t>
   </si>
   <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
+    <t>This test validates the complete administrative workflow for registering and authorizing a new provider within the Plumbers. The automation navigates to the Add Providers module to dynamically create a unique pumbler profile, populating operational data including provider service radius, service time, address and banking details. Following creation, the script transitions to the Compliance phase, where it filters for the new pumbler in the "Pending Documents" list, automates the upload of regulatory files, and sets document expiry dates. The workflow then triggers  the Final Approval and verifying the pumbler successful migration to the active provider List, ensuring end-to-end data consistency and functional status transitions. Following verification, the script executes a comprehensive financial audit by performing both credit and debit transactions within the store’s wallet to ensure backend accounting synchronization.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The WE1 Application is deployed and the Login URL is reachable (https://dev.we1.co/#/login)  and configured as base.url in config.properties.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Super Admin credentials (email and password) are configured in the config.properties file.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddCityArea test suite must be always executed before this test. This is critical because the AddCityAdmin process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
+RunSheet: AddCityArea</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>System State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Store and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
+RunSheet: AddStore
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
 2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
 3.Verify Delivery Services,verify,,"//div[contains(text(),'☰ ON-DEMAND SERVICES')]"
 4.Click Home Icon Plumbers,click,,"//div[@role='row'][.//span[text()='Plumbers']]//i[@title='Home']"
@@ -731,667 +1391,32 @@
 74.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
 75.Click Submit, click, , "//button[normalize-space()='Submit']"
 76.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-77.wait,1000,,</t>
-  </si>
-  <si>
-    <t>This test validates the complete administrative workflow for registering and authorizing a new provider within the Plumbers. The automation navigates to the Add Providers module to dynamically create a unique pumbler profile, populating operational data including provider service radius, service time, address and banking details. Following creation, the script transitions to the Compliance phase, where it filters for the new pumbler in the "Pending Documents" list, automates the upload of regulatory files, and sets document expiry dates. The workflow then triggers  the Final Approval and verifying the pumbler successful migration to the active provider List, ensuring end-to-end data consistency and functional status transitions. Following verification, the script executes a comprehensive financial audit by performing both credit and debit transactions within the store’s wallet to ensure backend accounting synchronization.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-System State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The WE1 Application is deployed and the Login URL is reachable (https://dev.we1.co/#/login)  and configured as base.url in config.properties.
+77.Click Back, click, , "//button[normalize-space()='Back']"
+78.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+79.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+80.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
+81.Click Reject Document,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
+82.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+83.Rejection Reason,type,document insufficent,"//textarea[@id='swal2-textarea']"
+84..Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+85.Click Back, click, , "//button[@class='buttonWidget']"
+86.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+87.Scroll Grid, tab, 13, "//input[@aria-label='Provider Name Filter Input']"
+88.Click Block Provider,click,,"//i[@title='Block Provider']"
+89.Click Block  Yes,click,,"//button[normalize-space()='Yes']"
+90. Blocking Reason,type,customer complaints,"//textarea[@id='swal2-textarea']"
+91.Click block  Yes,click,,"//button[normalize-space()='Yes']"
+92.Click  Providers,click,,"//button[contains(., 'Providers')]"
+93.Select Blocked Providers,click,,"//div[contains(text(), 'Blocked Providers')]"
+94.Verify Blocked Provider,verify,,"//div[normalize-space()='☰ Blocked Plumbers Service Providers']"
+95.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+96.Scroll Grid, tab, 12, "//input[@aria-label='Provider Name Filter Input']"
+97.Click Unblock Provider,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+98.Click  Providers,click,,"//button[contains(., 'Providers')]"
+99.Select Provider List,click,,"//div[contains(text(), 'Provider List')]"
+100.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+101.wait,1000,,
 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Access Rights:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A valid Super Admin account exists in the database.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Data Availability: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Super Admin credentials (email and password) are configured in the config.properties file.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The AddCityArea test suite must be always executed before this test. This is critical because the AddCityAdmin process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
-RunSheet: AddCityArea</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>System State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Store and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
-RunSheet: AddStore
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
-</t>
-    </r>
   </si>
 </sst>
 </file>
@@ -1812,7 +1837,7 @@
         <v>28</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1881,13 +1906,13 @@
         <v>47</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1960,7 +1985,7 @@
         <v>30</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2035,7 +2060,7 @@
         <v>48</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -2100,7 +2125,7 @@
         <v>53</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2172,7 +2197,7 @@
         <v>52</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2244,7 +2269,7 @@
         <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2316,7 +2341,7 @@
         <v>50</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2388,7 +2413,7 @@
         <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2460,7 +2485,7 @@
         <v>54</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
54th commit: Test Independency Implemented
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8045004-928D-402B-B284-8248C5F535FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9777751-6E80-4F3A-AB33-A5CE5692B1DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -311,73 +311,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>Data Dependency:</t>
     </r>
     <r>
@@ -456,346 +389,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Navigation State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Store and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
     </r>
   </si>
   <si>
@@ -1599,6 +1192,546 @@
 73.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
 74.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
 75.wait,1000,,</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SuperAdminLogin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SuperAdminLogin
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SuperAdminLogin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SuperAdminLogin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SuperAdminLogin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Store and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SuperAdminLogin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2091,10 +2224,10 @@
         <v>48</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2151,22 +2284,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2239,7 +2372,7 @@
         <v>30</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2311,10 +2444,10 @@
         <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -2376,10 +2509,10 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2448,10 +2581,10 @@
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2520,10 +2653,10 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2592,10 +2725,10 @@
         <v>36</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2664,10 +2797,10 @@
         <v>40</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2736,10 +2869,10 @@
         <v>44</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
55th commit: Provider Service & Category Creation Test Suite Completed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9777751-6E80-4F3A-AB33-A5CE5692B1DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5906194-B0F4-4F0F-998D-7C24FF6A1CAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -542,105 +542,6 @@
   </si>
   <si>
     <t>This test validates the end-to-end lifecycle of a professional service vertical by dynamically creating a localized "Painter" service, onboarding a new provider with comprehensive operational and banking details, and configuring specific service categories and commercial packages. The workflow ensures functional integration between the service definition and provider availability, concluding with a verification of administrative controls by updating localized metadata and successfully deactivating the service to confirm state transition integrity.</t>
-  </si>
-  <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-3.Verify Delivery Services,verify,,"//div[normalize-space()='ON-DEMAND SERVICES']"
-4.Click  Add New Services,click,,"//button[normalize-space()='Add New Services']"
-5.Enter Service Name, type, Painter{randomAlpha}&gt;&gt; serviceName, "//input[@placeholder='Service Name']"
-6.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
-7.Enter Service Name Arabic, type, دهان, "//input[@placeholder='Service Name (in Arabic)']"
-8.Enter Service Name Hindi, type, पेंटर, "//input[@placeholder='Service Name (in Hindi)']"
-9.Enter Slug, type, painter, "//input[@placeholder='Slug']"
-10.Upload Service Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file' and @accept='image/*']"
-11.wait,2000,,
-12.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-13.Select Activate,click,,"//li[@aria-label='Activate']"
-14.Open Select City Dropdown,click,,"//div[contains(@class, 'p-multiselect-label-container')]"
-15.Select {areaName},click,,"//li[contains(@aria-label, '{areaName}')]"
-16.Click  Submit,click,,"//button[normalize-space()='Submit']"
-17.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
-18.Click Home Icon ,click,,"//i[@title='Home']"
-19.Click  Providers,click,,"//button[contains(., 'Providers')]"
-20.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
-21.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
-22.Enter Provider Full Name, type, Painter{randomAlpha}&gt;&gt; painterName, "//input[@placeholder='Provider Full Name']"
-23.Upload Painter Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file']"
-24.Enter Email, type, Painter_{timestamp}@gmail.com&gt;&gt;painterEmail, "//input[@placeholder='Unique Email']"
-25.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
-26.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
-27.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
-28.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
-29.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
-30.Enter Provider Address, type, painter chennai, "//input[@placeholder='Enter provider Address']"
-31.wait,1000,,
-32.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
-33.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
-34.wait,1000,,
-35.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
-36.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
-37.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
-38.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
-39.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
-40.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
-41.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
-42.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
-43.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
-44.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
-45.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
-46.Enter Accont Holder Name, type, {painterName}, "//input[@placeholder='Account Holder Name']"
-47.Enter Payment Email Address, type, {painterEmail}, "//input[@placeholder='Email Address for Payment Notification']"
-48.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
-49.Click Save, click, , "//button[@type='submit']"
-50.Verify Sucess, verify, , "//div[@aria-label='Info']"
-51.Filter Painter List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
-52.Click  Providers,click,,"//button[normalize-space()='Category']"
-53.Click  Add New Category,click,,"//button[normalize-space()='ADD CATEGORY']"
-54.Enter Category Name, type,residential painter, "//input[@placeholder='Enter the category name']"
-55.Enter Category Name Tamil, type, குடியிருப்பு பெயிண்டர், "//input[@placeholder='Category Name (in Tamil)']"
-56.Enter Category Name Arabic, type, دهان سكني, "//input[@placeholder='Category Name (in Arabic)']"
-57.Enter Category Name Hindi, type, आवासीय पेंटर, "//input[@placeholder='Category Name (in Hindi)']"
-58.Open Category status Dropdown,click,,"//span[@aria-label='Select a category status']"
-59.Select Activate,click,,"//li[@aria-label='Active']"
-60.Upload Category Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file' and @accept='image/*']"
-61.wait,2000,,
-62.Click  Submit,click,,"//button[normalize-space()='Submit']"
-63.Filter Category Name,type,residential painter,"//input[@aria-label='Category Name Filter Input']"
-64.Click  Providers,click,,"//button[contains(., 'Providers')]"
-65.Select Provider List,click,,"//div[normalize-space()='Provider List']"
-66.Filter Painter List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
-67.Scroll Grid, tab, 7, "//input[@aria-label='Provider Name Filter Input']"
-68.Click Package Icon,click,,"//i[@class='bi bi-box-seam cursor-pointer gridIcon Navigate']"
-69.Click  Add Package,click,,"//button[normalize-space()='Add Package']"
-70.Open Category  Dropdown,click,,"//span[@aria-label='Package Category']"
-71.Select Activate,click,,"//li[@aria-label='residential painter']"
-72.Enter Package Name, type, Premium, "//input[@placeholder='Package Name']"
-73.Enter Amount, type, 1000, "//input[@placeholder='Amount Value']"
-74.Open Max Book Quantity  Dropdown,click,,"//span[@aria-label='Package Max Book Quantity']"
-75.Select 4,click,,"//li[@aria-label='4']"
-76.Open Status Dropdown,click,,"//span[@aria-label='select Status']"
-77.Select Activate,click,,"//li[@aria-label='Activate']"
-78.Enter Description, type, Premium residential painting package, "//textarea[@placeholder='Description']"
-79.Click  Submit,click,,"//button[normalize-space()='Submit']"
-80.wait,1000,,
-81.Click  back,click,,"//button[normalize-space()='Back']"
-82.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-83.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-84.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
-85.Click Edit Icon ,click,,"//i[@title='Edit']"
-86.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
-87.Enter Service Name Arabic, type, دهان, "//input[@placeholder='Service Name (in Arabic)']"
-88.Enter Service Name Hindi, type, पेंटर, "//input[@placeholder='Service Name (in Hindi)']"
-89.Scroll Grid, tab, 4, "//input[@placeholder='Service Name (in Hindi)']"
-90.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-91.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
-92.Click  Submit,click,,"//button[normalize-space()='Submit']"
-93.Click  back,click,,"//button[normalize-space()='Back']"
-94.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-95.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-96.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
-97.wait,1000,,</t>
   </si>
   <si>
     <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
@@ -1732,6 +1633,135 @@
       <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
 </t>
     </r>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
+3.Verify Delivery Services,verify,,"//div[normalize-space()='ON-DEMAND SERVICES']"
+4.Click  Add New Services,click,,"//button[normalize-space()='Add New Services']"
+5.Enter Service Name, type, Painter{randomAlpha}&gt;&gt; serviceName, "//input[@placeholder='Service Name']"
+6.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
+7.Enter Service Name Arabic, type, دهان, "//input[@placeholder='Service Name (in Arabic)']"
+8.Enter Service Name Hindi, type, पेंटर, "//input[@placeholder='Service Name (in Hindi)']"
+9.Enter Slug, type, painter, "//input[@placeholder='Slug']"
+10.Upload Service Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file' and @accept='image/*']"
+11.wait,2000,,
+12.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+13.Select Activate,click,,"//li[@aria-label='Activate']"
+14.Open Select City Dropdown,click,,"//div[contains(@class, 'p-multiselect-label-container')]"
+15.Select {areaName},click,,"//li[contains(@aria-label, '{areaName}')]"
+16.Click  Submit,click,,"//button[normalize-space()='Submit']"
+17.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
+18.Click Home Icon ,click,,"//i[@title='Home']"
+19.Click Settings ,click,,"//button[contains(., 'Settings')]"
+20.Click Requirment Document ,click,,"//div[normalize-space()='Required Document']"
+21.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
+22.Enter Name, type, Address Proof, "//input[@placeholder='Type here']"
+23.Open status Dropdown,click,,"//span[@aria-label='Status']"
+24.Select Active,click,,"//li[@aria-label='Active']"
+25.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
+26.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
+27.Click Submit ,click,,"//button[normalize-space()='Submit']"
+28.Verify Sucess, verify, , "//div[@aria-label='Info']"
+29.Filter Document List,type,Address Proof,"//input[@aria-label='Name Filter Input']"
+30.Click Settings ,click,,"//button[contains(., 'Settings')]"
+31.Click Promocode ,click,,"//div[normalize-space()='Promocode']"
+32.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
+33.Click Close ,click,,"//button[normalize-space()='Close']"
+34.Click  Providers,click,,"//button[contains(., 'Providers')]"
+35.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
+36.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
+37.Enter Provider Full Name, type, Painter{randomAlpha}&gt;&gt; painterName, "//input[@placeholder='Provider Full Name']"
+38.Upload Painter Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file']"
+39.Enter Email, type, Painter_{timestamp}@gmail.com&gt;&gt;painterEmail, "//input[@placeholder='Unique Email']"
+40.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
+41.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
+42.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
+43.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
+44.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
+45.Enter Provider Address, type, painter chennai, "//input[@placeholder='Enter provider Address']"
+46.wait,1000,,
+47.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
+48.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
+49.wait,1000,,
+50.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
+51.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
+52.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
+53.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
+54.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
+55.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
+56.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
+57.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
+58.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
+59.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
+60.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
+61.Enter Accont Holder Name, type, {painterName}, "//input[@placeholder='Account Holder Name']"
+62.Enter Payment Email Address, type, {painterEmail}, "//input[@placeholder='Email Address for Payment Notification']"
+63.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
+64.Click Save, click, , "//button[@type='submit']"
+65.Verify Sucess, verify, , "//div[@aria-label='Info']"
+66.Filter Painter List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
+67.Click  Providers,click,,"//button[contains(., 'Providers')]"
+68.Select Pending Document Providers,click,,"//div[normalize-space()='Pending Document Providers']"
+69.Filter Plumber List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
+70.Click Document Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+71. Provider Required Documents,verify,,"//div[contains(text(),'Documents')]"
+72.FilterDocumet List,type,Address Proof,"//input[@aria-label='Document Name Filter Input']"
+73.Add Address Proof,click,,"(//i[contains(@class, 'Edit')])[1]"
+74.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
+75.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+76.Click Submit, click, , "//button[normalize-space()='Submit']"
+77.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+78.FilterDocumet List,type,Address Proof,"//input[@aria-label='Document Name Filter Input']"
+79.Click Approve Store,click,,"//div[@row-index='0']//i[contains(@class, 'bi-hand-thumbs-up-fill')]"
+80.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+81.Click Back, click, , "//button[@class='buttonWidget']"
+82.Click  Providers,click,,"//button[normalize-space()='Category']"
+83.Click  Add New Category,click,,"//button[normalize-space()='ADD CATEGORY']"
+84.Enter Category Name, type,residential painter, "//input[@placeholder='Enter the category name']"
+85.Enter Category Name Tamil, type, குடியிருப்பு பெயிண்டர், "//input[@placeholder='Category Name (in Tamil)']"
+86.Enter Category Name Arabic, type, دهان سكني, "//input[@placeholder='Category Name (in Arabic)']"
+87.Enter Category Name Hindi, type, आवासीय पेंटर, "//input[@placeholder='Category Name (in Hindi)']"
+88.Open Category status Dropdown,click,,"//span[@aria-label='Select a category status']"
+89.Select Activate,click,,"//li[@aria-label='Active']"
+90.Upload Category Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file' and @accept='image/*']"
+91.wait,2000,,
+92.Click  Submit,click,,"//button[normalize-space()='Submit']"
+93.Filter Category Name,type,residential painter,"//input[@aria-label='Category Name Filter Input']"
+94.Click  Providers,click,,"//button[contains(., 'Providers')]"
+95.Select Provider List,click,,"//div[normalize-space()='Provider List']"
+96.Filter Painter List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
+97.Scroll Grid, tab, 7, "//input[@aria-label='Provider Name Filter Input']"
+98.Click Package Icon,click,,"//i[@class='bi bi-box-seam cursor-pointer gridIcon Navigate']"
+99.Click  Add Package,click,,"//button[normalize-space()='Add Package']"
+100.Open Category  Dropdown,click,,"//span[@aria-label='Package Category']"
+101.Select Activate,click,,"//li[@aria-label='residential painter']"
+102.Enter Package Name, type, Premium, "//input[@placeholder='Package Name']"
+103.Enter Amount, type, 1000, "//input[@placeholder='Amount Value']"
+104.Open Max Book Quantity  Dropdown,click,,"//span[@aria-label='Package Max Book Quantity']"
+105.Select 4,click,,"//li[@aria-label='4']"
+106.Open Status Dropdown,click,,"//span[@aria-label='select Status']"
+107.Select Activate,click,,"//li[@aria-label='Activate']"
+108.Enter Description, type, Premium residential painting package, "//textarea[@placeholder='Description']"
+109.Click  Submit,click,,"//button[normalize-space()='Submit']"
+110.wait,1000,,
+111.Click  back,click,,"//button[normalize-space()='Back']"
+112.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
+113.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
+114.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
+115.Click Edit Icon ,click,,"//i[@title='Edit']"
+116.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
+117.Enter Service Name Arabic, type, دهان, "//input[@placeholder='Service Name (in Arabic)']"
+118.Enter Service Name Hindi, type, पेंटर, "//input[@placeholder='Service Name (in Hindi)']"
+119.Scroll Grid, tab, 4, "//input[@placeholder='Service Name (in Hindi)']"
+120.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+121.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
+122.Click  Submit,click,,"//button[normalize-space()='Submit']"
+123.Click  back,click,,"//button[normalize-space()='Back']"
+124.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
+125.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
+126.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
+127.wait,1000,,</t>
   </si>
 </sst>
 </file>
@@ -2224,10 +2254,10 @@
         <v>48</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2296,7 +2326,7 @@
         <v>56</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>55</v>
@@ -2372,7 +2402,7 @@
         <v>30</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2444,7 +2474,7 @@
         <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>50</v>
@@ -2509,10 +2539,10 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2581,10 +2611,10 @@
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2653,10 +2683,10 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2725,10 +2755,10 @@
         <v>36</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2797,7 +2827,7 @@
         <v>40</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>51</v>
@@ -2869,10 +2899,10 @@
         <v>44</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
56th commit: Add Customer Test Suite Completed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5906194-B0F4-4F0F-998D-7C24FF6A1CAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5975E62-0B34-4610-AD6C-9E3AB6E2EC46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
-    <sheet name="AddCityArea" sheetId="1" r:id="rId2"/>
-    <sheet name="AddCityAdmin" sheetId="2" r:id="rId3"/>
-    <sheet name="AddAutoDriver" sheetId="3" r:id="rId4"/>
-    <sheet name="AddBikeDriver" sheetId="4" r:id="rId5"/>
-    <sheet name="AddTaxiDriver" sheetId="5" r:id="rId6"/>
-    <sheet name="AddStore" sheetId="7" r:id="rId7"/>
-    <sheet name="StoreOperations" sheetId="8" r:id="rId8"/>
-    <sheet name="StoreStatusManagement" sheetId="10" r:id="rId9"/>
-    <sheet name="AddProvider" sheetId="11" r:id="rId10"/>
-    <sheet name="ProviderServiceCategoryCreation" sheetId="12" r:id="rId11"/>
+    <sheet name="AddCustomer" sheetId="13" r:id="rId2"/>
+    <sheet name="AddCityArea" sheetId="1" r:id="rId3"/>
+    <sheet name="AddCityAdmin" sheetId="2" r:id="rId4"/>
+    <sheet name="AddAutoDriver" sheetId="3" r:id="rId5"/>
+    <sheet name="AddBikeDriver" sheetId="4" r:id="rId6"/>
+    <sheet name="AddTaxiDriver" sheetId="5" r:id="rId7"/>
+    <sheet name="AddStore" sheetId="7" r:id="rId8"/>
+    <sheet name="StoreOperations" sheetId="8" r:id="rId9"/>
+    <sheet name="StoreStatusManagement" sheetId="10" r:id="rId10"/>
+    <sheet name="AddProvider" sheetId="11" r:id="rId11"/>
+    <sheet name="ProviderServiceCategoryCreation" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="77">
   <si>
     <t>City Area</t>
   </si>
@@ -73,9 +74,6 @@
     <t>CityAdmin</t>
   </si>
   <si>
-    <t>TC_CA_02_add_city_admin</t>
-  </si>
-  <si>
     <t>SA_TS_3</t>
   </si>
   <si>
@@ -100,22 +98,10 @@
     <t>Validate that the admin can successfully add a new taxi driver by entering valid driver details and vehicle details and approve him from pendind documents by adding documents and verify he is coming in on approved drivers list.</t>
   </si>
   <si>
-    <t>TC_CA_05_add_verify_taxi_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_04_add_verify_bike_driver</t>
-  </si>
-  <si>
     <t>Validate that the admin can successfully add a new Auto driver by entering valid driver details and vehicle details and approve him from pendind documents by adding documents and verify he is coming in on approved drivers list .</t>
   </si>
   <si>
-    <t>TC_CA_03_add_verify_auto_driver</t>
-  </si>
-  <si>
     <t>SA_TS_0</t>
-  </si>
-  <si>
-    <t>TC_CA_01_add_city_area</t>
   </si>
   <si>
     <t>TC_CA_00_super_admin_login</t>
@@ -167,9 +153,6 @@
     <t>SA_TS_6</t>
   </si>
   <si>
-    <t>TC_CA_06_add_store</t>
-  </si>
-  <si>
     <t>Add New Store &amp; Approve</t>
   </si>
   <si>
@@ -182,9 +165,6 @@
     <t>Store Operations</t>
   </si>
   <si>
-    <t>TC_CA_07_store_oprerations</t>
-  </si>
-  <si>
     <t>This test validates the end-to-end lifecycle of a delivery store's operational setup, focusing on catalog management, financial provisioning, and logistics readiness. The workflow begins by navigating through the delivery services hierarchy to locate a specific store, where it performs a menu expansion by adding new products with precise attributes including pricing, imagery, and discount logic. Following inventory setup, the script executes a comprehensive financial audit by performing both credit and debit transactions within the store’s wallet to ensure backend accounting synchronization. Finally, the test secures the store's fulfillment capabilities by registering a new private driver, capturing personal and vehicle details alongside document uploads, thereby ensuring the merchant is fully prepared to manage products, finances, and last-mile delivery.</t>
   </si>
   <si>
@@ -194,9 +174,6 @@
     <t>Store Status Mangement</t>
   </si>
   <si>
-    <t>TC_CA_08_store_status_management</t>
-  </si>
-  <si>
     <t>This test validates the complete lifecycle of a store within a delivery services platform, beginning with the creation of a new store (using dynamic timestamps for uniqueness) and the configuration of its operational settings, bank details, and timing. It then navigates through various administrative states, including uploading and verifying compliance documents, moving the store from a pending status to approved, and then testing the blocking/unblocking functionality. Finally, the script validates the rejection workflow by moving a store to the rejected list with a specific reason, ensuring that status transitions and data filtering across the "Store List," "Pending," and "Blocked" modules are functioning as expected.</t>
   </si>
   <si>
@@ -204,9 +181,6 @@
   </si>
   <si>
     <t>Add New Provider &amp; Approve</t>
-  </si>
-  <si>
-    <t>TC_CA_09_add_provider</t>
   </si>
   <si>
     <t>This test validates the complete administrative workflow for registering and authorizing a new provider within the Plumbers. The automation navigates to the Add Providers module to dynamically create a unique pumbler profile, populating operational data including provider service radius, service time, address and banking details. Following creation, the script transitions to the Compliance phase, where it filters for the new pumbler in the "Pending Documents" list, automates the upload of regulatory files, and sets document expiry dates. The workflow then triggers  the Final Approval and verifying the pumbler successful migration to the active provider List, ensuring end-to-end data consistency and functional status transitions. Following verification, the script executes a comprehensive financial audit by performing both credit and debit transactions within the store’s wallet to ensure backend accounting synchronization.</t>
@@ -463,9 +437,6 @@
   </si>
   <si>
     <t>SA_TS_10</t>
-  </si>
-  <si>
-    <t>TC_CA_10_provider_new_service&amp;category_creation</t>
   </si>
   <si>
     <t>Add New Provider Service &amp;  Category</t>
@@ -1762,6 +1733,127 @@
 125.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
 126.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
 127.wait,1000,,</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>TC_CA_01_add_customer</t>
+  </si>
+  <si>
+    <t>TC_CA_02_add_city_area</t>
+  </si>
+  <si>
+    <t>TC_CA_03_add_city_admin</t>
+  </si>
+  <si>
+    <t>TC_CA_04_add_verify_auto_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_05_add_verify_bike_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_06_add_verify_taxi_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_07_add_store</t>
+  </si>
+  <si>
+    <t>TC_CA_08_store_oprerations</t>
+  </si>
+  <si>
+    <t>TC_CA_09_store_status_management</t>
+  </si>
+  <si>
+    <t>TC_CA_10_add_provider</t>
+  </si>
+  <si>
+    <t>SA_TS_11</t>
+  </si>
+  <si>
+    <t>TC_CA_11_provider_new_service&amp;category_creation</t>
+  </si>
+  <si>
+    <t>Validate the end-to-end creation of a Customer.</t>
+  </si>
+  <si>
+    <t>1. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+2.Click  Add Customers,click,,"//span[normalize-space()='Add customers']"
+3. Verify Add Customer Heading,verify,,"//div[normalize-space()='Add Customer']"
+4.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "//label[contains(., 'Customer Full Name')]/following::input[1]"
+5.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "//input[@type='email']"
+6.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+7.Enter Video Call Limit, type, 60, "//label[contains(., 'User Used Video Call Limit in Minutes')]/following::input[1]"
+8.Open Gender,click,,"//span[@aria-label='select gender']"
+9.Select Male,click,,"//li[@aria-label='Male']"
+10.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "//input[@type='file' and @accept='image/*']"
+11.Click Submit, click, , "//button[normalize-space()='Submit']"
+12.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+13. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+14. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+15.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
+16. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+17.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+18.Click Edit Icon ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+19.Click Close, click, , "//button[normalize-space()='Close']"
+20.Click Wallet Icon ,click,,"//i[@title='Wallet']"
+21.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
+22.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
+23.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+24.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
+25.Click Submit, click, , "//button[normalize-space()='Submit']"
+26.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+27.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
+28.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
+29.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+30.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
+31.Click Submit, click, , "//button[normalize-space()='Submit']"
+32.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+33. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+34. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+35.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
+36. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+37.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+38.Click Loyalty Points Icon,click,,"//i[@title='Loyalty Points']"
+38.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
+39.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
+40.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
+41.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+42.Select Add Points,click,,"//li[@role='option'][contains(.,'Add Points')]"
+43.Enter Points, type, 30, "//input[@placeholder='Enter Points']"
+44.Click Submit, click, , "//button[normalize-space()='Submit']"
+45.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+46.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
+47.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
+48.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
+49.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+50.Select Deduct Points,click,,"//li[@role='option'][contains(.,'Deduct Points')]"
+51.Enter Points, type, 10, "//input[@placeholder='Enter Points']"
+52.Click Submit, click, , "//button[normalize-space()='Submit']"
+53.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+54. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+55. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+56.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
+57. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+58.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+59.Click Disable  Icon,click,,"//i[@title='Disable']"
+60.Click Disable  User  Yes,click,,"//button[normalize-space()='Yes']"
+61.Disable Reason,type,Client Complaints,"//textarea[@id='swal2-textarea']"
+62.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+63.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+64. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+65. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+66.Click  Blocked Customers,click,,"//span[normalize-space()='Blocked customers']"
+67.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+68.Scroll Grid, tab, 10, "//input[@aria-label='Customer Name Filter Input']"
+69.Click Enable  Icon,click,,"//i[@title='Status']"
+70.Click Enable  Yes,click,,"//button[normalize-space()='Yes']"
+71. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+72. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+73.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
+74. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+75.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+76.wait,1000,,</t>
   </si>
 </sst>
 </file>
@@ -2167,22 +2259,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2201,6 +2293,78 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57207608-1AD9-408F-B018-55A141C9A651}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F63FB6C5-854C-4D7D-9CEB-846B4D7D2F52}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2242,22 +2406,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2272,7 +2436,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{319ADEF0-2336-4246-BBC3-461C4994D500}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2314,22 +2478,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2345,6 +2509,82 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46ECEE02-404F-4AF1-8311-95653C3B218B}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="31.6640625" customWidth="1"/>
+    <col min="5" max="5" width="53.21875" customWidth="1"/>
+    <col min="6" max="6" width="29" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2387,22 +2627,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2420,7 +2660,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9466ABF-463D-46B5-A321-4AC4765F1CE7}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2462,22 +2702,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
+        <v>65</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -2485,7 +2725,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7A75689-8D07-4A99-AA90-48806EECB90F}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2530,19 +2770,19 @@
         <v>13</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2557,7 +2797,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4197A722-266E-4219-9B46-8F4D56D7D7A1}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2599,22 +2839,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2629,7 +2869,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{790BFFF3-3BE5-4068-A6FF-6214BEDD72BA}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2671,22 +2911,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>18</v>
-      </c>
       <c r="C2" s="7" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2701,7 +2941,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C456A73-57BC-411E-B40E-DADED30882CB}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2743,22 +2983,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2773,7 +3013,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86A4538F-421E-4B0B-A965-0382A5BEF523}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2815,22 +3055,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2843,76 +3083,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57207608-1AD9-408F-B018-55A141C9A651}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="26.77734375" customWidth="1"/>
-    <col min="4" max="4" width="34.109375" customWidth="1"/>
-    <col min="5" max="5" width="69.33203125" customWidth="1"/>
-    <col min="6" max="6" width="31.77734375" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="8"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
57th commit: Recrussive Multi Sheet Test Running Implemented
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5975E62-0B34-4610-AD6C-9E3AB6E2EC46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E01377E0-D7D6-4F7D-8806-AF4655A26B74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -440,76 +440,6 @@
   </si>
   <si>
     <t>Add New Provider Service &amp;  Category</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The AddCityArea test suite must be always executed before this test. This is critical because the ProviderCategoryCreation process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
-RunSheet: AddCityArea
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
   </si>
   <si>
     <t>This test validates the end-to-end lifecycle of a professional service vertical by dynamically creating a localized "Painter" service, onboarding a new provider with comprehensive operational and banking details, and configuring specific service categories and commercial packages. The workflow ensures functional integration between the service definition and provider availability, concluding with a verification of administrative controls by updating localized metadata and successfully deactivating the service to confirm state transition integrity.</t>
@@ -720,110 +650,6 @@
 50.Click Doc Icon,click,,"//i[@title='Document']"
 51.Click Eye Icon,click,,"//i[@title='View']"
 52.wait,1000,,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-3.Verify Delivery Services,verify,,"//div[contains(text(),'ON-DEMAND SERVICES')]"
-4.Click Home Icon Plumbers,click,,"//div[@role='row'][.//span[text()='Plumbers']]//i[@title='Home']"
-5.Verify Plumbers Summary,verify,,"//div[contains(text(),'Plumbers Summary')]"
-6.Click  Providers,click,,"//button[contains(., 'Providers')]"
-7.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
-8.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
-9.Enter Provider Full Name, type, Plumber{randomAlpha}&gt;&gt; plumberName, "//input[@placeholder='Provider Full Name']"
-10.Upload Plumber Image, uploadfile, "src/main/resources/test-data/plumber.jpg", "//input[@type='file']"
-11.Enter Email, type, Plumber_{timestamp}@gmail.com&gt;&gt;plumberEmail, "//input[@placeholder='Unique Email']"
-12.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
-13.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
-14.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
-15.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
-16.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
-17..Enter Provider Address, type, plumber chennai, "//input[@placeholder='Enter provider Address']"
-18.wait,1000,,
-19.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
-20.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
-21.wait,1000,,
-22.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
-23.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
-24.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
-25.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
-26.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
-27.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
-28.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
-29.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
-30.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
-31.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
-32.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
-33.Enter Accont Holder Name, type, {plumberName}, "//input[@placeholder='Account Holder Name']"
-34.Enter Payment Email Address, type, {plumberEmail}, "//input[@placeholder='Email Address for Payment Notification']"
-35.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
-36.Click Save, click, , "//button[@type='submit']"
-37.Verify Sucess, verify, , "//div[@aria-label='Info']"
-38.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-39.Click  Providers,click,,"//button[contains(., 'Providers')]"
-40.Select Pending Document Providers,click,,"//div[normalize-space()='Pending Document Providers']"
-41.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-42.Click Document Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-43. Provider Required Documents,verify,,"//div[contains(text(),'Documents')]"
-44.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
-45.Add Address Proof,click,,"(//i[contains(@class, 'Edit')])[1]"
-46.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-47.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-48.Click Submit, click, , "//button[normalize-space()='Submit']"
-49.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-50.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
-51.Click Approve Store,click,,"//div[@row-index='0']//i[contains(@class, 'bi-hand-thumbs-up-fill')]"
-52.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-53.Click Back, click, , "//button[@class='buttonWidget']"
-54.Click  Providers,click,,"//button[contains(., 'Providers')]"
-55.Select Provider List,click,,"//div[normalize-space()='Provider List']"
-56.Verify Approved Provider,verify,,"//div[normalize-space()='Approved Plumbers Service Providers']"
-57.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-58.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-59.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
-60.Click Back, click, , "//button[@class='buttonWidget']"
-61.Verify Approved Provider,verify,,"//div[normalize-space()='Approved Plumbers Service Providers']"
-62.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-63.Scroll Grid, tab, 11, "//input[@aria-label='Provider Name Filter Input']"
-64.Click Wallet Icon,click,,"//i[@class='bi bi-cash-stack cursor-pointer gridIcon Navigate']"
-65.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
-66.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
-67.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-68.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
-69.Click Submit, click, , "//button[normalize-space()='Submit']"
-70.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-71.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
-72.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
-73.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-74.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
-75.Click Submit, click, , "//button[normalize-space()='Submit']"
-76.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-77.Click Back, click, , "//button[normalize-space()='Back']"
-78.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-79.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-80.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
-81.Click Reject Document,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
-82.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-83.Rejection Reason,type,document insufficent,"//textarea[@id='swal2-textarea']"
-84..Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-85.Click Back, click, , "//button[@class='buttonWidget']"
-86.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-87.Scroll Grid, tab, 13, "//input[@aria-label='Provider Name Filter Input']"
-88.Click Block Provider,click,,"//i[@title='Block Provider']"
-89.Click Block  Yes,click,,"//button[normalize-space()='Yes']"
-90. Blocking Reason,type,customer complaints,"//textarea[@id='swal2-textarea']"
-91.Click block  Yes,click,,"//button[normalize-space()='Yes']"
-92.Click  Providers,click,,"//button[contains(., 'Providers')]"
-93.Select Blocked Providers,click,,"//div[contains(text(), 'Blocked Providers')]"
-94.Verify Blocked Provider,verify,,"//div[normalize-space()='Blocked Plumbers Service Providers']"
-95.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-96.Scroll Grid, tab, 12, "//input[@aria-label='Provider Name Filter Input']"
-97.Click Unblock Provider,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-98.Click  Providers,click,,"//button[contains(., 'Providers')]"
-99.Select Provider List,click,,"//div[contains(text(), 'Provider List')]"
-100.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-101.wait,1000,,
-</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
@@ -1606,135 +1432,6 @@
     </r>
   </si>
   <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-3.Verify Delivery Services,verify,,"//div[normalize-space()='ON-DEMAND SERVICES']"
-4.Click  Add New Services,click,,"//button[normalize-space()='Add New Services']"
-5.Enter Service Name, type, Painter{randomAlpha}&gt;&gt; serviceName, "//input[@placeholder='Service Name']"
-6.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
-7.Enter Service Name Arabic, type, دهان, "//input[@placeholder='Service Name (in Arabic)']"
-8.Enter Service Name Hindi, type, पेंटर, "//input[@placeholder='Service Name (in Hindi)']"
-9.Enter Slug, type, painter, "//input[@placeholder='Slug']"
-10.Upload Service Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file' and @accept='image/*']"
-11.wait,2000,,
-12.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-13.Select Activate,click,,"//li[@aria-label='Activate']"
-14.Open Select City Dropdown,click,,"//div[contains(@class, 'p-multiselect-label-container')]"
-15.Select {areaName},click,,"//li[contains(@aria-label, '{areaName}')]"
-16.Click  Submit,click,,"//button[normalize-space()='Submit']"
-17.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
-18.Click Home Icon ,click,,"//i[@title='Home']"
-19.Click Settings ,click,,"//button[contains(., 'Settings')]"
-20.Click Requirment Document ,click,,"//div[normalize-space()='Required Document']"
-21.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
-22.Enter Name, type, Address Proof, "//input[@placeholder='Type here']"
-23.Open status Dropdown,click,,"//span[@aria-label='Status']"
-24.Select Active,click,,"//li[@aria-label='Active']"
-25.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
-26.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
-27.Click Submit ,click,,"//button[normalize-space()='Submit']"
-28.Verify Sucess, verify, , "//div[@aria-label='Info']"
-29.Filter Document List,type,Address Proof,"//input[@aria-label='Name Filter Input']"
-30.Click Settings ,click,,"//button[contains(., 'Settings')]"
-31.Click Promocode ,click,,"//div[normalize-space()='Promocode']"
-32.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
-33.Click Close ,click,,"//button[normalize-space()='Close']"
-34.Click  Providers,click,,"//button[contains(., 'Providers')]"
-35.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
-36.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
-37.Enter Provider Full Name, type, Painter{randomAlpha}&gt;&gt; painterName, "//input[@placeholder='Provider Full Name']"
-38.Upload Painter Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file']"
-39.Enter Email, type, Painter_{timestamp}@gmail.com&gt;&gt;painterEmail, "//input[@placeholder='Unique Email']"
-40.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
-41.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
-42.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
-43.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
-44.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
-45.Enter Provider Address, type, painter chennai, "//input[@placeholder='Enter provider Address']"
-46.wait,1000,,
-47.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
-48.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
-49.wait,1000,,
-50.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
-51.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
-52.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
-53.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
-54.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
-55.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
-56.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
-57.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
-58.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
-59.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
-60.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
-61.Enter Accont Holder Name, type, {painterName}, "//input[@placeholder='Account Holder Name']"
-62.Enter Payment Email Address, type, {painterEmail}, "//input[@placeholder='Email Address for Payment Notification']"
-63.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
-64.Click Save, click, , "//button[@type='submit']"
-65.Verify Sucess, verify, , "//div[@aria-label='Info']"
-66.Filter Painter List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
-67.Click  Providers,click,,"//button[contains(., 'Providers')]"
-68.Select Pending Document Providers,click,,"//div[normalize-space()='Pending Document Providers']"
-69.Filter Plumber List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
-70.Click Document Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-71. Provider Required Documents,verify,,"//div[contains(text(),'Documents')]"
-72.FilterDocumet List,type,Address Proof,"//input[@aria-label='Document Name Filter Input']"
-73.Add Address Proof,click,,"(//i[contains(@class, 'Edit')])[1]"
-74.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-75.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-76.Click Submit, click, , "//button[normalize-space()='Submit']"
-77.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-78.FilterDocumet List,type,Address Proof,"//input[@aria-label='Document Name Filter Input']"
-79.Click Approve Store,click,,"//div[@row-index='0']//i[contains(@class, 'bi-hand-thumbs-up-fill')]"
-80.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-81.Click Back, click, , "//button[@class='buttonWidget']"
-82.Click  Providers,click,,"//button[normalize-space()='Category']"
-83.Click  Add New Category,click,,"//button[normalize-space()='ADD CATEGORY']"
-84.Enter Category Name, type,residential painter, "//input[@placeholder='Enter the category name']"
-85.Enter Category Name Tamil, type, குடியிருப்பு பெயிண்டர், "//input[@placeholder='Category Name (in Tamil)']"
-86.Enter Category Name Arabic, type, دهان سكني, "//input[@placeholder='Category Name (in Arabic)']"
-87.Enter Category Name Hindi, type, आवासीय पेंटर, "//input[@placeholder='Category Name (in Hindi)']"
-88.Open Category status Dropdown,click,,"//span[@aria-label='Select a category status']"
-89.Select Activate,click,,"//li[@aria-label='Active']"
-90.Upload Category Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file' and @accept='image/*']"
-91.wait,2000,,
-92.Click  Submit,click,,"//button[normalize-space()='Submit']"
-93.Filter Category Name,type,residential painter,"//input[@aria-label='Category Name Filter Input']"
-94.Click  Providers,click,,"//button[contains(., 'Providers')]"
-95.Select Provider List,click,,"//div[normalize-space()='Provider List']"
-96.Filter Painter List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
-97.Scroll Grid, tab, 7, "//input[@aria-label='Provider Name Filter Input']"
-98.Click Package Icon,click,,"//i[@class='bi bi-box-seam cursor-pointer gridIcon Navigate']"
-99.Click  Add Package,click,,"//button[normalize-space()='Add Package']"
-100.Open Category  Dropdown,click,,"//span[@aria-label='Package Category']"
-101.Select Activate,click,,"//li[@aria-label='residential painter']"
-102.Enter Package Name, type, Premium, "//input[@placeholder='Package Name']"
-103.Enter Amount, type, 1000, "//input[@placeholder='Amount Value']"
-104.Open Max Book Quantity  Dropdown,click,,"//span[@aria-label='Package Max Book Quantity']"
-105.Select 4,click,,"//li[@aria-label='4']"
-106.Open Status Dropdown,click,,"//span[@aria-label='select Status']"
-107.Select Activate,click,,"//li[@aria-label='Activate']"
-108.Enter Description, type, Premium residential painting package, "//textarea[@placeholder='Description']"
-109.Click  Submit,click,,"//button[normalize-space()='Submit']"
-110.wait,1000,,
-111.Click  back,click,,"//button[normalize-space()='Back']"
-112.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-113.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-114.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
-115.Click Edit Icon ,click,,"//i[@title='Edit']"
-116.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
-117.Enter Service Name Arabic, type, دهان, "//input[@placeholder='Service Name (in Arabic)']"
-118.Enter Service Name Hindi, type, पेंटर, "//input[@placeholder='Service Name (in Hindi)']"
-119.Scroll Grid, tab, 4, "//input[@placeholder='Service Name (in Hindi)']"
-120.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-121.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
-122.Click  Submit,click,,"//button[normalize-space()='Submit']"
-123.Click  back,click,,"//button[normalize-space()='Back']"
-124.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-125.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-126.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
-127.wait,1000,,</t>
-  </si>
-  <si>
     <t>Customer</t>
   </si>
   <si>
@@ -1854,6 +1551,325 @@
 74. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
 75.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
 76.wait,1000,,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
+3.Verify Delivery Services,verify,,"//div[contains(text(),'ON-DEMAND SERVICES')]"
+4.Filter service List,type,Plumbers,"//input[@aria-label='Services Filter Input']"
+5.Click Home Icon Plumbers,click,,"//div[@role='row'][.//span[text()='Plumbers']]//i[@title='Home']"
+6.Verify Plumbers Summary,verify,,"//div[contains(text(),'Plumbers Summary')]"
+7.Click  Providers,click,,"//button[contains(., 'Providers')]"
+8.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
+9.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
+10.Enter Provider Full Name, type, Plumber{randomAlpha}&gt;&gt; plumberName, "//input[@placeholder='Provider Full Name']"
+11.Upload Plumber Image, uploadfile, "src/main/resources/test-data/plumber.jpg", "//input[@type='file']"
+12.Enter Email, type, Plumber_{timestamp}@gmail.com&gt;&gt;plumberEmail, "//input[@placeholder='Unique Email']"
+13.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
+14.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
+15.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
+16.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
+17.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
+18.Enter Provider Address, type, plumber chennai, "//input[@placeholder='Enter provider Address']"
+19.wait,1000,,
+20.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
+21.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
+22.wait,1000,,
+23.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
+24.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
+25.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
+26.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
+27.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
+28.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
+29.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
+30.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
+31.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
+32.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
+33.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
+34.Enter Accont Holder Name, type, {plumberName}, "//input[@placeholder='Account Holder Name']"
+35.Enter Payment Email Address, type, {plumberEmail}, "//input[@placeholder='Email Address for Payment Notification']"
+36.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
+37.Click Save, click, , "//button[@type='submit']"
+38.Verify Sucess, verify, , "//div[@aria-label='Info']"
+39.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+40.Click  Providers,click,,"//button[contains(., 'Providers')]"
+41.Select Pending Document Providers,click,,"//div[normalize-space()='Pending Document Providers']"
+42.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+43.Click Document Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+44. Provider Required Documents,verify,,"//div[contains(text(),'Documents')]"
+45.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
+46.Add Address Proof,click,,"(//i[contains(@class, 'Edit')])[1]"
+47.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
+48.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+49.Click Submit, click, , "//button[normalize-space()='Submit']"
+50.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+51.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
+52.Click Approve Store,click,,"//div[@row-index='0']//i[contains(@class, 'bi-hand-thumbs-up-fill')]"
+53.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+54.Click Back, click, , "//button[@class='buttonWidget']"
+55.Click  Providers,click,,"//button[contains(., 'Providers')]"
+56.Select Provider List,click,,"//div[normalize-space()='Provider List']"
+57.Verify Approved Provider,verify,,"//div[normalize-space()='Approved Plumbers Service Providers']"
+58.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+59.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+60.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
+61.Click Back, click, , "//button[@class='buttonWidget']"
+62.Verify Approved Provider,verify,,"//div[normalize-space()='Approved Plumbers Service Providers']"
+63.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+64.Scroll Grid, tab, 11, "//input[@aria-label='Provider Name Filter Input']"
+65.Click Wallet Icon,click,,"//i[@class='bi bi-cash-stack cursor-pointer gridIcon Navigate']"
+66.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
+67.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
+68.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+69.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
+70.Click Submit, click, , "//button[normalize-space()='Submit']"
+71.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+72.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
+73.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
+74.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+75.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
+76.Click Submit, click, , "//button[normalize-space()='Submit']"
+77.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+78.Click Back, click, , "//button[normalize-space()='Back']"
+79.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+80.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+81.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
+82.Click Reject Document,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
+83.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+84.Rejection Reason,type,document insufficent,"//textarea[@id='swal2-textarea']"
+85..Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+86.Click Back, click, , "//button[@class='buttonWidget']"
+87.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+88.Scroll Grid, tab, 13, "//input[@aria-label='Provider Name Filter Input']"
+89.Click Block Provider,click,,"//i[@title='Block Provider']"
+90.Click Block  Yes,click,,"//button[normalize-space()='Yes']"
+91. Blocking Reason,type,customer complaints,"//textarea[@id='swal2-textarea']"
+92.Click block  Yes,click,,"//button[normalize-space()='Yes']"
+93.Click  Providers,click,,"//button[contains(., 'Providers')]"
+94.Select Blocked Providers,click,,"//div[contains(text(), 'Blocked Providers')]"
+95.Verify Blocked Provider,verify,,"//div[normalize-space()='Blocked Plumbers Service Providers']"
+96.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+97.Scroll Grid, tab, 12, "//input[@aria-label='Provider Name Filter Input']"
+98.Click Unblock Provider,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+99.Click  Providers,click,,"//button[contains(., 'Providers')]"
+100.Select Provider List,click,,"//div[contains(text(), 'Provider List')]"
+101.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
+102.wait,1000,,
+</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The AddCityArea test suite must be always executed before this test. This is critical because the ProviderCategoryCreation process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
+RunSheet: AddCustomer,AddCityArea
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
+3.Verify Delivery Services,verify,,"//div[normalize-space()='ON-DEMAND SERVICES']"
+4.Click  Add New Services,click,,"//button[normalize-space()='Add New Services']"
+5.Enter Service Name, type, Painter{randomAlpha}&gt;&gt; serviceName, "//input[@placeholder='Service Name']"
+6.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
+7.Enter Service Name Arabic, type, دهان, "//input[@placeholder='Service Name (in Arabic)']"
+8.Enter Service Name Hindi, type, पेंटर, "//input[@placeholder='Service Name (in Hindi)']"
+9.Enter Slug, type, painter, "//input[@placeholder='Slug']"
+10.Upload Service Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file' and @accept='image/*']"
+11.wait,2000,,
+12.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+13.Select Activate,click,,"//li[@aria-label='Activate']"
+14.Open Select City Dropdown,click,,"//div[contains(@class, 'p-multiselect-label-container')]"
+15.Select {areaName},click,,"//li[contains(@aria-label, '{areaName}')]"
+16.Click  Submit,click,,"//button[normalize-space()='Submit']"
+17.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
+18.Click Home Icon ,click,,"//i[@title='Home']"
+19.Click Settings ,click,,"//button[contains(., 'Settings')]"
+20.Click Requirment Document ,click,,"//div[normalize-space()='Required Document']"
+21.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
+22.Enter Name, type, Address Proof, "//input[@placeholder='Type here']"
+23.Open status Dropdown,click,,"//span[@aria-label='Status']"
+24.Select Active,click,,"//li[@aria-label='Active']"
+25.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
+26.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
+27.Click Submit ,click,,"//button[normalize-space()='Submit']"
+28.Verify Sucess, verify, , "//div[@aria-label='Info']"
+29.Filter Document List,type,Address Proof,"//input[@aria-label='Name Filter Input']"
+30.Click Settings ,click,,"//button[contains(., 'Settings')]"
+31.Click Promocode ,click,,"//div[normalize-space()='Promocode']"
+32.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
+33.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
+34.Select User,click,,"//li[@aria-label='{customerName}']"
+35.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
+35.Enter Code Name, type, GoldMember001, "//input[@placeholder='Code Name']"
+36.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
+37.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
+38.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
+39.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
+40.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
+41.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
+42.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
+43.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
+44.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
+45.Click Submit ,click,,"//button[normalize-space()='Submit']"
+46.Verify Sucess, verify, , "//div[@aria-label='Info']"
+47.Filter PromoCode List,type,GoldMember001,"//input[@aria-label='Promocode Filter Input']"
+48.Click  Providers,click,,"//button[contains(., 'Providers')]"
+49.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
+50.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
+51.Enter Provider Full Name, type, Painter{randomAlpha}&gt;&gt; painterName, "//input[@placeholder='Provider Full Name']"
+52.Upload Painter Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file']"
+53.Enter Email, type, Painter_{timestamp}@gmail.com&gt;&gt;painterEmail, "//input[@placeholder='Unique Email']"
+54.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
+55.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
+56.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
+57.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
+58.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
+59.Enter Provider Address, type, painter chennai, "//input[@placeholder='Enter provider Address']"
+60.wait,1000,,
+61.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
+62.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
+63.wait,1000,,
+64.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
+65.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
+66.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
+67.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
+68.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
+69.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
+70.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
+71.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
+72.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
+73.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
+74.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
+75.Enter Accont Holder Name, type, {painterName}, "//input[@placeholder='Account Holder Name']"
+76.Enter Payment Email Address, type, {painterEmail}, "//input[@placeholder='Email Address for Payment Notification']"
+77.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
+78.Click Save, click, , "//button[@type='submit']"
+79.Verify Sucess, verify, , "//div[@aria-label='Info']"
+80.Filter Painter List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
+81.Click  Providers,click,,"//button[contains(., 'Providers')]"
+82.Select Pending Document Providers,click,,"//div[normalize-space()='Pending Document Providers']"
+83.Filter Plumber List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
+84.Click Document Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+85. Provider Required Documents,verify,,"//div[contains(text(),'Documents')]"
+86.FilterDocumet List,type,Address Proof,"//input[@aria-label='Document Name Filter Input']"
+87.Add Address Proof,click,,"(//i[contains(@class, 'Edit')])[1]"
+88.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
+89.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+90.Click Submit, click, , "//button[normalize-space()='Submit']"
+91.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+92.FilterDocumet List,type,Address Proof,"//input[@aria-label='Document Name Filter Input']"
+93.Click Approve Store,click,,"//div[@row-index='0']//i[contains(@class, 'bi-hand-thumbs-up-fill')]"
+94.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+95.Click Back, click, , "//button[@class='buttonWidget']"
+96.Click  Providers,click,,"//button[normalize-space()='Category']"
+97.Click  Add New Category,click,,"//button[normalize-space()='ADD CATEGORY']"
+98.Enter Category Name, type,residential painter, "//input[@placeholder='Enter the category name']"
+99.Enter Category Name Tamil, type, குடியிருப்பு பெயிண்டர், "//input[@placeholder='Category Name (in Tamil)']"
+100.Enter Category Name Arabic, type, دهان سكني, "//input[@placeholder='Category Name (in Arabic)']"
+101.Enter Category Name Hindi, type, आवासीय पेंटर, "//input[@placeholder='Category Name (in Hindi)']"
+102.Open Category status Dropdown,click,,"//span[@aria-label='Select a category status']"
+103.Select Activate,click,,"//li[@aria-label='Active']"
+104.Upload Category Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file' and @accept='image/*']"
+105.wait,2000,,
+106.Click  Submit,click,,"//button[normalize-space()='Submit']"
+107.Filter Category Name,type,residential painter,"//input[@aria-label='Category Name Filter Input']"
+108.Click  Providers,click,,"//button[contains(., 'Providers')]"
+109.Select Provider List,click,,"//div[normalize-space()='Provider List']"
+110.Filter Painter List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
+111.Scroll Grid, tab, 7, "//input[@aria-label='Provider Name Filter Input']"
+112.Click Package Icon,click,,"//i[@class='bi bi-box-seam cursor-pointer gridIcon Navigate']"
+113.Click  Add Package,click,,"//button[normalize-space()='Add Package']"
+114.Open Category  Dropdown,click,,"//span[@aria-label='Package Category']"
+115.Select Activate,click,,"//li[@aria-label='residential painter']"
+116.Enter Package Name, type, Premium, "//input[@placeholder='Package Name']"
+117.Enter Amount, type, 1000, "//input[@placeholder='Amount Value']"
+118.Open Max Book Quantity  Dropdown,click,,"//span[@aria-label='Package Max Book Quantity']"
+119.Select 4,click,,"//li[@aria-label='4']"
+120.Open Status Dropdown,click,,"//span[@aria-label='select Status']"
+121.Select Activate,click,,"//li[@aria-label='Activate']"
+122.Enter Description, type, Premium residential painting package, "//textarea[@placeholder='Description']"
+123.Click  Submit,click,,"//button[normalize-space()='Submit']"
+124.wait,1000,,
+125.Click  back,click,,"//button[normalize-space()='Back']"
+126.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
+127.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
+128.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
+129.Click Edit Icon ,click,,"//i[@title='Edit']"
+130.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
+131.Enter Service Name Arabic, type, دهان, "//input[@placeholder='Service Name (in Arabic)']"
+132.Enter Service Name Hindi, type, पेंटर, "//input[@placeholder='Service Name (in Hindi)']"
+133.Scroll Grid, tab, 4, "//input[@placeholder='Service Name (in Hindi)']"
+134.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+135.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
+136.Click  Submit,click,,"//button[normalize-space()='Submit']"
+137.Click  back,click,,"//button[normalize-space()='Back']"
+138.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
+139.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
+140.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
+141.wait,1000,,</t>
   </si>
 </sst>
 </file>
@@ -2340,16 +2356,16 @@
         <v>35</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>36</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2412,16 +2428,16 @@
         <v>38</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>39</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2478,22 +2494,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2554,19 +2570,19 @@
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2633,7 +2649,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>26</v>
@@ -2642,7 +2658,7 @@
         <v>25</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2708,13 +2724,13 @@
         <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>41</v>
@@ -2773,16 +2789,16 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2845,16 +2861,16 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2917,16 +2933,16 @@
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2989,16 +3005,16 @@
         <v>29</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>30</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3061,13 +3077,13 @@
         <v>32</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>42</v>

</xml_diff>

<commit_message>
58th commit: Delievery Service Complete Lifecycle Test Suite Implemented
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E01377E0-D7D6-4F7D-8806-AF4655A26B74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDD1D2D9-E568-4E54-879E-EC5DC14D4004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -23,8 +23,9 @@
     <sheet name="AddStore" sheetId="7" r:id="rId8"/>
     <sheet name="StoreOperations" sheetId="8" r:id="rId9"/>
     <sheet name="StoreStatusManagement" sheetId="10" r:id="rId10"/>
-    <sheet name="AddProvider" sheetId="11" r:id="rId11"/>
-    <sheet name="ProviderServiceCategoryCreation" sheetId="12" r:id="rId12"/>
+    <sheet name="DeliveryServiceCompleteTest" sheetId="14" r:id="rId11"/>
+    <sheet name="AddProvider" sheetId="11" r:id="rId12"/>
+    <sheet name="ProviderServiceCompleteTest" sheetId="12" r:id="rId13"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="83">
   <si>
     <t>City Area</t>
   </si>
@@ -440,9 +441,6 @@
   </si>
   <si>
     <t>Add New Provider Service &amp;  Category</t>
-  </si>
-  <si>
-    <t>This test validates the end-to-end lifecycle of a professional service vertical by dynamically creating a localized "Painter" service, onboarding a new provider with comprehensive operational and banking details, and configuring specific service categories and commercial packages. The workflow ensures functional integration between the service definition and provider availability, concluding with a verification of administrative controls by updating localized metadata and successfully deactivating the service to confirm state transition integrity.</t>
   </si>
   <si>
     <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
@@ -1462,13 +1460,7 @@
     <t>TC_CA_09_store_status_management</t>
   </si>
   <si>
-    <t>TC_CA_10_add_provider</t>
-  </si>
-  <si>
     <t>SA_TS_11</t>
-  </si>
-  <si>
-    <t>TC_CA_11_provider_new_service&amp;category_creation</t>
   </si>
   <si>
     <t>Validate the end-to-end creation of a Customer.</t>
@@ -1658,79 +1650,27 @@
 </t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The AddCityArea test suite must be always executed before this test. This is critical because the ProviderCategoryCreation process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
-RunSheet: AddCustomer,AddCityArea
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
+    <t>TC_CA_10_delivery_service_complete_test</t>
+  </si>
+  <si>
+    <t>TC_CA_11_add_provider</t>
+  </si>
+  <si>
+    <t>TC_CA_12_provider_service_full_lifecycle_test</t>
+  </si>
+  <si>
+    <t>Add New Delivery Service &amp;  Category</t>
+  </si>
+  <si>
+    <t>SA_TS_12</t>
+  </si>
+  <si>
+    <t>This test validates the end-to-end lifecycle of a professional service vertical by dynamically creating a localized "Painter" service featuring multi-language support in Tamil, Arabic, and Hindi. The workflow spans from initial service definition and the configuration of governance controls—such as mandatory Address Proof documents and promotional campaigns—to a comprehensive Provider Onboarding phase involving banking details, operational scheduling, and document approval. The process concludes by verifying functional integrity through the assignment of Premium commercial packages and administrative metadata updates, ultimately confirming state transition integrity by successfully deactivating the service.</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-3.Verify Delivery Services,verify,,"//div[normalize-space()='ON-DEMAND SERVICES']"
+2.Click Provider Services,click,,"//h2[contains(text(), 'Provider Services')]"
+3.Verify Provider Services,verify,,"//div[normalize-space()='ON-DEMAND SERVICES']"
 4.Click  Add New Services,click,,"//button[normalize-space()='Add New Services']"
 5.Enter Service Name, type, Painter{randomAlpha}&gt;&gt; serviceName, "//input[@placeholder='Service Name']"
 6.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
@@ -1870,6 +1810,320 @@
 139.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
 140.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
 141.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[@class='fa-solid fa-user-shield iconstyle']"
+2.Click Delivery Services,click,,"//h2[normalize-space()='Delivery Services']"
+3.Verify Delivery Services,verify,,"//div[normalize-space()='DELIVERY SERVICES']"
+4.Click  Add Service Category,click,,"//button[normalize-space()='Add Service Category']"
+5.Enter Category Name, type, milk Delivery{randomAlpha}&gt;&gt; deliveryName, "//input[@placeholder='Category Name']"
+6.Enter Slug, type, Milk Delivery, "//input[@placeholder='Slug']"
+7.Upload Category Image, uploadfile, "src/main/resources/test-data/milkman.jpg", "//input[@type='file' and @accept='image/*']"
+8.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+9.Select Activate,click,,"//li[@aria-label='Activate']"
+10.Open Category Flow Dropdown,click,,"//label[contains(., 'Category Flow')]/following-sibling::p-dropdown"
+11.Select default flow(food-delivery),click,,"//li[@aria-label='default flow(food-delivery)']"
+12.Enter Delivery Name Tamil, type,பால்காரர், "//input[@placeholder='Enter in Tamil']"
+13.Enter Delivery Name Arabic, type, لبّان, "//input[@placeholder='Enter in Arabic']"
+14.Enter Delivery Name Hindi, type, दूधवाला, "//input[@placeholder='Enter in Hindi']"
+15.Click  Submit,click,,"//button[normalize-space()='Submit']"
+16.Verify Sucess, verify, , "//div[@aria-label='Info']"
+17.Filter Services List,type,{deliveryName},"//input[@aria-label='Services Filter Input']"
+18.Click Home Icon ,click,,"//i[@title='Home']"
+19.Click Settings ,click,,"//button[contains(., 'Settings')]"
+20.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
+21.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
+22.Enter Name, type, Address Proof, "//input[@placeholder='Type here']"
+23.Open status Dropdown,click,,"//span[@aria-label='select status']"
+24.Select Active,click,,"//li[@aria-label='Active']"
+25.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
+26.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
+27.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
+28.Click  Require Proof Number,click,,"//div[./div[contains(text(), 'Require Proof Number')]]//input"
+29.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
+30.Click Submit ,click,,"//button[normalize-space()='Submit']"
+31.Verify Sucess, verify, , "//div[@aria-label='Info']"
+32.Filter Document List,type,Address Proof,"//input[@aria-label='Name Filter Input']"
+33.wait,2000,,
+33.Click Settings ,click,,"//button[contains(., 'Settings')]"
+34.Click Promocode ,click,,"//div[normalize-space()='Promocode']"
+35.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
+36.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
+37.Select User,click,,"//li[@aria-label='{customerName}']"
+38.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
+39.Enter Code Name, type, GoldMember001, "//input[@placeholder='Code Name']"
+40.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
+41.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
+42.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
+43.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
+44.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
+45.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
+46.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
+47.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
+48.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
+49.Click Submit ,click,,"//button[normalize-space()='Submit']"
+50.Verify Sucess, verify, , "//div[@aria-label='Info']"
+51.Filter PromoCode List,type,GoldMember001,"//input[@aria-label='promocode Filter Input']"
+52.wait,2000,,
+53.Click Settings ,click,,"//button[contains(., 'Settings')]"
+54.Click Service Settings ,click,,"//div[normalize-space()='Service Settings']"
+55.Enter Driver Serach Radius, type, 50, "//span[contains(text(), 'Driver search Radius')]/ancestor::app-input//input"
+56.Open Tax Type Dropdown,click,,"//span[@aria-label='Select Tax Type']"
+57.Select Amount,click,,"//li[@aria-label='Amount']"
+58.Enter Tax, type, 20, "//span[contains(text(), 'Tax')]/ancestor::app-input//input"
+59.Open Platform Fee Type Dropdown,click,,"//span[@aria-label='Seelct Type']"
+60.Select Amount,click,,"//li[@aria-label='Amount']"
+61.Enter Platform Fee, type, 20, "//span[contains(text(), 'Platform Fee')]/ancestor::app-input//input"
+62.Enter Cancel Charge (in %):, type, 20, "//span[contains(text(), 'Cancel Charge (in %):')]/ancestor::app-input//input"
+63.Enter Driver Accept Timeout (in Second):, type, 20, "//span[contains(text(), 'Driver Accept Timeout (in Second):')]/ancestor::app-input//input"
+64.Click Submit ,click,,"//button[normalize-space()='Submit']"
+65.Verify Sucess, verify, , "//div[@aria-label='Info']"
+66.Click  Stores,click,,"//button[contains(., 'Stores')]"
+67.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
+68.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Add Store')]"
+69.Enter Store Name, type, amul_{timestamp} &gt;&gt; milkStore, "//input[@placeholder='Store Name']"
+70.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
+71.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
+72.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
+73. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
+74.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
+75.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
+76.Enter Short Description, type, amul taste of india, "//input[@placeholder="Type here"]"
+77.Upload Banner Image, uploadfile, "src/main/resources/test-data/amulbanner.jpg", "//input[@type='file']"
+78.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
+79.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
+80.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
+81.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
+82.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+83..Enter Store Address, type, Amul chennai, "//input[@placeholder='Search location']"
+84.wait,1000,,
+85.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
+86.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
+87.wait,1000,,
+88.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
+89.Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
+90.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
+91.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
+92.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
+93.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
+94.Enter Contact Person Full Name, type, storeowner_{timestamp} &gt;&gt; storeOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
+95.Enter Email, type, amul_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
+96.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
+97.Upload Store Image, uploadfile, "src/main/resources/test-data/milkbooth.jpeg", "(//input[@type='file'])[2]"
+98.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
+99.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
+100.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
+101.Enter Accont Holder Name, type, {storeOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
+102.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
+103.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
+104.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
+105.Enter From Time, type, 100000, "(//label[contains(.,'From Time')]/following-sibling::input)[1]"
+106.Enter To Time, type, 220000, "(//label[contains(.,'To Time')]/following-sibling::input)[1]"
+107.Submit Add Store,click,,"//button[normalize-space()='Submit']"
+108. Verify Success Message,verify,,"//div[@aria-label='Info']"
+109.Click  Stores,click,,"//button[contains(., 'Stores')]"
+110.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+111.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
+112.Filter Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
+113.Click  Stores,click,,"//button[contains(., 'Stores')]"
+114.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
+115.Verify Add Store,verify,,"//div[normalize-space()='Pending Documents Store']"
+116.Filter Pending Document Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
+117.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+118.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
+119. Store Required Documents,verify,,"//div[contains(text(),'Documents')]"
+120.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+121.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
+122.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+123.Click Submit, click, , "//button[normalize-space()='Submit']"
+124.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+125.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+126.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+127.Click Back, click, , "//button[@class='buttonWidget']"
+128.Click  Stores,click,,"//button[contains(., 'Stores')]"
+129.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+130.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
+131.Filter Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
+132.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+133.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
+134.Click Back, click, , "//button[@class='buttonWidget']"
+135.Click Category, click, , "//button[normalize-space()='Category']"
+136.Click  Add New Category,click,,"//button[normalize-space()='Add Category']"
+137.Enter Category Name, type,curd, "//span[contains(text(), 'Category Name')]/ancestor::app-input//input"
+138.Enter Category Name Arabic, type, رائب, "//span[contains(text(), 'Language Value (in Arabic)')]/ancestor::app-input//input"
+139.Enter Category Name Tamil, type, தயிர், "//span[contains(text(), 'Language Value (in Tamil)')]/ancestor::app-input//input"
+140.Enter Category Name Hindi, type, दही, "//span[contains(text(), 'Language Value (in Hindi)')]/ancestor::app-input//input"
+141.Open Category status Dropdown,click,,"//span[@aria-label='status']"
+142.Select Active,click,,"//li[@aria-label='active']"
+143.Upload Category Image, uploadfile, "src/main/resources/test-data/curd.jpeg", "//input[@type='file' and @accept='image/*']"
+144.wait,2000,,
+145.Enter Slug Name, type, curd, "//span[text()='Slug']/ancestor::app-input//input"
+146.Click  Submit,click,,"//button[normalize-space()='Submit']"
+147.Verify Success Message,verify,,"//div[@aria-label='Info']"
+148.Filter Category Name,type,curd,"//input[@aria-label='Category Name Filter Input']"
+149.Click  Stores,click,,"//button[contains(., 'Stores')]"
+150.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+151.Filter Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
+152.Scroll Grid, tab, 9, "//input[@aria-label='Store Name Filter Input']"
+153.Click Product Icon,click,,"//i[@title='Product View']"
+154.Click  Add  Products,click,,"//button[normalize-space()='Add Products']"
+155.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[1]"
+156.Select curd,click,,"//li[@role='option'][contains(.,'curd')]"
+157.wait,1000,,
+158.Click badge,click,,"//i[@class='fa-solid fa-user-shield iconstyle']"
+159.Click Delivery Services,click,,"//h2[normalize-space()='Delivery Services']"
+160.Verify Delivery Services,verify,,"//div[normalize-space()='DELIVERY SERVICES']"
+161.Filter Services List,type,{deliveryName},"//input[@aria-label='Services Filter Input']"
+162.Click Edit Icon ,click,,"//i[@title='Edit']"
+163.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+164.wait,1000,,
+164.Select Dectivate,click,,"//li[@aria-label='Deactivate']"
+165.Click Submit ,click,,"//button[normalize-space()='Submit']"
+166.Filter Services List,type,{deliveryName},"//input[@aria-label='Services Filter Input']"
+167.wait,1000,,</t>
+  </si>
+  <si>
+    <t>This test validates the end-to-end lifecycle of a localized delivery service by dynamically creating a "Milk Delivery" vertical, onboarding a store provider with comprehensive operational, banking, and scheduling details, and configuring necessary administrative prerequisites including mandatory document requirements, promotional codes, and global service settings (taxes, fees, and search radii). The workflow ensures full functional integration by verifying the provider's document approval process and the successful addition of localized product categories like "Curd" (translated in Tamil, Arabic, and Hindi). The test concludes by performing an administrative state transition, deactivating the service to confirm systemic integrity and the proper functioning of administrative controls across the entire service ecosystem.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The AddCustomer test suite must be always executed before this test. This is critical because the DelieveryServiceCompleteTest process utilizes the dynamic {customerName} variable generated and stored during the AddCustomer creation phase.
+RunSheet:AddCustomer
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The AddCustomer,AddCityArea test suite must be always executed before this test. This is critical because the ProviderServiceCompleteTest process utilizes the dynamic {areaName},{customerName} variable generated and stored during the AddCityArea and AddCustomer creation phase.
+RunSheet: AddCustomer,AddCityArea
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2356,16 +2610,16 @@
         <v>35</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>36</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2381,6 +2635,78 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73960651-1493-478A-BEDA-A31CF297E315}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F63FB6C5-854C-4D7D-9CEB-846B4D7D2F52}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2422,22 +2748,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>39</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2452,7 +2778,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{319ADEF0-2336-4246-BBC3-461C4994D500}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2494,22 +2820,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B2" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>44</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>45</v>
+        <v>77</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2570,19 +2896,19 @@
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>60</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2649,7 +2975,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>26</v>
@@ -2658,7 +2984,7 @@
         <v>25</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2724,13 +3050,13 @@
         <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>41</v>
@@ -2789,16 +3115,16 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2861,16 +3187,16 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2933,16 +3259,16 @@
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3005,16 +3331,16 @@
         <v>29</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>30</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3077,13 +3403,13 @@
         <v>32</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>42</v>

</xml_diff>

<commit_message>
59th commit: Transport Service Complete Lifecycle Test Suite Implemented
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDD1D2D9-E568-4E54-879E-EC5DC14D4004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD43FB45-8218-4D83-8BD6-6AF59D997736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="10" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -20,12 +20,13 @@
     <sheet name="AddAutoDriver" sheetId="3" r:id="rId5"/>
     <sheet name="AddBikeDriver" sheetId="4" r:id="rId6"/>
     <sheet name="AddTaxiDriver" sheetId="5" r:id="rId7"/>
-    <sheet name="AddStore" sheetId="7" r:id="rId8"/>
-    <sheet name="StoreOperations" sheetId="8" r:id="rId9"/>
-    <sheet name="StoreStatusManagement" sheetId="10" r:id="rId10"/>
-    <sheet name="DeliveryServiceCompleteTest" sheetId="14" r:id="rId11"/>
-    <sheet name="AddProvider" sheetId="11" r:id="rId12"/>
-    <sheet name="ProviderServiceCompleteTest" sheetId="12" r:id="rId13"/>
+    <sheet name="TransportServiceCompleteTest" sheetId="15" r:id="rId8"/>
+    <sheet name="AddStore" sheetId="7" r:id="rId9"/>
+    <sheet name="StoreOperations" sheetId="8" r:id="rId10"/>
+    <sheet name="StoreStatusManagement" sheetId="10" r:id="rId11"/>
+    <sheet name="DeliveryServiceCompleteTest" sheetId="14" r:id="rId12"/>
+    <sheet name="AddProvider" sheetId="11" r:id="rId13"/>
+    <sheet name="ProviderServiceCompleteTest" sheetId="12" r:id="rId14"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="89">
   <si>
     <t>City Area</t>
   </si>
@@ -1449,15 +1450,6 @@
   </si>
   <si>
     <t>TC_CA_06_add_verify_taxi_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_07_add_store</t>
-  </si>
-  <si>
-    <t>TC_CA_08_store_oprerations</t>
-  </si>
-  <si>
-    <t>TC_CA_09_store_status_management</t>
   </si>
   <si>
     <t>SA_TS_11</t>
@@ -1648,15 +1640,6 @@
 101.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
 102.wait,1000,,
 </t>
-  </si>
-  <si>
-    <t>TC_CA_10_delivery_service_complete_test</t>
-  </si>
-  <si>
-    <t>TC_CA_11_add_provider</t>
-  </si>
-  <si>
-    <t>TC_CA_12_provider_service_full_lifecycle_test</t>
   </si>
   <si>
     <t>Add New Delivery Service &amp;  Category</t>
@@ -2124,6 +2107,282 @@
       <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
 </t>
     </r>
+  </si>
+  <si>
+    <t>Add New Transport Service ,Vehicle Type &amp;  driver</t>
+  </si>
+  <si>
+    <t>TC_CA_08_add_store</t>
+  </si>
+  <si>
+    <t>TC_CA_09_store_oprerations</t>
+  </si>
+  <si>
+    <t>TC_CA_10_store_status_management</t>
+  </si>
+  <si>
+    <t>TC_CA_11_delivery_service_complete_test</t>
+  </si>
+  <si>
+    <t>TC_CA_12_add_provider</t>
+  </si>
+  <si>
+    <t>SA_TS_13</t>
+  </si>
+  <si>
+    <t>TC_CA_13_provider_service_full_lifecycle_test</t>
+  </si>
+  <si>
+    <t>TC_CA_07_transport_service_complete_test</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddCustomer,AddCityArea test suite must be always executed before this test. This is critical because the TransportServiceCompleteTest process utilizes the dynamic {areaName},{customerName} variable generated and stored during the AddCityArea and AddCustomer creation phase.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AddCustomer,AddCityArea</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>This test validates the end-to-end operational lifecycle of a comprehensive Transport Service ecosystem by dynamically creating a localized "Bus Ride" category with multilingual support and city-specific accessibility. The workflow integrates complex administrative configurations, including the establishment of tiered vehicle types (e.g., Volvo) with granular fare structures, promotional code management for targeted user segments, and global service parameters such as driver search radii, tax implications, and platform fees. Furthermore, the test verifies the robustness of the onboarding pipeline by simulating driver registration—complete with banking and vehicle documentation—and exercising the mandatory document approval framework to transition a driver from "Pending" to "Approved" status. The cycle concludes by establishing loyalty program parameters and performing a systemic deactivation of the transport category, ensuring that administrative controls effectively manage service availability and data integrity across the entire transport infrastructure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+2. Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+3.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
+4.Click  Add Category,click,,"//button[normalize-space()='Add Category']"
+5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "//input[@placeholder='Service Name']"
+6.Enter Service Name Arabic, type, رحلة بالحافلة, "//input[@placeholder='Service Name (in Arabic)']"
+7.Enter Slug, type, Bus Ride, "//input[@placeholder='Slug']"
+8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "//input[@type='file' and @accept='image/*']"
+9.wait,2000,,
+10.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+11.Select Activate,click,,"//li[@aria-label='Activate']"
+12.Open Select City Dropdown,click,,"//span[text()='Select City']/ancestor::app-drop-down//div[contains(@class, 'p-multiselect-label-container')]"
+13.Select {areaName},click,,"//li[@aria-label='{areaName}']"
+14.Click  Submit,click,,"//button[normalize-space()='Submit']"
+15.Verify Sucess, verify, , "//div[@aria-label='Info']"
+16.wait,2000,,
+17.Click  back,click,,"//button[normalize-space()='Back']"
+18.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+19.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+20.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
+21.Click Home Icon ,click,,"//i[@title='Home']"
+22.Click Settings ,click,,"//button[contains(., 'Settings')]"
+23.Click Vehicle Type,click,,"//div[normalize-space()='Vehicle Type']"
+24.Click Add Vehicle Type,click,,"//button[normalize-space()='Add Vehicle Type']"
+25.Enter Vehicle Type Name, type, volvo, "//input[@placeholder='Type here']"
+26.Enter Cost For Km, type, 150, "//input[@placeholder='Cost For Km']"
+27.Enter Time Fare Per Min, type,10, "//input[@placeholder='Time Fare Per Min']"
+28.Enter Base fare, type,100, "//input[@placeholder='Base fare']"
+29.Enter Min Fare Amount, type,50, "//input[@placeholder='Min Fare Amount']"
+30.Enter Rental Cost For Km, type,30, "//input[@placeholder='Rental Cost For Km']"
+31.Enter Rental Amount For 1 Hour, type,50, "//input[@placeholder='Rental Amount For 1 Hour']"
+32.Enter Rental Km Limit For 1 Hour, type,50, "//input[@placeholder='Rental Km Limit For 1 Hour']"
+33.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "//app-image-upload//input[@type='file' and @accept='image/*']"
+34.Click Surcharge Time Checkbox, click, , "//div[text()='EveryDay']/preceding-sibling::mat-checkbox"
+35.Enter From Time, type, 100000, "//app-time-picker//input[@type='time']"
+36.Enter To Time, type, 220000, "(//app-time-picker//input[@type='time'])[2]"
+37.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+38.Select Active,click,,"//li[@aria-label='Active']"
+39.Click  Submit,click,,"//button[normalize-space()='Submit']"
+40.Verify Sucess, verify, , "//div[@aria-label='Info']"
+41.Click Settings ,click,,"//button[contains(., 'Settings')]"
+42.Click Promocode,click,,"//div[normalize-space()='Promocode']"
+43.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
+44.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
+45.Select User,click,,"//li[@aria-label='{customerName}']"
+46.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
+47.Enter Code Name, type, GoldMember001, "//input[@placeholder='Code Name']"
+48.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
+49.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
+50.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
+51.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
+52.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
+53.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
+54.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
+55.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
+56.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
+57.Click Submit ,click,,"//button[normalize-space()='Submit']"
+58.Verify Sucess, verify, , "//div[@aria-label='Info']"
+59.wait,2000,,
+60.Click Settings ,click,,"//button[contains(., 'Settings')]"
+61.Click Service Settings ,click,,"//div[normalize-space()='Service Setting']"
+62.Enter Driver Accept Timeout, type, 60, "//label[contains(., "Driver Accept Timeout")]/following::input[1]"
+63.Enter Driver Serach Radius, type, 50, "//label[contains(., "Driver Search Radius")]/following::input[1]"
+64.Open Tax Type Dropdown,click,,"//span[@aria-label='Select Tax Rype']"
+65.Select Amount,click,,"//li[@aria-label='Amount']"
+66.Enter Tax, type, 20, "//label[contains(., 'Tax')]/following::input[1]"
+67.Open Platform Fee Type Dropdown,click,,"//label[contains(., 'Platform Fee Type')]/following::span[@role='combobox']"
+68.Select Amount,click,,"//li[@aria-label='Amount']"
+69.Enter Platform Fee, type, 20, "//label[contains(., "Platform Fee")]/following::input[1]"
+70.Click Submit ,click,,"//button[normalize-space()='Submit']"
+71.Verify Sucess, verify, , "//div[@aria-label='Info']"
+72.wait,1000,,
+73.Click Settings ,click,,"//button[contains(., 'Settings')]"
+74.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
+75.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
+76.Enter Name, type, Driving License, "//label[contains(., 'Name')]/following::input[1]"
+77.Open status Dropdown,click,,"//label[contains(., 'Status')]/following::div[contains(@class, 'p-dropdown')]"
+78.Select Active,click,,"//li[@aria-label='Active']"
+79.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
+80.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
+81.Click  Require Proof Number,click,,"//div[./div[contains(text(), 'Require Proof Number')]]//input"
+82.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
+83.Click Submit ,click,,"//button[normalize-space()='Submit']"
+84.Verify Sucess, verify, , "//div[@aria-label='Info']"
+85.Filter Document List,type,Driving License,"//input[@aria-label='Name Filter Input']"
+86.wait,1000,,
+88.Click Settings ,click,,"//button[contains(., 'Settings')]"
+89.Click Customer Loyalty Settings,click,,"//div[text()=' Customer Loyalty Settings ']"
+90.Open status Allow Customer loyalty points,click,,"//label[contains(., 'Allow Customer loyalty points')]/following::div[contains(@class, 'p-dropdown')]"
+91.Select ON,click,,"//li[@role='option']//span[text()='ON']"
+92.Enter Minimum order amount for eligibility to redeem loyalty points, type, 25,"//label[contains(., 'Minimum order amount for eligibility to redeem loyalty points')]/following::input[1]"
+93.Enter Loyalty points redeem per order (in %) (% of order amount), type, 10,"//label[contains(., 'Loyalty points redeem per order (in %) (% of order amount)')]/following::input[1]"
+94.Enter Loyalty points per default currency (for ex. $1 = 10 points), type, 5,"//label[contains(., 'Loyalty points per default currency (for ex. $1 = 10 points)')]/following::input[1]"
+95.Click Submit ,click,,"//button[normalize-space()='Submit']"
+96.Verify Sucess, verify, , "//div[@aria-label='Info']"
+97.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+98.Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+99.Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+100.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+101.Select Bus Ride Option,click,,"//span[normalize-space()='{transportName}']"
+102.Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+103.Enter Driver Name, type, busdriver_{timestamp} &gt;&gt; busDriverName, "//label[contains(.,'Full Name')]/following::input[1]"
+104.Enter Email, type, busdriver_{timestamp}@gmail.com&gt;&gt;busEmail, "//label[contains(.,'Email')]/following::input[1]"
+105.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+106.Upload Profile Image, uploadfile, "src/main/resources/test-data/busdriver.jpg", "//input[@type='file']"
+107.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+108.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+109.Select  volvo Option,click,,"//li[@role='option']//span[text()='volvo']"
+110.Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+111.Enter Vehicle Company, type, tata, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+112.Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+113. Enter Model Name, type, deisel, "//label[contains(.,'Model Name')]/following::input[1]"
+114.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/busvolvo.jpeg", "(//input[@type='file'])[2]"
+115. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+116.Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+117.Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+118.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+119.Enter Account Holder Name, type, {busDriverName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+120.Enter Payment Email Address, type, {busEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+121.Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+122.Click Submit, click, , "//button[contains(.,'Submit')]"
+123.Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+124.Wait for Toast to hide, wait, 1000,
+125.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+126.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+127.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+128.Filter by Name,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
+129.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+130.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+131.FilterDocumet List,type,Driving License,"//input[@aria-label='Document Name Filter Input']"
+132.Add Driving License,click,,"//i[@title='Edit']"
+133.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+134.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+135.Click Submit, click, , "//button[normalize-space()='Submit']"
+136.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+137.Click Approve Driver,click,,"//i[@title='Approve']"
+138.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+139.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+140.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+141.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+142.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+143.Filter Approved Driver,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
+144.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+145.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+146.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
+147.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
+148.Click Edit Icon ,click,,"//i[@title='Edit']"
+149.Scroll Grid, tab, 5, "//input[@placeholder='Service Name']"
+150.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+151.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
+152.Click  Submit,click,,"//button[normalize-space()='Submit']"
+153.Verify Sucess, verify, , "//div[@aria-label='Info']"
+154.wait,2000,,
+</t>
   </si>
 </sst>
 </file>
@@ -2563,6 +2822,78 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86A4538F-421E-4B0B-A965-0382A5BEF523}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57207608-1AD9-408F-B018-55A141C9A651}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2604,13 +2935,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>35</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>36</v>
@@ -2634,7 +2965,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73960651-1493-478A-BEDA-A31CF297E315}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2676,22 +3007,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2706,7 +3037,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F63FB6C5-854C-4D7D-9CEB-846B4D7D2F52}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2748,19 +3079,19 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>39</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>57</v>
@@ -2778,7 +3109,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{319ADEF0-2336-4246-BBC3-461C4994D500}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2820,22 +3151,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>44</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2902,10 +3233,10 @@
         <v>59</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>52</v>
@@ -3284,6 +3615,79 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4DB4E5D-EBF5-4B6A-BF83-7934D70C5535}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="38" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C456A73-57BC-411E-B40E-DADED30882CB}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3325,13 +3729,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>30</v>
@@ -3353,76 +3757,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86A4538F-421E-4B0B-A965-0382A5BEF523}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="26.77734375" customWidth="1"/>
-    <col min="4" max="4" width="34.109375" customWidth="1"/>
-    <col min="5" max="5" width="69.33203125" customWidth="1"/>
-    <col min="6" max="6" width="31.77734375" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="8"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
61th commit: Test Data Cleanup Implemented
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD43FB45-8218-4D83-8BD6-6AF59D997736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F2D75D5-BB7B-4C50-99D8-79CD03D65142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="10" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="11" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -27,6 +27,7 @@
     <sheet name="DeliveryServiceCompleteTest" sheetId="14" r:id="rId12"/>
     <sheet name="AddProvider" sheetId="11" r:id="rId13"/>
     <sheet name="ProviderServiceCompleteTest" sheetId="12" r:id="rId14"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId15"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="95">
   <si>
     <t>City Area</t>
   </si>
@@ -116,34 +117,6 @@
   </si>
   <si>
     <t>Verify successful authentication of the Super Admin role using valid credentials and Dashboard access validation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-2. Click City area menu,click,,"//span[normalize-space()='City area']"
-3. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
-4. Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
-5. Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
-6. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
-7. Open Status Dropdown,click,,"//span[@aria-label='select status']"
-8. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-9. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
-10. Click Submit,click,,"//button[normalize-space()='Submit']"
-11. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
-12. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
-13. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
-14. Click Add Category,click,,"//button[normalize-space()='Add Category']"
-15. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
-16. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
-17. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
-18. Click close,click,,"//button[normalize-space()='Close']"
-19. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-20. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-21. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
-22. Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
-23. Open Select City Dropdown,click,,"//select[@id='cityId']"
-24. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-25. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
-</t>
   </si>
   <si>
     <t>Validate the end-to-end creation of a City Area, including status configuration and polygon mapping. Verify data persistence by ensuring the new area is correctly listed and available for selection in 'City Wise Manage Services' in ' Transport Service ' and 'City Admin' modules.</t>
@@ -2384,12 +2357,174 @@
 154.wait,2000,,
 </t>
   </si>
+  <si>
+    <t>SA_TS_14</t>
+  </si>
+  <si>
+    <t>Clean The Test Data Created During Test Run</t>
+  </si>
+  <si>
+    <t>TC_CA_14_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>This test phase ensures the long-term stability and performance of the QA environment by executing a systematic Automated Data Cleanup strategy. Leveraging localized SQL Hooks with built-in safety firewalls, the workflow identifies and removes dynamically generated test artifacts—including unique City Areas, Provider profiles, and administrative accounts—created during the regression suite. By targeting specific records using variable-driven WHERE clauses, the script maintains database referential integrity, prevents record duplication in subsequent runs, and ensures the test environment remains in a pristine, 'ready-state' for continuous integration</t>
+  </si>
+  <si>
+    <t>1.Remove Test Area,sql delete,,"DELETE FROM we1.admin_area_list WHERE name = '{areaName}';"
+2.wait,2000,,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+2. Click City area menu,click,,"//span[normalize-space()='City area']"
+3. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
+4. Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
+5. Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
+6. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
+7. Open Status Dropdown,click,,"//span[@aria-label='select status']"
+8. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+9. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
+10. Click Submit,click,,"//button[normalize-space()='Submit']"
+11. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
+12. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
+13. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
+14. Click Add Category,click,,"//button[normalize-space()='Add Category']"
+15. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
+16. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
+17. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
+18. Click close,click,,"//button[normalize-space()='Close']"
+19. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+20. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+21. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
+22. Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
+23. Open Select City Dropdown,click,,"//select[@id='cityId']"
+24. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
+25. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
+</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CRITICAL SYSTEM WARNING: DATABASE INTEGRITY PROTOCOL</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-----------------------------------------</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">This sheet contains SQL Hooks that execute directly against the we1 Production/Staging database. DO NOT modify the SQL syntax, remove variable placeholders (e.g., {areaName}), or edit the WHERE clauses.
+Unauthorized changes may result in irreversible data loss or database corruption. If modifications are required, please contact the Automation Lead or the Database Administrator.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PASSWORD TO EDIT SHEET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> :eit6190
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.
+RunSheet: SuperAdminLogin
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2409,6 +2544,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2803,7 +2946,7 @@
         <v>23</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2863,22 +3006,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2935,22 +3078,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3007,22 +3150,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3079,22 +3222,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>39</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3151,22 +3294,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>84</v>
-      </c>
       <c r="D2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>72</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3178,6 +3321,80 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="n2KwI2T0nM4kUyp7LiUODpwAG/galVyQSDtsZl0yUO+rjA55NBZcPk6XHtPhEPr+7rDS1I7x7D4NXk32F3GmoA==" saltValue="GAfl83kbCDLkZxzinmefRw==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3227,19 +3444,19 @@
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="D2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3306,16 +3523,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3381,16 +3598,16 @@
         <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -3446,16 +3663,16 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3518,16 +3735,16 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3584,22 +3801,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3656,22 +3873,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3729,22 +3946,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
61th commit: Test Data Cleanup Implemented On Existing Frame Work
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F2D75D5-BB7B-4C50-99D8-79CD03D65142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA7C2B5A-73CC-4484-9D74-B97A6F10A87D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="11" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -461,330 +461,6 @@
 42. Verify Success Message,verify,,"//div[@aria-label='Info']"
 43.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
 </t>
-  </si>
-  <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-6. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-7. Enter Driver Name, type, autodriver_{timestamp} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-8. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
-9. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-10. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-11. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-12.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-13.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
-14. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-15.Enter Vehicle Company, type, bajaj, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-16. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-17. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-18. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-19. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-20. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-21. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-22. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-23. Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-24. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-25. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-26. Click Submit, click, , "//button[contains(.,'Submit')]"
-27. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-28. Wait for Toast to hide, wait, 1000,
-29.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-31.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-32.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-33.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-34. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-35.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-36.Add Driving License,click,,"//i[@title='Edit']"
-37.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-38.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-39.Click Submit, click, , "//button[normalize-space()='Submit']"
-40.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-41.Click Approve Driver,click,,"//i[@title='Approve']"
-42.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-43.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-44.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-45.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-46.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-47.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-48.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-49.Click Doc Icon,click,,"//i[@title='Document']"
-50.Click Eye Icon,click,,"//i[@title='View']"
-51.wait,1000,,</t>
-  </si>
-  <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-3. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-4. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-5.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-6.Select Bike Ride Option,click,,"//span[normalize-space()='Bike Ride']"
-7. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-8. Enter Driver Name, type, bikedriver_{timestamp} &gt;&gt; bikeName, "//label[contains(.,'Full Name')]/following::input[1]"
-9. Enter Email, type, bikedriver_{timestamp}@gmail.com&gt;&gt;bikeEmail, "//label[contains(.,'Email')]/following::input[1]"
-10. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-11. Upload Profile Image, uploadfile, "src/main/resources/test-data/bikedriver.jpg", "//input[@type='file']"
-12. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-13.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-14.Select  Scooter Option,click,,"//li[@role='option']//span[text()='Scooter']"
-15. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-16.Enter Vehicle Company, type, honda, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-17. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
-18. Enter Model Name, type, activa, "//label[contains(.,'Model Name')]/following::input[1]"
-19. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/bike.jpg", "(//input[@type='file'])[2]"
-20. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-21. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-22. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-23. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-24. Enter Account Holder Name, type, {bikeName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-25. Enter Payment Email Address, type, {bikeEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-26. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-27. Click Submit, click, , "//button[contains(.,'Submit')]"
-28. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-29. Wait for Toast to hide, wait, 1000,
-30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-31.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-32.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-33.Filter by Name,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
-34.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-35. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-36.FilterDocumet List,type,Vehicle Permit Copy,"//input[@aria-label='Document Name Filter Input']"
-37.Add Vehicle Permit Copy,click,,"//i[@title='Edit']"
-38.Upload Vehicle Permit Copy, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-39.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-40.Click Submit, click, , "//button[normalize-space()='Submit']"
-41.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-42.Click Approve Driver,click,,"//i[@title='Approve']"
-43.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-44.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-46.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-47.Approved Drivers List,verify,,"//div[contains(text(),' Approved Drivers List')]"
-48.Filter Approved Driver,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
-49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-50.Click Doc Icon,click,,"//i[@title='Document']"
-51.Click Eye Icon,click,,"//i[@title='View']"
-52.wait,1000,,</t>
-  </si>
-  <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-3. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-4. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-5.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-6.Select Taxi Ride Option,click,,"//span[normalize-space()='Taxi Ride']"
-7. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-8. Enter Driver Name, type, taxidriver_{timestamp} &gt;&gt; taxiName, "//label[contains(.,'Full Name')]/following::input[1]"
-9. Enter Email, type, taxidriver_{timestamp}@gmail.com&gt;&gt;taxiEmail, "//label[contains(.,'Email')]/following::input[1]"
-10. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-11. Upload Profile Image, uploadfile, "src/main/resources/test-data/taxidriver.jpg", "//input[@type='file']"
-12. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-13.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-14.Select  Suv Option,click,,"//li[@role='option']//span[text()='SUV']"
-15. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-16.Enter Vehicle Company, type, toyota, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-17. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
-18. Enter Model Name, type, etios, "//label[contains(.,'Model Name')]/following::input[1]"
-19.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/taxi.jpg", "(//input[@type='file'])[2]"
-20. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-21. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-22. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-23. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-24. Enter Account Holder Name, type, {taxiName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-25. Enter Payment Email Address, type, {taxiEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-26. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-27. Click Submit, click, , "//button[contains(.,'Submit')]"
-28. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-29. Wait for Toast to hide, wait, 1000,
-30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-31.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-32.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-33.Filter by Name,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
-34.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-35. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-36.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-37.Add Driving License,click,,"//i[@title='Edit']"
-38.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-39.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-40.Click Submit, click, , "//button[normalize-space()='Submit']"
-41.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-42.Click Approve Driver,click,,"//i[@title='Approve']"
-43.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-44.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-46.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-47.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-48.Filter Approved Driver,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
-49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-50.Click Doc Icon,click,,"//i[@title='Document']"
-51.Click Eye Icon,click,,"//i[@title='View']"
-52.wait,1000,,</t>
-  </si>
-  <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
-3.Verify Delivery Services,verify,,"//div[contains(text(),' DELIVERY SERVICES')]"
-4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
-5.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
-6.Click  Stores,click,,"//button[contains(., 'Stores')]"
-7.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
-8.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Add Store')]"
-9.Enter Store Name, type, bilal_{timestamp} &gt;&gt; storeName, "//input[@placeholder='Store Name']"
-10.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
-11.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
-12.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
-13. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
-14.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
-15.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
-16.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
-17.Upload Banner Image, uploadfile, "src/main/resources/test-data/kfcbanner.jpg", "//input[@type='file']"
-18.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
-19.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
-20.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
-21.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
-22.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-23..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
-24.wait,1000,,
-25.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
-26.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
-27.wait,1000,,
-28.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
-29.Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
-30.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
-31.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
-32.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
-33.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
-34.Enter Contact Person Full Name, type, storeowner_{timestamp} &gt;&gt; storeOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
-35.Enter Email, type, kfc_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
-36.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
-37.Upload Store Image, uploadfile, "src/main/resources/test-data/kfcstore.jpg", "(//input[@type='file'])[2]"
-38.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
-39.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
-40.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
-41.Enter Accont Holder Name, type, {storeOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
-42.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
-43.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
-44.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
-45.Enter From Time, type, 100000, "(//label[contains(.,'From Time')]/following-sibling::input)[1]"
-46.Enter To Time, type, 220000, "(//label[contains(.,'To Time')]/following-sibling::input)[1]"
-47.Submit Add Store,click,,"//button[normalize-space()='Submit']"
-48. Verify Success Message,verify,,"//div[@aria-label='Info']"
-49.Click  Stores,click,,"//button[contains(., 'Stores')]"
-50.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-51.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-52.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-53.Click  Stores,click,,"//button[contains(., 'Stores')]"
-54.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
-55.Verify Add Store,verify,,"//div[normalize-space()='Pending Documents Store']"
-56.Filter Pending Document Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-57.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-58.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-59. Store Required Documents,verify,,"//div[contains(text(),'Documents')]"
-60.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-61.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-62.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-63.Click Submit, click, , "//button[normalize-space()='Submit']"
-64.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-65.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-66.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-67.Click Back, click, , "//button[@class='buttonWidget']"
-68.Click  Stores,click,,"//button[contains(., 'Stores')]"
-69.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-70.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-71.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-72.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-73.Click Block Icon,click,,"//i[@title='Blocked']"
-74.Click Block  Yes,click,,"//button[normalize-space()='Yes']"
-75.Click  Stores,click,,"//button[contains(., 'Stores')]"
-76.Select Blocked Store,click,,"//div[normalize-space()='Blocked Stores']"
-77.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-78.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-79.Click unBlock Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
-80.Click  Stores,click,,"//button[contains(., 'Stores')]"
-81.Select Rejected Store,click,,"//div[normalize-space()='Rejected Stores']"
-82.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-83.Scroll Grid, tab, 7, "//input[@aria-label='Store Name Filter Input']"
-84.Click Approve Icon,click,,"//i[@title='Approve']"
-85.Click  Stores,click,,"//button[contains(., 'Stores')]"
-86.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-87.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-88.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-89.Click Doc Icon,click,,"//i[@title='Document']"
-90.Click UnApprove Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
-91.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-92.Rejection Reason,type,document insufficent,"//textarea[@id='swal2-textarea']"
-93.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-94.wait,1000,,</t>
-  </si>
-  <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
-3.Verify Delivery Services,verify,,"//div[contains(text(),'DELIVERY SERVICES')]"
-4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
-5.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
-6.Click  Stores,click,,"//button[contains(., 'Stores')]"
-7.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-8.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-9.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-10.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-11.Click Product Icon,click,,"//i[@title='Product View']"
-12.Click  Add  Products,click,,"//button[normalize-space()='Add Products']"
-13.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[1]"
-14.Select Grill Chicken,click,,"//li[@role='option'][contains(.,'Grill Chicken')]"
-15.Enter Product Name, type, Grill Chicken, "//label[contains(.,'Product Name')]/following-sibling::input"
-16.Enter Product Amount, type, 500, "//label[contains(.,'Product Amount')]/following-sibling::input"
-17.Enter Product Description, type, KFC special grill chicken, "//label[contains(text(),'Product Description')]/following-sibling::textarea"
-18.Upload Product Image, uploadfile, "src/main/resources/test-data/grillchicken.jpg", "//input[@type='file' and @accept='image/*']"
-19.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[2]"
-20.Select Activate,click,,"//li[@role='option'][contains(.,'Activate')]"
-21.Open Discount Type Dropdown,click,,"//label[contains(.,'Discount Type')]/following-sibling::select/option[text()='Discount in Amount']"
-22.Enter Discount Amount, type, 50, "//label[contains(.,'Discount Amount')]/following-sibling::input"
-23.Click Save, click, , "//button[normalize-space()='Save']"
-24.Verify Saved Succesfully, verify, , "//div[@aria-label='Product added successfully']"
-25.Verify Store Products,verify,,"//div[normalize-space()='Store Products']"
-26.Filter Product List,type,Grill Chicken,"//input[@aria-label='Product Name Filter Input']"
-27.Click Back, click, , "//button[normalize-space()='Back']"
-28.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-29.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-30.Click Wallet Icon,click,,"//i[@title='Wallet']"
-31.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
-32.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
-33.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-34.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
-35.Click Submit, click, , "//button[normalize-space()='Submit']"
-36.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-37.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
-38.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
-39.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-40.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
-41.Click Submit, click, , "//button[normalize-space()='Submit']"
-42.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-43.Click Back, click, , "//button[normalize-space()='Back']"
-44.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-45.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-46.Click Drivers Icon,click,,"//i[@title='Drivers']"
-47.Click Add Private Driver, click, , "//button[normalize-space()='Add Private Driver']"
-48.Enter Driver Name, type, kfcdriver_{timestamp} &gt;&gt; kfcdriverName, "//label[contains(., 'Driver Full Name')]/following-sibling::div//input"
-49.Enter Email, type, kfcdriver_{timestamp}@gmail.com, "//label[contains(., 'Email')]/following-sibling::div//input"
-50.Enter Contact Number, type, {randomPhone}, "//label[contains(., 'Contact No')]/following-sibling::div//input"
-51.Upload Profile Image, uploadfile, "src/main/resources/test-data/bikedriver.jpg", "//input[@type='file' and @accept='image/*']"
-52. Select Male Gender, click, , "//div[contains(text(), 'Male')]/preceding-sibling::mat-radio-button"
-53.Click Vehicle Type Dropdown,click,,"//label[contains(., 'Vehicle Type')]/following-sibling::p-dropdown"
-54.Select  Scooter Option,click,,"//li[@role='option'][contains(.,'Scooter')]"
-55. Enter Model Year, type, 2013, "//label[span[text()='Model Year']]/following::input[1]"
-56.Enter Vehicle Company, type, honda, "//label[contains(., 'Vehicle Company')]/following-sibling::div//input"
-57. Enter Plate No, type, KL-01-AB-1634, "//label[contains(., 'Plate No')]/following-sibling::div//input"
-58. Enter Model Name, type, activa, "//label[contains(., 'Model Name')]/following-sibling::div//input"
-59. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/bike.jpg", "(//app-image-upload//input[@type='file'])[2]"
-60. Enter Vehicle Color, type, white, "//label[contains(., 'Vehicle Color')]/following::input[1]"
-61. Click Submit, click, , "//button[contains(.,'Submit')]"
-62. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-63.Filter Driver List,type,{kfcdriverName},"//input[@aria-label='Driver Name Filter Input']"
-64.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
-65.wait,1000,,</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
@@ -1429,85 +1105,6 @@
   </si>
   <si>
     <t>Validate the end-to-end creation of a Customer.</t>
-  </si>
-  <si>
-    <t>1. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-2.Click  Add Customers,click,,"//span[normalize-space()='Add customers']"
-3. Verify Add Customer Heading,verify,,"//div[normalize-space()='Add Customer']"
-4.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "//label[contains(., 'Customer Full Name')]/following::input[1]"
-5.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "//input[@type='email']"
-6.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-7.Enter Video Call Limit, type, 60, "//label[contains(., 'User Used Video Call Limit in Minutes')]/following::input[1]"
-8.Open Gender,click,,"//span[@aria-label='select gender']"
-9.Select Male,click,,"//li[@aria-label='Male']"
-10.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "//input[@type='file' and @accept='image/*']"
-11.Click Submit, click, , "//button[normalize-space()='Submit']"
-12.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-13. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-14. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-15.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
-16. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-17.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-18.Click Edit Icon ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-19.Click Close, click, , "//button[normalize-space()='Close']"
-20.Click Wallet Icon ,click,,"//i[@title='Wallet']"
-21.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
-22.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
-23.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-24.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
-25.Click Submit, click, , "//button[normalize-space()='Submit']"
-26.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-27.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
-28.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
-29.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-30.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
-31.Click Submit, click, , "//button[normalize-space()='Submit']"
-32.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-33. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-34. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-35.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
-36. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-37.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-38.Click Loyalty Points Icon,click,,"//i[@title='Loyalty Points']"
-38.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
-39.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
-40.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
-41.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-42.Select Add Points,click,,"//li[@role='option'][contains(.,'Add Points')]"
-43.Enter Points, type, 30, "//input[@placeholder='Enter Points']"
-44.Click Submit, click, , "//button[normalize-space()='Submit']"
-45.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-46.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
-47.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
-48.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
-49.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-50.Select Deduct Points,click,,"//li[@role='option'][contains(.,'Deduct Points')]"
-51.Enter Points, type, 10, "//input[@placeholder='Enter Points']"
-52.Click Submit, click, , "//button[normalize-space()='Submit']"
-53.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-54. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-55. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-56.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
-57. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-58.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-59.Click Disable  Icon,click,,"//i[@title='Disable']"
-60.Click Disable  User  Yes,click,,"//button[normalize-space()='Yes']"
-61.Disable Reason,type,Client Complaints,"//textarea[@id='swal2-textarea']"
-62.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-63.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-64. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-65. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-66.Click  Blocked Customers,click,,"//span[normalize-space()='Blocked customers']"
-67.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-68.Scroll Grid, tab, 10, "//input[@aria-label='Customer Name Filter Input']"
-69.Click Enable  Icon,click,,"//i[@title='Status']"
-70.Click Enable  Yes,click,,"//button[normalize-space()='Yes']"
-71. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-72. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-73.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
-74. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-75.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-76.wait,1000,,</t>
   </si>
   <si>
     <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
@@ -1624,148 +1221,987 @@
     <t>This test validates the end-to-end lifecycle of a professional service vertical by dynamically creating a localized "Painter" service featuring multi-language support in Tamil, Arabic, and Hindi. The workflow spans from initial service definition and the configuration of governance controls—such as mandatory Address Proof documents and promotional campaigns—to a comprehensive Provider Onboarding phase involving banking details, operational scheduling, and document approval. The process concludes by verifying functional integrity through the assignment of Premium commercial packages and administrative metadata updates, ultimately confirming state transition integrity by successfully deactivating the service.</t>
   </si>
   <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-2.Click Provider Services,click,,"//h2[contains(text(), 'Provider Services')]"
-3.Verify Provider Services,verify,,"//div[normalize-space()='ON-DEMAND SERVICES']"
-4.Click  Add New Services,click,,"//button[normalize-space()='Add New Services']"
-5.Enter Service Name, type, Painter{randomAlpha}&gt;&gt; serviceName, "//input[@placeholder='Service Name']"
-6.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
-7.Enter Service Name Arabic, type, دهان, "//input[@placeholder='Service Name (in Arabic)']"
-8.Enter Service Name Hindi, type, पेंटर, "//input[@placeholder='Service Name (in Hindi)']"
-9.Enter Slug, type, painter, "//input[@placeholder='Slug']"
-10.Upload Service Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file' and @accept='image/*']"
-11.wait,2000,,
-12.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-13.Select Activate,click,,"//li[@aria-label='Activate']"
-14.Open Select City Dropdown,click,,"//div[contains(@class, 'p-multiselect-label-container')]"
-15.Select {areaName},click,,"//li[contains(@aria-label, '{areaName}')]"
-16.Click  Submit,click,,"//button[normalize-space()='Submit']"
-17.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
-18.Click Home Icon ,click,,"//i[@title='Home']"
-19.Click Settings ,click,,"//button[contains(., 'Settings')]"
-20.Click Requirment Document ,click,,"//div[normalize-space()='Required Document']"
-21.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
-22.Enter Name, type, Address Proof, "//input[@placeholder='Type here']"
-23.Open status Dropdown,click,,"//span[@aria-label='Status']"
-24.Select Active,click,,"//li[@aria-label='Active']"
-25.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
-26.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
-27.Click Submit ,click,,"//button[normalize-space()='Submit']"
-28.Verify Sucess, verify, , "//div[@aria-label='Info']"
-29.Filter Document List,type,Address Proof,"//input[@aria-label='Name Filter Input']"
-30.Click Settings ,click,,"//button[contains(., 'Settings')]"
-31.Click Promocode ,click,,"//div[normalize-space()='Promocode']"
-32.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
-33.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
-34.Select User,click,,"//li[@aria-label='{customerName}']"
-35.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
-35.Enter Code Name, type, GoldMember001, "//input[@placeholder='Code Name']"
-36.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
-37.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
-38.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
-39.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
-40.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
-41.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
-42.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
-43.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
-44.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
-45.Click Submit ,click,,"//button[normalize-space()='Submit']"
-46.Verify Sucess, verify, , "//div[@aria-label='Info']"
-47.Filter PromoCode List,type,GoldMember001,"//input[@aria-label='Promocode Filter Input']"
-48.Click  Providers,click,,"//button[contains(., 'Providers')]"
-49.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
-50.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
-51.Enter Provider Full Name, type, Painter{randomAlpha}&gt;&gt; painterName, "//input[@placeholder='Provider Full Name']"
-52.Upload Painter Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file']"
-53.Enter Email, type, Painter_{timestamp}@gmail.com&gt;&gt;painterEmail, "//input[@placeholder='Unique Email']"
-54.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
-55.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
-56.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
-57.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
-58.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
-59.Enter Provider Address, type, painter chennai, "//input[@placeholder='Enter provider Address']"
-60.wait,1000,,
-61.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
-62.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
-63.wait,1000,,
-64.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
-65.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
-66.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
-67.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
-68.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
-69.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
-70.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
-71.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
-72.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
-73.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
-74.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
-75.Enter Accont Holder Name, type, {painterName}, "//input[@placeholder='Account Holder Name']"
-76.Enter Payment Email Address, type, {painterEmail}, "//input[@placeholder='Email Address for Payment Notification']"
-77.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
-78.Click Save, click, , "//button[@type='submit']"
-79.Verify Sucess, verify, , "//div[@aria-label='Info']"
-80.Filter Painter List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
-81.Click  Providers,click,,"//button[contains(., 'Providers')]"
-82.Select Pending Document Providers,click,,"//div[normalize-space()='Pending Document Providers']"
-83.Filter Plumber List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
-84.Click Document Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-85. Provider Required Documents,verify,,"//div[contains(text(),'Documents')]"
-86.FilterDocumet List,type,Address Proof,"//input[@aria-label='Document Name Filter Input']"
-87.Add Address Proof,click,,"(//i[contains(@class, 'Edit')])[1]"
-88.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-89.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-90.Click Submit, click, , "//button[normalize-space()='Submit']"
-91.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-92.FilterDocumet List,type,Address Proof,"//input[@aria-label='Document Name Filter Input']"
-93.Click Approve Store,click,,"//div[@row-index='0']//i[contains(@class, 'bi-hand-thumbs-up-fill')]"
-94.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-95.Click Back, click, , "//button[@class='buttonWidget']"
-96.Click  Providers,click,,"//button[normalize-space()='Category']"
-97.Click  Add New Category,click,,"//button[normalize-space()='ADD CATEGORY']"
-98.Enter Category Name, type,residential painter, "//input[@placeholder='Enter the category name']"
-99.Enter Category Name Tamil, type, குடியிருப்பு பெயிண்டர், "//input[@placeholder='Category Name (in Tamil)']"
-100.Enter Category Name Arabic, type, دهان سكني, "//input[@placeholder='Category Name (in Arabic)']"
-101.Enter Category Name Hindi, type, आवासीय पेंटर, "//input[@placeholder='Category Name (in Hindi)']"
-102.Open Category status Dropdown,click,,"//span[@aria-label='Select a category status']"
-103.Select Activate,click,,"//li[@aria-label='Active']"
-104.Upload Category Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file' and @accept='image/*']"
-105.wait,2000,,
-106.Click  Submit,click,,"//button[normalize-space()='Submit']"
-107.Filter Category Name,type,residential painter,"//input[@aria-label='Category Name Filter Input']"
-108.Click  Providers,click,,"//button[contains(., 'Providers')]"
-109.Select Provider List,click,,"//div[normalize-space()='Provider List']"
-110.Filter Painter List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
-111.Scroll Grid, tab, 7, "//input[@aria-label='Provider Name Filter Input']"
-112.Click Package Icon,click,,"//i[@class='bi bi-box-seam cursor-pointer gridIcon Navigate']"
-113.Click  Add Package,click,,"//button[normalize-space()='Add Package']"
-114.Open Category  Dropdown,click,,"//span[@aria-label='Package Category']"
-115.Select Activate,click,,"//li[@aria-label='residential painter']"
-116.Enter Package Name, type, Premium, "//input[@placeholder='Package Name']"
-117.Enter Amount, type, 1000, "//input[@placeholder='Amount Value']"
-118.Open Max Book Quantity  Dropdown,click,,"//span[@aria-label='Package Max Book Quantity']"
-119.Select 4,click,,"//li[@aria-label='4']"
-120.Open Status Dropdown,click,,"//span[@aria-label='select Status']"
-121.Select Activate,click,,"//li[@aria-label='Activate']"
-122.Enter Description, type, Premium residential painting package, "//textarea[@placeholder='Description']"
-123.Click  Submit,click,,"//button[normalize-space()='Submit']"
-124.wait,1000,,
-125.Click  back,click,,"//button[normalize-space()='Back']"
-126.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-127.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-128.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
-129.Click Edit Icon ,click,,"//i[@title='Edit']"
-130.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
-131.Enter Service Name Arabic, type, دهان, "//input[@placeholder='Service Name (in Arabic)']"
-132.Enter Service Name Hindi, type, पेंटर, "//input[@placeholder='Service Name (in Hindi)']"
-133.Scroll Grid, tab, 4, "//input[@placeholder='Service Name (in Hindi)']"
-134.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-135.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
-136.Click  Submit,click,,"//button[normalize-space()='Submit']"
-137.Click  back,click,,"//button[normalize-space()='Back']"
-138.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-139.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-140.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
-141.wait,1000,,</t>
+    <t>This test validates the end-to-end lifecycle of a localized delivery service by dynamically creating a "Milk Delivery" vertical, onboarding a store provider with comprehensive operational, banking, and scheduling details, and configuring necessary administrative prerequisites including mandatory document requirements, promotional codes, and global service settings (taxes, fees, and search radii). The workflow ensures full functional integration by verifying the provider's document approval process and the successful addition of localized product categories like "Curd" (translated in Tamil, Arabic, and Hindi). The test concludes by performing an administrative state transition, deactivating the service to confirm systemic integrity and the proper functioning of administrative controls across the entire service ecosystem.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The AddCustomer test suite must be always executed before this test. This is critical because the DelieveryServiceCompleteTest process utilizes the dynamic {customerName} variable generated and stored during the AddCustomer creation phase.
+RunSheet:AddCustomer
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The AddCustomer,AddCityArea test suite must be always executed before this test. This is critical because the ProviderServiceCompleteTest process utilizes the dynamic {areaName},{customerName} variable generated and stored during the AddCityArea and AddCustomer creation phase.
+RunSheet: AddCustomer,AddCityArea
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Add New Transport Service ,Vehicle Type &amp;  driver</t>
+  </si>
+  <si>
+    <t>TC_CA_08_add_store</t>
+  </si>
+  <si>
+    <t>TC_CA_09_store_oprerations</t>
+  </si>
+  <si>
+    <t>TC_CA_10_store_status_management</t>
+  </si>
+  <si>
+    <t>TC_CA_11_delivery_service_complete_test</t>
+  </si>
+  <si>
+    <t>TC_CA_12_add_provider</t>
+  </si>
+  <si>
+    <t>SA_TS_13</t>
+  </si>
+  <si>
+    <t>TC_CA_13_provider_service_full_lifecycle_test</t>
+  </si>
+  <si>
+    <t>TC_CA_07_transport_service_complete_test</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddCustomer,AddCityArea test suite must be always executed before this test. This is critical because the TransportServiceCompleteTest process utilizes the dynamic {areaName},{customerName} variable generated and stored during the AddCityArea and AddCustomer creation phase.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AddCustomer,AddCityArea</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>This test validates the end-to-end operational lifecycle of a comprehensive Transport Service ecosystem by dynamically creating a localized "Bus Ride" category with multilingual support and city-specific accessibility. The workflow integrates complex administrative configurations, including the establishment of tiered vehicle types (e.g., Volvo) with granular fare structures, promotional code management for targeted user segments, and global service parameters such as driver search radii, tax implications, and platform fees. Furthermore, the test verifies the robustness of the onboarding pipeline by simulating driver registration—complete with banking and vehicle documentation—and exercising the mandatory document approval framework to transition a driver from "Pending" to "Approved" status. The cycle concludes by establishing loyalty program parameters and performing a systemic deactivation of the transport category, ensuring that administrative controls effectively manage service availability and data integrity across the entire transport infrastructure.</t>
+  </si>
+  <si>
+    <t>SA_TS_14</t>
+  </si>
+  <si>
+    <t>Clean The Test Data Created During Test Run</t>
+  </si>
+  <si>
+    <t>TC_CA_14_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>This test phase ensures the long-term stability and performance of the QA environment by executing a systematic Automated Data Cleanup strategy. Leveraging localized SQL Hooks with built-in safety firewalls, the workflow identifies and removes dynamically generated test artifacts—including unique City Areas, Provider profiles, and administrative accounts—created during the regression suite. By targeting specific records using variable-driven WHERE clauses, the script maintains database referential integrity, prevents record duplication in subsequent runs, and ensures the test environment remains in a pristine, 'ready-state' for continuous integration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+2. Click City area menu,click,,"//span[normalize-space()='City area']"
+3. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
+4. Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
+5. Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
+6. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
+7. Open Status Dropdown,click,,"//span[@aria-label='select status']"
+8. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+9. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
+10. Click Submit,click,,"//button[normalize-space()='Submit']"
+11. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
+12. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
+13. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
+14. Click Add Category,click,,"//button[normalize-space()='Add Category']"
+15. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
+16. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
+17. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
+18. Click close,click,,"//button[normalize-space()='Close']"
+19. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+20. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+21. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
+22. Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
+23. Open Select City Dropdown,click,,"//select[@id='cityId']"
+24. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
+25. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
+</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CRITICAL SYSTEM WARNING: DATABASE INTEGRITY PROTOCOL</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-----------------------------------------</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">This sheet contains SQL Hooks that execute directly against the we1 Production/Staging database. DO NOT modify the SQL syntax, remove variable placeholders (e.g., {areaName}), or edit the WHERE clauses.
+Unauthorized changes may result in irreversible data loss or database corruption. If modifications are required, please contact the Automation Lead or the Database Administrator.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PASSWORD TO EDIT SHEET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> :eit6190
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.
+RunSheet: SuperAdminLogin
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+2.Click  Add Customers,click,,"//span[normalize-space()='Add customers']"
+3. Verify Add Customer Heading,verify,,"//div[normalize-space()='Add Customer']"
+4.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "//label[contains(., 'Customer Full Name')]/following::input[1]"
+5.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "//input[@type='email']"
+6.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+7.Enter Video Call Limit, type, 60, "//label[contains(., 'User Used Video Call Limit in Minutes')]/following::input[1]"
+8.Open Gender,click,,"//span[@aria-label='select gender']"
+9.Select Male,click,,"//li[@aria-label='Male']"
+10.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "//input[@type='file' and @accept='image/*']"
+11.Click Submit, click, , "//button[normalize-space()='Submit']"
+12.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+13. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+14. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+15.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
+16. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+17.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+18.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
+19.Click Edit Icon ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+20.Click Close, click, , "//button[normalize-space()='Close']"
+21.Click Wallet Icon ,click,,"//i[@title='Wallet']"
+22.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
+23.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
+24.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+25.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
+26.Click Submit, click, , "//button[normalize-space()='Submit']"
+27.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+28.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
+29.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
+30.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+31.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
+32.Click Submit, click, , "//button[normalize-space()='Submit']"
+33.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+34. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+35. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+36.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
+37. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+38.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+39.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
+40.Click Loyalty Points Icon,click,,"//i[@title='Loyalty Points']"
+41.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
+42.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
+43.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
+44.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+45.Select Add Points,click,,"//li[@role='option'][contains(.,'Add Points')]"
+46.Enter Points, type, 30, "//input[@placeholder='Enter Points']"
+47.Click Submit, click, , "//button[normalize-space()='Submit']"
+48.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+49.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
+50.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
+51.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
+52.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+53.Select Deduct Points,click,,"//li[@role='option'][contains(.,'Deduct Points')]"
+54.Enter Points, type, 10, "//input[@placeholder='Enter Points']"
+55.Click Submit, click, , "//button[normalize-space()='Submit']"
+56.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+57. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+58. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+59.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
+60. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+61.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+62.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
+63.Click Disable  Icon,click,,"//i[@title='Block']"
+64.Click Disable  User  Yes,click,,"//button[normalize-space()='Yes']"
+65.Disable Reason,type,Client Complaints,"//textarea[@id='swal2-textarea']"
+66.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+67.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+68. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+69. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+70.Click  Blocked Customers,click,,"//span[normalize-space()='Blocked customers']"
+71.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+72.Scroll Grid, tab, 10, "//input[@aria-label='Customer Name Filter Input']"
+73.Click Enable  Icon,click,,"//i[@title='Status']"
+74.Click Enable  Yes,click,,"//button[normalize-space()='Yes']"
+75. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+76. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+77.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
+78. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+79.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+80.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+6. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
+7. Enter Driver Name, type, autodriver_{timestamp} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+8. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+9. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+10. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+11. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+12.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+13.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
+14. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+15.Enter Vehicle Company, type, autoCompany{randomAlpha}&gt;&gt; autoCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+16. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+17. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+18. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+19. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+20. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+21. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+22. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+23. Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+24. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+25. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+26. Click Submit, click, , "//button[contains(.,'Submit')]"
+27. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+28. Wait for Toast to hide, wait, 1000,
+29.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+32.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+33.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+34. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+35.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+36.Add Driving License,click,,"//i[@title='Edit']"
+37.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+38.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+39.Click Submit, click, , "//button[normalize-space()='Submit']"
+40.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+41.Click Approve Driver,click,,"//i[@title='Approve']"
+42.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+43.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+44.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+45.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+46.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+47.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+48.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+49.Click Doc Icon,click,,"//i[@title='Document']"
+50.Click Eye Icon,click,,"//i[@title='View']"
+51.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+3. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+4. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+5.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+6.Select Bike Ride Option,click,,"//span[normalize-space()='Bike Ride']"
+7. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+8. Enter Driver Name, type, bikedriver_{timestamp} &gt;&gt; bikeName, "//label[contains(.,'Full Name')]/following::input[1]"
+9. Enter Email, type, bikedriver_{timestamp}@gmail.com&gt;&gt;bikeEmail, "//label[contains(.,'Email')]/following::input[1]"
+10. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+11. Upload Profile Image, uploadfile, "src/main/resources/test-data/bikedriver.jpg", "//input[@type='file']"
+12. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+13.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+14.Select  Scooter Option,click,,"//li[@role='option']//span[text()='Scooter']"
+15. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+16.Enter Vehicle Company, type, bikeCompany{randomAlpha}&gt;&gt; bikeCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+17. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+18. Enter Model Name, type, activa, "//label[contains(.,'Model Name')]/following::input[1]"
+19. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/bike.jpg", "(//input[@type='file'])[2]"
+20. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+21. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+22. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+23. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+24. Enter Account Holder Name, type, {bikeName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+25. Enter Payment Email Address, type, {bikeEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+26. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+27. Click Submit, click, , "//button[contains(.,'Submit')]"
+28. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+29. Wait for Toast to hide, wait, 1000,
+30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+32.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+33.Filter by Name,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
+34.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+35. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+36.FilterDocumet List,type,Vehicle Permit Copy,"//input[@aria-label='Document Name Filter Input']"
+37.Add Vehicle Permit Copy,click,,"//i[@title='Edit']"
+38.Upload Vehicle Permit Copy, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+39.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+40.Click Submit, click, , "//button[normalize-space()='Submit']"
+41.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+42.Click Approve Driver,click,,"//i[@title='Approve']"
+43.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+44.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+46.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+47.Approved Drivers List,verify,,"//div[contains(text(),' Approved Drivers List')]"
+48.Filter Approved Driver,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
+49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+50.Click Doc Icon,click,,"//i[@title='Document']"
+51.Click Eye Icon,click,,"//i[@title='View']"
+52.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+3. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+4. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+5.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+6.Select Taxi Ride Option,click,,"//span[normalize-space()='Taxi Ride']"
+7. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+8. Enter Driver Name, type, taxidriver_{timestamp} &gt;&gt; taxiName, "//label[contains(.,'Full Name')]/following::input[1]"
+9. Enter Email, type, taxidriver_{timestamp}@gmail.com&gt;&gt;taxiEmail, "//label[contains(.,'Email')]/following::input[1]"
+10. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+11. Upload Profile Image, uploadfile, "src/main/resources/test-data/taxidriver.jpg", "//input[@type='file']"
+12. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+13.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+14.Select  Suv Option,click,,"//li[@role='option']//span[text()='SUV']"
+15. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+16.Enter Vehicle Company, type, taxiCompany{randomAlpha}&gt;&gt; taxiCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+17. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+18. Enter Model Name, type, etios, "//label[contains(.,'Model Name')]/following::input[1]"
+19.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/taxi.jpg", "(//input[@type='file'])[2]"
+20. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+21. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+22. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+23. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+24. Enter Account Holder Name, type, {taxiName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+25. Enter Payment Email Address, type, {taxiEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+26. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+27. Click Submit, click, , "//button[contains(.,'Submit')]"
+28. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+29. Wait for Toast to hide, wait, 1000,
+30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+32.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+33.Filter by Name,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
+34.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+35. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+36.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+37.Add Driving License,click,,"//i[@title='Edit']"
+38.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+39.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+40.Click Submit, click, , "//button[normalize-space()='Submit']"
+41.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+42.Click Approve Driver,click,,"//i[@title='Approve']"
+43.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+44.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+46.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+47.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+48.Filter Approved Driver,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
+49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+50.Click Doc Icon,click,,"//i[@title='Document']"
+51.Click Eye Icon,click,,"//i[@title='View']"
+52.wait,1000,,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+2. Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+3.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
+4.Click  Add Category,click,,"//button[normalize-space()='Add Category']"
+5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "//input[@placeholder='Service Name']"
+6.Enter Service Name Arabic, type, رحلة بالحافلة, "//input[@placeholder='Service Name (in Arabic)']"
+7.Enter Slug, type, Bus Ride, "//input[@placeholder='Slug']"
+8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "//input[@type='file' and @accept='image/*']"
+9.wait,2000,,
+10.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+11.Select Activate,click,,"//li[@aria-label='Activate']"
+12.Open Select City Dropdown,click,,"//span[text()='Select City']/ancestor::app-drop-down//div[contains(@class, 'p-multiselect-label-container')]"
+13.Select {areaName},click,,"//li[@aria-label='{areaName}']"
+14.Click  Submit,click,,"//button[normalize-space()='Submit']"
+15.Verify Sucess, verify, , "//div[@aria-label='Info']"
+16.wait,2000,,
+17.Click  back,click,,"//button[normalize-space()='Back']"
+18.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+19.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+20.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
+21.Click Home Icon ,click,,"//i[@title='Home']"
+22.Click Settings ,click,,"//button[contains(., 'Settings')]"
+23.Click Vehicle Type,click,,"//div[normalize-space()='Vehicle Type']"
+24.Click Add Vehicle Type,click,,"//button[normalize-space()='Add Vehicle Type']"
+25.Enter Vehicle Type Name, type, volvo{randomAlpha}&gt;&gt;busTypeName, "//input[@placeholder='Type here']"
+26.Enter Cost For Km, type, 150, "//input[@placeholder='Cost For Km']"
+27.Enter Time Fare Per Min, type,10, "//input[@placeholder='Time Fare Per Min']"
+28.Enter Base fare, type,100, "//input[@placeholder='Base fare']"
+29.Enter Min Fare Amount, type,50, "//input[@placeholder='Min Fare Amount']"
+30.Enter Rental Cost For Km, type,30, "//input[@placeholder='Rental Cost For Km']"
+31.Enter Rental Amount For 1 Hour, type,50, "//input[@placeholder='Rental Amount For 1 Hour']"
+32.Enter Rental Km Limit For 1 Hour, type,50, "//input[@placeholder='Rental Km Limit For 1 Hour']"
+33.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "//app-image-upload//input[@type='file' and @accept='image/*']"
+34.Click Surcharge Time Checkbox, click, , "//div[text()='EveryDay']/preceding-sibling::mat-checkbox"
+35.Enter From Time, type, 100000, "//app-time-picker//input[@type='time']"
+36.Enter To Time, type, 220000, "(//app-time-picker//input[@type='time'])[2]"
+37.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+38.Select Active,click,,"//li[@aria-label='Active']"
+39.Click  Submit,click,,"//button[normalize-space()='Submit']"
+40.Verify Sucess, verify, , "//div[@aria-label='Info']"
+41.Click Settings ,click,,"//button[contains(., 'Settings')]"
+42.Click Promocode,click,,"//div[normalize-space()='Promocode']"
+43.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
+44.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
+45.Select User,click,,"//li[@aria-label='{customerName}']"
+46.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
+47.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; promoCodeName, "//input[@placeholder='Code Name']"
+48.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
+49.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
+50.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
+51.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
+52.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
+53.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
+54.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
+55.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
+56.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
+57.Click Submit ,click,,"//button[normalize-space()='Submit']"
+58.Verify Sucess, verify, , "//div[@aria-label='Info']"
+59.wait,2000,,
+60.Click Settings ,click,,"//button[contains(., 'Settings')]"
+61.Click Service Settings ,click,,"//div[normalize-space()='Service Setting']"
+62.Enter Driver Accept Timeout, type, 60, "//label[contains(., "Driver Accept Timeout")]/following::input[1]"
+63.Enter Driver Serach Radius, type, 50, "//label[contains(., "Driver Search Radius")]/following::input[1]"
+64.Open Tax Type Dropdown,click,,"//span[@aria-label='Select Tax Rype']"
+65.Select Amount,click,,"//li[@aria-label='Amount']"
+66.Enter Tax, type, 20, "//label[contains(., 'Tax')]/following::input[1]"
+67.Open Platform Fee Type Dropdown,click,,"//label[contains(., 'Platform Fee Type')]/following::span[@role='combobox']"
+68.Select Amount,click,,"//li[@aria-label='Amount']"
+69.Enter Platform Fee, type, 20, "//label[contains(., "Platform Fee")]/following::input[1]"
+70.Click Submit ,click,,"//button[normalize-space()='Submit']"
+71.Verify Sucess, verify, , "//div[@aria-label='Info']"
+72.wait,1000,,
+73.Click Settings ,click,,"//button[contains(., 'Settings')]"
+74.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
+75.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
+76.Enter Name, type, documet{randomAlpha}&gt;&gt; documentName, "//label[contains(., 'Name')]/following::input[1]"
+77.Open status Dropdown,click,,"//label[contains(., 'Status')]/following::div[contains(@class, 'p-dropdown')]"
+78.Select Active,click,,"//li[@aria-label='Active']"
+79.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
+80.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
+81.Click  Require Proof Number,click,,"//div[./div[contains(text(), 'Require Proof Number')]]//input"
+82.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
+83.Click Submit ,click,,"//button[normalize-space()='Submit']"
+84.Verify Sucess, verify, , "//div[@aria-label='Info']"
+85.Filter Document List,type,{documentName},"//input[@aria-label='Name Filter Input']"
+86.wait,1000,,
+88.Click Settings ,click,,"//button[contains(., 'Settings')]"
+89.Click Customer Loyalty Settings,click,,"//div[text()=' Customer Loyalty Settings ']"
+90.Open status Allow Customer loyalty points,click,,"//label[contains(., 'Allow Customer loyalty points')]/following::div[contains(@class, 'p-dropdown')]"
+91.Select ON,click,,"//li[@role='option']//span[text()='ON']"
+92.Enter Minimum order amount for eligibility to redeem loyalty points, type, 25,"//label[contains(., 'Minimum order amount for eligibility to redeem loyalty points')]/following::input[1]"
+93.Enter Loyalty points redeem per order (in %) (% of order amount), type, 10,"//label[contains(., 'Loyalty points redeem per order (in %) (% of order amount)')]/following::input[1]"
+94.Enter Loyalty points per default currency (for ex. $1 = 10 points), type, 5,"//label[contains(., 'Loyalty points per default currency (for ex. $1 = 10 points)')]/following::input[1]"
+95.Click Submit ,click,,"//button[normalize-space()='Submit']"
+96.Verify Sucess, verify, , "//div[@aria-label='Info']"
+97.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+98.Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+99.Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+100.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+101.Select Bus Ride Option,click,,"//span[normalize-space()='{transportName}']"
+102.Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+103.Enter Driver Name, type, busdriver_{timestamp} &gt;&gt; busDriverName, "//label[contains(.,'Full Name')]/following::input[1]"
+104.Enter Email, type, busdriver_{timestamp}@gmail.com&gt;&gt;busEmail, "//label[contains(.,'Email')]/following::input[1]"
+105.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+106.Upload Profile Image, uploadfile, "src/main/resources/test-data/busdriver.jpg", "//input[@type='file']"
+107.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+108.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+109.Select  volvo Option,click,,"//li[@role='option']//span[text()='{busTypeName}']"
+110.Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+111.Enter Vehicle Company, type, busCompany{randomAlpha}&gt;&gt; busCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+112.Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+113. Enter Model Name, type, deisel, "//label[contains(.,'Model Name')]/following::input[1]"
+114.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/busvolvo.jpeg", "(//input[@type='file'])[2]"
+115. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+116.Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+117.Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+118.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+119.Enter Account Holder Name, type, {busDriverName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+120.Enter Payment Email Address, type, {busEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+121.Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+122.Click Submit, click, , "//button[contains(.,'Submit')]"
+123.Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+124.Wait for Toast to hide, wait, 1000,
+125.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+126.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+127.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+128.Filter by Name,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
+129.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+130.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+131.FilterDocumet List,type,{documentName},"//input[@aria-label='Document Name Filter Input']"
+132.Add Driving License,click,,"//i[@title='Edit']"
+133.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+134.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+135.Click Submit, click, , "//button[normalize-space()='Submit']"
+136.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+137.Click Approve Driver,click,,"//i[@title='Approve']"
+138.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+139.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+140.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+141.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+142.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+143.Filter Approved Driver,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
+144.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+145.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+146.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
+147.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
+148.Click Edit Icon ,click,,"//i[@title='Edit']"
+149.Scroll Grid, tab, 5, "//input[@placeholder='Service Name']"
+150.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+151.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
+152.Click  Submit,click,,"//button[normalize-space()='Submit']"
+153.Verify Sucess, verify, , "//div[@aria-label='Info']"
+154.wait,2000,,
+</t>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
+3.Verify Delivery Services,verify,,"//div[contains(text(),'DELIVERY SERVICES')]"
+4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
+5.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
+6.Click  Stores,click,,"//button[contains(., 'Stores')]"
+7.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+8.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
+9.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+10.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+11.Click Product Icon,click,,"//i[@title='Product View']"
+12.Click  Add  Products,click,,"//button[normalize-space()='Add Products']"
+13.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[1]"
+14.Select Grill Chicken,click,,"//li[@role='option'][contains(.,'Grill Chicken')]"
+15.Enter Product Name, type, kfcProduct{randomAlpha}&gt;&gt; kfcProductName, "//label[contains(.,'Product Name')]/following-sibling::input"
+16.Enter Product Amount, type, 500, "//label[contains(.,'Product Amount')]/following-sibling::input"
+17.Enter Product Description, type, KFC special grill chicken, "//label[contains(text(),'Product Description')]/following-sibling::textarea"
+18.Upload Product Image, uploadfile, "src/main/resources/test-data/grillchicken.jpg", "//input[@type='file' and @accept='image/*']"
+19.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[2]"
+20.Select Activate,click,,"//li[@role='option'][contains(.,'Activate')]"
+21.Open Discount Type Dropdown,click,,"//label[contains(.,'Discount Type')]/following-sibling::select/option[text()='Discount in Amount']"
+22.Enter Discount Amount, type, 50, "//label[contains(.,'Discount Amount')]/following-sibling::input"
+23.Click Save, click, , "//button[normalize-space()='Save']"
+24.Verify Saved Succesfully, verify, , "//div[@aria-label='Product added successfully']"
+25.Verify Store Products,verify,,"//div[normalize-space()='Store Products']"
+26.Filter Product List,type,{kfcProductName},"//input[@aria-label='Product Name Filter Input']"
+27.Click Back, click, , "//button[normalize-space()='Back']"
+28.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+29.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+30.Click Wallet Icon,click,,"//i[@title='Wallet']"
+31.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
+32.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
+33.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+34.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
+35.Click Submit, click, , "//button[normalize-space()='Submit']"
+36.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+37.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
+38.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
+39.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+40.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
+41.Click Submit, click, , "//button[normalize-space()='Submit']"
+42.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+43.Click Back, click, , "//button[normalize-space()='Back']"
+44.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+45.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+46.Click Drivers Icon,click,,"//i[@title='Drivers']"
+47.Click Add Private Driver, click, , "//button[normalize-space()='Add Private Driver']"
+48.Enter Driver Name, type, kfcdriver_{timestamp} &gt;&gt; kfcdriverName, "//label[contains(., 'Driver Full Name')]/following-sibling::div//input"
+49.Enter Email, type, kfcdriver_{timestamp}@gmail.com, "//label[contains(., 'Email')]/following-sibling::div//input"
+50.Enter Contact Number, type, {randomPhone}, "//label[contains(., 'Contact No')]/following-sibling::div//input"
+51.Upload Profile Image, uploadfile, "src/main/resources/test-data/bikedriver.jpg", "//input[@type='file' and @accept='image/*']"
+52. Select Male Gender, click, , "//div[contains(text(), 'Male')]/preceding-sibling::mat-radio-button"
+53.Click Vehicle Type Dropdown,click,,"//label[contains(., 'Vehicle Type')]/following-sibling::p-dropdown"
+54.Select  Scooter Option,click,,"//li[@role='option'][contains(.,'Scooter')]"
+55. Enter Model Year, type, 2013, "//label[span[text()='Model Year']]/following::input[1]"
+56.Enter Vehicle Company, type, kfcBikeCompany{randomAlpha}&gt;&gt; kfcBikeCompanyName, "//label[contains(., 'Vehicle Company')]/following-sibling::div//input"
+57. Enter Plate No, type, KL-01-AB-1634, "//label[contains(., 'Plate No')]/following-sibling::div//input"
+58. Enter Model Name, type, activa, "//label[contains(., 'Model Name')]/following-sibling::div//input"
+59. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/bike.jpg", "(//app-image-upload//input[@type='file'])[2]"
+60. Enter Vehicle Color, type, white, "//label[contains(., 'Vehicle Color')]/following::input[1]"
+61. Click Submit, click, , "//button[contains(.,'Submit')]"
+62. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+63.Filter Driver List,type,{kfcdriverName},"//input[@aria-label='Driver Name Filter Input']"
+64.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
+65.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
+3.Verify Delivery Services,verify,,"//div[contains(text(),' DELIVERY SERVICES')]"
+4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
+5.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
+6.Click  Stores,click,,"//button[contains(., 'Stores')]"
+7.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
+8.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Add Store')]"
+9.Enter Store Name, type, bilal_{timestamp} &gt;&gt; hotelName, "//input[@placeholder='Store Name']"
+10.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
+11.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
+12.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
+13. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
+14.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
+15.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
+16.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
+17.Upload Banner Image, uploadfile, "src/main/resources/test-data/kfcbanner.jpg", "//input[@type='file']"
+18.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
+19.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
+20.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
+21.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
+22.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+23..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
+24.wait,1000,,
+25.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
+26.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
+27.wait,1000,,
+28.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
+29.Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
+30.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
+31.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
+32.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
+33.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
+34.Enter Contact Person Full Name, type, bilalowner_{timestamp} &gt;&gt; hotelOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
+35.Enter Email, type, bilal_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
+36.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
+37.Upload Store Image, uploadfile, "src/main/resources/test-data/kfcstore.jpg", "(//input[@type='file'])[2]"
+38.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
+39.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
+40.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
+41.Enter Accont Holder Name, type, {hotelOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
+42.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
+43.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
+44.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
+45.Enter From Time, type, 100000, "(//label[contains(.,'From Time')]/following-sibling::input)[1]"
+46.Enter To Time, type, 220000, "(//label[contains(.,'To Time')]/following-sibling::input)[1]"
+47.Submit Add Store,click,,"//button[normalize-space()='Submit']"
+48. Verify Success Message,verify,,"//div[@aria-label='Info']"
+49.Click  Stores,click,,"//button[contains(., 'Stores')]"
+50.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+51.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
+52.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
+53.Click  Stores,click,,"//button[contains(., 'Stores')]"
+54.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
+55.Verify Add Store,verify,,"//div[normalize-space()='Pending Documents Store']"
+56.Filter Pending Document Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
+57.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+58.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
+59. Store Required Documents,verify,,"//div[contains(text(),'Documents')]"
+60.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+61.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
+62.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+63.Click Submit, click, , "//button[normalize-space()='Submit']"
+64.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+65.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+66.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+67.Click Back, click, , "//button[@class='buttonWidget']"
+68.Click  Stores,click,,"//button[contains(., 'Stores')]"
+69.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+70.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
+71.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
+72.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+73.Click Block Icon,click,,"//i[@title='Blocked']"
+74.Click Block  Yes,click,,"//button[normalize-space()='Yes']"
+75.Click  Stores,click,,"//button[contains(., 'Stores')]"
+76.Select Blocked Store,click,,"//div[normalize-space()='Blocked Stores']"
+77.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
+78.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+79.Click unBlock Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
+80.Click  Stores,click,,"//button[contains(., 'Stores')]"
+81.Select Rejected Store,click,,"//div[normalize-space()='Rejected Stores']"
+82.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
+83.Scroll Grid, tab, 7, "//input[@aria-label='Store Name Filter Input']"
+84.Click Approve Icon,click,,"//i[@title='Approve']"
+85.Click  Stores,click,,"//button[contains(., 'Stores')]"
+86.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+87.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
+88.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+89.Click Doc Icon,click,,"//i[@title='Document']"
+90.Click UnApprove Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
+91.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+92.Rejection Reason,type,document insufficent,"//textarea[@id='swal2-textarea']"
+93.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+94.wait,1000,,</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[@class='fa-solid fa-user-shield iconstyle']"
@@ -1789,7 +2225,7 @@
 19.Click Settings ,click,,"//button[contains(., 'Settings')]"
 20.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
 21.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
-22.Enter Name, type, Address Proof, "//input[@placeholder='Type here']"
+22.Enter Name, type, documet{randomAlpha}&gt;&gt; deliveryDocumentName, "//input[@placeholder='Type here']"
 23.Open status Dropdown,click,,"//span[@aria-label='select status']"
 24.Select Active,click,,"//li[@aria-label='Active']"
 25.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
@@ -1799,7 +2235,7 @@
 29.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
 30.Click Submit ,click,,"//button[normalize-space()='Submit']"
 31.Verify Sucess, verify, , "//div[@aria-label='Info']"
-32.Filter Document List,type,Address Proof,"//input[@aria-label='Name Filter Input']"
+32.Filter Document List,type,{deliveryDocumentName},"//input[@aria-label='Name Filter Input']"
 33.wait,2000,,
 33.Click Settings ,click,,"//button[contains(., 'Settings')]"
 34.Click Promocode ,click,,"//div[normalize-space()='Promocode']"
@@ -1807,7 +2243,7 @@
 36.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
 37.Select User,click,,"//li[@aria-label='{customerName}']"
 38.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
-39.Enter Code Name, type, GoldMember001, "//input[@placeholder='Code Name']"
+39.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; deliveryPromoCodeName, "//input[@placeholder='Code Name']"
 40.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
 41.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
 42.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
@@ -1819,7 +2255,7 @@
 48.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
 49.Click Submit ,click,,"//button[normalize-space()='Submit']"
 50.Verify Sucess, verify, , "//div[@aria-label='Info']"
-51.Filter PromoCode List,type,GoldMember001,"//input[@aria-label='promocode Filter Input']"
+51.Filter PromoCode List,type,{deliveryPromoCodeName},"//input[@aria-label='promocode Filter Input']"
 52.wait,2000,,
 53.Click Settings ,click,,"//button[contains(., 'Settings')]"
 54.Click Service Settings ,click,,"//div[normalize-space()='Service Settings']"
@@ -1862,14 +2298,14 @@
 91.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
 92.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
 93.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
-94.Enter Contact Person Full Name, type, storeowner_{timestamp} &gt;&gt; storeOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
+94.Enter Contact Person Full Name, type, amulStoreowner_{timestamp} &gt;&gt; milkStoreOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
 95.Enter Email, type, amul_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
 96.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
 97.Upload Store Image, uploadfile, "src/main/resources/test-data/milkbooth.jpeg", "(//input[@type='file'])[2]"
 98.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
 99.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
 100.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
-101.Enter Accont Holder Name, type, {storeOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
+101.Enter Accont Holder Name, type, {milkStoreOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
 102.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
 103.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
 104.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
@@ -1905,7 +2341,7 @@
 134.Click Back, click, , "//button[@class='buttonWidget']"
 135.Click Category, click, , "//button[normalize-space()='Category']"
 136.Click  Add New Category,click,,"//button[normalize-space()='Add Category']"
-137.Enter Category Name, type,curd, "//span[contains(text(), 'Category Name')]/ancestor::app-input//input"
+137.Enter Category Name, type,curd{randomAlpha}&gt;&gt; MilkCategoryName, "//span[contains(text(), 'Category Name')]/ancestor::app-input//input"
 138.Enter Category Name Arabic, type, رائب, "//span[contains(text(), 'Language Value (in Arabic)')]/ancestor::app-input//input"
 139.Enter Category Name Tamil, type, தயிர், "//span[contains(text(), 'Language Value (in Tamil)')]/ancestor::app-input//input"
 140.Enter Category Name Hindi, type, दही, "//span[contains(text(), 'Language Value (in Hindi)')]/ancestor::app-input//input"
@@ -1916,7 +2352,7 @@
 145.Enter Slug Name, type, curd, "//span[text()='Slug']/ancestor::app-input//input"
 146.Click  Submit,click,,"//button[normalize-space()='Submit']"
 147.Verify Success Message,verify,,"//div[@aria-label='Info']"
-148.Filter Category Name,type,curd,"//input[@aria-label='Category Name Filter Input']"
+148.Filter Category Name,type,{MilkCategoryName},"//input[@aria-label='Category Name Filter Input']"
 149.Click  Stores,click,,"//button[contains(., 'Stores')]"
 150.Select Store List,click,,"//div[contains(text(), 'Store List')]"
 151.Filter Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
@@ -1924,7 +2360,7 @@
 153.Click Product Icon,click,,"//i[@title='Product View']"
 154.Click  Add  Products,click,,"//button[normalize-space()='Add Products']"
 155.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[1]"
-156.Select curd,click,,"//li[@role='option'][contains(.,'curd')]"
+156.Select curd,click,,"//li[@role='option'][contains(.,'{MilkCategoryName}')]"
 157.wait,1000,,
 158.Click badge,click,,"//i[@class='fa-solid fa-user-shield iconstyle']"
 159.Click Delivery Services,click,,"//h2[normalize-space()='Delivery Services']"
@@ -1939,585 +2375,195 @@
 167.wait,1000,,</t>
   </si>
   <si>
-    <t>This test validates the end-to-end lifecycle of a localized delivery service by dynamically creating a "Milk Delivery" vertical, onboarding a store provider with comprehensive operational, banking, and scheduling details, and configuring necessary administrative prerequisites including mandatory document requirements, promotional codes, and global service settings (taxes, fees, and search radii). The workflow ensures full functional integration by verifying the provider's document approval process and the successful addition of localized product categories like "Curd" (translated in Tamil, Arabic, and Hindi). The test concludes by performing an administrative state transition, deactivating the service to confirm systemic integrity and the proper functioning of administrative controls across the entire service ecosystem.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The AddCustomer test suite must be always executed before this test. This is critical because the DelieveryServiceCompleteTest process utilizes the dynamic {customerName} variable generated and stored during the AddCustomer creation phase.
-RunSheet:AddCustomer
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The AddCustomer,AddCityArea test suite must be always executed before this test. This is critical because the ProviderServiceCompleteTest process utilizes the dynamic {areaName},{customerName} variable generated and stored during the AddCityArea and AddCustomer creation phase.
-RunSheet: AddCustomer,AddCityArea
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <t>Add New Transport Service ,Vehicle Type &amp;  driver</t>
-  </si>
-  <si>
-    <t>TC_CA_08_add_store</t>
-  </si>
-  <si>
-    <t>TC_CA_09_store_oprerations</t>
-  </si>
-  <si>
-    <t>TC_CA_10_store_status_management</t>
-  </si>
-  <si>
-    <t>TC_CA_11_delivery_service_complete_test</t>
-  </si>
-  <si>
-    <t>TC_CA_12_add_provider</t>
-  </si>
-  <si>
-    <t>SA_TS_13</t>
-  </si>
-  <si>
-    <t>TC_CA_13_provider_service_full_lifecycle_test</t>
-  </si>
-  <si>
-    <t>TC_CA_07_transport_service_complete_test</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The AddCustomer,AddCityArea test suite must be always executed before this test. This is critical because the TransportServiceCompleteTest process utilizes the dynamic {areaName},{customerName} variable generated and stored during the AddCityArea and AddCustomer creation phase.</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-RunSheet: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>AddCustomer,AddCityArea</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <t>This test validates the end-to-end operational lifecycle of a comprehensive Transport Service ecosystem by dynamically creating a localized "Bus Ride" category with multilingual support and city-specific accessibility. The workflow integrates complex administrative configurations, including the establishment of tiered vehicle types (e.g., Volvo) with granular fare structures, promotional code management for targeted user segments, and global service parameters such as driver search radii, tax implications, and platform fees. Furthermore, the test verifies the robustness of the onboarding pipeline by simulating driver registration—complete with banking and vehicle documentation—and exercising the mandatory document approval framework to transition a driver from "Pending" to "Approved" status. The cycle concludes by establishing loyalty program parameters and performing a systemic deactivation of the transport category, ensuring that administrative controls effectively manage service availability and data integrity across the entire transport infrastructure.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
-2. Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
-3.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
-4.Click  Add Category,click,,"//button[normalize-space()='Add Category']"
-5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "//input[@placeholder='Service Name']"
-6.Enter Service Name Arabic, type, رحلة بالحافلة, "//input[@placeholder='Service Name (in Arabic)']"
-7.Enter Slug, type, Bus Ride, "//input[@placeholder='Slug']"
-8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "//input[@type='file' and @accept='image/*']"
-9.wait,2000,,
-10.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-11.Select Activate,click,,"//li[@aria-label='Activate']"
-12.Open Select City Dropdown,click,,"//span[text()='Select City']/ancestor::app-drop-down//div[contains(@class, 'p-multiselect-label-container')]"
-13.Select {areaName},click,,"//li[@aria-label='{areaName}']"
-14.Click  Submit,click,,"//button[normalize-space()='Submit']"
-15.Verify Sucess, verify, , "//div[@aria-label='Info']"
-16.wait,2000,,
-17.Click  back,click,,"//button[normalize-space()='Back']"
-18.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
-19.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
-20.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
-21.Click Home Icon ,click,,"//i[@title='Home']"
-22.Click Settings ,click,,"//button[contains(., 'Settings')]"
-23.Click Vehicle Type,click,,"//div[normalize-space()='Vehicle Type']"
-24.Click Add Vehicle Type,click,,"//button[normalize-space()='Add Vehicle Type']"
-25.Enter Vehicle Type Name, type, volvo, "//input[@placeholder='Type here']"
-26.Enter Cost For Km, type, 150, "//input[@placeholder='Cost For Km']"
-27.Enter Time Fare Per Min, type,10, "//input[@placeholder='Time Fare Per Min']"
-28.Enter Base fare, type,100, "//input[@placeholder='Base fare']"
-29.Enter Min Fare Amount, type,50, "//input[@placeholder='Min Fare Amount']"
-30.Enter Rental Cost For Km, type,30, "//input[@placeholder='Rental Cost For Km']"
-31.Enter Rental Amount For 1 Hour, type,50, "//input[@placeholder='Rental Amount For 1 Hour']"
-32.Enter Rental Km Limit For 1 Hour, type,50, "//input[@placeholder='Rental Km Limit For 1 Hour']"
-33.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "//app-image-upload//input[@type='file' and @accept='image/*']"
-34.Click Surcharge Time Checkbox, click, , "//div[text()='EveryDay']/preceding-sibling::mat-checkbox"
-35.Enter From Time, type, 100000, "//app-time-picker//input[@type='time']"
-36.Enter To Time, type, 220000, "(//app-time-picker//input[@type='time'])[2]"
-37.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-38.Select Active,click,,"//li[@aria-label='Active']"
-39.Click  Submit,click,,"//button[normalize-space()='Submit']"
-40.Verify Sucess, verify, , "//div[@aria-label='Info']"
-41.Click Settings ,click,,"//button[contains(., 'Settings')]"
-42.Click Promocode,click,,"//div[normalize-space()='Promocode']"
-43.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
-44.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
-45.Select User,click,,"//li[@aria-label='{customerName}']"
-46.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
-47.Enter Code Name, type, GoldMember001, "//input[@placeholder='Code Name']"
-48.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
-49.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
-50.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
-51.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
-52.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
-53.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
-54.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
-55.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
-56.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
-57.Click Submit ,click,,"//button[normalize-space()='Submit']"
-58.Verify Sucess, verify, , "//div[@aria-label='Info']"
-59.wait,2000,,
-60.Click Settings ,click,,"//button[contains(., 'Settings')]"
-61.Click Service Settings ,click,,"//div[normalize-space()='Service Setting']"
-62.Enter Driver Accept Timeout, type, 60, "//label[contains(., "Driver Accept Timeout")]/following::input[1]"
-63.Enter Driver Serach Radius, type, 50, "//label[contains(., "Driver Search Radius")]/following::input[1]"
-64.Open Tax Type Dropdown,click,,"//span[@aria-label='Select Tax Rype']"
-65.Select Amount,click,,"//li[@aria-label='Amount']"
-66.Enter Tax, type, 20, "//label[contains(., 'Tax')]/following::input[1]"
-67.Open Platform Fee Type Dropdown,click,,"//label[contains(., 'Platform Fee Type')]/following::span[@role='combobox']"
-68.Select Amount,click,,"//li[@aria-label='Amount']"
-69.Enter Platform Fee, type, 20, "//label[contains(., "Platform Fee")]/following::input[1]"
-70.Click Submit ,click,,"//button[normalize-space()='Submit']"
-71.Verify Sucess, verify, , "//div[@aria-label='Info']"
-72.wait,1000,,
-73.Click Settings ,click,,"//button[contains(., 'Settings')]"
-74.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
-75.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
-76.Enter Name, type, Driving License, "//label[contains(., 'Name')]/following::input[1]"
-77.Open status Dropdown,click,,"//label[contains(., 'Status')]/following::div[contains(@class, 'p-dropdown')]"
-78.Select Active,click,,"//li[@aria-label='Active']"
-79.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
-80.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
-81.Click  Require Proof Number,click,,"//div[./div[contains(text(), 'Require Proof Number')]]//input"
-82.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
-83.Click Submit ,click,,"//button[normalize-space()='Submit']"
-84.Verify Sucess, verify, , "//div[@aria-label='Info']"
-85.Filter Document List,type,Driving License,"//input[@aria-label='Name Filter Input']"
-86.wait,1000,,
-88.Click Settings ,click,,"//button[contains(., 'Settings')]"
-89.Click Customer Loyalty Settings,click,,"//div[text()=' Customer Loyalty Settings ']"
-90.Open status Allow Customer loyalty points,click,,"//label[contains(., 'Allow Customer loyalty points')]/following::div[contains(@class, 'p-dropdown')]"
-91.Select ON,click,,"//li[@role='option']//span[text()='ON']"
-92.Enter Minimum order amount for eligibility to redeem loyalty points, type, 25,"//label[contains(., 'Minimum order amount for eligibility to redeem loyalty points')]/following::input[1]"
-93.Enter Loyalty points redeem per order (in %) (% of order amount), type, 10,"//label[contains(., 'Loyalty points redeem per order (in %) (% of order amount)')]/following::input[1]"
-94.Enter Loyalty points per default currency (for ex. $1 = 10 points), type, 5,"//label[contains(., 'Loyalty points per default currency (for ex. $1 = 10 points)')]/following::input[1]"
-95.Click Submit ,click,,"//button[normalize-space()='Submit']"
-96.Verify Sucess, verify, , "//div[@aria-label='Info']"
-97.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-98.Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-99.Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-100.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-101.Select Bus Ride Option,click,,"//span[normalize-space()='{transportName}']"
-102.Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-103.Enter Driver Name, type, busdriver_{timestamp} &gt;&gt; busDriverName, "//label[contains(.,'Full Name')]/following::input[1]"
-104.Enter Email, type, busdriver_{timestamp}@gmail.com&gt;&gt;busEmail, "//label[contains(.,'Email')]/following::input[1]"
-105.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-106.Upload Profile Image, uploadfile, "src/main/resources/test-data/busdriver.jpg", "//input[@type='file']"
-107.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-108.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-109.Select  volvo Option,click,,"//li[@role='option']//span[text()='volvo']"
-110.Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-111.Enter Vehicle Company, type, tata, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-112.Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
-113. Enter Model Name, type, deisel, "//label[contains(.,'Model Name')]/following::input[1]"
-114.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/busvolvo.jpeg", "(//input[@type='file'])[2]"
-115. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-116.Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-117.Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-118.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-119.Enter Account Holder Name, type, {busDriverName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-120.Enter Payment Email Address, type, {busEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-121.Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-122.Click Submit, click, , "//button[contains(.,'Submit')]"
-123.Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-124.Wait for Toast to hide, wait, 1000,
-125.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-126.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-127.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-128.Filter by Name,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
-129.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-130.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-131.FilterDocumet List,type,Driving License,"//input[@aria-label='Document Name Filter Input']"
-132.Add Driving License,click,,"//i[@title='Edit']"
-133.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-134.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-135.Click Submit, click, , "//button[normalize-space()='Submit']"
-136.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-137.Click Approve Driver,click,,"//i[@title='Approve']"
-138.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-139.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-140.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-141.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-142.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-143.Filter Approved Driver,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
-144.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
-145.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
-146.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
-147.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
-148.Click Edit Icon ,click,,"//i[@title='Edit']"
-149.Scroll Grid, tab, 5, "//input[@placeholder='Service Name']"
-150.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-151.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
-152.Click  Submit,click,,"//button[normalize-space()='Submit']"
-153.Verify Sucess, verify, , "//div[@aria-label='Info']"
-154.wait,2000,,
-</t>
-  </si>
-  <si>
-    <t>SA_TS_14</t>
-  </si>
-  <si>
-    <t>Clean The Test Data Created During Test Run</t>
-  </si>
-  <si>
-    <t>TC_CA_14_test_data_cleanup</t>
-  </si>
-  <si>
-    <t>This test phase ensures the long-term stability and performance of the QA environment by executing a systematic Automated Data Cleanup strategy. Leveraging localized SQL Hooks with built-in safety firewalls, the workflow identifies and removes dynamically generated test artifacts—including unique City Areas, Provider profiles, and administrative accounts—created during the regression suite. By targeting specific records using variable-driven WHERE clauses, the script maintains database referential integrity, prevents record duplication in subsequent runs, and ensures the test environment remains in a pristine, 'ready-state' for continuous integration</t>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
+2.Click Provider Services,click,,"//h2[contains(text(), 'Provider Services')]"
+3.Verify Provider Services,verify,,"//div[normalize-space()='ON-DEMAND SERVICES']"
+4.Click  Add New Services,click,,"//button[normalize-space()='Add New Services']"
+5.Enter Service Name, type, Painter{randomAlpha}&gt;&gt; serviceName, "//input[@placeholder='Service Name']"
+6.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
+7.Enter Service Name Arabic, type, دهان, "//input[@placeholder='Service Name (in Arabic)']"
+8.Enter Service Name Hindi, type, पेंटर, "//input[@placeholder='Service Name (in Hindi)']"
+9.Enter Slug, type, painter, "//input[@placeholder='Slug']"
+10.Upload Service Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file' and @accept='image/*']"
+11.wait,2000,,
+12.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+13.Select Activate,click,,"//li[@aria-label='Activate']"
+14.Open Select City Dropdown,click,,"//div[contains(@class, 'p-multiselect-label-container')]"
+15.Select {areaName},click,,"//li[contains(@aria-label, '{areaName}')]"
+16.Click  Submit,click,,"//button[normalize-space()='Submit']"
+17.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
+18.Click Home Icon ,click,,"//i[@title='Home']"
+19.Click Settings ,click,,"//button[contains(., 'Settings')]"
+20.Click Requirment Document ,click,,"//div[normalize-space()='Required Document']"
+21.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
+22.Enter Name, type, documet{randomAlpha}&gt;&gt; providerDocumentName, "//input[@placeholder='Type here']"
+23.Open status Dropdown,click,,"//span[@aria-label='Status']"
+24.Select Active,click,,"//li[@aria-label='Active']"
+25.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
+26.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
+27.Click Submit ,click,,"//button[normalize-space()='Submit']"
+28.Verify Sucess, verify, , "//div[@aria-label='Info']"
+29.Filter Document List,type,{providerDocumentName},"//input[@aria-label='Name Filter Input']"
+30.Click Settings ,click,,"//button[contains(., 'Settings')]"
+31.Click Promocode ,click,,"//div[normalize-space()='Promocode']"
+32.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
+33.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
+34.Select User,click,,"//li[@aria-label='{customerName}']"
+35.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
+35.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; providerPromoCodeName, "//input[@placeholder='Code Name']"
+36.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
+37.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
+38.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
+39.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
+40.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
+41.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
+42.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
+43.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
+44.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
+45.Click Submit ,click,,"//button[normalize-space()='Submit']"
+46.Verify Sucess, verify, , "//div[@aria-label='Info']"
+47.Filter PromoCode List,type,{providerPromoCodeName},"//input[@aria-label='Promocode Filter Input']"
+48.Click  Providers,click,,"//button[contains(., 'Providers')]"
+49.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
+50.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
+51.Enter Provider Full Name, type, Painter{randomAlpha}&gt;&gt; painterName, "//input[@placeholder='Provider Full Name']"
+52.Upload Painter Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file']"
+53.Enter Email, type, Painter_{timestamp}@gmail.com&gt;&gt;painterEmail, "//input[@placeholder='Unique Email']"
+54.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
+55.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
+56.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
+57.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
+58.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
+59.Enter Provider Address, type, painter chennai, "//input[@placeholder='Enter provider Address']"
+60.wait,1000,,
+61.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
+62.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
+63.wait,1000,,
+64.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
+65.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
+66.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
+67.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
+68.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
+69.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
+70.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
+71.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
+72.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
+73.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
+74.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
+75.Enter Accont Holder Name, type, {painterName}, "//input[@placeholder='Account Holder Name']"
+76.Enter Payment Email Address, type, {painterEmail}, "//input[@placeholder='Email Address for Payment Notification']"
+77.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
+78.Click Save, click, , "//button[@type='submit']"
+79.Verify Sucess, verify, , "//div[@aria-label='Info']"
+80.Filter Painter List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
+81.Click  Providers,click,,"//button[contains(., 'Providers')]"
+82.Select Pending Document Providers,click,,"//div[normalize-space()='Pending Document Providers']"
+83.Filter Plumber List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
+84.Click Document Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+85. Provider Required Documents,verify,,"//div[contains(text(),'Documents')]"
+86.FilterDocumet List,type,{providerDocumentName},"//input[@aria-label='Document Name Filter Input']"
+87.Add Address Proof,click,,"(//i[contains(@class, 'Edit')])[1]"
+88.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
+89.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+90.Click Submit, click, , "//button[normalize-space()='Submit']"
+91.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+92.FilterDocumet List,type,{providerDocumentName},"//input[@aria-label='Document Name Filter Input']"
+93.Click Approve Store,click,,"//div[@row-index='0']//i[contains(@class, 'bi-hand-thumbs-up-fill')]"
+94.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+95.Click Back, click, , "//button[@class='buttonWidget']"
+96.Click  Providers,click,,"//button[normalize-space()='Category']"
+97.Click  Add New Category,click,,"//button[normalize-space()='ADD CATEGORY']"
+98.Enter Category Name, type,residentialPainter{randomAlpha}&gt;&gt; painterCategoryName, "//input[@placeholder='Enter the category name']"
+99.Enter Category Name Tamil, type, குடியிருப்பு பெயிண்டர், "//input[@placeholder='Category Name (in Tamil)']"
+100.Enter Category Name Arabic, type, دهان سكني, "//input[@placeholder='Category Name (in Arabic)']"
+101.Enter Category Name Hindi, type, आवासीय पेंटर, "//input[@placeholder='Category Name (in Hindi)']"
+102.Open Category status Dropdown,click,,"//span[@aria-label='Select a category status']"
+103.Select Activate,click,,"//li[@aria-label='Active']"
+104.Upload Category Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file' and @accept='image/*']"
+105.wait,2000,,
+106.Click  Submit,click,,"//button[normalize-space()='Submit']"
+107.Filter Category Name,type,{painterCategoryName},"//input[@aria-label='Category Name Filter Input']"
+108.Click  Providers,click,,"//button[contains(., 'Providers')]"
+109.Select Provider List,click,,"//div[normalize-space()='Provider List']"
+110.Filter Painter List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
+111.Scroll Grid, tab, 7, "//input[@aria-label='Provider Name Filter Input']"
+112.Click Package Icon,click,,"//i[@class='bi bi-box-seam cursor-pointer gridIcon Navigate']"
+113.Click  Add Package,click,,"//button[normalize-space()='Add Package']"
+114.Open Category  Dropdown,click,,"//span[@aria-label='Package Category']"
+115.Select Activate,click,,"//li[@aria-label='{painterCategoryName}']"
+116.Enter Package Name, type, package{randomAlpha}&gt;&gt; packageName, "//input[@placeholder='Package Name']"
+117.Enter Amount, type, 1000, "//input[@placeholder='Amount Value']"
+118.Open Max Book Quantity  Dropdown,click,,"//span[@aria-label='Package Max Book Quantity']"
+119.Select 4,click,,"//li[@aria-label='4']"
+120.Open Status Dropdown,click,,"//span[@aria-label='select Status']"
+121.Select Activate,click,,"//li[@aria-label='Activate']"
+122.Enter Description, type, Premium residential painting package, "//textarea[@placeholder='Description']"
+123.Click  Submit,click,,"//button[normalize-space()='Submit']"
+124.wait,1000,,
+125.Click  back,click,,"//button[normalize-space()='Back']"
+126.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
+127.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
+128.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
+129.Click Edit Icon ,click,,"//i[@title='Edit']"
+130.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
+131.Enter Service Name Arabic, type, دهان, "//input[@placeholder='Service Name (in Arabic)']"
+132.Enter Service Name Hindi, type, पेंटर, "//input[@placeholder='Service Name (in Hindi)']"
+133.Scroll Grid, tab, 4, "//input[@placeholder='Service Name (in Hindi)']"
+134.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+135.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
+136.Click  Submit,click,,"//button[normalize-space()='Submit']"
+137.Click  back,click,,"//button[normalize-space()='Back']"
+138.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
+139.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
+140.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
+141.wait,1000,,</t>
   </si>
   <si>
     <t>1.Remove Test Area,sql delete,,"DELETE FROM we1.admin_area_list WHERE name = '{areaName}';"
-2.wait,2000,,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-2. Click City area menu,click,,"//span[normalize-space()='City area']"
-3. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
-4. Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
-5. Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
-6. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
-7. Open Status Dropdown,click,,"//span[@aria-label='select status']"
-8. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-9. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
-10. Click Submit,click,,"//button[normalize-space()='Submit']"
-11. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
-12. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
-13. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
-14. Click Add Category,click,,"//button[normalize-space()='Add Category']"
-15. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
-16. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
-17. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
-18. Click close,click,,"//button[normalize-space()='Close']"
-19. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-20. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-21. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
-22. Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
-23. Open Select City Dropdown,click,,"//select[@id='cityId']"
-24. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-25. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
-</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>CRITICAL SYSTEM WARNING: DATABASE INTEGRITY PROTOCOL</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-----------------------------------------</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">This sheet contains SQL Hooks that execute directly against the we1 Production/Staging database. DO NOT modify the SQL syntax, remove variable placeholders (e.g., {areaName}), or edit the WHERE clauses.
-Unauthorized changes may result in irreversible data loss or database corruption. If modifications are required, please contact the Automation Lead or the Database Administrator.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PASSWORD TO EDIT SHEET</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> :eit6190
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.
-RunSheet: SuperAdminLogin
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
+2.Remove Customer,sql delete,,"DELETE FROM we1.users WHERE first_name = '{customerName}';"
+3.Remove City Admin,sql delete,,"DELETE FROM we1.super_admin WHERE name = '{adminName}';"
+4.Remove Auto Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{autoName}';"
+5.Remove Auto Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{autoName}';"
+6.Remove Auto Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{autoCompanyName}';"
+7.Remove Bike Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{bikeName}';"
+8.Remove Bike Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{bikeName}';"
+9.Remove Bike Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{bikeCompanyName}';"
+10.Remove Taxi Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{taxiName}';"
+11.Remove Taxi Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{taxiName}';"
+12.Remove Taxi Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{taxiCompanyName}';"
+13.Remove Bus Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{busDriverName}';"
+14.Remove Bus Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{busDriverName}';"
+15.Remove Bus Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{busCompanyName}';"
+16.Remove Bus Driver Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{documentName}';"
+17.Remove Transport Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{promoCodeName}';"
+18.Remove Bus Vehicle Variation Volvo,sql delete,,"DELETE FROM we1.transport_vehicle_type WHERE name = '{busTypeName}';"
+19.Remove  Transport Ride,sql delete,,"DELETE FROM we1.service_category WHERE name = '{transportName}';"
+20.Remove Kfc Private Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{kfcdriverName}';"
+21.Remove Kfc Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{kfcBikeCompanyName}';"
+22.Remove Kfc Product Details,sql delete,,"DELETE FROM we1.store_product_details WHERE name = '{kfcProductName}';"
+23.Remove Kfc Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{storeOwner}';"
+24.Remove Kfc Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{storeOwner}';"
+25.Remove Kfc Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{storeName}';"
+26.Remove Bilal Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{hotelOwner}';"
+27.Remove Bilal Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{hotelOwner}';"
+28.Remove Bilal Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{hotelName}';"
+29.Remove Amul Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{milkStoreOwner}';"
+30.Remove Amul Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{milkStoreOwner}';"
+31.Remove Amul Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{milkStore}';"
+32.Remove Curd Product Category,sql delete,,"DELETE FROM we1.store_product_category WHERE name = '{MilkCategoryName}';"
+33.Remove Delievery Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{deliveryDocumentName}';"
+34.Remove Delievery Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{deliveryPromoCodeName}';"
+35.Remove  Deleivrey Service,sql delete,,"DELETE FROM we1.service_category WHERE name = '{deliveryName}';"
+36.Remove Plumber Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{plumberName}';"
+37.Remove Plumber Provider Details,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{plumberName}';"
+38.Remove Painter Package,sql delete,,"DELETE FROM we1.other_service_provider_packages WHERE name = '{packageName}';"
+39.Remove Painter Sub Category,sql delete,,"DELETE FROM we1.other_service_sub_category WHERE name = '{painterCategoryName}';"
+40.Remove Provider Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{providerDocumentName}';"
+41.Remove Provider Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{providerPromoCodeName}';"
+42.Remove Painter Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{painterName}';"
+43.Remove Painter From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{painterName}';"
+44.Remove Provider Service,sql delete,,"DELETE FROM we1.service_category WHERE name = '{serviceName}';"
+45.wait,2000,,</t>
   </si>
 </sst>
 </file>
@@ -3012,13 +3058,13 @@
         <v>31</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>49</v>
+        <v>90</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>41</v>
@@ -3084,16 +3130,16 @@
         <v>34</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>35</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>48</v>
+        <v>91</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3150,22 +3196,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3222,22 +3268,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>38</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3294,22 +3340,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>71</v>
+        <v>93</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3366,22 +3412,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3392,7 +3438,7 @@
       <c r="E3" s="8"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="n2KwI2T0nM4kUyp7LiUODpwAG/galVyQSDtsZl0yUO+rjA55NBZcPk6XHtPhEPr+7rDS1I7x7D4NXk32F3GmoA==" saltValue="GAfl83kbCDLkZxzinmefRw==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="DqE1814P8bOJA2mrdcTnqHRVqCJMD/2LmSxLLnNa47sn/9DqPhga1D3bKgFI0NpAFAU7XBeAvjl+0K9pV6Ij3g==" saltValue="JBa6gN7OIbu41Q1IhDHnzw==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -3444,19 +3490,19 @@
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3523,16 +3569,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3598,7 +3644,7 @@
         <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>26</v>
@@ -3663,16 +3709,16 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>45</v>
+        <v>86</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3735,16 +3781,16 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>46</v>
+        <v>87</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3807,16 +3853,16 @@
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>47</v>
+        <v>88</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3876,19 +3922,19 @@
         <v>30</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="9" t="s">
-        <v>84</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3952,16 +3998,16 @@
         <v>28</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>29</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
62th commit: Read Me Updated and Multiple Database Run Implemented
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA7C2B5A-73CC-4484-9D74-B97A6F10A87D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8DAE119-D7FC-4BEB-BED4-55AC025B7B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="11" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -1883,162 +1883,6 @@
 50.Click Doc Icon,click,,"//i[@title='Document']"
 51.Click Eye Icon,click,,"//i[@title='View']"
 52.wait,1000,,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
-2. Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
-3.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
-4.Click  Add Category,click,,"//button[normalize-space()='Add Category']"
-5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "//input[@placeholder='Service Name']"
-6.Enter Service Name Arabic, type, رحلة بالحافلة, "//input[@placeholder='Service Name (in Arabic)']"
-7.Enter Slug, type, Bus Ride, "//input[@placeholder='Slug']"
-8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "//input[@type='file' and @accept='image/*']"
-9.wait,2000,,
-10.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-11.Select Activate,click,,"//li[@aria-label='Activate']"
-12.Open Select City Dropdown,click,,"//span[text()='Select City']/ancestor::app-drop-down//div[contains(@class, 'p-multiselect-label-container')]"
-13.Select {areaName},click,,"//li[@aria-label='{areaName}']"
-14.Click  Submit,click,,"//button[normalize-space()='Submit']"
-15.Verify Sucess, verify, , "//div[@aria-label='Info']"
-16.wait,2000,,
-17.Click  back,click,,"//button[normalize-space()='Back']"
-18.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
-19.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
-20.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
-21.Click Home Icon ,click,,"//i[@title='Home']"
-22.Click Settings ,click,,"//button[contains(., 'Settings')]"
-23.Click Vehicle Type,click,,"//div[normalize-space()='Vehicle Type']"
-24.Click Add Vehicle Type,click,,"//button[normalize-space()='Add Vehicle Type']"
-25.Enter Vehicle Type Name, type, volvo{randomAlpha}&gt;&gt;busTypeName, "//input[@placeholder='Type here']"
-26.Enter Cost For Km, type, 150, "//input[@placeholder='Cost For Km']"
-27.Enter Time Fare Per Min, type,10, "//input[@placeholder='Time Fare Per Min']"
-28.Enter Base fare, type,100, "//input[@placeholder='Base fare']"
-29.Enter Min Fare Amount, type,50, "//input[@placeholder='Min Fare Amount']"
-30.Enter Rental Cost For Km, type,30, "//input[@placeholder='Rental Cost For Km']"
-31.Enter Rental Amount For 1 Hour, type,50, "//input[@placeholder='Rental Amount For 1 Hour']"
-32.Enter Rental Km Limit For 1 Hour, type,50, "//input[@placeholder='Rental Km Limit For 1 Hour']"
-33.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "//app-image-upload//input[@type='file' and @accept='image/*']"
-34.Click Surcharge Time Checkbox, click, , "//div[text()='EveryDay']/preceding-sibling::mat-checkbox"
-35.Enter From Time, type, 100000, "//app-time-picker//input[@type='time']"
-36.Enter To Time, type, 220000, "(//app-time-picker//input[@type='time'])[2]"
-37.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-38.Select Active,click,,"//li[@aria-label='Active']"
-39.Click  Submit,click,,"//button[normalize-space()='Submit']"
-40.Verify Sucess, verify, , "//div[@aria-label='Info']"
-41.Click Settings ,click,,"//button[contains(., 'Settings')]"
-42.Click Promocode,click,,"//div[normalize-space()='Promocode']"
-43.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
-44.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
-45.Select User,click,,"//li[@aria-label='{customerName}']"
-46.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
-47.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; promoCodeName, "//input[@placeholder='Code Name']"
-48.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
-49.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
-50.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
-51.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
-52.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
-53.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
-54.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
-55.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
-56.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
-57.Click Submit ,click,,"//button[normalize-space()='Submit']"
-58.Verify Sucess, verify, , "//div[@aria-label='Info']"
-59.wait,2000,,
-60.Click Settings ,click,,"//button[contains(., 'Settings')]"
-61.Click Service Settings ,click,,"//div[normalize-space()='Service Setting']"
-62.Enter Driver Accept Timeout, type, 60, "//label[contains(., "Driver Accept Timeout")]/following::input[1]"
-63.Enter Driver Serach Radius, type, 50, "//label[contains(., "Driver Search Radius")]/following::input[1]"
-64.Open Tax Type Dropdown,click,,"//span[@aria-label='Select Tax Rype']"
-65.Select Amount,click,,"//li[@aria-label='Amount']"
-66.Enter Tax, type, 20, "//label[contains(., 'Tax')]/following::input[1]"
-67.Open Platform Fee Type Dropdown,click,,"//label[contains(., 'Platform Fee Type')]/following::span[@role='combobox']"
-68.Select Amount,click,,"//li[@aria-label='Amount']"
-69.Enter Platform Fee, type, 20, "//label[contains(., "Platform Fee")]/following::input[1]"
-70.Click Submit ,click,,"//button[normalize-space()='Submit']"
-71.Verify Sucess, verify, , "//div[@aria-label='Info']"
-72.wait,1000,,
-73.Click Settings ,click,,"//button[contains(., 'Settings')]"
-74.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
-75.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
-76.Enter Name, type, documet{randomAlpha}&gt;&gt; documentName, "//label[contains(., 'Name')]/following::input[1]"
-77.Open status Dropdown,click,,"//label[contains(., 'Status')]/following::div[contains(@class, 'p-dropdown')]"
-78.Select Active,click,,"//li[@aria-label='Active']"
-79.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
-80.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
-81.Click  Require Proof Number,click,,"//div[./div[contains(text(), 'Require Proof Number')]]//input"
-82.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
-83.Click Submit ,click,,"//button[normalize-space()='Submit']"
-84.Verify Sucess, verify, , "//div[@aria-label='Info']"
-85.Filter Document List,type,{documentName},"//input[@aria-label='Name Filter Input']"
-86.wait,1000,,
-88.Click Settings ,click,,"//button[contains(., 'Settings')]"
-89.Click Customer Loyalty Settings,click,,"//div[text()=' Customer Loyalty Settings ']"
-90.Open status Allow Customer loyalty points,click,,"//label[contains(., 'Allow Customer loyalty points')]/following::div[contains(@class, 'p-dropdown')]"
-91.Select ON,click,,"//li[@role='option']//span[text()='ON']"
-92.Enter Minimum order amount for eligibility to redeem loyalty points, type, 25,"//label[contains(., 'Minimum order amount for eligibility to redeem loyalty points')]/following::input[1]"
-93.Enter Loyalty points redeem per order (in %) (% of order amount), type, 10,"//label[contains(., 'Loyalty points redeem per order (in %) (% of order amount)')]/following::input[1]"
-94.Enter Loyalty points per default currency (for ex. $1 = 10 points), type, 5,"//label[contains(., 'Loyalty points per default currency (for ex. $1 = 10 points)')]/following::input[1]"
-95.Click Submit ,click,,"//button[normalize-space()='Submit']"
-96.Verify Sucess, verify, , "//div[@aria-label='Info']"
-97.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-98.Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-99.Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-100.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-101.Select Bus Ride Option,click,,"//span[normalize-space()='{transportName}']"
-102.Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-103.Enter Driver Name, type, busdriver_{timestamp} &gt;&gt; busDriverName, "//label[contains(.,'Full Name')]/following::input[1]"
-104.Enter Email, type, busdriver_{timestamp}@gmail.com&gt;&gt;busEmail, "//label[contains(.,'Email')]/following::input[1]"
-105.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-106.Upload Profile Image, uploadfile, "src/main/resources/test-data/busdriver.jpg", "//input[@type='file']"
-107.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-108.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-109.Select  volvo Option,click,,"//li[@role='option']//span[text()='{busTypeName}']"
-110.Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-111.Enter Vehicle Company, type, busCompany{randomAlpha}&gt;&gt; busCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-112.Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
-113. Enter Model Name, type, deisel, "//label[contains(.,'Model Name')]/following::input[1]"
-114.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/busvolvo.jpeg", "(//input[@type='file'])[2]"
-115. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-116.Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-117.Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-118.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-119.Enter Account Holder Name, type, {busDriverName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-120.Enter Payment Email Address, type, {busEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-121.Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-122.Click Submit, click, , "//button[contains(.,'Submit')]"
-123.Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-124.Wait for Toast to hide, wait, 1000,
-125.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-126.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-127.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-128.Filter by Name,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
-129.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-130.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-131.FilterDocumet List,type,{documentName},"//input[@aria-label='Document Name Filter Input']"
-132.Add Driving License,click,,"//i[@title='Edit']"
-133.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-134.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-135.Click Submit, click, , "//button[normalize-space()='Submit']"
-136.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-137.Click Approve Driver,click,,"//i[@title='Approve']"
-138.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-139.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-140.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-141.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-142.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-143.Filter Approved Driver,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
-144.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
-145.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
-146.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
-147.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
-148.Click Edit Icon ,click,,"//i[@title='Edit']"
-149.Scroll Grid, tab, 5, "//input[@placeholder='Service Name']"
-150.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-151.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
-152.Click  Submit,click,,"//button[normalize-space()='Submit']"
-153.Verify Sucess, verify, , "//div[@aria-label='Info']"
-154.wait,2000,,
-</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
@@ -2564,6 +2408,164 @@
 43.Remove Painter From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{painterName}';"
 44.Remove Provider Service,sql delete,,"DELETE FROM we1.service_category WHERE name = '{serviceName}';"
 45.wait,2000,,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+2. Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+3.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
+4.Click  Add Category,click,,"//button[normalize-space()='Add Category']"
+5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "//input[@placeholder='Service Name']"
+6.Enter Service Name Arabic, type, رحلة بالحافلة, "//input[@placeholder='Service Name (in Arabic)']"
+7.Enter Slug, type, Bus Ride, "//input[@placeholder='Slug']"
+8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "//input[@type='file' and @accept='image/*']"
+9.wait,2000,,
+10.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+11.Select Activate,click,,"//li[@aria-label='Activate']"
+12.Open Select City Dropdown,click,,"//span[text()='Select City']/ancestor::app-drop-down//div[contains(@class, 'p-multiselect-label-container')]"
+13.Select {areaName},click,,"//li[@aria-label='{areaName}']"
+14.Click  Submit,click,,"//button[normalize-space()='Submit']"
+15.Verify Sucess, verify, , "//div[@aria-label='Info']"
+16.wait,2000,,
+17.Click  back,click,,"//button[normalize-space()='Back']"
+18.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+19.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+20.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
+21.Click Home Icon ,click,,"//i[@title='Home']"
+22.Click Settings ,click,,"//button[contains(., 'Settings')]"
+23.Click Vehicle Type,click,,"//div[normalize-space()='Vehicle Type']"
+24.Click Add Vehicle Type,click,,"//button[normalize-space()='Add Vehicle Type']"
+25.Enter Vehicle Type Name, type, volvo{randomAlpha}&gt;&gt;busTypeName, "//input[@placeholder='Type here']"
+26.Enter Cost For Km, type, 150, "//input[@placeholder='Cost For Km']"
+27.Enter Time Fare Per Min, type,10, "//input[@placeholder='Time Fare Per Min']"
+28.Enter Base fare, type,100, "//input[@placeholder='Base fare']"
+29.Enter Min Fare Amount, type,50, "//input[@placeholder='Min Fare Amount']"
+30.Enter Rental Cost For Km, type,30, "//input[@placeholder='Rental Cost For Km']"
+31.Enter Rental Amount For 1 Hour, type,50, "//input[@placeholder='Rental Amount For 1 Hour']"
+32.Enter Rental Km Limit For 1 Hour, type,50, "//input[@placeholder='Rental Km Limit For 1 Hour']"
+33.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "//app-image-upload//input[@type='file' and @accept='image/*']"
+34.Click Surcharge Time Checkbox, click, , "//div[text()='EveryDay']/preceding-sibling::mat-checkbox"
+35.Enter From Time, type, 100000, "//app-time-picker//input[@type='time']"
+36.Enter To Time, type, 220000, "(//app-time-picker//input[@type='time'])[2]"
+37.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+38.Select Active,click,,"//li[@aria-label='Active']"
+39.Click  Submit,click,,"//button[normalize-space()='Submit']"
+40.Verify Sucess, verify, , "//div[@aria-label='Info']"
+41.Click Settings ,click,,"//button[contains(., 'Settings')]"
+42.Click Promocode,click,,"//div[normalize-space()='Promocode']"
+43.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
+44.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
+45.Select User,click,,"//li[@aria-label='{customerName}']"
+46.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
+47.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; promoCodeName, "//input[@placeholder='Code Name']"
+48.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
+49.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
+50.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
+51.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
+52.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
+53.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
+54.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
+55.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
+56.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
+57.Click Submit ,click,,"//button[normalize-space()='Submit']"
+58.Verify Sucess, verify, , "//div[@aria-label='Info']"
+59.wait,2000,,
+60.Click Settings ,click,,"//button[contains(., 'Settings')]"
+61.Click Service Settings ,click,,"//div[normalize-space()='Service Setting']"
+62.Enter Driver Accept Timeout, type, 60, "//label[contains(., "Driver Accept Timeout")]/following::input[1]"
+63.Enter Driver Serach Radius, type, 50, "//label[contains(., "Driver Search Radius")]/following::input[1]"
+64.Open Tax Type Dropdown,click,,"//span[@aria-label='Select Tax Rype']"
+65.Select Amount,click,,"//li[@aria-label='Amount']"
+66.Enter Tax, type, 20, "//label[contains(., 'Tax')]/following::input[1]"
+67.Open Platform Fee Type Dropdown,click,,"//label[contains(., 'Platform Fee Type')]/following::span[@role='combobox']"
+68.Select Amount,click,,"//li[@aria-label='Amount']"
+69.Enter Platform Fee, type, 20, "//label[contains(., "Platform Fee")]/following::input[1]"
+70.Click Submit ,click,,"//button[normalize-space()='Submit']"
+71.Verify Sucess, verify, , "//div[@aria-label='Info']"
+72.wait,1000,,
+73.Click Settings ,click,,"//button[contains(., 'Settings')]"
+74.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
+75.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
+76.Enter Name, type, documet{randomAlpha}&gt;&gt; documentName, "//label[contains(., 'Name')]/following::input[1]"
+77.Open status Dropdown,click,,"//label[contains(., 'Status')]/following::div[contains(@class, 'p-dropdown')]"
+78.Select Active,click,,"//li[@aria-label='Active']"
+79.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
+80.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
+81.Click  Require Proof Number,click,,"//div[./div[contains(text(), 'Require Proof Number')]]//input"
+82.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
+83.Click Submit ,click,,"//button[normalize-space()='Submit']"
+84.Verify Sucess, verify, , "//div[@aria-label='Info']"
+85.Filter Document List,type,{documentName},"//input[@aria-label='Name Filter Input']"
+86.wait,1000,,
+88.Click Settings ,click,,"//button[contains(., 'Settings')]"
+89.Click Customer Loyalty Settings,click,,"//div[text()=' Customer Loyalty Settings ']"
+90.Open status Allow Customer loyalty points,click,,"//label[contains(., 'Allow Customer loyalty points')]/following::div[contains(@class, 'p-dropdown')]"
+91.Select ON,click,,"//li[@role='option']//span[text()='ON']"
+92.Enter Minimum order amount for eligibility to redeem loyalty points, type, 25,"//label[contains(., 'Minimum order amount for eligibility to redeem loyalty points')]/following::input[1]"
+93.Enter Loyalty points redeem per order (in %) (% of order amount), type, 10,"//label[contains(., 'Loyalty points redeem per order (in %) (% of order amount)')]/following::input[1]"
+94.Enter Loyalty points per default currency (for ex. $1 = 10 points), type, 5,"//label[contains(., 'Loyalty points per default currency (for ex. $1 = 10 points)')]/following::input[1]"
+95.Click Submit ,click,,"//button[normalize-space()='Submit']"
+96.Verify Sucess, verify, , "//div[@aria-label='Info']"
+97.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+98.Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+99.Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+100.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+101.Select Bus Ride Option,click,,"//span[normalize-space()='{transportName}']"
+102.Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+103.Enter Driver Name, type, busdriver_{timestamp} &gt;&gt; busDriverName, "//label[contains(.,'Full Name')]/following::input[1]"
+104.Enter Email, type, busdriver_{timestamp}@gmail.com&gt;&gt;busEmail, "//label[contains(.,'Email')]/following::input[1]"
+105.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+106.Upload Profile Image, uploadfile, "src/main/resources/test-data/busdriver.jpg", "//input[@type='file']"
+107.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+108.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+109.Select  volvo Option,click,,"//li[@role='option']//span[text()='{busTypeName}']"
+110.Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+111.Enter Vehicle Company, type, busCompany{randomAlpha}&gt;&gt; busCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+112.Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+113. Enter Model Name, type, deisel, "//label[contains(.,'Model Name')]/following::input[1]"
+114.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/busvolvo.jpeg", "(//input[@type='file'])[2]"
+115. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+116.Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+117.Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+118.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+119.Enter Account Holder Name, type, {busDriverName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+120.Enter Payment Email Address, type, {busEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+121.Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+122.Click Submit, click, , "//button[contains(.,'Submit')]"
+123.Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+124.Wait for Toast to hide, wait, 1000,
+125.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+126.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+127.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+128.Filter by Name,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
+129.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+130.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+131.FilterDocumet List,type,{documentName},"//input[@aria-label='Document Name Filter Input']"
+132.Add Driving License,click,,"//i[@title='Edit']"
+133.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+134.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+135.Click Submit, click, , "//button[normalize-space()='Submit']"
+136.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+137.Click Approve Driver,click,,"//i[@title='Approve']"
+138.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+139.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+140.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+141.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+142.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+143.Filter Approved Driver,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
+144.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+145.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+146.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
+147.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
+148.Click Edit Icon ,click,,"//i[@title='Edit']"
+149.wait,2000,,
+150.Scroll Grid, tab, 5, "//input[@placeholder='Service Name']"
+151.wait,2000,,
+152.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+153.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
+154.Click  Submit,click,,"//button[normalize-space()='Submit']"
+155.Verify Sucess, verify, , "//div[@aria-label='Info']"
+156.wait,2000,,
+</t>
   </si>
 </sst>
 </file>
@@ -3064,7 +3066,7 @@
         <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>41</v>
@@ -3136,7 +3138,7 @@
         <v>35</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>50</v>
@@ -3208,7 +3210,7 @@
         <v>65</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>66</v>
@@ -3352,7 +3354,7 @@
         <v>64</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>67</v>
@@ -3424,7 +3426,7 @@
         <v>82</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>84</v>
@@ -3438,7 +3440,7 @@
       <c r="E3" s="8"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="DqE1814P8bOJA2mrdcTnqHRVqCJMD/2LmSxLLnNa47sn/9DqPhga1D3bKgFI0NpAFAU7XBeAvjl+0K9pV6Ij3g==" saltValue="JBa6gN7OIbu41Q1IhDHnzw==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="atjs4lQ1+o6fSFUQ0qpte05fkgrHsWBNK0UOqkGvhk5aH4hAig+bv994FWadvg20PU7CWkefN+SDSjlYBHqE/Q==" saltValue="4xFzDJqljq8EGyX3Igns8Q==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -3931,7 +3933,7 @@
         <v>78</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>77</v>

</xml_diff>

<commit_message>
65th commit: Test Cases Updated after modification
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8DAE119-D7FC-4BEB-BED4-55AC025B7B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46C20AA4-614F-4D1E-AA49-DA772A16BE03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -27,7 +27,8 @@
     <sheet name="DeliveryServiceCompleteTest" sheetId="14" r:id="rId12"/>
     <sheet name="AddProvider" sheetId="11" r:id="rId13"/>
     <sheet name="ProviderServiceCompleteTest" sheetId="12" r:id="rId14"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId15"/>
+    <sheet name="SubscriptionPlanTest" sheetId="29" r:id="rId15"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId16"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="101">
   <si>
     <t>City Area</t>
   </si>
@@ -415,52 +416,6 @@
   </si>
   <si>
     <t>Add New Provider Service &amp;  Category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-4. Verify City Admin List,verify,,"//div[normalize-space()='City Admin List']"
-5. Click Add City Admin button,click,,"//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
-6. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
-7.Select Name field,click ,, "//input[@id='name']"
-8. Enter Admin Name, type, faizal_{timestamp} &gt;&gt; adminName, "//input[@id='name']"
-9.Select Email field,click,, "//input[@id='email']"
-10. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
-11.select the password field,click,, "//input[@id='password']"
-12.Enter the Password as "faizal@123". "//input[@id='password']"
-13.Open Select City Dropdown,click,,"//select[@id='cityId']"
-14.Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-15. Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
-16.Click on the "Customers" → "Add Customers" checkbox. "//label[normalize-space()='Add Customers']"
-17.Click on the "Customers" → "Verified Customers"checkbox. "//label[normalize-space()='Verified Customers']"
-18.Click on the "Customers" → "Non Verified Customers" checkbox. "//label[normalize-space()='Non Verified Customers']"
-19.Click on the "Customers" → "Blocked Customers" checkbox. "//label[normalize-space()='Blocked Customers']"
-20.Click on the "Customers" → "Deleted Customers" checkbox. "//label[normalize-space()='Deleted Customers']"
-21.Click on the "Customers" → "Pending Customers" checkbox. "//label[normalize-space()='Pending Customers']"
-22.Click on the "Providers" → "Transport Providers List" checkbox. "//label[normalize-space()='Transport Providers List']"
-23.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
-24.Click on the "Drivers" → "Approved Drivers" checkbox. "//label[normalize-space()='Approved Drivers']"
-25.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
-26.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
-27.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
-28.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
-29.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox. "//label[normalize-space()='Driver Subscription Plan']"
-30.Click on the "Cash Out" → "Driver Cash Out" checkbox. "//label[normalize-space()='Driver Cash Out']"
-31.Click on the "Report Issue" → "Customer Report Issues" checkbox. "//label[normalize-space()='Customer Report Issues']"
-32.Click on the "Report Issue" → "Driver Report Issues" checkbox. "//label[normalize-space()='Driver Report Issues']"
-33.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
-34.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
-35.Click on the "Report Issue" → "FAQs" checkbox. "(//h3[contains(.,'Report Issue')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
-36.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
-37.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
-38.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[h3[contains(.,'Website Settings')]]//label[contains(.,'Delivery')]"
-39.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[.//h3[contains(text(),'Website Settings')]]//label[contains(.,'Transport')]"
-40.Click on the "Website Settings" → "FAQs" checkbox. "(//h3[contains(.,'Website Settings')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
-41.Click on the "Add City Admin" button. "//button[@type='submit']"
-42. Verify Success Message,verify,,"//div[@aria-label='Info']"
-43.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
-</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
@@ -1490,38 +1445,7 @@
     <t>Clean The Test Data Created During Test Run</t>
   </si>
   <si>
-    <t>TC_CA_14_test_data_cleanup</t>
-  </si>
-  <si>
     <t>This test phase ensures the long-term stability and performance of the QA environment by executing a systematic Automated Data Cleanup strategy. Leveraging localized SQL Hooks with built-in safety firewalls, the workflow identifies and removes dynamically generated test artifacts—including unique City Areas, Provider profiles, and administrative accounts—created during the regression suite. By targeting specific records using variable-driven WHERE clauses, the script maintains database referential integrity, prevents record duplication in subsequent runs, and ensures the test environment remains in a pristine, 'ready-state' for continuous integration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-2. Click City area menu,click,,"//span[normalize-space()='City area']"
-3. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
-4. Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
-5. Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
-6. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
-7. Open Status Dropdown,click,,"//span[@aria-label='select status']"
-8. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-9. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
-10. Click Submit,click,,"//button[normalize-space()='Submit']"
-11. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
-12. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
-13. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
-14. Click Add Category,click,,"//button[normalize-space()='Add Category']"
-15. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
-16. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
-17. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
-18. Click close,click,,"//button[normalize-space()='Close']"
-19. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-20. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-21. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
-22. Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
-23. Open Select City Dropdown,click,,"//select[@id='cityId']"
-24. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-25. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
-</t>
   </si>
   <si>
     <r>
@@ -1640,249 +1564,6 @@
       <t xml:space="preserve">
 </t>
     </r>
-  </si>
-  <si>
-    <t>1. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-2.Click  Add Customers,click,,"//span[normalize-space()='Add customers']"
-3. Verify Add Customer Heading,verify,,"//div[normalize-space()='Add Customer']"
-4.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "//label[contains(., 'Customer Full Name')]/following::input[1]"
-5.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "//input[@type='email']"
-6.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-7.Enter Video Call Limit, type, 60, "//label[contains(., 'User Used Video Call Limit in Minutes')]/following::input[1]"
-8.Open Gender,click,,"//span[@aria-label='select gender']"
-9.Select Male,click,,"//li[@aria-label='Male']"
-10.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "//input[@type='file' and @accept='image/*']"
-11.Click Submit, click, , "//button[normalize-space()='Submit']"
-12.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-13. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-14. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-15.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
-16. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-17.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-18.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
-19.Click Edit Icon ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-20.Click Close, click, , "//button[normalize-space()='Close']"
-21.Click Wallet Icon ,click,,"//i[@title='Wallet']"
-22.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
-23.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
-24.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-25.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
-26.Click Submit, click, , "//button[normalize-space()='Submit']"
-27.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-28.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
-29.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
-30.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-31.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
-32.Click Submit, click, , "//button[normalize-space()='Submit']"
-33.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-34. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-35. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-36.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
-37. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-38.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-39.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
-40.Click Loyalty Points Icon,click,,"//i[@title='Loyalty Points']"
-41.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
-42.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
-43.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
-44.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-45.Select Add Points,click,,"//li[@role='option'][contains(.,'Add Points')]"
-46.Enter Points, type, 30, "//input[@placeholder='Enter Points']"
-47.Click Submit, click, , "//button[normalize-space()='Submit']"
-48.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-49.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
-50.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
-51.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
-52.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-53.Select Deduct Points,click,,"//li[@role='option'][contains(.,'Deduct Points')]"
-54.Enter Points, type, 10, "//input[@placeholder='Enter Points']"
-55.Click Submit, click, , "//button[normalize-space()='Submit']"
-56.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-57. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-58. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-59.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
-60. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-61.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-62.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
-63.Click Disable  Icon,click,,"//i[@title='Block']"
-64.Click Disable  User  Yes,click,,"//button[normalize-space()='Yes']"
-65.Disable Reason,type,Client Complaints,"//textarea[@id='swal2-textarea']"
-66.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-67.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-68. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-69. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-70.Click  Blocked Customers,click,,"//span[normalize-space()='Blocked customers']"
-71.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-72.Scroll Grid, tab, 10, "//input[@aria-label='Customer Name Filter Input']"
-73.Click Enable  Icon,click,,"//i[@title='Status']"
-74.Click Enable  Yes,click,,"//button[normalize-space()='Yes']"
-75. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-76. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-77.Click  Verified Customers,click,,"//span[normalize-space()='Verified customers']"
-78. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-79.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-80.wait,1000,,</t>
-  </si>
-  <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-6. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-7. Enter Driver Name, type, autodriver_{timestamp} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-8. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
-9. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-10. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-11. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-12.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-13.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
-14. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-15.Enter Vehicle Company, type, autoCompany{randomAlpha}&gt;&gt; autoCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-16. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-17. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-18. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-19. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-20. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-21. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-22. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-23. Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-24. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-25. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-26. Click Submit, click, , "//button[contains(.,'Submit')]"
-27. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-28. Wait for Toast to hide, wait, 1000,
-29.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-31.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-32.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-33.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-34. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-35.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-36.Add Driving License,click,,"//i[@title='Edit']"
-37.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-38.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-39.Click Submit, click, , "//button[normalize-space()='Submit']"
-40.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-41.Click Approve Driver,click,,"//i[@title='Approve']"
-42.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-43.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-44.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-45.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-46.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-47.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-48.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-49.Click Doc Icon,click,,"//i[@title='Document']"
-50.Click Eye Icon,click,,"//i[@title='View']"
-51.wait,1000,,</t>
-  </si>
-  <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-3. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-4. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-5.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-6.Select Bike Ride Option,click,,"//span[normalize-space()='Bike Ride']"
-7. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-8. Enter Driver Name, type, bikedriver_{timestamp} &gt;&gt; bikeName, "//label[contains(.,'Full Name')]/following::input[1]"
-9. Enter Email, type, bikedriver_{timestamp}@gmail.com&gt;&gt;bikeEmail, "//label[contains(.,'Email')]/following::input[1]"
-10. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-11. Upload Profile Image, uploadfile, "src/main/resources/test-data/bikedriver.jpg", "//input[@type='file']"
-12. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-13.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-14.Select  Scooter Option,click,,"//li[@role='option']//span[text()='Scooter']"
-15. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-16.Enter Vehicle Company, type, bikeCompany{randomAlpha}&gt;&gt; bikeCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-17. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
-18. Enter Model Name, type, activa, "//label[contains(.,'Model Name')]/following::input[1]"
-19. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/bike.jpg", "(//input[@type='file'])[2]"
-20. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-21. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-22. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-23. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-24. Enter Account Holder Name, type, {bikeName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-25. Enter Payment Email Address, type, {bikeEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-26. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-27. Click Submit, click, , "//button[contains(.,'Submit')]"
-28. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-29. Wait for Toast to hide, wait, 1000,
-30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-31.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-32.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-33.Filter by Name,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
-34.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-35. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-36.FilterDocumet List,type,Vehicle Permit Copy,"//input[@aria-label='Document Name Filter Input']"
-37.Add Vehicle Permit Copy,click,,"//i[@title='Edit']"
-38.Upload Vehicle Permit Copy, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-39.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-40.Click Submit, click, , "//button[normalize-space()='Submit']"
-41.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-42.Click Approve Driver,click,,"//i[@title='Approve']"
-43.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-44.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-46.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-47.Approved Drivers List,verify,,"//div[contains(text(),' Approved Drivers List')]"
-48.Filter Approved Driver,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
-49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-50.Click Doc Icon,click,,"//i[@title='Document']"
-51.Click Eye Icon,click,,"//i[@title='View']"
-52.wait,1000,,</t>
-  </si>
-  <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-3. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-4. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-5.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-6.Select Taxi Ride Option,click,,"//span[normalize-space()='Taxi Ride']"
-7. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-8. Enter Driver Name, type, taxidriver_{timestamp} &gt;&gt; taxiName, "//label[contains(.,'Full Name')]/following::input[1]"
-9. Enter Email, type, taxidriver_{timestamp}@gmail.com&gt;&gt;taxiEmail, "//label[contains(.,'Email')]/following::input[1]"
-10. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-11. Upload Profile Image, uploadfile, "src/main/resources/test-data/taxidriver.jpg", "//input[@type='file']"
-12. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-13.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-14.Select  Suv Option,click,,"//li[@role='option']//span[text()='SUV']"
-15. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-16.Enter Vehicle Company, type, taxiCompany{randomAlpha}&gt;&gt; taxiCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-17. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
-18. Enter Model Name, type, etios, "//label[contains(.,'Model Name')]/following::input[1]"
-19.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/taxi.jpg", "(//input[@type='file'])[2]"
-20. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-21. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-22. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-23. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-24. Enter Account Holder Name, type, {taxiName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-25. Enter Payment Email Address, type, {taxiEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-26. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-27. Click Submit, click, , "//button[contains(.,'Submit')]"
-28. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-29. Wait for Toast to hide, wait, 1000,
-30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-31.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-32.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-33.Filter by Name,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
-34.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-35. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-36.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-37.Add Driving License,click,,"//i[@title='Edit']"
-38.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-39.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-40.Click Submit, click, , "//button[normalize-space()='Submit']"
-41.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-42.Click Approve Driver,click,,"//i[@title='Approve']"
-43.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-44.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-46.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-47.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-48.Filter Approved Driver,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
-49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-50.Click Doc Icon,click,,"//i[@title='Document']"
-51.Click Eye Icon,click,,"//i[@title='View']"
-52.wait,1000,,</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
@@ -2410,6 +2091,214 @@
 45.wait,2000,,</t>
   </si>
   <si>
+    <t>Add New  Store, Provider , Driver &amp;  Customer Subscription Plan</t>
+  </si>
+  <si>
+    <t>TC_CA_14_subscription_plan_test</t>
+  </si>
+  <si>
+    <t>SA_TS_15</t>
+  </si>
+  <si>
+    <t>TC_CA_15_test_data_cleanup</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.
+RunSheet: SuperAdminLogin
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+2.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+3.Click Store subscription plan,click,,"//span[normalize-space()='Store subscription plan']"
+4.Verify Store Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Store']"
+5.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
+6.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+7.Select Food Delivery,click,,"//li[@aria-label='Food Delivery']"
+8.Enter Store Plan Name, type, StorePlan{randomAlpha}&gt;&gt; storeSubscriptionName, "//input[@placeholder='Plan Name']"
+9.Enter Store Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
+10.Enter Store Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
+11.Enter Store Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
+12.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
+13.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
+14.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
+15.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description(in Arabic)']"
+16.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description(in Tamil)']"
+17.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description(in Hindi)']"
+18.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+19.Select On,click,,"//li[@aria-label='on']"
+20.Click Submit ,click,,"//button[normalize-space()='Submit']"
+21.Filter Services List,type,{storeSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+22.Click Edit ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+23.Click Close ,click,,"//button[normalize-space()='Close']"
+24.Click Active ,click,,"//i[@title='Active']"
+25.wait,2000,,
+26.Click Deactive,click,,"//i[@title='Inactive']"
+27.wait,2000,,
+28.Click Delete Plan,click,,"//i[@class='bi bi-trash cursor-pointer gridIcon Delete']"
+29.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
+30.wait,3000,,
+31.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+32.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+33.Click Driver subscription plan,click,,"//span[normalize-space()='Driver subscription plan']"
+34.Verify Driver Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Driver']"
+35.Click  Add New Subscription,click,,"//button[normalize-space()='ADD']"
+36.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+37.Select Auto Ride,click,,"//li[@aria-label='Auto Ride']"
+38.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "//input[@placeholder='Plan Name']"
+39.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
+40.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil)']"
+41.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi)']"
+42.Enter Number Of Days, type,100, "//input[@placeholder='No. of Days ']"
+43.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No of Rides with Zero admin commission']"
+44.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
+45.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
+46.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description Arabic']"
+47.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description Tamil']"
+48.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description Hindi']"
+49.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+50.Select On,click,,"//li[@aria-label='on']"
+51.Click Submit ,click,,"//button[normalize-space()='Submit']"
+52.Filter Services List,type,{driverSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+53.Click Edit ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+54.Click Close ,click,,"//button[normalize-space()='Close']"
+55.Click Active ,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+56.wait,2000,,
+57.Click Deactive,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
+58.wait,2000,,
+59.Click Delete Plan,click,,"//i[@class='bi bi-trash cursor-pointer gridIcon Delete']"
+60.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
+61.wait,3000,,
+62.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+63.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+64.Click Provider subscription plan,click,,"//span[normalize-space()='Provider subscription plan']"
+65.Verify Provider Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Provider']"
+66.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
+67.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+68.Select Pest Control,click,,"//li[@aria-label='Pest Control']"
+69.Enter Provider Plan Name, type, ProviderPlan{randomAlpha}&gt;&gt; providerSubscriptionName, "//input[@placeholder='Plan Name']"
+70.Enter Provider Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic):']"
+71.Enter Provider Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
+72.Enter Provider Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
+73.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
+74.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price ']"
+75.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Enter Description(in English):']"
+76.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Enter Description(in Arabic):']"
+77.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Enter Description(in Tamil)']"
+78.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Enter Description(in Hindi']"
+79.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+80.Select On,click,,"//li[@aria-label='on']"
+81.Click Submit ,click,,"//button[normalize-space()='Submit']"
+82.Filter Services List,type,{providerSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+83.Click Edit ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+84.Click Close ,click,,"//button[normalize-space()='Close']"
+85.Click Active ,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+86.wait,2000,,
+87.Click Deactive,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
+88.wait,2000,,
+89.Click Delete Plan,click,,"//i[@class='bi bi-trash cursor-pointer gridIcon Delete']"
+90.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
+91.wait,3000,,
+92.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+93.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+94.Click Customer subscription plan,click,,"//span[normalize-space()='Customer subscription plan']"
+95.Verify Customer Subscription Plan Lists ,verify,,"//div[normalize-space()='Customer Subscription Plans']"
+96.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
+97.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+98.Select Pest Control,click,,"//li[@aria-label='Pest Control']"
+99.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; custometSubscriptionName, "//input[@placeholder='Plan Name']"
+100.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
+101.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
+102.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
+103.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
+104.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No Of Free Rides']"
+105.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
+106.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
+107.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description(in Arabic)']"
+108.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description(in Tamil)']"
+109.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description(in Hindi)']"
+110.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+111.Select On,click,,"//li[@aria-label='on']"
+112.Click Submit ,click,,"//button[normalize-space()='Submit']"
+113.Filter Services List,type,{custometSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+114.Click Edit ,click,,"//i[@title='Edit Plan']"
+115.Click Close ,click,,"//button[normalize-space()='Close']"
+116.Click Active ,click,,"//i[@title='Activate Plan']"
+117.wait,2000,,
+118.Click Deactive,click,,"//i[@title='Deactivate Plan']"
+119.wait,2000,,
+120.Click Delete Plan,click,,"//i[@title='Delete Plan']"
+121.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
+122.wait,3000,,
+</t>
+  </si>
+  <si>
+    <t>This test case validates the end-to-end management of subscription plan architectures across four distinct user entities: Store, Driver, Provider, and Customer. The workflow systematically executes the creation of localized "Premium" plans for various service categories—such as Food Delivery and Pest Control—featuring integrated multi-language support in Arabic, Tamil, and Hindi. The validation cycle spans from defining plan durations, pricing, and free-ride quotas to conducting administrative audits including localized description verification, active/inactive state toggling, and data filtering. The process concludes by confirming the operational lifecycle through record modification and final deletion, ensuring the functional stability and localized integrity of the platform’s commercial monetization modules.</t>
+  </si>
+  <si>
     <t xml:space="preserve">1.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
 2. Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
 3.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
@@ -2434,138 +2323,471 @@
 22.Click Settings ,click,,"//button[contains(., 'Settings')]"
 23.Click Vehicle Type,click,,"//div[normalize-space()='Vehicle Type']"
 24.Click Add Vehicle Type,click,,"//button[normalize-space()='Add Vehicle Type']"
-25.Enter Vehicle Type Name, type, volvo{randomAlpha}&gt;&gt;busTypeName, "//input[@placeholder='Type here']"
-26.Enter Cost For Km, type, 150, "//input[@placeholder='Cost For Km']"
-27.Enter Time Fare Per Min, type,10, "//input[@placeholder='Time Fare Per Min']"
-28.Enter Base fare, type,100, "//input[@placeholder='Base fare']"
-29.Enter Min Fare Amount, type,50, "//input[@placeholder='Min Fare Amount']"
-30.Enter Rental Cost For Km, type,30, "//input[@placeholder='Rental Cost For Km']"
-31.Enter Rental Amount For 1 Hour, type,50, "//input[@placeholder='Rental Amount For 1 Hour']"
-32.Enter Rental Km Limit For 1 Hour, type,50, "//input[@placeholder='Rental Km Limit For 1 Hour']"
-33.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "//app-image-upload//input[@type='file' and @accept='image/*']"
-34.Click Surcharge Time Checkbox, click, , "//div[text()='EveryDay']/preceding-sibling::mat-checkbox"
-35.Enter From Time, type, 100000, "//app-time-picker//input[@type='time']"
-36.Enter To Time, type, 220000, "(//app-time-picker//input[@type='time'])[2]"
-37.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-38.Select Active,click,,"//li[@aria-label='Active']"
-39.Click  Submit,click,,"//button[normalize-space()='Submit']"
-40.Verify Sucess, verify, , "//div[@aria-label='Info']"
-41.Click Settings ,click,,"//button[contains(., 'Settings')]"
-42.Click Promocode,click,,"//div[normalize-space()='Promocode']"
-43.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
-44.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
-45.Select User,click,,"//li[@aria-label='{customerName}']"
-46.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
-47.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; promoCodeName, "//input[@placeholder='Code Name']"
-48.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
-49.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
-50.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
-51.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
-52.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
-53.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
-54.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
-55.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
-56.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
-57.Click Submit ,click,,"//button[normalize-space()='Submit']"
-58.Verify Sucess, verify, , "//div[@aria-label='Info']"
-59.wait,2000,,
-60.Click Settings ,click,,"//button[contains(., 'Settings')]"
-61.Click Service Settings ,click,,"//div[normalize-space()='Service Setting']"
-62.Enter Driver Accept Timeout, type, 60, "//label[contains(., "Driver Accept Timeout")]/following::input[1]"
-63.Enter Driver Serach Radius, type, 50, "//label[contains(., "Driver Search Radius")]/following::input[1]"
-64.Open Tax Type Dropdown,click,,"//span[@aria-label='Select Tax Rype']"
-65.Select Amount,click,,"//li[@aria-label='Amount']"
-66.Enter Tax, type, 20, "//label[contains(., 'Tax')]/following::input[1]"
-67.Open Platform Fee Type Dropdown,click,,"//label[contains(., 'Platform Fee Type')]/following::span[@role='combobox']"
+25.Enter Vehicle Type Name, type, volvo{randomAlpha}&gt;&gt;busTypeName, "//input[@placeholder='Enter Vehicle Type']"
+26.Enter Base Fare, type, 150, "//input[@placeholder='Enter base fare']"
+27.Enter Free Waiting Time , type, 10, "//label[contains(., 'Free Waiting Time')]/following::input[1]"
+28.Open Wating Charge Dropdown,click,"//label[contains(., 'Waiting Charge Type')]/following-sibling::p-dropdown//span[@role='combobox']"
+29.Select Amount,click,,"//li[@aria-label='Amount']"
+30.Enter Waiting Rate , type, 10, "//input[@placeholder='Waiting Rate (per min)']"
+31.Enter Included Trip Waiting , type, 10, "//input[@placeholder='Included Trip Waiting']"
+32.Open Pickup Charge Dropdown,click,"//label[contains(., 'Pickup Charge Type')]/following-sibling::p-dropdown//span[@role='combobox']"
+33.Select Amount,click,,"//li[@aria-label='Amount']"
+34.Enter Pickup Fee , type, 10, "//input[@placeholder='Pickup Fee (Per Km)']"
+35.Open Customer Fee Dropdown,click,"//label[contains(., 'Customer Fee Type')]/following-sibling::p-dropdown//span[@role='combobox']"
+36.Select Amount,click,,"//li[@aria-label='Amount']"
+37.Enter Customer Fee , type,50, "//input[@placeholder='Customer Fee']"
+38.Open Driver Fee Dropdown,click,"//label[contains(., 'Driver Fee Type')]/following-sibling::p-dropdown//span[@role='combobox']"
+39.Select Amount,click,,"//li[@aria-label='Amout']"
+40.Enter Driver Fee , type,50, "//input[@placeholder='Driver Fee']"
+41.Open Status Dropdown,click,"//label[contains(., 'Status')]/following-sibling::p-dropdown//span[@role='combobox']"
+42.Select Active,click,,"//li[@aria-label='Active']"
+43.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "//app-image-upload//input[@type='file' and @accept='image/*']"
+44.Click Surcharge Time Checkbox, click, , "//div[text()='EveryDay']/preceding-sibling::mat-checkbox"
+45.Enter From Time, type, 100000, "//app-time-picker//input[@type='time']"
+46.Enter To Time, type, 220000, "(//app-time-picker//input[@type='time'])[2]"
+47.Click  Submit,click,,"//button[normalize-space()='Submit']"
+48.Verify Sucess, verify, , "//div[@aria-label='Info']"
+49.Click Settings ,click,,"//button[contains(., 'Settings')]"
+50.Click Promocode,click,,"//div[normalize-space()='Promocode']"
+46.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
+47.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
+48.Select User,click,,"//li[@aria-label='{customerName}']"
+49.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
+50.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; promoCodeName, "//input[@placeholder='Code Name']"
+51.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
+52.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
+53.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
+54.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
+55.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
+56.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
+57.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
+58.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
+59.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
+60.Click Submit ,click,,"//button[normalize-space()='Submit']"
+61.Verify Sucess, verify, , "//div[@aria-label='Info']"
+62.wait,2000,,
+63.Click Settings ,click,,"//button[contains(., 'Settings')]"
+64.Click Service Settings ,click,,"//div[normalize-space()='Service Setting']"
+65.Enter Driver Accept Timeout, type, 60, "//label[contains(., "Driver Accept Timeout")]/following::input[1]"
+66.Enter Driver Serach Radius, type, 50, "//label[contains(., "Driver Search Radius")]/following::input[1]"
+67.Open Tax Type Dropdown,click,,"//span[@aria-label='Select Tax Rype']"
 68.Select Amount,click,,"//li[@aria-label='Amount']"
-69.Enter Platform Fee, type, 20, "//label[contains(., "Platform Fee")]/following::input[1]"
-70.Click Submit ,click,,"//button[normalize-space()='Submit']"
-71.Verify Sucess, verify, , "//div[@aria-label='Info']"
-72.wait,1000,,
-73.Click Settings ,click,,"//button[contains(., 'Settings')]"
-74.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
-75.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
-76.Enter Name, type, documet{randomAlpha}&gt;&gt; documentName, "//label[contains(., 'Name')]/following::input[1]"
-77.Open status Dropdown,click,,"//label[contains(., 'Status')]/following::div[contains(@class, 'p-dropdown')]"
-78.Select Active,click,,"//li[@aria-label='Active']"
-79.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
-80.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
-81.Click  Require Proof Number,click,,"//div[./div[contains(text(), 'Require Proof Number')]]//input"
-82.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
-83.Click Submit ,click,,"//button[normalize-space()='Submit']"
-84.Verify Sucess, verify, , "//div[@aria-label='Info']"
-85.Filter Document List,type,{documentName},"//input[@aria-label='Name Filter Input']"
-86.wait,1000,,
-88.Click Settings ,click,,"//button[contains(., 'Settings')]"
-89.Click Customer Loyalty Settings,click,,"//div[text()=' Customer Loyalty Settings ']"
-90.Open status Allow Customer loyalty points,click,,"//label[contains(., 'Allow Customer loyalty points')]/following::div[contains(@class, 'p-dropdown')]"
-91.Select ON,click,,"//li[@role='option']//span[text()='ON']"
-92.Enter Minimum order amount for eligibility to redeem loyalty points, type, 25,"//label[contains(., 'Minimum order amount for eligibility to redeem loyalty points')]/following::input[1]"
-93.Enter Loyalty points redeem per order (in %) (% of order amount), type, 10,"//label[contains(., 'Loyalty points redeem per order (in %) (% of order amount)')]/following::input[1]"
-94.Enter Loyalty points per default currency (for ex. $1 = 10 points), type, 5,"//label[contains(., 'Loyalty points per default currency (for ex. $1 = 10 points)')]/following::input[1]"
-95.Click Submit ,click,,"//button[normalize-space()='Submit']"
-96.Verify Sucess, verify, , "//div[@aria-label='Info']"
-97.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-98.Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-99.Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-100.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-101.Select Bus Ride Option,click,,"//span[normalize-space()='{transportName}']"
-102.Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-103.Enter Driver Name, type, busdriver_{timestamp} &gt;&gt; busDriverName, "//label[contains(.,'Full Name')]/following::input[1]"
-104.Enter Email, type, busdriver_{timestamp}@gmail.com&gt;&gt;busEmail, "//label[contains(.,'Email')]/following::input[1]"
-105.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-106.Upload Profile Image, uploadfile, "src/main/resources/test-data/busdriver.jpg", "//input[@type='file']"
-107.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-108.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-109.Select  volvo Option,click,,"//li[@role='option']//span[text()='{busTypeName}']"
-110.Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-111.Enter Vehicle Company, type, busCompany{randomAlpha}&gt;&gt; busCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-112.Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
-113. Enter Model Name, type, deisel, "//label[contains(.,'Model Name')]/following::input[1]"
-114.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/busvolvo.jpeg", "(//input[@type='file'])[2]"
-115. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-116.Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-117.Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-118.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-119.Enter Account Holder Name, type, {busDriverName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-120.Enter Payment Email Address, type, {busEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-121.Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-122.Click Submit, click, , "//button[contains(.,'Submit')]"
-123.Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-124.Wait for Toast to hide, wait, 1000,
-125.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-126.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-127.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-128.Filter by Name,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
-129.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-130.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-131.FilterDocumet List,type,{documentName},"//input[@aria-label='Document Name Filter Input']"
-132.Add Driving License,click,,"//i[@title='Edit']"
-133.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-134.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-135.Click Submit, click, , "//button[normalize-space()='Submit']"
-136.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-137.Click Approve Driver,click,,"//i[@title='Approve']"
+69.Enter Tax, type, 20, "//label[contains(., 'Tax')]/following::input[1]"
+70.Open Platform Fee Type Dropdown,click,,"//label[contains(., 'Platform Fee Type')]/following::span[@role='combobox']"
+71.Select Amount,click,,"//li[@aria-label='Amount']"
+72.Enter Platform Fee, type, 20, "//label[contains(., "Platform Fee")]/following::input[1]"
+73.Click Submit ,click,,"//button[normalize-space()='Submit']"
+74.Verify Sucess, verify, , "//div[@aria-label='Info']"
+75.wait,1000,,
+76.Click Settings ,click,,"//button[contains(., 'Settings')]"
+77.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
+78.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
+79.Enter Name, type, documet{randomAlpha}&gt;&gt; documentName, "//label[contains(., 'Name')]/following::input[1]"
+80.Open status Dropdown,click,,"//label[contains(., 'Status')]/following::div[contains(@class, 'p-dropdown')]"
+81.Select Active,click,,"//li[@aria-label='Active']"
+82.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
+83.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
+84.Click  Require Proof Number,click,,"//div[./div[contains(text(), 'Require Proof Number')]]//input"
+85.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
+86.Click Submit ,click,,"//button[normalize-space()='Submit']"
+87.Verify Sucess, verify, , "//div[@aria-label='Info']"
+88.Filter Document List,type,{documentName},"//input[@aria-label='Name Filter Input']"
+89.wait,1000,,
+90.Click Settings ,click,,"//button[contains(., 'Settings')]"
+91.Click Customer Loyalty Settings,click,,"//div[text()=' Customer Loyalty Settings ']"
+92.Open status Allow Customer loyalty points,click,,"//label[contains(., 'Allow Customer loyalty points')]/following::div[contains(@class, 'p-dropdown')]"
+93.Select ON,click,,"//li[@role='option']//span[text()='ON']"
+94.Enter Minimum order amount for eligibility to redeem loyalty points, type, 25,"//label[contains(., 'Minimum order amount for eligibility to redeem loyalty points')]/following::input[1]"
+95.Enter Loyalty points redeem per order (in %) (% of order amount), type, 10,"//label[contains(., 'Loyalty points redeem per order (in %) (% of order amount)')]/following::input[1]"
+96.Enter Loyalty points per default currency (for ex. $1 = 10 points), type, 5,"//label[contains(., 'Loyalty points per default currency (for ex. $1 = 10 points)')]/following::input[1]"
+97.Click Submit ,click,,"//button[normalize-space()='Submit']"
+98.Verify Sucess, verify, , "//div[@aria-label='Info']"
+99.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+100.Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+101.Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+102.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+103.Select Bus Ride Option,click,,"//span[normalize-space()='{transportName}']"
+104.Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+105.Enter Driver Name, type, busdriver_{timestamp} &gt;&gt; busDriverName, "//label[contains(.,'Full Name')]/following::input[1]"
+106.Enter Email, type, busdriver_{timestamp}@gmail.com&gt;&gt;busEmail, "//label[contains(.,'Email')]/following::input[1]"
+107.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+108.Upload Profile Image, uploadfile, "src/main/resources/test-data/busdriver.jpg", "//input[@type='file']"
+109.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+110.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+111.Select  volvo Option,click,,"//li[@role='option']//span[text()='{busTypeName}']"
+112.Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+113.Enter Vehicle Company, type, busCompany{randomAlpha}&gt;&gt; busCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+114.Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+115. Enter Model Name, type, deisel, "//label[contains(.,'Model Name')]/following::input[1]"
+116.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/busvolvo.jpeg", "(//input[@type='file'])[2]"
+117. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+118.Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+119.Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+120.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+121.Enter Account Holder Name, type, {busDriverName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+122.Enter Payment Email Address, type, {busEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+123.Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+124.Click Submit, click, , "//button[contains(.,'Submit')]"
+125.Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+126.Wait for Toast to hide, wait, 1000,
+127.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+128.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+129.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
+130.Filter by Name,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
+131.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+132.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+133.FilterDocumet List,type,{documentName},"//input[@aria-label='Document Name Filter Input']"
+134.Add Driving License,click,,"//i[@title='Edit']"
+135.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+136.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+137.Click Submit, click, , "//button[normalize-space()='Submit']"
 138.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-139.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-140.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-141.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-142.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-143.Filter Approved Driver,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
-144.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
-145.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
-146.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
-147.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
-148.Click Edit Icon ,click,,"//i[@title='Edit']"
-149.wait,2000,,
-150.Scroll Grid, tab, 5, "//input[@placeholder='Service Name']"
+139.Click Approve Driver,click,,"//i[@title='Approve']"
+140.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+141.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+142.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+143.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+144.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+145.Filter Approved Driver,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
+146.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+147.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+148.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
+149.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
+150.Click Edit Icon ,click,,"//i[@title='Edit']"
 151.wait,2000,,
-152.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-153.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
-154.Click  Submit,click,,"//button[normalize-space()='Submit']"
-155.Verify Sucess, verify, , "//div[@aria-label='Info']"
-156.wait,2000,,
+152.Scroll Grid, tab, 5, "//input[@placeholder='Service Name']"
+153.wait,2000,,
+154.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+155.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
+156.Click  Submit,click,,"//button[normalize-space()='Submit']"
+157.Verify Sucess, verify, , "//div[@aria-label='Info']"
+158.wait,2000,,
 </t>
+  </si>
+  <si>
+    <t>1. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+2.Click  Add Customers,click,,"//span[normalize-space()='Add Customers']"
+3. Verify Add Customer Heading,verify,,"//div[normalize-space()='Add Customer']"
+4.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "//label[contains(., 'Customer Full Name')]/following::input[1]"
+5.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "//input[@type='email']"
+6.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+7.Enter Video Call Limit, type, 60, "//label[contains(., 'User Used Video Call Limit in Minutes')]/following::input[1]"
+8.Open Gender,click,,"//span[@aria-label='select gender']"
+9.Select Male,click,,"//li[@aria-label='Male']"
+10.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "//input[@type='file' and @accept='image/*']"
+11.Click Submit, click, , "//button[normalize-space()='Submit']"
+12.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+13. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+14. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+15.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
+16. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+17.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+18.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
+19.Click Edit Icon ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+20.Click Close, click, , "//button[normalize-space()='Close']"
+21.Click Wallet Icon ,click,,"//i[@title='Wallet']"
+22.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
+23.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
+24.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+25.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
+26.Click Submit, click, , "//button[normalize-space()='Submit']"
+27.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+28.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
+29.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
+30.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+31.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
+32.Click Submit, click, , "//button[normalize-space()='Submit']"
+33.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+34. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+35. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+36.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
+37. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+38.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+39.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
+40.Click Loyalty Points Icon,click,,"//i[@title='Loyalty Points']"
+41.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
+42.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
+43.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
+44.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+45.Select Add Points,click,,"//li[@role='option'][contains(.,'Add Points')]"
+46.Enter Points, type, 30, "//input[@placeholder='Enter Points']"
+47.Click Submit, click, , "//button[normalize-space()='Submit']"
+48.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+49.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
+50.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
+51.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
+52.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+53.Select Deduct Points,click,,"//li[@role='option'][contains(.,'Deduct Points')]"
+54.Enter Points, type, 10, "//input[@placeholder='Enter Points']"
+55.Click Submit, click, , "//button[normalize-space()='Submit']"
+56.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+57. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+58. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+59.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
+60. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+61.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+62.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
+63.Click Disable  Icon,click,,"//i[@title='Block']"
+64.Click Disable  User  Yes,click,,"//button[normalize-space()='Yes']"
+65.Disable Reason,type,Client Complaints,"//textarea[@id='swal2-textarea']"
+66.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+67.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+68. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+69. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+70.Click  Blocked Customers,click,,"//span[normalize-space()='Blocked Customers']"
+71.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+72.Scroll Grid, tab, 10, "//input[@aria-label='Customer Name Filter Input']"
+73.Click Enable  Icon,click,,"//i[@title='Status']"
+74.Click Enable  Yes,click,,"//button[normalize-space()='Yes']"
+75. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+76. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+77.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
+78. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+79.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+80.wait,1000,,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+2. Click City area menu,click,,"//span[normalize-space()='City Area']"
+3. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
+4. Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
+5. Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
+6. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
+7. Open Status Dropdown,click,,"//span[@aria-label='select status']"
+8. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+9.Enter City Area, type, triplicane, "//input[@placeholder='Search location']"
+10.wait,1000,,
+11.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
+12.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
+13.wait,1000,,
+14. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
+15. Click Submit,click,,"//button[normalize-space()='Submit']"
+16. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
+17. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
+18. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
+19. Click Add Category,click,,"//button[normalize-space()='Add Category']"
+20. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
+21. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
+22. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
+23. Click close,click,,"//button[normalize-space()='Close']"
+19. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+24. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+25. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
+26. Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
+27. Open Select City Dropdown,click,,"//select[@id='cityId']"
+28. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
+29. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+4. Verify City Admin List,verify,,"//div[normalize-space()='City Admin List']"
+5. Click Add City Admin button,click,,"//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
+6. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
+7.Select Name field,click ,, "//input[@id='name']"
+8. Enter Admin Name, type, faizal{randomAlpha} &gt;&gt; adminName, "//input[@id='name']"
+9.Select Email field,click,, "//input[@id='email']"
+10. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
+11.select the password field,click,, "//input[@id='password']"
+12.Enter the Password as "faizal@123". "//input[@id='password']"
+13.Open Select City Dropdown,click,,"//select[@id='cityId']"
+14.Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
+15. Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
+16.Click on the "Customers" → "Add Customers" checkbox. "//label[normalize-space()='Add Customers']"
+17.Click on the "Customers" → "Verified Customers"checkbox. "//label[normalize-space()='Verified Customers']"
+18.Click on the "Customers" → "Non Verified Customers" checkbox. "//label[normalize-space()='Non Verified Customers']"
+19.Click on the "Customers" → "Blocked Customers" checkbox. "//label[normalize-space()='Blocked Customers']"
+20.Click on the "Customers" → "Deleted Customers" checkbox. "//label[normalize-space()='Deleted Customers']"
+21.Click on the "Customers" → "Pending Customers" checkbox. "//label[normalize-space()='Pending Customers']"
+22.Click on the "Providers" → "Transport Providers List" checkbox. "//label[normalize-space()='Transport Providers List']"
+23.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
+24.Click on the "Drivers" → "Approved Drivers" checkbox. "//label[normalize-space()='Approved Drivers']"
+25.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
+26.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
+27.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
+28.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
+29.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox. "//label[normalize-space()='Driver Subscription Plan']"
+30.Click on the "Cash Out" → "Driver Cash Out" checkbox. "//label[normalize-space()='Driver Cash Out']"
+31.Click on the "Report Issue" → "Customer Report Issues" checkbox. "//label[normalize-space()='Customer Report Issues']"
+32.Click on the "Report Issue" → "Driver Report Issues" checkbox. "//label[normalize-space()='Driver Report Issues']"
+33.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
+34.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
+35.Click on the "Report Issue" → "FAQs" checkbox. "(//h3[contains(.,'Report Issue')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
+36.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
+37.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
+38.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[h3[contains(.,'Website Settings')]]//label[contains(.,'Delivery')]"
+39.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[.//h3[contains(text(),'Website Settings')]]//label[contains(.,'Transport')]"
+40.Click on the "Website Settings" → "FAQs" checkbox. "(//h3[contains(.,'Website Settings')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
+41.Click on the "Add City Admin" button. "//button[@type='submit']"
+42. Verify Success Message,verify,,"//div[@aria-label='Info']"
+43.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
+</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+6. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
+7. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+8. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+9. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+10. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+11. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+12.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+13.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
+14. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+15.Enter Vehicle Company, type, autoCompany{randomAlpha}&gt;&gt; autoCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+16. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+17. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+18. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+19. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+20. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+21. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+22. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+23. Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+24. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+25. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+26. Click Submit, click, , "//button[contains(.,'Submit')]"
+27. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+28. Wait for Toast to hide, wait, 1000,
+29.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+32.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+33.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+34.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+35. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+36.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+37.Add Driving License,click,,"//i[@title='Edit']"
+38.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+39.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+40.Click Submit, click, , "//button[normalize-space()='Submit']"
+41.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+42.Click Approve Driver,click,,"//i[@title='Approve']"
+43.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+43.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+46.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+47.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+48.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+50.Click Doc Icon,click,,"//i[@title='Document']"
+51.Click Eye Icon,click,,"//i[@title='View']"
+52.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+3. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+4. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+5.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+6.Select Bike Ride Option,click,,"//span[normalize-space()='Bike Ride']"
+7. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+8. Enter Driver Name, type, bikedriver{randomAlpha}&gt;&gt; bikeName, "//label[contains(.,'Full Name')]/following::input[1]"
+9. Enter Email, type, bikedriver_{timestamp}@gmail.com&gt;&gt;bikeEmail, "//label[contains(.,'Email')]/following::input[1]"
+10. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+11. Upload Profile Image, uploadfile, "src/main/resources/test-data/bikedriver.jpg", "//input[@type='file']"
+12. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+13.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+14.Select  Scooter Option,click,,"//li[@role='option']//span[text()='Scooter']"
+15. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+16.Enter Vehicle Company, type, bikeCompany{randomAlpha}&gt;&gt; bikeCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+17. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+18. Enter Model Name, type, activa, "//label[contains(.,'Model Name')]/following::input[1]"
+19. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/bike.jpg", "(//input[@type='file'])[2]"
+20. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+21. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+22. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+23. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+24. Enter Account Holder Name, type, {bikeName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+25. Enter Payment Email Address, type, {bikeEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+26. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+27. Click Submit, click, , "//button[contains(.,'Submit')]"
+28. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+29. Wait for Toast to hide, wait, 1000,
+30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+32.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+33.Filter by Name,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
+34.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+35.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+36.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+37.FilterDocumet List,type,Vehicle Permit Copy,"//input[@aria-label='Document Name Filter Input']"
+38.Add Vehicle Permit Copy,click,,"//i[@title='Edit']"
+39.Upload Vehicle Permit Copy, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+40.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+41.Click Submit, click, , "//button[normalize-space()='Submit']"
+42.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+43.Click Approve Driver,click,,"//i[@title='Approve']"
+44.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+46.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+47.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+48.Approved Drivers List,verify,,"//div[contains(text(),' Approved Drivers List')]"
+49.Filter Approved Driver,type,{bikeName},"//input[@aria-label='Driver Name Filter Input']"
+50.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+51.Click Doc Icon,click,,"//i[@title='Document']"
+52.Click Eye Icon,click,,"//i[@title='View']"
+53.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+3. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+4. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+5.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+6.Select Taxi Ride Option,click,,"//span[normalize-space()='Taxi Ride']"
+7. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+8. Enter Driver Name, type, taxidriver{randomAlpha} &gt;&gt; taxiName, "//label[contains(.,'Full Name')]/following::input[1]"
+9. Enter Email, type, taxidriver_{timestamp}@gmail.com&gt;&gt;taxiEmail, "//label[contains(.,'Email')]/following::input[1]"
+10. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+11. Upload Profile Image, uploadfile, "src/main/resources/test-data/taxidriver.jpg", "//input[@type='file']"
+12. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+13.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+14.Select  Suv Option,click,,"//li[@role='option']//span[text()='SUV']"
+15. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+16.Enter Vehicle Company, type, taxiCompany{randomAlpha}&gt;&gt; taxiCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+17. Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+18. Enter Model Name, type, etios, "//label[contains(.,'Model Name')]/following::input[1]"
+19.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/taxi.jpg", "(//input[@type='file'])[2]"
+20. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+21. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+22. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+23. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+24. Enter Account Holder Name, type, {taxiName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+25. Enter Payment Email Address, type, {taxiEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+26. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+27. Click Submit, click, , "//button[contains(.,'Submit')]"
+28. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+29. Wait for Toast to hide, wait, 1000,
+30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+32.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+33.Filter by Name,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
+34.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+35.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+36. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+37.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+38.Add Driving License,click,,"//i[@title='Edit']"
+39.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+40.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+41.Click Submit, click, , "//button[normalize-space()='Submit']"
+42.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+43.Click Approve Driver,click,,"//i[@title='Approve']"
+44.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+46.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+47.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+48.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+49.Filter Approved Driver,type,{taxiName},"//input[@aria-label='Driver Name Filter Input']"
+50.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+51.Click Doc Icon,click,,"//i[@title='Document']"
+52.Click Eye Icon,click,,"//i[@title='View']"
+53.wait,1000,,</t>
   </si>
 </sst>
 </file>
@@ -3060,13 +3282,13 @@
         <v>31</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>41</v>
@@ -3132,16 +3354,16 @@
         <v>34</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>35</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3198,22 +3420,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3270,22 +3492,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>38</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3342,22 +3564,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3373,6 +3595,78 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0F6277B-DBCF-4BFF-819C-1E90748D3258}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3414,22 +3708,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="E2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3440,7 +3734,7 @@
       <c r="E3" s="8"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="atjs4lQ1+o6fSFUQ0qpte05fkgrHsWBNK0UOqkGvhk5aH4hAig+bv994FWadvg20PU7CWkefN+SDSjlYBHqE/Q==" saltValue="4xFzDJqljq8EGyX3Igns8Q==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -3492,19 +3786,19 @@
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3571,16 +3865,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3646,13 +3940,13 @@
         <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>44</v>
+        <v>97</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>40</v>
@@ -3711,16 +4005,16 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3783,16 +4077,16 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3855,16 +4149,16 @@
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3924,19 +4218,19 @@
         <v>30</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>94</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4000,16 +4294,16 @@
         <v>28</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>29</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
66th commit: Test Cases Updated Transport Test modification
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46C20AA4-614F-4D1E-AA49-DA772A16BE03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{261120D6-711C-4106-94A9-C451F48FF5F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="102">
   <si>
     <t>City Area</t>
   </si>
@@ -2299,172 +2299,6 @@
     <t>This test case validates the end-to-end management of subscription plan architectures across four distinct user entities: Store, Driver, Provider, and Customer. The workflow systematically executes the creation of localized "Premium" plans for various service categories—such as Food Delivery and Pest Control—featuring integrated multi-language support in Arabic, Tamil, and Hindi. The validation cycle spans from defining plan durations, pricing, and free-ride quotas to conducting administrative audits including localized description verification, active/inactive state toggling, and data filtering. The process concludes by confirming the operational lifecycle through record modification and final deletion, ensuring the functional stability and localized integrity of the platform’s commercial monetization modules.</t>
   </si>
   <si>
-    <t xml:space="preserve">1.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
-2. Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
-3.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
-4.Click  Add Category,click,,"//button[normalize-space()='Add Category']"
-5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "//input[@placeholder='Service Name']"
-6.Enter Service Name Arabic, type, رحلة بالحافلة, "//input[@placeholder='Service Name (in Arabic)']"
-7.Enter Slug, type, Bus Ride, "//input[@placeholder='Slug']"
-8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "//input[@type='file' and @accept='image/*']"
-9.wait,2000,,
-10.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-11.Select Activate,click,,"//li[@aria-label='Activate']"
-12.Open Select City Dropdown,click,,"//span[text()='Select City']/ancestor::app-drop-down//div[contains(@class, 'p-multiselect-label-container')]"
-13.Select {areaName},click,,"//li[@aria-label='{areaName}']"
-14.Click  Submit,click,,"//button[normalize-space()='Submit']"
-15.Verify Sucess, verify, , "//div[@aria-label='Info']"
-16.wait,2000,,
-17.Click  back,click,,"//button[normalize-space()='Back']"
-18.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
-19.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
-20.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
-21.Click Home Icon ,click,,"//i[@title='Home']"
-22.Click Settings ,click,,"//button[contains(., 'Settings')]"
-23.Click Vehicle Type,click,,"//div[normalize-space()='Vehicle Type']"
-24.Click Add Vehicle Type,click,,"//button[normalize-space()='Add Vehicle Type']"
-25.Enter Vehicle Type Name, type, volvo{randomAlpha}&gt;&gt;busTypeName, "//input[@placeholder='Enter Vehicle Type']"
-26.Enter Base Fare, type, 150, "//input[@placeholder='Enter base fare']"
-27.Enter Free Waiting Time , type, 10, "//label[contains(., 'Free Waiting Time')]/following::input[1]"
-28.Open Wating Charge Dropdown,click,"//label[contains(., 'Waiting Charge Type')]/following-sibling::p-dropdown//span[@role='combobox']"
-29.Select Amount,click,,"//li[@aria-label='Amount']"
-30.Enter Waiting Rate , type, 10, "//input[@placeholder='Waiting Rate (per min)']"
-31.Enter Included Trip Waiting , type, 10, "//input[@placeholder='Included Trip Waiting']"
-32.Open Pickup Charge Dropdown,click,"//label[contains(., 'Pickup Charge Type')]/following-sibling::p-dropdown//span[@role='combobox']"
-33.Select Amount,click,,"//li[@aria-label='Amount']"
-34.Enter Pickup Fee , type, 10, "//input[@placeholder='Pickup Fee (Per Km)']"
-35.Open Customer Fee Dropdown,click,"//label[contains(., 'Customer Fee Type')]/following-sibling::p-dropdown//span[@role='combobox']"
-36.Select Amount,click,,"//li[@aria-label='Amount']"
-37.Enter Customer Fee , type,50, "//input[@placeholder='Customer Fee']"
-38.Open Driver Fee Dropdown,click,"//label[contains(., 'Driver Fee Type')]/following-sibling::p-dropdown//span[@role='combobox']"
-39.Select Amount,click,,"//li[@aria-label='Amout']"
-40.Enter Driver Fee , type,50, "//input[@placeholder='Driver Fee']"
-41.Open Status Dropdown,click,"//label[contains(., 'Status')]/following-sibling::p-dropdown//span[@role='combobox']"
-42.Select Active,click,,"//li[@aria-label='Active']"
-43.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "//app-image-upload//input[@type='file' and @accept='image/*']"
-44.Click Surcharge Time Checkbox, click, , "//div[text()='EveryDay']/preceding-sibling::mat-checkbox"
-45.Enter From Time, type, 100000, "//app-time-picker//input[@type='time']"
-46.Enter To Time, type, 220000, "(//app-time-picker//input[@type='time'])[2]"
-47.Click  Submit,click,,"//button[normalize-space()='Submit']"
-48.Verify Sucess, verify, , "//div[@aria-label='Info']"
-49.Click Settings ,click,,"//button[contains(., 'Settings')]"
-50.Click Promocode,click,,"//div[normalize-space()='Promocode']"
-46.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
-47.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
-48.Select User,click,,"//li[@aria-label='{customerName}']"
-49.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
-50.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; promoCodeName, "//input[@placeholder='Code Name']"
-51.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
-52.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
-53.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
-54.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
-55.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
-56.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
-57.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
-58.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
-59.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
-60.Click Submit ,click,,"//button[normalize-space()='Submit']"
-61.Verify Sucess, verify, , "//div[@aria-label='Info']"
-62.wait,2000,,
-63.Click Settings ,click,,"//button[contains(., 'Settings')]"
-64.Click Service Settings ,click,,"//div[normalize-space()='Service Setting']"
-65.Enter Driver Accept Timeout, type, 60, "//label[contains(., "Driver Accept Timeout")]/following::input[1]"
-66.Enter Driver Serach Radius, type, 50, "//label[contains(., "Driver Search Radius")]/following::input[1]"
-67.Open Tax Type Dropdown,click,,"//span[@aria-label='Select Tax Rype']"
-68.Select Amount,click,,"//li[@aria-label='Amount']"
-69.Enter Tax, type, 20, "//label[contains(., 'Tax')]/following::input[1]"
-70.Open Platform Fee Type Dropdown,click,,"//label[contains(., 'Platform Fee Type')]/following::span[@role='combobox']"
-71.Select Amount,click,,"//li[@aria-label='Amount']"
-72.Enter Platform Fee, type, 20, "//label[contains(., "Platform Fee")]/following::input[1]"
-73.Click Submit ,click,,"//button[normalize-space()='Submit']"
-74.Verify Sucess, verify, , "//div[@aria-label='Info']"
-75.wait,1000,,
-76.Click Settings ,click,,"//button[contains(., 'Settings')]"
-77.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
-78.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
-79.Enter Name, type, documet{randomAlpha}&gt;&gt; documentName, "//label[contains(., 'Name')]/following::input[1]"
-80.Open status Dropdown,click,,"//label[contains(., 'Status')]/following::div[contains(@class, 'p-dropdown')]"
-81.Select Active,click,,"//li[@aria-label='Active']"
-82.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
-83.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
-84.Click  Require Proof Number,click,,"//div[./div[contains(text(), 'Require Proof Number')]]//input"
-85.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
-86.Click Submit ,click,,"//button[normalize-space()='Submit']"
-87.Verify Sucess, verify, , "//div[@aria-label='Info']"
-88.Filter Document List,type,{documentName},"//input[@aria-label='Name Filter Input']"
-89.wait,1000,,
-90.Click Settings ,click,,"//button[contains(., 'Settings')]"
-91.Click Customer Loyalty Settings,click,,"//div[text()=' Customer Loyalty Settings ']"
-92.Open status Allow Customer loyalty points,click,,"//label[contains(., 'Allow Customer loyalty points')]/following::div[contains(@class, 'p-dropdown')]"
-93.Select ON,click,,"//li[@role='option']//span[text()='ON']"
-94.Enter Minimum order amount for eligibility to redeem loyalty points, type, 25,"//label[contains(., 'Minimum order amount for eligibility to redeem loyalty points')]/following::input[1]"
-95.Enter Loyalty points redeem per order (in %) (% of order amount), type, 10,"//label[contains(., 'Loyalty points redeem per order (in %) (% of order amount)')]/following::input[1]"
-96.Enter Loyalty points per default currency (for ex. $1 = 10 points), type, 5,"//label[contains(., 'Loyalty points per default currency (for ex. $1 = 10 points)')]/following::input[1]"
-97.Click Submit ,click,,"//button[normalize-space()='Submit']"
-98.Verify Sucess, verify, , "//div[@aria-label='Info']"
-99.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-100.Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-101.Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-102.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-103.Select Bus Ride Option,click,,"//span[normalize-space()='{transportName}']"
-104.Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-105.Enter Driver Name, type, busdriver_{timestamp} &gt;&gt; busDriverName, "//label[contains(.,'Full Name')]/following::input[1]"
-106.Enter Email, type, busdriver_{timestamp}@gmail.com&gt;&gt;busEmail, "//label[contains(.,'Email')]/following::input[1]"
-107.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-108.Upload Profile Image, uploadfile, "src/main/resources/test-data/busdriver.jpg", "//input[@type='file']"
-109.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-110.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-111.Select  volvo Option,click,,"//li[@role='option']//span[text()='{busTypeName}']"
-112.Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-113.Enter Vehicle Company, type, busCompany{randomAlpha}&gt;&gt; busCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-114.Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
-115. Enter Model Name, type, deisel, "//label[contains(.,'Model Name')]/following::input[1]"
-116.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/busvolvo.jpeg", "(//input[@type='file'])[2]"
-117. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-118.Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-119.Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-120.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-121.Enter Account Holder Name, type, {busDriverName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-122.Enter Payment Email Address, type, {busEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-123.Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-124.Click Submit, click, , "//button[contains(.,'Submit')]"
-125.Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-126.Wait for Toast to hide, wait, 1000,
-127.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-128.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-129.Click Pending Documents,click,,"//span[normalize-space()='Pending documents']"
-130.Filter by Name,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
-131.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-132.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-133.FilterDocumet List,type,{documentName},"//input[@aria-label='Document Name Filter Input']"
-134.Add Driving License,click,,"//i[@title='Edit']"
-135.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-136.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-137.Click Submit, click, , "//button[normalize-space()='Submit']"
-138.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-139.Click Approve Driver,click,,"//i[@title='Approve']"
-140.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-141.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-142.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-143.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-144.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-145.Filter Approved Driver,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
-146.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
-147.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
-148.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
-149.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
-150.Click Edit Icon ,click,,"//i[@title='Edit']"
-151.wait,2000,,
-152.Scroll Grid, tab, 5, "//input[@placeholder='Service Name']"
-153.wait,2000,,
-154.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-155.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
-156.Click  Submit,click,,"//button[normalize-space()='Submit']"
-157.Verify Sucess, verify, , "//div[@aria-label='Info']"
-158.wait,2000,,
-</t>
-  </si>
-  <si>
     <t>1. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
 2.Click  Add Customers,click,,"//span[normalize-space()='Add Customers']"
 3. Verify Add Customer Heading,verify,,"//div[normalize-space()='Add Customer']"
@@ -2788,6 +2622,189 @@
 51.Click Doc Icon,click,,"//i[@title='Document']"
 52.Click Eye Icon,click,,"//i[@title='View']"
 53.wait,1000,,</t>
+  </si>
+  <si>
+    <t>Super Admin Login</t>
+  </si>
+  <si>
+    <t>1.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+2. Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+3.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
+4.Click  Add Category,click,,"//button[normalize-space()='Add Category']"
+5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "//input[@placeholder='Service Name']"
+6.Enter Service Name Arabic, type, رحلة بالحافلة, "//input[@placeholder='Service Name (in Arabic)']"
+7.Enter Slug, type, Bus Ride, "//input[@placeholder='Slug']"
+8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "//input[@type='file' and @accept='image/*']"
+9.wait,2000,,
+10.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+11.Select Activate,click,,"//li[@aria-label='Activate']"
+12.Open Select City Dropdown,click,,"//span[text()='Select City']/ancestor::app-drop-down//div[contains(@class, 'p-multiselect-label-container')]"
+13.Select {areaName},click,,"//li[@aria-label='{areaName}']"
+14.Click  Submit,click,,"//button[normalize-space()='Submit']"
+15.Verify Sucess, verify, , "//div[@aria-label='Info']"
+16.wait,2000,,
+17.Click  back,click,,"//button[normalize-space()='Back']"
+18.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+19.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+20.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
+21.Click Home Icon ,click,,"//i[@title='Home']"
+22.Click Settings ,click,,"//button[contains(., 'Settings')]"
+23.Click Vehicle Type,click,,"//div[normalize-space()='Vehicle Type']"
+24.Click Add Vehicle Type,click,,"//button[normalize-space()='Add Vehicle Type']"
+25.Enter Vehicle Type Name, type, volvo{randomAlpha}&gt;&gt;busTypeName, "//input[@placeholder='Enter Vehicle Type']"
+26.Enter Base Fare, type, 150, "//input[@placeholder='Enter base fare']"
+27.Enter Base Fare Max Kilometer, type, 10, "//input[@placeholder='Enter Base Fare KM Limit']"
+28.Open Extra Distance Fare Dropdown,click,"//label[contains(., 'Extra Distance Fare Type')]/following-sibling::p-dropdown"
+29.Select Amount,click,,"//li[@aria-label='Amount']"
+30.Enter Extra Distance Fare , type, 10, "//input[@placeholder='Extra Distance Fare (Per Km)']"
+31.Enter Free Waiting Time , type, 10, "//label[contains(., 'Free Waiting Time')]/following::input[1]"
+32.Open Waiting Charge Dropdown,click,"((//label[contains(., 'Waiting Charge Type')]/following::p-dropdown)[1])"
+33.Select Amount,click,,"//li[@aria-label='Amount']"
+34.Enter Waiting Rate , type, 10, "//input[@placeholder='Waiting Rate (per min)']"
+35.Enter Included Trip Waiting , type, 10, "//input[@placeholder='Included Trip Waiting']"
+36.Open Trip Waiting Charge Dropdown,click,"((//label[contains(., 'Waiting Charge Type')]/following::p-dropdown)[2])"
+37.Select Amount,click,,"//li[@aria-label='Amount']"
+38.Enter Trip Waiting Rate , type,50, "//input[@placeholder='Trip Waiting Rate (per min)']"
+39.Enter Free Pickup Distance , type,5, "//input[@placeholder='Free Pickup Distance (In kms)']"
+40.Open Pickup Charge Dropdown,click,"//label[contains(., 'Pickup Charge Type')]/following-sibling::p-dropdown"
+41.Select Amount,click,,"//li[@aria-label='Amount']"
+42.Enter Pickup Fee, type,50, "//input[@placeholder='Pickup Fee (Per Km)']"
+43.Open Customer Fee  Dropdown,click,"//span[@aria-label='Customer Fee Type']"
+44.Select Amount,click,,"//li[@aria-label='Amount']"
+45.Enter Customer Fee, type,50, "//input[@placeholder='Customer Fee']"
+46.Open Customer GST  Dropdown,click,"//label[contains(., 'Customer GST type')]/following-sibling::p-dropdown"
+47.Select Amount,click,,"//li[@aria-label='Amount']"
+48.Enter  GST amount, type,50, "//input[contains(@placeholder,'Enter GST amount or percentage')]"
+49.Open Driver Fee  Dropdown,click,"//span[@aria-label='Driver Fee Type']"
+50.Select Amount,click,,"//li[@aria-label='Amount']"
+51.Enter  Driver Fee, type,50, "//input[@placeholder='Driver Fee']"
+52.Open Driver GST  Dropdown,click,"//label[contains(., 'Driver GST type')]/following-sibling::p-dropdown"
+53.Select Amount,click,,"//li[@aria-label='Amount']"
+54.Enter Driver Gst,type,50," //input[@placeholder='Driver GST in amount or percentage']"
+55.Open Status Dropdown,click,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+56.Select Active,click,,"//li[@aria-label='Active']"
+57.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "//app-image-upload//input[@type='file' and @accept='image/*']"
+58.Enter Notifiacation,type,50,"//input[@placeholder='User will be notified when pickup km exceeds this']"
+59.Enter Driver Request ETA,type,50,"//input[@placeholder='Enter Driver ETA Limit']"
+60.Enter Driver Request KM,type,50,"//input[@placeholder='Driver Request KM Limit']"
+61.Click Surcharge Time Checkbox, click, , "//div[text()='EveryDay']/preceding-sibling::mat-checkbox"
+62.Enter From Time, type, 100000AM, "((//input[@placeholder='--:--:-- --'])[1])"
+63.Enter To Time, type, 220000PM, "((//input[@placeholder='--:--:-- --'])[2])"
+64.Open  Dropdown,click,"((//span[@aria-label='select type'])[1])"
+65.Select Amount,click,,"//li[@aria-label='Amount']"
+66.Enter  Price, type,50, "//input[@placeholder='Enter Price']"
+67.Click  Submit,click,,"//button[normalize-space()='Submit']"
+68.Verify Sucess, verify, , "//div[@aria-label='Info']"
+69.Click Settings ,click,,"//button[contains(., 'Settings')]"
+70.Click Promocode,click,,"//div[normalize-space()='Promocode']"
+71.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
+72.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
+73.Select User,click,,"//li[@aria-label='{customerName}']"
+74.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
+75.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; promoCodeName, "//input[@placeholder='Code Name']"
+76.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
+77.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
+78.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
+79.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
+80.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
+81.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
+82.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
+83.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
+84.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
+85.Click Submit ,click,,"//button[normalize-space()='Submit']"
+86.Verify Sucess, verify, , "//div[@aria-label='Info']"
+87.wait,2000,,
+88.Click Settings ,click,,"//button[contains(., 'Settings')]"
+89.Click Service Settings ,click,,"//div[normalize-space()='Service Setting']"
+90.Enter Driver Accept Timeout, type, 60, "//label[contains(., "Driver Accept Timeout")]/following::input[1]"
+91.Enter Driver Serach Radius, type, 50, "//label[contains(., "Driver Search Radius")]/following::input[1]"
+92.Click Submit ,click,,"//button[normalize-space()='Submit']"
+93.Verify Sucess, verify, , "//div[@aria-label='Info']"
+94.wait,1000,,
+95.Click Settings ,click,,"//button[contains(., 'Settings')]"
+96.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
+97.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
+98.Enter Name, type, documet{randomAlpha}&gt;&gt; documentName, "//label[contains(., 'Name')]/following::input[1]"
+99.Open status Dropdown,click,,"//label[contains(., 'Status')]/following::div[contains(@class, 'p-dropdown')]"
+100.Select Active,click,,"//li[@aria-label='Active']"
+101.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
+102.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
+103.Click  Require Proof Number,click,,"//div[./div[contains(text(), 'Require Proof Number')]]//input"
+104.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
+105.Click Submit ,click,,"//button[normalize-space()='Submit']"
+106.Verify Sucess, verify, , "//div[@aria-label='Info']"
+107.Filter Document List,type,{documentName},"//input[@aria-label='Name Filter Input']"
+108.wait,1000,,
+109.Click Settings ,click,,"//button[contains(., 'Settings')]"
+110.Click Customer Loyalty Settings,click,,"//div[text()=' Customer Loyalty Settings ']"
+111.Open status Allow Customer loyalty points,click,,"//label[contains(., 'Allow Customer loyalty points')]/following::div[contains(@class, 'p-dropdown')]"
+112.Select ON,click,,"//li[@role='option']//span[text()='ON']"
+113.Enter Minimum order amount for eligibility to redeem loyalty points, type, 100,"//label[contains(., 'Minimum order amount for eligibility to redeem loyalty points')]/following::input[1]"
+114.Enter Loyalty points redeem per order (in %) (% of order amount), type, 10,"//label[contains(., 'Loyalty points redeem per order (in %) (% of order amount)')]/following::input[1]"
+115.Enter Loyalty points per default currency (for ex. $1 = 10 points), type, 5,"//label[contains(., 'Loyalty points per default currency (for ex. $1 = 10 points)')]/following::input[1]"
+116.Click Submit ,click,,"//button[normalize-space()='Submit']"
+117.Verify Sucess, verify, , "//div[@aria-label='Info']"
+118.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+119.Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+120.Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+121.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+122.Select Bus Ride Option,click,,"//span[normalize-space()='{transportName}']"
+123.Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+124.Enter Driver Name, type, busdriver_{timestamp} &gt;&gt; busDriverName, "//label[contains(.,'Full Name')]/following::input[1]"
+125.Enter Email, type, busdriver_{timestamp}@gmail.com&gt;&gt;busEmail, "//label[contains(.,'Email')]/following::input[1]"
+126.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+127.Upload Profile Image, uploadfile, "src/main/resources/test-data/busdriver.jpg", "//input[@type='file']"
+128.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+129.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+130.Select  volvo Option,click,,"//li[@role='option']//span[text()='{busTypeName}']"
+131.Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+132.Enter Vehicle Company, type, busCompany{randomAlpha}&gt;&gt; busCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+133.Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
+134. Enter Model Name, type, deisel, "//label[contains(.,'Model Name')]/following::input[1]"
+135.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/busvolvo.jpeg", "(//input[@type='file'])[2]"
+136. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+137.Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+138.Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+139.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+140.Enter Account Holder Name, type, {busDriverName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+141.Enter Payment Email Address, type, {busEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+142.Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+143.Click Submit, click, , "//button[contains(.,'Submit')]"
+144.Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+145.Wait for Toast to hide, wait, 1000,
+146.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+147.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+148.Click Pending Documents,click,," //span[normalize-space()='Pending Documents']"
+149.Filter by Name,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
+150.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+151.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+152.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+153.FilterDocumet List,type,{documentName},"//input[@aria-label='Document Name Filter Input']"
+154.Add Driving License,click,,"//i[@title='Edit']"
+155.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+156.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+157.Click Submit, click, , "//button[normalize-space()='Submit']"
+158.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+159.Click Approve Driver,click,,"//i[@title='Approve']"
+160.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+161.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+162.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+163.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+164.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+165.Filter Approved Driver,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
+166.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+167.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+168.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
+169.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
+170.Click Edit Icon ,click,,"//i[@title='Edit']"
+171.wait,2000,,
+172.Scroll Grid, tab, 5, "//input[@placeholder='Service Name']"
+173.wait,2000,,
+174.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+175.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
+176.Click  Submit,click,,"//button[normalize-space()='Submit']"
+177.Verify Sucess, verify, , "//div[@aria-label='Info']"
+178.wait,2000,,</t>
   </si>
 </sst>
 </file>
@@ -3204,7 +3221,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
@@ -3795,7 +3812,7 @@
         <v>59</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>45</v>
@@ -3871,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>45</v>
@@ -3946,7 +3963,7 @@
         <v>26</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>40</v>
@@ -4011,7 +4028,7 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>46</v>
@@ -4083,7 +4100,7 @@
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>47</v>
@@ -4155,7 +4172,7 @@
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>48</v>
@@ -4227,7 +4244,7 @@
         <v>77</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>76</v>

</xml_diff>

<commit_message>
67th commit: Test Cases Completely Working Again
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{261120D6-711C-4106-94A9-C451F48FF5F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94A5C8B5-77AB-4EB0-99FB-DFF0B202A1FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="11" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -416,83 +416,6 @@
   </si>
   <si>
     <t>Add New Provider Service &amp;  Category</t>
-  </si>
-  <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
-3.Verify Delivery Services,verify,,"//div[contains(text(),'DELIVERY SERVICES')]"
-4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
-5.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
-6.Click  Stores,click,,"//button[contains(., 'Stores')]"
-7.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
-8.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Add Store')]"
-9.Enter Store Name, type, KFC_{timestamp} &gt;&gt; storeName, "//input[@placeholder='Store Name']"
-10.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
-11.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
-12.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
-13. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
-14.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
-15.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
-16.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
-17.Upload Banner Image, uploadfile, "src/main/resources/test-data/kfcbanner.jpg", "//input[@type='file']"
-18.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
-19.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
-20.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
-21.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
-22.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-23..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
-24.wait,1000,,
-25.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
-26.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
-27.wait,1000,,
-28.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
-29.Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
-30.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
-31.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
-32.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
-33.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
-34.Enter Contact Person Full Name, type, storeowner_{timestamp} &gt;&gt; storeOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
-35.Enter Email, type, kfc_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
-36.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
-37.Upload Store Image, uploadfile, "src/main/resources/test-data/kfcstore.jpg", "(//input[@type='file'])[2]"
-38.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
-39.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
-40.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
-41.Enter Accont Holder Name, type, {storeOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
-42.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
-43.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
-44.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
-45.Enter From Time, type, 100000, "(//label[contains(.,'From Time')]/following-sibling::input)[1]"
-46.Enter To Time, type, 220000, "(//label[contains(.,'To Time')]/following-sibling::input)[1]"
-47.Submit Add Store,click,,"//button[normalize-space()='Submit']"
-48. Verify Success Message,verify,,"//div[@aria-label='Info']"
-49.Click  Stores,click,,"//button[contains(., 'Stores')]"
-50.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-51.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-52.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-53.Click  Stores,click,,"//button[contains(., 'Stores')]"
-54.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
-55.Verify Add Store,verify,,"//div[normalize-space()='Pending Documents Store']"
-56.Filter Pending Document Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-57.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-58.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-59. Store Required Documents,verify,,"//div[contains(text(),'Documents')]"
-60.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-61.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-62.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-63.Click Submit, click, , "//button[normalize-space()='Submit']"
-64.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-65.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-66.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-67.Click Back, click, , "//button[@class='buttonWidget']"
-68.Click  Stores,click,,"//button[contains(., 'Stores')]"
-69.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-70.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-71.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-72.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-73.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-74.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
-75.wait,1000,,</t>
   </si>
   <si>
     <r>
@@ -1631,273 +1554,6 @@
 63.Filter Driver List,type,{kfcdriverName},"//input[@aria-label='Driver Name Filter Input']"
 64.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
 65.wait,1000,,</t>
-  </si>
-  <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
-3.Verify Delivery Services,verify,,"//div[contains(text(),' DELIVERY SERVICES')]"
-4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
-5.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
-6.Click  Stores,click,,"//button[contains(., 'Stores')]"
-7.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
-8.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Add Store')]"
-9.Enter Store Name, type, bilal_{timestamp} &gt;&gt; hotelName, "//input[@placeholder='Store Name']"
-10.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
-11.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
-12.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
-13. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
-14.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
-15.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
-16.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
-17.Upload Banner Image, uploadfile, "src/main/resources/test-data/kfcbanner.jpg", "//input[@type='file']"
-18.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
-19.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
-20.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
-21.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
-22.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-23..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
-24.wait,1000,,
-25.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
-26.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
-27.wait,1000,,
-28.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
-29.Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
-30.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
-31.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
-32.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
-33.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
-34.Enter Contact Person Full Name, type, bilalowner_{timestamp} &gt;&gt; hotelOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
-35.Enter Email, type, bilal_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
-36.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
-37.Upload Store Image, uploadfile, "src/main/resources/test-data/kfcstore.jpg", "(//input[@type='file'])[2]"
-38.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
-39.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
-40.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
-41.Enter Accont Holder Name, type, {hotelOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
-42.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
-43.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
-44.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
-45.Enter From Time, type, 100000, "(//label[contains(.,'From Time')]/following-sibling::input)[1]"
-46.Enter To Time, type, 220000, "(//label[contains(.,'To Time')]/following-sibling::input)[1]"
-47.Submit Add Store,click,,"//button[normalize-space()='Submit']"
-48. Verify Success Message,verify,,"//div[@aria-label='Info']"
-49.Click  Stores,click,,"//button[contains(., 'Stores')]"
-50.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-51.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-52.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
-53.Click  Stores,click,,"//button[contains(., 'Stores')]"
-54.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
-55.Verify Add Store,verify,,"//div[normalize-space()='Pending Documents Store']"
-56.Filter Pending Document Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
-57.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-58.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-59. Store Required Documents,verify,,"//div[contains(text(),'Documents')]"
-60.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-61.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-62.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-63.Click Submit, click, , "//button[normalize-space()='Submit']"
-64.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-65.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-66.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-67.Click Back, click, , "//button[@class='buttonWidget']"
-68.Click  Stores,click,,"//button[contains(., 'Stores')]"
-69.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-70.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-71.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
-72.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-73.Click Block Icon,click,,"//i[@title='Blocked']"
-74.Click Block  Yes,click,,"//button[normalize-space()='Yes']"
-75.Click  Stores,click,,"//button[contains(., 'Stores')]"
-76.Select Blocked Store,click,,"//div[normalize-space()='Blocked Stores']"
-77.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
-78.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-79.Click unBlock Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
-80.Click  Stores,click,,"//button[contains(., 'Stores')]"
-81.Select Rejected Store,click,,"//div[normalize-space()='Rejected Stores']"
-82.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
-83.Scroll Grid, tab, 7, "//input[@aria-label='Store Name Filter Input']"
-84.Click Approve Icon,click,,"//i[@title='Approve']"
-85.Click  Stores,click,,"//button[contains(., 'Stores')]"
-86.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-87.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
-88.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-89.Click Doc Icon,click,,"//i[@title='Document']"
-90.Click UnApprove Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
-91.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-92.Rejection Reason,type,document insufficent,"//textarea[@id='swal2-textarea']"
-93.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-94.wait,1000,,</t>
-  </si>
-  <si>
-    <t>1.Click badge,click,,"//i[@class='fa-solid fa-user-shield iconstyle']"
-2.Click Delivery Services,click,,"//h2[normalize-space()='Delivery Services']"
-3.Verify Delivery Services,verify,,"//div[normalize-space()='DELIVERY SERVICES']"
-4.Click  Add Service Category,click,,"//button[normalize-space()='Add Service Category']"
-5.Enter Category Name, type, milk Delivery{randomAlpha}&gt;&gt; deliveryName, "//input[@placeholder='Category Name']"
-6.Enter Slug, type, Milk Delivery, "//input[@placeholder='Slug']"
-7.Upload Category Image, uploadfile, "src/main/resources/test-data/milkman.jpg", "//input[@type='file' and @accept='image/*']"
-8.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-9.Select Activate,click,,"//li[@aria-label='Activate']"
-10.Open Category Flow Dropdown,click,,"//label[contains(., 'Category Flow')]/following-sibling::p-dropdown"
-11.Select default flow(food-delivery),click,,"//li[@aria-label='default flow(food-delivery)']"
-12.Enter Delivery Name Tamil, type,பால்காரர், "//input[@placeholder='Enter in Tamil']"
-13.Enter Delivery Name Arabic, type, لبّان, "//input[@placeholder='Enter in Arabic']"
-14.Enter Delivery Name Hindi, type, दूधवाला, "//input[@placeholder='Enter in Hindi']"
-15.Click  Submit,click,,"//button[normalize-space()='Submit']"
-16.Verify Sucess, verify, , "//div[@aria-label='Info']"
-17.Filter Services List,type,{deliveryName},"//input[@aria-label='Services Filter Input']"
-18.Click Home Icon ,click,,"//i[@title='Home']"
-19.Click Settings ,click,,"//button[contains(., 'Settings')]"
-20.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
-21.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
-22.Enter Name, type, documet{randomAlpha}&gt;&gt; deliveryDocumentName, "//input[@placeholder='Type here']"
-23.Open status Dropdown,click,,"//span[@aria-label='select status']"
-24.Select Active,click,,"//li[@aria-label='Active']"
-25.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
-26.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
-27.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
-28.Click  Require Proof Number,click,,"//div[./div[contains(text(), 'Require Proof Number')]]//input"
-29.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
-30.Click Submit ,click,,"//button[normalize-space()='Submit']"
-31.Verify Sucess, verify, , "//div[@aria-label='Info']"
-32.Filter Document List,type,{deliveryDocumentName},"//input[@aria-label='Name Filter Input']"
-33.wait,2000,,
-33.Click Settings ,click,,"//button[contains(., 'Settings')]"
-34.Click Promocode ,click,,"//div[normalize-space()='Promocode']"
-35.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
-36.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
-37.Select User,click,,"//li[@aria-label='{customerName}']"
-38.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
-39.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; deliveryPromoCodeName, "//input[@placeholder='Code Name']"
-40.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
-41.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
-42.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
-43.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
-44.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
-45.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
-46.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
-47.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
-48.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
-49.Click Submit ,click,,"//button[normalize-space()='Submit']"
-50.Verify Sucess, verify, , "//div[@aria-label='Info']"
-51.Filter PromoCode List,type,{deliveryPromoCodeName},"//input[@aria-label='promocode Filter Input']"
-52.wait,2000,,
-53.Click Settings ,click,,"//button[contains(., 'Settings')]"
-54.Click Service Settings ,click,,"//div[normalize-space()='Service Settings']"
-55.Enter Driver Serach Radius, type, 50, "//span[contains(text(), 'Driver search Radius')]/ancestor::app-input//input"
-56.Open Tax Type Dropdown,click,,"//span[@aria-label='Select Tax Type']"
-57.Select Amount,click,,"//li[@aria-label='Amount']"
-58.Enter Tax, type, 20, "//span[contains(text(), 'Tax')]/ancestor::app-input//input"
-59.Open Platform Fee Type Dropdown,click,,"//span[@aria-label='Seelct Type']"
-60.Select Amount,click,,"//li[@aria-label='Amount']"
-61.Enter Platform Fee, type, 20, "//span[contains(text(), 'Platform Fee')]/ancestor::app-input//input"
-62.Enter Cancel Charge (in %):, type, 20, "//span[contains(text(), 'Cancel Charge (in %):')]/ancestor::app-input//input"
-63.Enter Driver Accept Timeout (in Second):, type, 20, "//span[contains(text(), 'Driver Accept Timeout (in Second):')]/ancestor::app-input//input"
-64.Click Submit ,click,,"//button[normalize-space()='Submit']"
-65.Verify Sucess, verify, , "//div[@aria-label='Info']"
-66.Click  Stores,click,,"//button[contains(., 'Stores')]"
-67.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
-68.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Add Store')]"
-69.Enter Store Name, type, amul_{timestamp} &gt;&gt; milkStore, "//input[@placeholder='Store Name']"
-70.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
-71.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
-72.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
-73. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
-74.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
-75.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
-76.Enter Short Description, type, amul taste of india, "//input[@placeholder="Type here"]"
-77.Upload Banner Image, uploadfile, "src/main/resources/test-data/amulbanner.jpg", "//input[@type='file']"
-78.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
-79.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
-80.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
-81.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
-82.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-83..Enter Store Address, type, Amul chennai, "//input[@placeholder='Search location']"
-84.wait,1000,,
-85.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
-86.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
-87.wait,1000,,
-88.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
-89.Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
-90.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
-91.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
-92.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
-93.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
-94.Enter Contact Person Full Name, type, amulStoreowner_{timestamp} &gt;&gt; milkStoreOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
-95.Enter Email, type, amul_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
-96.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
-97.Upload Store Image, uploadfile, "src/main/resources/test-data/milkbooth.jpeg", "(//input[@type='file'])[2]"
-98.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
-99.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
-100.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
-101.Enter Accont Holder Name, type, {milkStoreOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
-102.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
-103.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
-104.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
-105.Enter From Time, type, 100000, "(//label[contains(.,'From Time')]/following-sibling::input)[1]"
-106.Enter To Time, type, 220000, "(//label[contains(.,'To Time')]/following-sibling::input)[1]"
-107.Submit Add Store,click,,"//button[normalize-space()='Submit']"
-108. Verify Success Message,verify,,"//div[@aria-label='Info']"
-109.Click  Stores,click,,"//button[contains(., 'Stores')]"
-110.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-111.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-112.Filter Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
-113.Click  Stores,click,,"//button[contains(., 'Stores')]"
-114.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
-115.Verify Add Store,verify,,"//div[normalize-space()='Pending Documents Store']"
-116.Filter Pending Document Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
-117.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-118.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-119. Store Required Documents,verify,,"//div[contains(text(),'Documents')]"
-120.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-121.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-122.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-123.Click Submit, click, , "//button[normalize-space()='Submit']"
-124.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-125.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-126.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-127.Click Back, click, , "//button[@class='buttonWidget']"
-128.Click  Stores,click,,"//button[contains(., 'Stores')]"
-129.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-130.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-131.Filter Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
-132.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-133.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-134.Click Back, click, , "//button[@class='buttonWidget']"
-135.Click Category, click, , "//button[normalize-space()='Category']"
-136.Click  Add New Category,click,,"//button[normalize-space()='Add Category']"
-137.Enter Category Name, type,curd{randomAlpha}&gt;&gt; MilkCategoryName, "//span[contains(text(), 'Category Name')]/ancestor::app-input//input"
-138.Enter Category Name Arabic, type, رائب, "//span[contains(text(), 'Language Value (in Arabic)')]/ancestor::app-input//input"
-139.Enter Category Name Tamil, type, தயிர், "//span[contains(text(), 'Language Value (in Tamil)')]/ancestor::app-input//input"
-140.Enter Category Name Hindi, type, दही, "//span[contains(text(), 'Language Value (in Hindi)')]/ancestor::app-input//input"
-141.Open Category status Dropdown,click,,"//span[@aria-label='status']"
-142.Select Active,click,,"//li[@aria-label='active']"
-143.Upload Category Image, uploadfile, "src/main/resources/test-data/curd.jpeg", "//input[@type='file' and @accept='image/*']"
-144.wait,2000,,
-145.Enter Slug Name, type, curd, "//span[text()='Slug']/ancestor::app-input//input"
-146.Click  Submit,click,,"//button[normalize-space()='Submit']"
-147.Verify Success Message,verify,,"//div[@aria-label='Info']"
-148.Filter Category Name,type,{MilkCategoryName},"//input[@aria-label='Category Name Filter Input']"
-149.Click  Stores,click,,"//button[contains(., 'Stores')]"
-150.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-151.Filter Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
-152.Scroll Grid, tab, 9, "//input[@aria-label='Store Name Filter Input']"
-153.Click Product Icon,click,,"//i[@title='Product View']"
-154.Click  Add  Products,click,,"//button[normalize-space()='Add Products']"
-155.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[1]"
-156.Select curd,click,,"//li[@role='option'][contains(.,'{MilkCategoryName}')]"
-157.wait,1000,,
-158.Click badge,click,,"//i[@class='fa-solid fa-user-shield iconstyle']"
-159.Click Delivery Services,click,,"//h2[normalize-space()='Delivery Services']"
-160.Verify Delivery Services,verify,,"//div[normalize-space()='DELIVERY SERVICES']"
-161.Filter Services List,type,{deliveryName},"//input[@aria-label='Services Filter Input']"
-162.Click Edit Icon ,click,,"//i[@title='Edit']"
-163.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-164.wait,1000,,
-164.Select Dectivate,click,,"//li[@aria-label='Deactivate']"
-165.Click Submit ,click,,"//button[normalize-space()='Submit']"
-166.Filter Services List,type,{deliveryName},"//input[@aria-label='Services Filter Input']"
-167.wait,1000,,</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
@@ -2169,131 +1825,6 @@
       </rPr>
       <t>The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
-2.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
-3.Click Store subscription plan,click,,"//span[normalize-space()='Store subscription plan']"
-4.Verify Store Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Store']"
-5.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
-6.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
-7.Select Food Delivery,click,,"//li[@aria-label='Food Delivery']"
-8.Enter Store Plan Name, type, StorePlan{randomAlpha}&gt;&gt; storeSubscriptionName, "//input[@placeholder='Plan Name']"
-9.Enter Store Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
-10.Enter Store Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
-11.Enter Store Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
-12.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
-13.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
-14.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
-15.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description(in Arabic)']"
-16.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description(in Tamil)']"
-17.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description(in Hindi)']"
-18.Open status Dropdown,click,,"//span[@aria-label='select Status']"
-19.Select On,click,,"//li[@aria-label='on']"
-20.Click Submit ,click,,"//button[normalize-space()='Submit']"
-21.Filter Services List,type,{storeSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
-22.Click Edit ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-23.Click Close ,click,,"//button[normalize-space()='Close']"
-24.Click Active ,click,,"//i[@title='Active']"
-25.wait,2000,,
-26.Click Deactive,click,,"//i[@title='Inactive']"
-27.wait,2000,,
-28.Click Delete Plan,click,,"//i[@class='bi bi-trash cursor-pointer gridIcon Delete']"
-29.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
-30.wait,3000,,
-31.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
-32.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
-33.Click Driver subscription plan,click,,"//span[normalize-space()='Driver subscription plan']"
-34.Verify Driver Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Driver']"
-35.Click  Add New Subscription,click,,"//button[normalize-space()='ADD']"
-36.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
-37.Select Auto Ride,click,,"//li[@aria-label='Auto Ride']"
-38.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "//input[@placeholder='Plan Name']"
-39.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
-40.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil)']"
-41.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi)']"
-42.Enter Number Of Days, type,100, "//input[@placeholder='No. of Days ']"
-43.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No of Rides with Zero admin commission']"
-44.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
-45.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
-46.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description Arabic']"
-47.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description Tamil']"
-48.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description Hindi']"
-49.Open status Dropdown,click,,"//span[@aria-label='select Status']"
-50.Select On,click,,"//li[@aria-label='on']"
-51.Click Submit ,click,,"//button[normalize-space()='Submit']"
-52.Filter Services List,type,{driverSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
-53.Click Edit ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-54.Click Close ,click,,"//button[normalize-space()='Close']"
-55.Click Active ,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-56.wait,2000,,
-57.Click Deactive,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
-58.wait,2000,,
-59.Click Delete Plan,click,,"//i[@class='bi bi-trash cursor-pointer gridIcon Delete']"
-60.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
-61.wait,3000,,
-62.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
-63.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
-64.Click Provider subscription plan,click,,"//span[normalize-space()='Provider subscription plan']"
-65.Verify Provider Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Provider']"
-66.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
-67.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
-68.Select Pest Control,click,,"//li[@aria-label='Pest Control']"
-69.Enter Provider Plan Name, type, ProviderPlan{randomAlpha}&gt;&gt; providerSubscriptionName, "//input[@placeholder='Plan Name']"
-70.Enter Provider Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic):']"
-71.Enter Provider Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
-72.Enter Provider Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
-73.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
-74.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price ']"
-75.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Enter Description(in English):']"
-76.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Enter Description(in Arabic):']"
-77.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Enter Description(in Tamil)']"
-78.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Enter Description(in Hindi']"
-79.Open status Dropdown,click,,"//span[@aria-label='select Status']"
-80.Select On,click,,"//li[@aria-label='on']"
-81.Click Submit ,click,,"//button[normalize-space()='Submit']"
-82.Filter Services List,type,{providerSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
-83.Click Edit ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-84.Click Close ,click,,"//button[normalize-space()='Close']"
-85.Click Active ,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-86.wait,2000,,
-87.Click Deactive,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
-88.wait,2000,,
-89.Click Delete Plan,click,,"//i[@class='bi bi-trash cursor-pointer gridIcon Delete']"
-90.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
-91.wait,3000,,
-92.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
-93.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
-94.Click Customer subscription plan,click,,"//span[normalize-space()='Customer subscription plan']"
-95.Verify Customer Subscription Plan Lists ,verify,,"//div[normalize-space()='Customer Subscription Plans']"
-96.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
-97.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
-98.Select Pest Control,click,,"//li[@aria-label='Pest Control']"
-99.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; custometSubscriptionName, "//input[@placeholder='Plan Name']"
-100.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
-101.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
-102.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
-103.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
-104.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No Of Free Rides']"
-105.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
-106.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
-107.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description(in Arabic)']"
-108.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description(in Tamil)']"
-109.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description(in Hindi)']"
-110.Open status Dropdown,click,,"//span[@aria-label='select Status']"
-111.Select On,click,,"//li[@aria-label='on']"
-112.Click Submit ,click,,"//button[normalize-space()='Submit']"
-113.Filter Services List,type,{custometSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
-114.Click Edit ,click,,"//i[@title='Edit Plan']"
-115.Click Close ,click,,"//button[normalize-space()='Close']"
-116.Click Active ,click,,"//i[@title='Activate Plan']"
-117.wait,2000,,
-118.Click Deactive,click,,"//i[@title='Deactivate Plan']"
-119.wait,2000,,
-120.Click Delete Plan,click,,"//i[@title='Delete Plan']"
-121.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
-122.wait,3000,,
-</t>
   </si>
   <si>
     <t>This test case validates the end-to-end management of subscription plan architectures across four distinct user entities: Store, Driver, Provider, and Customer. The workflow systematically executes the creation of localized "Premium" plans for various service categories—such as Food Delivery and Pest Control—featuring integrated multi-language support in Arabic, Tamil, and Hindi. The validation cycle spans from defining plan durations, pricing, and free-ride quotas to conducting administrative audits including localized description verification, active/inactive state toggling, and data filtering. The process concludes by confirming the operational lifecycle through record modification and final deletion, ensuring the functional stability and localized integrity of the platform’s commercial monetization modules.</t>
@@ -2805,6 +2336,476 @@
 176.Click  Submit,click,,"//button[normalize-space()='Submit']"
 177.Verify Sucess, verify, , "//div[@aria-label='Info']"
 178.wait,2000,,</t>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
+3.Verify Delivery Services,verify,,"//div[contains(text(),'DELIVERY SERVICES')]"
+4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
+5.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
+6.Click  Stores,click,,"//button[contains(., 'Stores')]"
+7.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
+8.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Add Store')]"
+9.Enter Store Name, type, KFC_{timestamp} &gt;&gt; storeName, "//input[@placeholder='Store Name']"
+10.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
+11.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
+12.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
+13. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
+14.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
+15.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
+16.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
+17.Upload Banner Image, uploadfile, "src/main/resources/test-data/kfcbanner.jpg", "//input[@type='file']"
+18.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
+19.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
+20.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
+21.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
+22.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+23..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
+24.wait,1000,,
+25.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
+26.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
+27.wait,1000,,
+28.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
+29.Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
+30.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
+31.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
+32.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
+33.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
+34.Enter Contact Person Full Name, type, storeowner_{timestamp} &gt;&gt; storeOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
+35.Enter Email, type, kfc_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
+36.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
+37.Upload Store Image, uploadfile, "src/main/resources/test-data/kfcstore.jpg", "(//input[@type='file'])[2]"
+38.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
+39.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
+40.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
+41.Enter Accont Holder Name, type, {storeOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
+42.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
+43.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
+44.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
+45.Enter From Time, type, 100000AM, "((//input[@placeholder='--:--:-- --'])[1])"
+46.Enter To Time, type, 100000PM, "((//input[@placeholder='--:--:-- --'])[2])"
+47.Submit Add Store,click,,"//button[normalize-space()='Submit']"
+48. Verify Success Message,verify,,"//div[@aria-label='Info']"
+49.Click  Stores,click,,"//button[contains(., 'Stores')]"
+50.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+51.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
+52.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+53.Click  Stores,click,,"//button[contains(., 'Stores')]"
+54.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
+55.Verify Add Store,verify,,"//div[normalize-space()='Pending Documents Store']"
+56.Filter Pending Document Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+57.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+58.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
+59. Store Required Documents,verify,,"//div[contains(text(),'Documents')]"
+60.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+61.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
+62.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+63.Click Submit, click, , "//button[normalize-space()='Submit']"
+64.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+65.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+66.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+67.Click Back, click, , "//button[@class='buttonWidget']"
+68.Click  Stores,click,,"//button[contains(., 'Stores')]"
+69.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+70.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
+71.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
+72.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+73.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
+74.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
+75.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
+2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
+3.Verify Delivery Services,verify,,"//div[contains(text(),' DELIVERY SERVICES')]"
+4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
+5.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
+6.Click  Stores,click,,"//button[contains(., 'Stores')]"
+7.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
+8.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Add Store')]"
+9.Enter Store Name, type, bilal_{timestamp} &gt;&gt; hotelName, "//input[@placeholder='Store Name']"
+10.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
+11.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
+12.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
+13. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
+14.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
+15.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
+16.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
+17.Upload Banner Image, uploadfile, "src/main/resources/test-data/kfcbanner.jpg", "//input[@type='file']"
+18.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
+19.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
+20.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
+21.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
+22.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+23..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
+24.wait,1000,,
+25.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
+26.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
+27.wait,1000,,
+28.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
+29.Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
+30.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
+31.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
+32.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
+33.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
+34.Enter Contact Person Full Name, type, bilalowner_{timestamp} &gt;&gt; hotelOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
+35.Enter Email, type, bilal_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
+36.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
+37.Upload Store Image, uploadfile, "src/main/resources/test-data/kfcstore.jpg", "(//input[@type='file'])[2]"
+38.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
+39.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
+40.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
+41.Enter Accont Holder Name, type, {hotelOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
+42.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
+43.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
+44.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
+45.Enter From Time, type, 100000AM, "((//input[@placeholder='--:--:-- --'])[1])"
+46.Enter To Time, type, 100000PM, "((//input[@placeholder='--:--:-- --'])[2])"
+47.Submit Add Store,click,,"//button[normalize-space()='Submit']"
+48. Verify Success Message,verify,,"//div[@aria-label='Info']"
+49.Click  Stores,click,,"//button[contains(., 'Stores')]"
+50.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+51.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
+52.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
+53.Click  Stores,click,,"//button[contains(., 'Stores')]"
+54.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
+55.Verify Add Store,verify,,"//div[normalize-space()='Pending Documents Store']"
+56.Filter Pending Document Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
+57.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+58.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
+59. Store Required Documents,verify,,"//div[contains(text(),'Documents')]"
+60.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+61.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
+62.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+63.Click Submit, click, , "//button[normalize-space()='Submit']"
+64.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+65.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+66.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+67.Click Back, click, , "//button[@class='buttonWidget']"
+68.Click  Stores,click,,"//button[contains(., 'Stores')]"
+69.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+70.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
+71.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
+72.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+73.Click Block Icon,click,,"//i[@title='Blocked']"
+74.Click Block  Yes,click,,"//button[normalize-space()='Yes']"
+75.Click  Stores,click,,"//button[contains(., 'Stores')]"
+76.Select Blocked Store,click,,"//div[normalize-space()='Blocked Stores']"
+77.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
+78.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+79.Click unBlock Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
+80.Click  Stores,click,,"//button[contains(., 'Stores')]"
+81.Select Rejected Store,click,,"//div[normalize-space()='Rejected Stores']"
+82.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
+83.Scroll Grid, tab, 7, "//input[@aria-label='Store Name Filter Input']"
+84.Click Approve Icon,click,,"//i[@title='Approve']"
+85.Click  Stores,click,,"//button[contains(., 'Stores')]"
+86.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+87.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
+88.wait,3000,,
+89.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+90.Click Doc Icon,click,,"//i[@title='Document']"
+91.Click UnApprove Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
+92.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+93.Rejection Reason,type,document insufficent,"//textarea[@id='swal2-textarea']"
+94.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+95.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[@class='fa-solid fa-user-shield iconstyle']"
+2.Click Delivery Services,click,,"//h2[normalize-space()='Delivery Services']"
+3.Verify Delivery Services,verify,,"//div[normalize-space()='DELIVERY SERVICES']"
+4.Click  Add Service Category,click,,"//button[normalize-space()='Add Service Category']"
+5.Enter Category Name, type, milk Delivery{randomAlpha}&gt;&gt; deliveryName, "//input[@placeholder='Category Name']"
+6.Enter Slug, type, Milk Delivery, "//input[@placeholder='Slug']"
+7.Upload Category Image, uploadfile, "src/main/resources/test-data/milkman.jpg", "//input[@type='file' and @accept='image/*']"
+8.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+9.Select Activate,click,,"//li[@aria-label='Activate']"
+10.Open Category Flow Dropdown,click,,"//label[contains(., 'Category Flow')]/following-sibling::p-dropdown"
+11.Select default flow(food-delivery),click,,"//li[@aria-label='default flow(food-delivery)']"
+12.Enter Delivery Name Tamil, type,பால்காரர், "//input[@placeholder='Enter in Tamil']"
+13.Enter Delivery Name Arabic, type, لبّان, "//input[@placeholder='Enter in Arabic']"
+14.Enter Delivery Name Hindi, type, दूधवाला, "//input[@placeholder='Enter in Hindi']"
+15.Click  Submit,click,,"//button[normalize-space()='Submit']"
+16.Verify Sucess, verify, , "//div[@aria-label='Info']"
+17.Filter Services List,type,{deliveryName},"//input[@aria-label='Services Filter Input']"
+18.Click Home Icon ,click,,"//i[@title='Home']"
+19.Click Settings ,click,,"//button[contains(., 'Settings')]"
+20.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
+21.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
+22.Enter Name, type, documet{randomAlpha}&gt;&gt; deliveryDocumentName, "//input[@placeholder='Type here']"
+23.Open status Dropdown,click,,"//span[@aria-label='select status']"
+24.Select Active,click,,"//li[@aria-label='Active']"
+25.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
+26.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
+27.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
+28.Click  Require Proof Number,click,,"//div[./div[contains(text(), 'Require Proof Number')]]//input"
+29.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
+30.Click Submit ,click,,"//button[normalize-space()='Submit']"
+31.Verify Sucess, verify, , "//div[@aria-label='Info']"
+32.Filter Document List,type,{deliveryDocumentName},"//input[@aria-label='Name Filter Input']"
+33.wait,2000,,
+33.Click Settings ,click,,"//button[contains(., 'Settings')]"
+34.Click Promocode ,click,,"//div[normalize-space()='Promocode']"
+35.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
+36.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
+37.Select User,click,,"//li[@aria-label='{customerName}']"
+38.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
+39.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; deliveryPromoCodeName, "//input[@placeholder='Code Name']"
+40.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
+41.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
+42.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
+43.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
+44.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
+45.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
+46.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
+47.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
+48.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
+49.Click Submit ,click,,"//button[normalize-space()='Submit']"
+50.Verify Sucess, verify, , "//div[@aria-label='Info']"
+51.Filter PromoCode List,type,{deliveryPromoCodeName},"//input[@aria-label='promocode Filter Input']"
+52.wait,2000,,
+53.Click Settings ,click,,"//button[contains(., 'Settings')]"
+54.Click Service Settings ,click,,"//div[normalize-space()='Service Settings']"
+55.Enter Driver Serach Radius, type, 50, "//span[contains(text(), 'Driver search Radius')]/ancestor::app-input//input"
+56.Open Tax Type Dropdown,click,,"//span[@aria-label='Select Tax Type']"
+57.Select Amount,click,,"//li[@aria-label='Amount']"
+58.Enter Tax, type, 20, "//span[contains(text(), 'Tax')]/ancestor::app-input//input"
+59.Open Platform Fee Type Dropdown,click,,"//span[@aria-label='Seelct Type']"
+60.Select Amount,click,,"//li[@aria-label='Amount']"
+61.Enter Platform Fee, type, 20, "//span[contains(text(), 'Platform Fee')]/ancestor::app-input//input"
+62.Enter Cancel Charge (in %):, type, 20, "//span[contains(text(), 'Cancel Charge (in %):')]/ancestor::app-input//input"
+63.Enter Driver Accept Timeout (in Second):, type, 20, "//span[contains(text(), 'Driver Accept Timeout (in Second):')]/ancestor::app-input//input"
+64.Click Submit ,click,,"//button[normalize-space()='Submit']"
+65.Verify Sucess, verify, , "//div[@aria-label='Info']"
+66.Click  Stores,click,,"//button[contains(., 'Stores')]"
+67.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
+68.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Add Store')]"
+69.Enter Store Name, type, amul_{timestamp} &gt;&gt; milkStore, "//input[@placeholder='Store Name']"
+70.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
+71.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
+72.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
+73. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
+74.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
+75.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
+76.Enter Short Description, type, amul taste of india, "//input[@placeholder="Type here"]"
+77.Upload Banner Image, uploadfile, "src/main/resources/test-data/amulbanner.jpg", "//input[@type='file']"
+78.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
+79.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
+80.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
+81.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
+82.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+83..Enter Store Address, type, Amul chennai, "//input[@placeholder='Search location']"
+84.wait,1000,,
+85.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
+86.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
+87.wait,1000,,
+88.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
+89.Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
+90.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
+91.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
+92.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
+93.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
+94.Enter Contact Person Full Name, type, amulStoreowner_{timestamp} &gt;&gt; milkStoreOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
+95.Enter Email, type, amul_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
+96.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
+97.Upload Store Image, uploadfile, "src/main/resources/test-data/milkbooth.jpeg", "(//input[@type='file'])[2]"
+98.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
+99.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
+100.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
+101.Enter Accont Holder Name, type, {milkStoreOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
+102.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
+103.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
+104.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
+105.Enter From Time, type, 100000AM, "((//input[@placeholder='--:--:-- --'])[1])"
+106.Enter To Time, type, 100000PM, "((//input[@placeholder='--:--:-- --'])[2])"
+107.Submit Add Store,click,,"//button[normalize-space()='Submit']"
+108. Verify Success Message,verify,,"//div[@aria-label='Info']"
+109.Click  Stores,click,,"//button[contains(., 'Stores')]"
+110.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+111.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
+112.Filter Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
+113.Click  Stores,click,,"//button[contains(., 'Stores')]"
+114.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
+115.Verify Add Store,verify,,"//div[normalize-space()='Pending Documents Store']"
+116.Filter Pending Document Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
+117.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+118.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
+119. Store Required Documents,verify,,"//div[contains(text(),'Documents')]"
+120.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+121.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
+122.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
+123.Click Submit, click, , "//button[normalize-space()='Submit']"
+124.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+125.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+126.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+127.Click Back, click, , "//button[@class='buttonWidget']"
+128.Click  Stores,click,,"//button[contains(., 'Stores')]"
+129.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+130.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
+131.Filter Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
+132.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
+133.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
+134.Click Back, click, , "//button[@class='buttonWidget']"
+135.Click Category, click, , "//button[normalize-space()='Category']"
+136.Click  Add New Category,click,,"//button[normalize-space()='Add Category']"
+137.Enter Category Name, type,curd{randomAlpha}&gt;&gt; MilkCategoryName, "//span[contains(text(), 'Category Name')]/ancestor::app-input//input"
+138.Enter Category Name Arabic, type, رائب, "//span[contains(text(), 'Language Value (in Arabic)')]/ancestor::app-input//input"
+139.Enter Category Name Tamil, type, தயிர், "//span[contains(text(), 'Language Value (in Tamil)')]/ancestor::app-input//input"
+140.Enter Category Name Hindi, type, दही, "//span[contains(text(), 'Language Value (in Hindi)')]/ancestor::app-input//input"
+141.Open Category status Dropdown,click,,"//span[@aria-label='status']"
+142.Select Active,click,,"//li[@aria-label='active']"
+143.Upload Category Image, uploadfile, "src/main/resources/test-data/curd.jpeg", "//input[@type='file' and @accept='image/*']"
+144.wait,2000,,
+145.Enter Slug Name, type, curd, "//span[text()='Slug']/ancestor::app-input//input"
+146.Click  Submit,click,,"//button[normalize-space()='Submit']"
+147.Verify Success Message,verify,,"//div[@aria-label='Info']"
+148.Filter Category Name,type,{MilkCategoryName},"//input[@aria-label='Category Name Filter Input']"
+149.Click  Stores,click,,"//button[contains(., 'Stores')]"
+150.Select Store List,click,,"//div[contains(text(), 'Store List')]"
+151.Filter Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
+152.Scroll Grid, tab, 9, "//input[@aria-label='Store Name Filter Input']"
+153.Click Product Icon,click,,"//i[@title='Product View']"
+154.Click  Add  Products,click,,"//button[normalize-space()='Add Products']"
+155.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[1]"
+156.Select curd,click,,"//li[@role='option'][contains(.,'{MilkCategoryName}')]"
+157.wait,1000,,
+158.Click badge,click,,"//i[@class='fa-solid fa-user-shield iconstyle']"
+159.Click Delivery Services,click,,"//h2[normalize-space()='Delivery Services']"
+160.Verify Delivery Services,verify,,"//div[normalize-space()='DELIVERY SERVICES']"
+161.Filter Services List,type,{deliveryName},"//input[@aria-label='Services Filter Input']"
+162.Click Edit Icon ,click,,"//i[@title='Edit']"
+163.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+164.wait,1000,,
+164.Select Dectivate,click,,"//li[@aria-label='Deactivate']"
+165.Click Submit ,click,,"//button[normalize-space()='Submit']"
+166.Filter Services List,type,{deliveryName},"//input[@aria-label='Services Filter Input']"
+167.wait,1000,,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+2.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+3.Click Store subscription plan,click,,"//span[normalize-space()='Store Subscription Plan']"
+4.Verify Store Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Store']"
+5.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
+6.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+7.Select Food Delivery,click,,"//li[@aria-label='Food Delivery']"
+8.Enter Store Plan Name, type, StorePlan{randomAlpha}&gt;&gt; storeSubscriptionName, "//input[@placeholder='Plan Name']"
+9.Enter Store Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
+10.Enter Store Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
+11.Enter Store Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
+12.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
+13.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
+14.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
+15.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description(in Arabic)']"
+16.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description(in Tamil)']"
+17.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description(in Hindi)']"
+18.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+19.Select On,click,,"//li[@aria-label='on']"
+20.Click Submit ,click,,"//button[normalize-space()='Submit']"
+21.Filter Services List,type,{storeSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+22.Click Edit ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+23.Click Close ,click,,"//button[normalize-space()='Close']"
+24.Click Active ,click,,"//i[@title='Active']"
+25.wait,2000,,
+26.Click Deactive,click,,"//i[@title='Inactive']"
+27.wait,2000,,
+28.Click Delete Plan,click,,"//i[@class='bi bi-trash cursor-pointer gridIcon Delete']"
+29.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
+30.wait,3000,,
+31.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+32.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+33.Click Driver subscription plan,click,,"//span[normalize-space()='Driver Subscription Plan']"
+34.Verify Driver Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Driver']"
+35.Click  Add New Subscription,click,,"//button[normalize-space()='ADD']"
+36.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+37.Select Auto Ride,click,,"//li[@aria-label='Auto Ride']"
+38.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "//input[@placeholder='Plan Name']"
+39.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
+40.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil)']"
+41.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi)']"
+42.Enter Number Of Days, type,100, "//input[@placeholder='No. of Days ']"
+43.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No of Rides with Zero admin commission']"
+44.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
+45.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
+46.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description Arabic']"
+47.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description Tamil']"
+48.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description Hindi']"
+49.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+50.Select On,click,,"//li[@aria-label='on']"
+51.Click Submit ,click,,"//button[normalize-space()='Submit']"
+52.Filter Services List,type,{driverSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+53.Click Edit ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+54.Click Close ,click,,"//button[normalize-space()='Close']"
+55.Click Active ,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+56.wait,2000,,
+57.Click Deactive,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
+58.wait,2000,,
+59.Click Delete Plan,click,,"//i[@class='bi bi-trash cursor-pointer gridIcon Delete']"
+60.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
+61.wait,3000,,
+62.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+63.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+64.Click Provider subscription plan,click,,"//span[normalize-space()='Provider Subscription Plan']"
+65.Verify Provider Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Provider']"
+66.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
+67.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+68.Select Pest Control,click,,"//li[@aria-label='Pest Control']"
+69.Enter Provider Plan Name, type, ProviderPlan{randomAlpha}&gt;&gt; providerSubscriptionName, "//input[@placeholder='Plan Name']"
+70.Enter Provider Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic):']"
+71.Enter Provider Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
+72.Enter Provider Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
+73.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
+74.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price ']"
+75.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Enter Description(in English):']"
+76.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Enter Description(in Arabic):']"
+77.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Enter Description(in Tamil)']"
+78.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Enter Description(in Hindi']"
+79.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+80.Select On,click,,"//li[@aria-label='on']"
+81.Click Submit ,click,,"//button[normalize-space()='Submit']"
+82.Filter Services List,type,{providerSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+83.Click Edit ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+84.Click Close ,click,,"//button[normalize-space()='Close']"
+85.Click Active ,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
+86.wait,2000,,
+87.Click Deactive,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
+88.wait,2000,,
+89.Click Delete Plan,click,,"//i[@class='bi bi-trash cursor-pointer gridIcon Delete']"
+90.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
+91.wait,3000,,
+92.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+93.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+94.Click Customer subscription plan,click,,"//span[normalize-space()='Customer subscription plan']"
+95.Verify Customer Subscription Plan Lists ,verify,,"//div[normalize-space()='Customer Subscription Plans']"
+96.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
+97.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+98.Select Pest Control,click,,"//li[@aria-label='Pest Control']"
+99.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; custometSubscriptionName, "//input[@placeholder='Plan Name']"
+100.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
+101.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
+102.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
+103.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
+104.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No Of Free Rides']"
+105.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
+106.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
+107.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description(in Arabic)']"
+108.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description(in Tamil)']"
+109.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description(in Hindi)']"
+110.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+111.Select On,click,,"//li[@aria-label='on']"
+112.Click Submit ,click,,"//button[normalize-space()='Submit']"
+113.Filter Services List,type,{custometSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+114.Click Edit ,click,,"//i[@title='Edit Plan']"
+115.Click Close ,click,,"//button[normalize-space()='Close']"
+116.Click Active ,click,,"//i[@title='Activate Plan']"
+117.wait,2000,,
+118.Click Deactive,click,,"//i[@title='Deactivate Plan']"
+119.wait,2000,,
+120.Click Delete Plan,click,,"//i[@title='Delete Plan']"
+121.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
+122.wait,3000,,
+</t>
   </si>
 </sst>
 </file>
@@ -3221,7 +3222,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
@@ -3299,13 +3300,13 @@
         <v>31</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>41</v>
@@ -3371,16 +3372,16 @@
         <v>34</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>35</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3437,22 +3438,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3509,22 +3510,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>38</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3581,22 +3582,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3653,22 +3654,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C2" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3725,22 +3726,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3803,19 +3804,19 @@
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3882,16 +3883,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3957,13 +3958,13 @@
         <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>40</v>
@@ -4022,16 +4023,16 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4094,16 +4095,16 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4166,16 +4167,16 @@
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4235,19 +4236,19 @@
         <v>30</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C2" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4311,16 +4312,16 @@
         <v>28</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>29</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>44</v>
+        <v>98</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
68th commit: 16 Test Cases Completed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94A5C8B5-77AB-4EB0-99FB-DFF0B202A1FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C57FD5A0-4207-47A3-8582-A69389F140A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="11" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2776,7 +2776,7 @@
 91.wait,3000,,
 92.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
 93.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
-94.Click Customer subscription plan,click,,"//span[normalize-space()='Customer subscription plan']"
+94.Click Customer subscription plan,click,,"//span[normalize-space()='Customer Subscription Plan']"
 95.Verify Customer Subscription Plan Lists ,verify,,"//div[normalize-space()='Customer Subscription Plans']"
 96.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
 97.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"

</xml_diff>

<commit_message>
69th commit: Transport City Admin Test Started
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C57FD5A0-4207-47A3-8582-A69389F140A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50EE8301-0A18-4945-8381-96D809E6A3AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="11" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -28,7 +28,8 @@
     <sheet name="AddProvider" sheetId="11" r:id="rId13"/>
     <sheet name="ProviderServiceCompleteTest" sheetId="12" r:id="rId14"/>
     <sheet name="SubscriptionPlanTest" sheetId="29" r:id="rId15"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId16"/>
+    <sheet name="AddTransportCityAdmin" sheetId="30" r:id="rId16"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId17"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="106">
   <si>
     <t>City Area</t>
   </si>
@@ -968,15 +969,6 @@
   </si>
   <si>
     <t>TC_CA_03_add_city_admin</t>
-  </si>
-  <si>
-    <t>TC_CA_04_add_verify_auto_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_05_add_verify_bike_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_06_add_verify_taxi_driver</t>
   </si>
   <si>
     <t>SA_TS_11</t>
@@ -1245,28 +1237,7 @@
     <t>Add New Transport Service ,Vehicle Type &amp;  driver</t>
   </si>
   <si>
-    <t>TC_CA_08_add_store</t>
-  </si>
-  <si>
-    <t>TC_CA_09_store_oprerations</t>
-  </si>
-  <si>
-    <t>TC_CA_10_store_status_management</t>
-  </si>
-  <si>
-    <t>TC_CA_11_delivery_service_complete_test</t>
-  </si>
-  <si>
-    <t>TC_CA_12_add_provider</t>
-  </si>
-  <si>
     <t>SA_TS_13</t>
-  </si>
-  <si>
-    <t>TC_CA_13_provider_service_full_lifecycle_test</t>
-  </si>
-  <si>
-    <t>TC_CA_07_transport_service_complete_test</t>
   </si>
   <si>
     <r>
@@ -1700,63 +1671,10 @@
 141.wait,1000,,</t>
   </si>
   <si>
-    <t>1.Remove Test Area,sql delete,,"DELETE FROM we1.admin_area_list WHERE name = '{areaName}';"
-2.Remove Customer,sql delete,,"DELETE FROM we1.users WHERE first_name = '{customerName}';"
-3.Remove City Admin,sql delete,,"DELETE FROM we1.super_admin WHERE name = '{adminName}';"
-4.Remove Auto Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{autoName}';"
-5.Remove Auto Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{autoName}';"
-6.Remove Auto Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{autoCompanyName}';"
-7.Remove Bike Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{bikeName}';"
-8.Remove Bike Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{bikeName}';"
-9.Remove Bike Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{bikeCompanyName}';"
-10.Remove Taxi Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{taxiName}';"
-11.Remove Taxi Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{taxiName}';"
-12.Remove Taxi Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{taxiCompanyName}';"
-13.Remove Bus Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{busDriverName}';"
-14.Remove Bus Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{busDriverName}';"
-15.Remove Bus Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{busCompanyName}';"
-16.Remove Bus Driver Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{documentName}';"
-17.Remove Transport Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{promoCodeName}';"
-18.Remove Bus Vehicle Variation Volvo,sql delete,,"DELETE FROM we1.transport_vehicle_type WHERE name = '{busTypeName}';"
-19.Remove  Transport Ride,sql delete,,"DELETE FROM we1.service_category WHERE name = '{transportName}';"
-20.Remove Kfc Private Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{kfcdriverName}';"
-21.Remove Kfc Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{kfcBikeCompanyName}';"
-22.Remove Kfc Product Details,sql delete,,"DELETE FROM we1.store_product_details WHERE name = '{kfcProductName}';"
-23.Remove Kfc Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{storeOwner}';"
-24.Remove Kfc Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{storeOwner}';"
-25.Remove Kfc Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{storeName}';"
-26.Remove Bilal Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{hotelOwner}';"
-27.Remove Bilal Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{hotelOwner}';"
-28.Remove Bilal Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{hotelName}';"
-29.Remove Amul Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{milkStoreOwner}';"
-30.Remove Amul Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{milkStoreOwner}';"
-31.Remove Amul Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{milkStore}';"
-32.Remove Curd Product Category,sql delete,,"DELETE FROM we1.store_product_category WHERE name = '{MilkCategoryName}';"
-33.Remove Delievery Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{deliveryDocumentName}';"
-34.Remove Delievery Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{deliveryPromoCodeName}';"
-35.Remove  Deleivrey Service,sql delete,,"DELETE FROM we1.service_category WHERE name = '{deliveryName}';"
-36.Remove Plumber Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{plumberName}';"
-37.Remove Plumber Provider Details,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{plumberName}';"
-38.Remove Painter Package,sql delete,,"DELETE FROM we1.other_service_provider_packages WHERE name = '{packageName}';"
-39.Remove Painter Sub Category,sql delete,,"DELETE FROM we1.other_service_sub_category WHERE name = '{painterCategoryName}';"
-40.Remove Provider Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{providerDocumentName}';"
-41.Remove Provider Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{providerPromoCodeName}';"
-42.Remove Painter Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{painterName}';"
-43.Remove Painter From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{painterName}';"
-44.Remove Provider Service,sql delete,,"DELETE FROM we1.service_category WHERE name = '{serviceName}';"
-45.wait,2000,,</t>
-  </si>
-  <si>
     <t>Add New  Store, Provider , Driver &amp;  Customer Subscription Plan</t>
   </si>
   <si>
-    <t>TC_CA_14_subscription_plan_test</t>
-  </si>
-  <si>
     <t>SA_TS_15</t>
-  </si>
-  <si>
-    <t>TC_CA_15_test_data_cleanup</t>
   </si>
   <si>
     <r>
@@ -2806,6 +2724,174 @@
 121.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
 122.wait,3000,,
 </t>
+  </si>
+  <si>
+    <t>SA_TS_16</t>
+  </si>
+  <si>
+    <t>TC_CA_16_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>TransportCityAdmin</t>
+  </si>
+  <si>
+    <t>1.Remove Test Area,sql delete,,"DELETE FROM we1.admin_area_list WHERE name = '{areaName}';"
+2.Remove Customer,sql delete,,"DELETE FROM we1.users WHERE first_name = '{customerName}';"
+3.Remove City Admin,sql delete,,"DELETE FROM we1.super_admin WHERE name = '{adminName}';"
+4.Remove Transport City Admin,sql delete,,"DELETE FROM we1.super_admin WHERE name = '{transAdminName}';"
+5.Remove Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{driverName}';"
+6.Remove  Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{driverName}';"
+7.Remove  Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{companyName}';"
+8.Remove Auto Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{autoName}';"
+9.Remove Auto Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{autoName}';"
+10.Remove Auto Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{autoCompanyName}';"
+11.Remove Bike Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{bikeName}';"
+12.Remove Bike Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{bikeName}';"
+13.Remove Bike Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{bikeCompanyName}';"
+14.Remove Taxi Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{taxiName}';"
+15.Remove Taxi Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{taxiName}';"
+16.Remove Taxi Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{taxiCompanyName}';"
+17.Remove Bus Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{busDriverName}';"
+18.Remove Bus Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{busDriverName}';"
+19.Remove Bus Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{busCompanyName}';"
+20.Remove Bus Driver Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{documentName}';"
+21.Remove Transport Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{promoCodeName}';"
+22.Remove Bus Vehicle Variation Volvo,sql delete,,"DELETE FROM we1.transport_vehicle_type WHERE name = '{busTypeName}';"
+23.Remove  Transport Ride,sql delete,,"DELETE FROM we1.service_category WHERE name = '{transportName}';"
+24.Remove Kfc Private Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{kfcdriverName}';"
+25.Remove Kfc Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{kfcBikeCompanyName}';"
+26.Remove Kfc Product Details,sql delete,,"DELETE FROM we1.store_product_details WHERE name = '{kfcProductName}';"
+27.Remove Kfc Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{storeOwner}';"
+28.Remove Kfc Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{storeOwner}';"
+29.Remove Kfc Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{storeName}';"
+30.Remove Bilal Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{hotelOwner}';"
+31.Remove Bilal Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{hotelOwner}';"
+32.Remove Bilal Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{hotelName}';"
+33.Remove Amul Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{milkStoreOwner}';"
+34.Remove Amul Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{milkStoreOwner}';"
+35.Remove Amul Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{milkStore}';"
+36.Remove Curd Product Category,sql delete,,"DELETE FROM we1.store_product_category WHERE name = '{MilkCategoryName}';"
+37.Remove Delievery Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{deliveryDocumentName}';"
+38.Remove Delievery Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{deliveryPromoCodeName}';"
+39.Remove  Deleivrey Service,sql delete,,"DELETE FROM we1.service_category WHERE name = '{deliveryName}';"
+40.Remove Plumber Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{plumberName}';"
+41.Remove Plumber Provider Details,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{plumberName}';"
+42.Remove Painter Package,sql delete,,"DELETE FROM we1.other_service_provider_packages WHERE name = '{packageName}';"
+43.Remove Painter Sub Category,sql delete,,"DELETE FROM we1.other_service_sub_category WHERE name = '{painterCategoryName}';"
+44.Remove Provider Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{providerDocumentName}';"
+45.Remove Provider Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{providerPromoCodeName}';"
+46.Remove Painter Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{painterName}';"
+47.Remove Painter From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{painterName}';"
+48.Remove Provider Service,sql delete,,"DELETE FROM we1.service_category WHERE name = '{serviceName}';"
+49.wait,2000,,</t>
+  </si>
+  <si>
+    <t>1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+4. Verify City Admin List,verify,,"//div[normalize-space()='City Admin List']"
+5. Click Add City Admin button,click,,"//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
+6. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
+7.Select Name field,click ,, "//input[@id='name']"
+8. Enter Admin Name, type, newAdmin{randomAlpha} &gt;&gt; transAdminName, "//input[@id='name']"
+9.Select Email field,click,, "//input[@id='email']"
+10. Enter Email, type, transAdmin_{timestamp}@gmail.com &gt;&gt; transAdminEmail, "//input[@id='email']"
+11.select the password field,click,, "//input[@id='password']"
+12.Enter the Password ,type,password{timestamp}&gt;&gt; transAdminPassword, "//input[@id='password']"
+13.Open Select City Dropdown,click,,"//select[@id='cityId']"
+14.Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
+15. Click on the "Transport Service" → "Bike Ride" checkbox. "//label[normalize-space()='Bike Ride']"
+16.Click on the "Transport Service" → "Taxi Ride" checkbox. "//label[normalize-space()='Taxi Ride']"
+17.Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
+18.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
+19.Click on the "Drivers" → "Approved Drivers" checkbox. "//label[normalize-space()='Approved Drivers']"
+20.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
+21.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
+22.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
+23.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
+24.Click on the "Add City Admin" button. "//button[@type='submit']"
+25. Verify Success Message,verify,,"//div[@aria-label='Info']"
+26.Filter admin name,type,{transAdminName},"//input[@aria-label='Name Filter Input']"
+27.wait,1000,,
+28.Click Logout Icon,click,,"//i[@class='fa-right-from-bracket fa-solid iconstyle']"
+29.Click Confirm Logout,click,,"//button[normalize-space()='Logout']"
+30.wait,1000,,
+31. Enter  Email , type , {transAdminEmail}, "//input[@placeholder='Enter your email']"
+32. Enter Password,type,{transAdminPassword}, "//input[@placeholder='Enter your password']"
+33. Click Login,click,,"//button[@type='submit']"
+34. Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
+35.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+36.Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+37. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+38.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+39.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+40.Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
+41.Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; driverName, "//label[contains(.,'Full Name')]/following::input[1]"
+42.Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;driverEmail, "//label[contains(.,'Email')]/following::input[1]"
+43.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+44.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+45.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+46.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+47.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
+48. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+49.Enter Vehicle Company, type, autoCompany{randomAlpha}&gt;&gt; companyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+50. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+51. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+52. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+53. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+54. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+55. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+56. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+57. Enter Account Holder Name, type,{driverName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+58.Enter Payment Email Address, type, {driverEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+59. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+60.Click Submit, click, , "//button[contains(.,'Submit')]"
+61.Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+62.wait,3000,,
+63.Click Logout Icon,click,,"//i[@class='fa-right-from-bracket fa-solid iconstyle']"
+64.Click Confirm Logout,click,,"//button[normalize-space()='Logout']"
+65.wait,1000,,
+66.Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
+67.Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
+68.Click Login,click,,"//button[@type='submit']"
+69.Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
+70.wait,1000,,</t>
+  </si>
+  <si>
+    <t>TC_CA_04_add_verify_auto_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_05_add_verify_bike_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_06_add_verify_taxi_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_07_transport_service_complete_test</t>
+  </si>
+  <si>
+    <t>TC_CA_08_add_store</t>
+  </si>
+  <si>
+    <t>TC_CA_9_store_oprerations</t>
+  </si>
+  <si>
+    <t>TC_CA_10_store_status_management</t>
+  </si>
+  <si>
+    <t>TC_CA_11_delivery_service_complete_test</t>
+  </si>
+  <si>
+    <t>TC_CA_12_add_provider</t>
+  </si>
+  <si>
+    <t>TC_CA_13_provider_service_full_lifecycle_test</t>
+  </si>
+  <si>
+    <t>TC_CA_14_subscription_plan_test</t>
+  </si>
+  <si>
+    <t>TC_CA_15_add_transport_city_admin</t>
   </si>
 </sst>
 </file>
@@ -3222,7 +3308,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
@@ -3300,13 +3386,13 @@
         <v>31</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>68</v>
+        <v>99</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>41</v>
@@ -3372,13 +3458,13 @@
         <v>34</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>69</v>
+        <v>100</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>35</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>48</v>
@@ -3438,22 +3524,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3510,19 +3596,19 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>71</v>
+        <v>102</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>38</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>49</v>
@@ -3582,22 +3668,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>73</v>
+        <v>103</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3654,22 +3740,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3685,6 +3771,71 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F6B7FC7-76CD-491F-AC51-1837B3B068AC}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="2" max="2" width="19.88671875" customWidth="1"/>
+    <col min="3" max="3" width="25.44140625" customWidth="1"/>
+    <col min="4" max="4" width="34.77734375" customWidth="1"/>
+    <col min="5" max="5" width="64" customWidth="1"/>
+    <col min="6" max="6" width="32.6640625" customWidth="1"/>
+    <col min="7" max="7" width="17.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3726,22 +3877,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3810,10 +3961,10 @@
         <v>51</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>44</v>
@@ -3889,7 +4040,7 @@
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>44</v>
@@ -3964,7 +4115,7 @@
         <v>26</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>40</v>
@@ -4023,13 +4174,13 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>54</v>
+        <v>94</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>45</v>
@@ -4095,13 +4246,13 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>55</v>
+        <v>95</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>46</v>
@@ -4167,13 +4318,13 @@
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>47</v>
@@ -4236,19 +4387,19 @@
         <v>30</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>76</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4312,13 +4463,13 @@
         <v>28</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>67</v>
+        <v>98</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>29</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>48</v>

</xml_diff>

<commit_message>
70th commit: Transport City Admin Test Completed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50EE8301-0A18-4945-8381-96D809E6A3AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C54B54-CC9F-40CE-9ADE-2888A9FBD2DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="13" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -2786,6 +2786,42 @@
 49.wait,2000,,</t>
   </si>
   <si>
+    <t>TC_CA_04_add_verify_auto_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_05_add_verify_bike_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_06_add_verify_taxi_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_07_transport_service_complete_test</t>
+  </si>
+  <si>
+    <t>TC_CA_08_add_store</t>
+  </si>
+  <si>
+    <t>TC_CA_9_store_oprerations</t>
+  </si>
+  <si>
+    <t>TC_CA_10_store_status_management</t>
+  </si>
+  <si>
+    <t>TC_CA_11_delivery_service_complete_test</t>
+  </si>
+  <si>
+    <t>TC_CA_12_add_provider</t>
+  </si>
+  <si>
+    <t>TC_CA_13_provider_service_full_lifecycle_test</t>
+  </si>
+  <si>
+    <t>TC_CA_14_subscription_plan_test</t>
+  </si>
+  <si>
+    <t>TC_CA_15_add_transport_city_admin</t>
+  </si>
+  <si>
     <t>1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
 2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
 3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
@@ -2847,51 +2883,23 @@
 59. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
 60.Click Submit, click, , "//button[contains(.,'Submit')]"
 61.Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-62.wait,3000,,
-63.Click Logout Icon,click,,"//i[@class='fa-right-from-bracket fa-solid iconstyle']"
-64.Click Confirm Logout,click,,"//button[normalize-space()='Logout']"
-65.wait,1000,,
-66.Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
-67.Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
-68.Click Login,click,,"//button[@type='submit']"
-69.Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
-70.wait,1000,,</t>
-  </si>
-  <si>
-    <t>TC_CA_04_add_verify_auto_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_05_add_verify_bike_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_06_add_verify_taxi_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_07_transport_service_complete_test</t>
-  </si>
-  <si>
-    <t>TC_CA_08_add_store</t>
-  </si>
-  <si>
-    <t>TC_CA_9_store_oprerations</t>
-  </si>
-  <si>
-    <t>TC_CA_10_store_status_management</t>
-  </si>
-  <si>
-    <t>TC_CA_11_delivery_service_complete_test</t>
-  </si>
-  <si>
-    <t>TC_CA_12_add_provider</t>
-  </si>
-  <si>
-    <t>TC_CA_13_provider_service_full_lifecycle_test</t>
-  </si>
-  <si>
-    <t>TC_CA_14_subscription_plan_test</t>
-  </si>
-  <si>
-    <t>TC_CA_15_add_transport_city_admin</t>
+62.wait,5000,,
+63.Click sidebar,click,,"//*[local-name()='svg' and @id='Layer_1']"
+64.wait,2000,,
+65.Check Transport Menu exists,element_present , , "//h2[normalize-space()='Transport Services']"
+66.wait,2000,,
+67.Check Deleivery Service exists, element_absent, , "//h2[normalize-space()='Delivery Services']"
+68.wait,2000,,
+69.Check Provider Service exists, element_absent, , "//h2[normalize-space()='Provider Services']"
+70.wait,2000,,
+71.Click Logout Icon,click,,"//h2[normalize-space()='Logout']"
+72.Click Confirm Logout,click,,"//button[normalize-space()='Logout']"
+73.wait,2000,,
+74.Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
+75.Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
+76.Click Login,click,,"//button[@type='submit']"
+77.Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
+78.wait,1000,,</t>
   </si>
 </sst>
 </file>
@@ -3386,7 +3394,7 @@
         <v>31</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>32</v>
@@ -3458,7 +3466,7 @@
         <v>34</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>35</v>
@@ -3530,7 +3538,7 @@
         <v>57</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>60</v>
@@ -3602,7 +3610,7 @@
         <v>37</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>38</v>
@@ -3674,7 +3682,7 @@
         <v>43</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>59</v>
@@ -3746,7 +3754,7 @@
         <v>73</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>76</v>
@@ -3818,13 +3826,13 @@
         <v>91</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>40</v>
@@ -4174,7 +4182,7 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
@@ -4246,7 +4254,7 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
@@ -4318,7 +4326,7 @@
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
@@ -4390,7 +4398,7 @@
         <v>63</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>66</v>
@@ -4463,7 +4471,7 @@
         <v>28</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
71th commit: Keyword Refrernce Page Updated
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C54B54-CC9F-40CE-9ADE-2888A9FBD2DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DE325C3-6743-41E9-95B4-355A2E8CAFE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="13" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="108">
   <si>
     <t>City Area</t>
   </si>
@@ -2900,6 +2900,99 @@
 76.Click Login,click,,"//button[@type='submit']"
 77.Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
 78.wait,1000,,</t>
+  </si>
+  <si>
+    <t>This test case validates the end-to-end lifecycle of an tranport city admin. The workflow initiates with the configuration of a new City Admin profile—integrating dynamic data generation for credentials and city mapping—while assigning permissions across specific transport services (Bike, Taxi, Auto) and driver management modules.The process systematically transitions from the super-admin creation phase to a live login validation, where the new admin’s restricted environment is audited to ensure the presence of authorized transport menus and the successful exclusion of unauthorized delivery and provider service modules. The validation cycle culminates in the execution of complex driver onboarding within the newly created admin account—spanning personal, vehicle, and banking data integration—thereby confirming the platform’s security architecture, hierarchical permission integrity, and the operational stability of city-specific administrative workflows.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddCityArea test suite must be always executed before this test. This is critical because the AddTransportCityAdmin process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
+RunSheet: AddCityArea</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>System State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -3829,13 +3922,13 @@
         <v>104</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>26</v>
+        <v>106</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>105</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>40</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
72th commit: All Test Cases Updated and Working
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DE325C3-6743-41E9-95B4-355A2E8CAFE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DD5F093-C7FB-4077-9FBF-20D6CCCC7834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1907,60 +1907,6 @@
 42. Verify Success Message,verify,,"//div[@aria-label='Info']"
 43.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
 </t>
-  </si>
-  <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-6. Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-7. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-8. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
-9. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-10. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-11. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-12.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-13.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
-14. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-15.Enter Vehicle Company, type, autoCompany{randomAlpha}&gt;&gt; autoCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-16. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-17. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-18. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-19. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-20. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-21. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-22. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-23. Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-24. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-25. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-26. Click Submit, click, , "//button[contains(.,'Submit')]"
-27. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-28. Wait for Toast to hide, wait, 1000,
-29.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-31.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-32.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-33.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-34.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-35. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-36.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-37.Add Driving License,click,,"//i[@title='Edit']"
-38.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-39.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-40.Click Submit, click, , "//button[normalize-space()='Submit']"
-41.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-42.Click Approve Driver,click,,"//i[@title='Approve']"
-43.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-43.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-46.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-47.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-48.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-50.Click Doc Icon,click,,"//i[@title='Document']"
-51.Click Eye Icon,click,,"//i[@title='View']"
-52.wait,1000,,</t>
   </si>
   <si>
     <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
@@ -2735,264 +2681,420 @@
     <t>TransportCityAdmin</t>
   </si>
   <si>
+    <t>TC_CA_04_add_verify_auto_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_05_add_verify_bike_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_06_add_verify_taxi_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_07_transport_service_complete_test</t>
+  </si>
+  <si>
+    <t>TC_CA_08_add_store</t>
+  </si>
+  <si>
+    <t>TC_CA_9_store_oprerations</t>
+  </si>
+  <si>
+    <t>TC_CA_10_store_status_management</t>
+  </si>
+  <si>
+    <t>TC_CA_11_delivery_service_complete_test</t>
+  </si>
+  <si>
+    <t>TC_CA_12_add_provider</t>
+  </si>
+  <si>
+    <t>TC_CA_13_provider_service_full_lifecycle_test</t>
+  </si>
+  <si>
+    <t>TC_CA_14_subscription_plan_test</t>
+  </si>
+  <si>
+    <t>TC_CA_15_add_transport_city_admin</t>
+  </si>
+  <si>
+    <t>This test case validates the end-to-end lifecycle of an tranport city admin. The workflow initiates with the configuration of a new City Admin profile—integrating dynamic data generation for credentials and city mapping—while assigning permissions across specific transport services (Bike, Taxi, Auto) and driver management modules.The process systematically transitions from the super-admin creation phase to a live login validation, where the new admin’s restricted environment is audited to ensure the presence of authorized transport menus and the successful exclusion of unauthorized delivery and provider service modules. The validation cycle culminates in the execution of complex driver onboarding within the newly created admin account—spanning personal, vehicle, and banking data integration—thereby confirming the platform’s security architecture, hierarchical permission integrity, and the operational stability of city-specific administrative workflows.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddCityArea test suite must be always executed before this test. This is critical because the AddTransportCityAdmin process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
+RunSheet: AddCityArea</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>System State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
+    </r>
+  </si>
+  <si>
     <t>1.Remove Test Area,sql delete,,"DELETE FROM we1.admin_area_list WHERE name = '{areaName}';"
 2.Remove Customer,sql delete,,"DELETE FROM we1.users WHERE first_name = '{customerName}';"
 3.Remove City Admin,sql delete,,"DELETE FROM we1.super_admin WHERE name = '{adminName}';"
-4.Remove Transport City Admin,sql delete,,"DELETE FROM we1.super_admin WHERE name = '{transAdminName}';"
-5.Remove Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{driverName}';"
-6.Remove  Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{driverName}';"
-7.Remove  Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{companyName}';"
-8.Remove Auto Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{autoName}';"
-9.Remove Auto Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{autoName}';"
-10.Remove Auto Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{autoCompanyName}';"
-11.Remove Bike Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{bikeName}';"
-12.Remove Bike Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{bikeName}';"
-13.Remove Bike Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{bikeCompanyName}';"
-14.Remove Taxi Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{taxiName}';"
-15.Remove Taxi Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{taxiName}';"
-16.Remove Taxi Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{taxiCompanyName}';"
-17.Remove Bus Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{busDriverName}';"
-18.Remove Bus Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{busDriverName}';"
-19.Remove Bus Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{busCompanyName}';"
-20.Remove Bus Driver Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{documentName}';"
-21.Remove Transport Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{promoCodeName}';"
-22.Remove Bus Vehicle Variation Volvo,sql delete,,"DELETE FROM we1.transport_vehicle_type WHERE name = '{busTypeName}';"
-23.Remove  Transport Ride,sql delete,,"DELETE FROM we1.service_category WHERE name = '{transportName}';"
-24.Remove Kfc Private Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{kfcdriverName}';"
-25.Remove Kfc Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{kfcBikeCompanyName}';"
-26.Remove Kfc Product Details,sql delete,,"DELETE FROM we1.store_product_details WHERE name = '{kfcProductName}';"
-27.Remove Kfc Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{storeOwner}';"
-28.Remove Kfc Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{storeOwner}';"
-29.Remove Kfc Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{storeName}';"
-30.Remove Bilal Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{hotelOwner}';"
-31.Remove Bilal Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{hotelOwner}';"
-32.Remove Bilal Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{hotelName}';"
-33.Remove Amul Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{milkStoreOwner}';"
-34.Remove Amul Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{milkStoreOwner}';"
-35.Remove Amul Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{milkStore}';"
-36.Remove Curd Product Category,sql delete,,"DELETE FROM we1.store_product_category WHERE name = '{MilkCategoryName}';"
-37.Remove Delievery Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{deliveryDocumentName}';"
-38.Remove Delievery Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{deliveryPromoCodeName}';"
-39.Remove  Deleivrey Service,sql delete,,"DELETE FROM we1.service_category WHERE name = '{deliveryName}';"
-40.Remove Plumber Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{plumberName}';"
-41.Remove Plumber Provider Details,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{plumberName}';"
-42.Remove Painter Package,sql delete,,"DELETE FROM we1.other_service_provider_packages WHERE name = '{packageName}';"
-43.Remove Painter Sub Category,sql delete,,"DELETE FROM we1.other_service_sub_category WHERE name = '{painterCategoryName}';"
-44.Remove Provider Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{providerDocumentName}';"
-45.Remove Provider Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{providerPromoCodeName}';"
-46.Remove Painter Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{painterName}';"
-47.Remove Painter From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{painterName}';"
-48.Remove Provider Service,sql delete,,"DELETE FROM we1.service_category WHERE name = '{serviceName}';"
-49.wait,2000,,</t>
-  </si>
-  <si>
-    <t>TC_CA_04_add_verify_auto_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_05_add_verify_bike_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_06_add_verify_taxi_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_07_transport_service_complete_test</t>
-  </si>
-  <si>
-    <t>TC_CA_08_add_store</t>
-  </si>
-  <si>
-    <t>TC_CA_9_store_oprerations</t>
-  </si>
-  <si>
-    <t>TC_CA_10_store_status_management</t>
-  </si>
-  <si>
-    <t>TC_CA_11_delivery_service_complete_test</t>
-  </si>
-  <si>
-    <t>TC_CA_12_add_provider</t>
-  </si>
-  <si>
-    <t>TC_CA_13_provider_service_full_lifecycle_test</t>
-  </si>
-  <si>
-    <t>TC_CA_14_subscription_plan_test</t>
-  </si>
-  <si>
-    <t>TC_CA_15_add_transport_city_admin</t>
-  </si>
-  <si>
-    <t>1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-4. Verify City Admin List,verify,,"//div[normalize-space()='City Admin List']"
-5. Click Add City Admin button,click,,"//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
-6. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
-7.Select Name field,click ,, "//input[@id='name']"
-8. Enter Admin Name, type, newAdmin{randomAlpha} &gt;&gt; transAdminName, "//input[@id='name']"
-9.Select Email field,click,, "//input[@id='email']"
-10. Enter Email, type, transAdmin_{timestamp}@gmail.com &gt;&gt; transAdminEmail, "//input[@id='email']"
-11.select the password field,click,, "//input[@id='password']"
-12.Enter the Password ,type,password{timestamp}&gt;&gt; transAdminPassword, "//input[@id='password']"
-13.Open Select City Dropdown,click,,"//select[@id='cityId']"
-14.Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-15. Click on the "Transport Service" → "Bike Ride" checkbox. "//label[normalize-space()='Bike Ride']"
-16.Click on the "Transport Service" → "Taxi Ride" checkbox. "//label[normalize-space()='Taxi Ride']"
-17.Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
-18.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
-19.Click on the "Drivers" → "Approved Drivers" checkbox. "//label[normalize-space()='Approved Drivers']"
-20.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
-21.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
-22.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
-23.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
-24.Click on the "Add City Admin" button. "//button[@type='submit']"
-25. Verify Success Message,verify,,"//div[@aria-label='Info']"
-26.Filter admin name,type,{transAdminName},"//input[@aria-label='Name Filter Input']"
-27.wait,1000,,
-28.Click Logout Icon,click,,"//i[@class='fa-right-from-bracket fa-solid iconstyle']"
-29.Click Confirm Logout,click,,"//button[normalize-space()='Logout']"
-30.wait,1000,,
-31. Enter  Email , type , {transAdminEmail}, "//input[@placeholder='Enter your email']"
-32. Enter Password,type,{transAdminPassword}, "//input[@placeholder='Enter your password']"
-33. Click Login,click,,"//button[@type='submit']"
-34. Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
-35.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-36.Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-37. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-38.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-39.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-40.Click Checkbox, click, , "//mat-checkbox[.//input[@id='mat-mdc-checkbox-1-input']]"
-41.Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; driverName, "//label[contains(.,'Full Name')]/following::input[1]"
-42.Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;driverEmail, "//label[contains(.,'Email')]/following::input[1]"
-43.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-44.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-45.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-46.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-47.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
-48. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-49.Enter Vehicle Company, type, autoCompany{randomAlpha}&gt;&gt; companyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-50. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-51. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-52. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-53. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-54. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-55. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-56. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-57. Enter Account Holder Name, type,{driverName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-58.Enter Payment Email Address, type, {driverEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-59. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-60.Click Submit, click, , "//button[contains(.,'Submit')]"
-61.Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-62.wait,5000,,
-63.Click sidebar,click,,"//*[local-name()='svg' and @id='Layer_1']"
-64.wait,2000,,
-65.Check Transport Menu exists,element_present , , "//h2[normalize-space()='Transport Services']"
-66.wait,2000,,
-67.Check Deleivery Service exists, element_absent, , "//h2[normalize-space()='Delivery Services']"
-68.wait,2000,,
-69.Check Provider Service exists, element_absent, , "//h2[normalize-space()='Provider Services']"
-70.wait,2000,,
-71.Click Logout Icon,click,,"//h2[normalize-space()='Logout']"
-72.Click Confirm Logout,click,,"//button[normalize-space()='Logout']"
-73.wait,2000,,
-74.Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
-75.Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
-76.Click Login,click,,"//button[@type='submit']"
-77.Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
-78.wait,1000,,</t>
-  </si>
-  <si>
-    <t>This test case validates the end-to-end lifecycle of an tranport city admin. The workflow initiates with the configuration of a new City Admin profile—integrating dynamic data generation for credentials and city mapping—while assigning permissions across specific transport services (Bike, Taxi, Auto) and driver management modules.The process systematically transitions from the super-admin creation phase to a live login validation, where the new admin’s restricted environment is audited to ensure the presence of authorized transport menus and the successful exclusion of unauthorized delivery and provider service modules. The validation cycle culminates in the execution of complex driver onboarding within the newly created admin account—spanning personal, vehicle, and banking data integration—thereby confirming the platform’s security architecture, hierarchical permission integrity, and the operational stability of city-specific administrative workflows.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The AddCityArea test suite must be always executed before this test. This is critical because the AddTransportCityAdmin process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
-RunSheet: AddCityArea</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>System State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
-    </r>
+4.Remove Auto Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{autoName}';"
+5.Remove Auto Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{autoName}';"
+6.Remove Auto Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{autoCompanyName}';"
+7.Remove Bike Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{bikeName}';"
+8.Remove Bike Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{bikeName}';"
+9.Remove Bike Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{bikeCompanyName}';"
+10.Remove Taxi Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{taxiName}';"
+11.Remove Taxi Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{taxiName}';"
+12.Remove Taxi Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{taxiCompanyName}';"
+13.Remove Bus Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{busDriverName}';"
+14.Remove Bus Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{busDriverName}';"
+15.Remove Bus Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{busCompanyName}';"
+16.Remove Bus Driver Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{documentName}';"
+17.Remove Transport Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{promoCodeName}';"
+18.Remove Bus Vehicle Variation Volvo,sql delete,,"DELETE FROM we1.transport_vehicle_type WHERE name = '{busTypeName}';"
+19.Remove  Transport Ride,sql delete,,"DELETE FROM we1.service_category WHERE name = '{transportName}';"
+20.Remove Kfc Private Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{kfcdriverName}';"
+21.Remove Kfc Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{kfcBikeCompanyName}';"
+22.Remove Kfc Product Details,sql delete,,"DELETE FROM we1.store_product_details WHERE name = '{kfcProductName}';"
+23.Remove Kfc Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{storeOwner}';"
+24.Remove Kfc Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{storeOwner}';"
+25.Remove Kfc Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{storeName}';"
+26.Remove Bilal Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{hotelOwner}';"
+27.Remove Bilal Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{hotelOwner}';"
+28.Remove Bilal Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{hotelName}';"
+29.Remove Amul Owner Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{milkStoreOwner}';"
+30.Remove Amul Owner From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{milkStoreOwner}';"
+31.Remove Amul Store Details,sql delete,,"DELETE FROM we1.store_details WHERE name = '{milkStore}';"
+32.Remove Curd Product Category,sql delete,,"DELETE FROM we1.store_product_category WHERE name = '{MilkCategoryName}';"
+33.Remove Delievery Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{deliveryDocumentName}';"
+34.Remove Delievery Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{deliveryPromoCodeName}';"
+35.Remove  Deleivrey Service,sql delete,,"DELETE FROM we1.service_category WHERE name = '{deliveryName}';"
+36.Remove Plumber Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{plumberName}';"
+37.Remove Plumber Provider Details,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{plumberName}';"
+38.Remove Painter Package,sql delete,,"DELETE FROM we1.other_service_provider_packages WHERE name = '{packageName}';"
+39.Remove Painter Sub Category,sql delete,,"DELETE FROM we1.other_service_sub_category WHERE name = '{painterCategoryName}';"
+40.Remove Provider Document,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{providerDocumentName}';"
+41.Remove Provider Service PromoCode,sql delete,,"DELETE FROM we1.promocode_details WHERE promo_code = '{providerPromoCodeName}';"
+42.Remove Painter Bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{painterName}';"
+43.Remove Painter From Providers,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{painterName}';"
+44.Remove Provider Service,sql delete,,"DELETE FROM we1.service_category WHERE name = '{serviceName}';"
+45.Remove Lorry Driver,sql delete,,"DELETE FROM we1.providers WHERE first_name = '{lorrydriverName}';"
+46.Remove Bus Driver bank Details,sql delete,,"DELETE FROM we1.provider_bank_details WHERE holder_name = '{lorrydriverName}';"
+47.Remove Lorry Vehicle Details,sql delete,,"DELETE FROM we1.transport_driver_details WHERE vehicle_company = '{lorrycompanyName}';"
+48.Remove Lorry Vehicle Variation tempo,sql delete,,"DELETE FROM we1.transport_vehicle_type WHERE name = '{lorryTypeName}';"
+49.Remove  Transport Ride,sql delete,,"DELETE FROM we1.service_category WHERE name = '{lorryTransportName}';"
+50.Remove Transport City Admin,sql delete,,"DELETE FROM we1.super_admin WHERE name = '{transAdminName}';"
+51.wait,2000,,</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+6. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+7. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+8. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+9. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+10. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+11. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+12.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+13.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
+14. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+15.Enter Vehicle Company, type, autoCompany{randomAlpha}&gt;&gt; autoCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+16. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+17. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+18. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+19. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+20. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+21. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+22. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+23. Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+24. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+25. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+26. Click Submit, click, , "//button[contains(.,'Submit')]"
+27. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+28. Wait for Toast to hide, wait, 1000,
+29.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+32.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+33.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+34.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+35. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+36.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+37.Add Driving License,click,,"//i[@title='Edit']"
+38.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+39.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+40.Click Submit, click, , "//button[normalize-space()='Submit']"
+41.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+42.Click Approve Driver,click,,"//i[@title='Approve']"
+43.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+43.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+46.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+47.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+48.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+50.Click Doc Icon,click,,"//i[@title='Document']"
+51.Click Eye Icon,click,,"//i[@title='View']"
+52.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+2.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+3.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
+4.Click  Add Category,click,,"//button[normalize-space()='Add Category']"
+5.Enter Service Name, type, lorryRide{randomAlpha}&gt;&gt;lorryTransportName, "//input[@placeholder='Service Name']"
+6.Enter Service Name Arabic, type, رحلة بالحافلة, "//input[@placeholder='Service Name (in Arabic)']"
+7.Enter Slug, type,{lorryTransportName}, "//input[@placeholder='Slug']"
+8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/lorry.png", "//input[@type='file' and @accept='image/*']"
+9.wait,2000,,
+10.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+11.Select Activate,click,,"//li[@aria-label='Activate']"
+12.Open Select City Dropdown,click,,"//span[text()='Select City']/ancestor::app-drop-down//div[contains(@class, 'p-multiselect-label-container')]"
+13.Select {areaName},click,,"//li[@aria-label='{areaName}']"
+14.Click  Submit,click,,"//button[normalize-space()='Submit']"
+15.Verify Sucess, verify, , "//div[@aria-label='Info']"
+16.wait,2000,,
+17.Click Dashboard Home Icon,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
+18.Click Dashboard menu,click,,"//h2[normalize-space()='Dashboard']"
+19.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+20.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+21.Filter Services List,type,{lorryTransportName},"//input[@aria-label='Services Filter Input']"
+22.Click Home Icon ,click,,"//i[@title='Home']"
+23.Click Settings ,click,,"//button[contains(., 'Settings')]"
+24.Click Vehicle Type,click,,"//div[normalize-space()='Vehicle Type']"
+25.Click Add Vehicle Type,click,,"//button[normalize-space()='Add Vehicle Type']"
+26.Enter Vehicle Type Name, type, tempo{randomAlpha}&gt;&gt;lorryTypeName, "//input[@placeholder='Enter Vehicle Type']"
+27.Enter Base Fare, type, 150, "//input[@placeholder='Enter base fare']"
+28.Enter Base Fare Max Kilometer, type, 10, "//input[@placeholder='Enter Base Fare KM Limit']"
+29.Open Extra Distance Fare Dropdown,click,"//label[contains(., 'Extra Distance Fare Type')]/following-sibling::p-dropdown"
+30.Select Amount,click,,"//li[@aria-label='Amount']"
+31.Enter Extra Distance Fare , type, 10, "//input[@placeholder='Extra Distance Fare (Per Km)']"
+32.Enter Free Waiting Time , type, 10, "//label[contains(., 'Free Waiting Time')]/following::input[1]"
+33.Open Waiting Charge Dropdown,click,"((//label[contains(., 'Waiting Charge Type')]/following::p-dropdown)[1])"
+34.Select Amount,click,,"//li[@aria-label='Amount']"
+35.Enter Waiting Rate , type, 10, "//input[@placeholder='Waiting Rate (per min)']"
+36.Enter Included Trip Waiting , type, 10, "//input[@placeholder='Included Trip Waiting']"
+37.Open Trip Waiting Charge Dropdown,click,"((//label[contains(., 'Waiting Charge Type')]/following::p-dropdown)[2])"
+38.Select Amount,click,,"//li[@aria-label='Amount']"
+39.Enter Trip Waiting Rate , type,50, "//input[@placeholder='Trip Waiting Rate (per min)']"
+40.Enter Free Pickup Distance , type,5, "//input[@placeholder='Free Pickup Distance (In kms)']"
+41.Open Pickup Charge Dropdown,click,"//label[contains(., 'Pickup Charge Type')]/following-sibling::p-dropdown"
+42.Select Amount,click,,"//li[@aria-label='Amount']"
+43.Enter Pickup Fee, type,50, "//input[@placeholder='Pickup Fee (Per Km)']"
+44.Open Customer Fee  Dropdown,click,"//span[@aria-label='Customer Fee Type']"
+45.Select Amount,click,,"//li[@aria-label='Amount']"
+46.Enter Customer Fee, type,50, "//input[@placeholder='Customer Fee']"
+47.Open Customer GST  Dropdown,click,"//label[contains(., 'Customer GST type')]/following-sibling::p-dropdown"
+48.Select Amount,click,,"//li[@aria-label='Amount']"
+49.Enter  GST amount, type,50, "//input[contains(@placeholder,'Enter GST amount or percentage')]"
+50.Open Driver Fee  Dropdown,click,"//span[@aria-label='Driver Fee Type']"
+51.Select Amount,click,,"//li[@aria-label='Amount']"
+52.Enter  Driver Fee, type,50, "//input[@placeholder='Driver Fee']"
+53.Open Driver GST  Dropdown,click,"//label[contains(., 'Driver GST type')]/following-sibling::p-dropdown"
+54.Select Amount,click,,"//li[@aria-label='Amount']"
+55.Enter Driver Gst,type,50," //input[@placeholder='Driver GST in amount or percentage']"
+56.Open Status Dropdown,click,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+57.Select Active,click,,"//li[@aria-label='Active']"
+58.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/tempo.jpg", "//app-image-upload//input[@type='file' and @accept='image/*']"
+59.Enter Notifiacation,type,50,"//input[@placeholder='User will be notified when pickup km exceeds this']"
+60.Enter Driver Request ETA,type,50,"//input[@placeholder='Enter Driver ETA Limit']"
+61.Enter Driver Request KM,type,50,"//input[@placeholder='Driver Request KM Limit']"
+62.Click Surcharge Time Checkbox, click, , "//div[text()='EveryDay']/preceding-sibling::mat-checkbox"
+63.Enter From Time, type, 100000AM, "((//input[@placeholder='--:--:-- --'])[1])"
+64.Enter To Time, type, 220000PM, "((//input[@placeholder='--:--:-- --'])[2])"
+65.Open  Dropdown,click,"((//span[@aria-label='select type'])[1])"
+66.Select Amount,click,,"//li[@aria-label='Amount']"
+67.Enter  Price, type,50, "//input[@placeholder='Enter Price']"
+68.Click  Submit,click,,"//button[normalize-space()='Submit']"
+69.Verify Sucess, verify, , "//div[@aria-label='Info']"
+70.wait,3000,,
+71.Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+72.Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+73. Verify City Admin List,verify,,"//div[normalize-space()='City Admin List']"
+74.Click Add City Admin button,click,,"//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
+75.Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
+76.Select Name field,click ,, "//input[@id='name']"
+77. Enter Admin Name, type, newAdmin{randomAlpha} &gt;&gt; transAdminName, "//input[@id='name']"
+78.Select Email field,click,, "//input[@id='email']"
+79. Enter Email, type, transAdmin_{timestamp}@gmail.com &gt;&gt; transAdminEmail, "//input[@id='email']"
+80.select the password field,click,, "//input[@id='password']"
+81.Enter the Password ,type,password{timestamp}&gt;&gt; transAdminPassword, "//input[@id='password']"
+82.Open Select City Dropdown,click,,"//select[@id='cityId']"
+83.Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
+84. Click on the "Transport Service" → "Bike Ride" checkbox. "//label[normalize-space()='Bike Ride']"
+85.Click on the "Transport Service" → "Taxi Ride" checkbox. "//label[normalize-space()='Taxi Ride']"
+86.Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
+87.Click on the "Transport Service" → "{lorryTransportName}" checkbox. "//label[normalize-space()='{lorryTransportName}']"
+88.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
+89.Click on the "Drivers" → "Approved Drivers" checkbox. "//label[normalize-space()='Approved Drivers']"
+90.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
+91.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
+92.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
+93.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
+94.Click on the "Drivers" → "Driver Peding Documents" checkbox. "//label[normalize-space()='Driver Peding Documents']"
+95.Click on the "Drivers" → "Driver Expired Documents" checkbox. "//label[normalize-space()='Driver Expired Documents']"
+96.Click on the "Add City Admin" button. "//button[@type='submit']"
+97. Verify Success Message,verify,,"//div[@aria-label='Info']"
+98.Filter admin name,type,{transAdminName},"//input[@aria-label='Name Filter Input']"
+99.wait,1000,,
+100.Click Logout Icon,click,,"//i[@class='fa-right-from-bracket fa-solid iconstyle']"
+101.Click Confirm Logout,click,,"//button[normalize-space()='Logout']"
+102.wait,1000,,
+103.Enter  Email , type , {transAdminEmail}, "//input[@placeholder='Enter your email']"
+104.Enter Password,type,{transAdminPassword}, "//input[@placeholder='Enter your password']"
+105.Click Login,click,,"//button[@type='submit']"
+106.Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
+107.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+108.Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+109.Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+110.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+111.Select Lorry Ride Option,click,,"//span[normalize-space()='{lorryTransportName}']"
+112.Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+113.Enter Driver Name, type, lorrydriver{randomAlpha} &gt;&gt; lorrydriverName, "//label[contains(.,'Full Name')]/following::input[1]"
+114.Enter Email, type, lorrydriver_{timestamp}@gmail.com&gt;&gt;lorrydriverEmail, "//label[contains(.,'Email')]/following::input[1]"
+115.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+116.Upload Profile Image, uploadfile, "src/main/resources/test-data/lorrydriver.jpg", "//input[@type='file']"
+117.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+118.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+119.Select  Lorry Option,click,,"//span[normalize-space()='{lorryTypeName}']"
+120. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+121.Enter Vehicle Company, type, lorryCompany{randomAlpha}&gt;&gt; lorrycompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+122. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+123.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+124.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/lorry.png", "(//input[@type='file'])[2]"
+125.Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+126.Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+127.Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+128.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+129.Enter Account Holder Name, type,{lorrydriverName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+130.Enter Payment Email Address, type, {driverEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+131.Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+132.Click Submit, click, , "//button[contains(.,'Submit')]"
+133.Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+134.wait,5000,,
+135.Click sidebar,click,,"//*[local-name()='svg' and @id='Layer_1']"
+136.wait,2000,,
+137.Check Transport Menu exists,element_present , , "//h2[normalize-space()='Transport Services']"
+138.wait,2000,,
+139.Check Deleivery Service exists, element_absent, , "//h2[normalize-space()='Delivery Services']"
+140.wait,2000,,
+141.Check Provider Service exists, element_absent, , "//h2[normalize-space()='Provider Services']"
+142.wait,2000,,
+143.Check Add Driver exists, element_present, , " //span[normalize-space()='Add Driver']"
+144.wait,2000,,
+145.Check Approved Driver exists, element_present, , " //span[normalize-space()='Approved Drivers']"
+146.wait,2000,,
+147. Check Un-Approved Drivers exists, element_present, , " //span[normalize-space()='Un-Approved Drivers']"
+148.wait,2000,,
+149.Check  Blocked Driver exists, element_present, , "//span[normalize-space()='Blocked Drivers']"
+150.wait,2000,,
+151.Check  Reject Driver exists, element_present, , "//span[normalize-space()='Reject Drivers']"
+152.wait,2000,,
+153.Check  Deleted Driver exists, element_present, , "//span[normalize-space()='Deleted Drivers']"
+154.wait,2000,,
+155.Check  Driver Documents exists, element_present, , "//span[normalize-space()='Driver Peding Documents']"
+156.wait,2000,,
+157.Check  Driver Expired Documents exists, element_present, , "//span[normalize-space()='Driver Expired Documents']"
+158.wait,2000,,
+159.Click Logout Icon,click,,"//h2[normalize-space()='Logout']"
+160.Click Confirm Logout,click,,"//button[normalize-space()='Logout']"
+161.wait,2000,,
+162.Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
+163.Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
+164.Click Login,click,,"//button[@type='submit']"
+165.Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
+166.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
+167.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
+168.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
+169.Filter Services List,type,{lorryTransportName},"//input[@aria-label='Services Filter Input']"
+170.Click Edit Icon ,click,,"//i[@title='Edit']"
+171.wait,2000,,
+172.Scroll Grid, tab, 5, "//input[@placeholder='Service Name']"
+173.wait,2000,,
+174.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
+175.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
+176.Click  Submit,click,,"//button[normalize-space()='Submit']"
+177.Verify Sucess, verify, , "//div[@aria-label='Info']"
+178.wait,2000,,</t>
   </si>
 </sst>
 </file>
@@ -3409,7 +3511,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
@@ -3487,7 +3589,7 @@
         <v>31</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>32</v>
@@ -3559,13 +3661,13 @@
         <v>34</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>35</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>48</v>
@@ -3631,13 +3733,13 @@
         <v>57</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>60</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>61</v>
@@ -3703,7 +3805,7 @@
         <v>37</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>38</v>
@@ -3775,7 +3877,7 @@
         <v>43</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>59</v>
@@ -3847,13 +3949,13 @@
         <v>73</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>76</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>75</v>
@@ -3916,19 +4018,19 @@
         <v>74</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -3978,19 +4080,19 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>70</v>
@@ -4275,13 +4377,13 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>45</v>
@@ -4347,13 +4449,13 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>46</v>
@@ -4419,13 +4521,13 @@
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>47</v>
@@ -4491,13 +4593,13 @@
         <v>63</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>66</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>65</v>
@@ -4564,13 +4666,13 @@
         <v>28</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>29</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>48</v>

</xml_diff>

<commit_message>
74th Commit :Sheet Loop Running For Database Stress Test Implemented
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT PROJECTS\ABCDautomationforUI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DD5F093-C7FB-4077-9FBF-20D6CCCC7834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5787D5C3-CA9B-4D1F-AE52-D3930F559C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -1746,88 +1746,6 @@
   </si>
   <si>
     <t>This test case validates the end-to-end management of subscription plan architectures across four distinct user entities: Store, Driver, Provider, and Customer. The workflow systematically executes the creation of localized "Premium" plans for various service categories—such as Food Delivery and Pest Control—featuring integrated multi-language support in Arabic, Tamil, and Hindi. The validation cycle spans from defining plan durations, pricing, and free-ride quotas to conducting administrative audits including localized description verification, active/inactive state toggling, and data filtering. The process concludes by confirming the operational lifecycle through record modification and final deletion, ensuring the functional stability and localized integrity of the platform’s commercial monetization modules.</t>
-  </si>
-  <si>
-    <t>1. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-2.Click  Add Customers,click,,"//span[normalize-space()='Add Customers']"
-3. Verify Add Customer Heading,verify,,"//div[normalize-space()='Add Customer']"
-4.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "//label[contains(., 'Customer Full Name')]/following::input[1]"
-5.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "//input[@type='email']"
-6.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-7.Enter Video Call Limit, type, 60, "//label[contains(., 'User Used Video Call Limit in Minutes')]/following::input[1]"
-8.Open Gender,click,,"//span[@aria-label='select gender']"
-9.Select Male,click,,"//li[@aria-label='Male']"
-10.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "//input[@type='file' and @accept='image/*']"
-11.Click Submit, click, , "//button[normalize-space()='Submit']"
-12.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-13. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-14. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-15.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
-16. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-17.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-18.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
-19.Click Edit Icon ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-20.Click Close, click, , "//button[normalize-space()='Close']"
-21.Click Wallet Icon ,click,,"//i[@title='Wallet']"
-22.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
-23.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
-24.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-25.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
-26.Click Submit, click, , "//button[normalize-space()='Submit']"
-27.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-28.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
-29.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
-30.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-31.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
-32.Click Submit, click, , "//button[normalize-space()='Submit']"
-33.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-34. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-35. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-36.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
-37. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-38.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-39.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
-40.Click Loyalty Points Icon,click,,"//i[@title='Loyalty Points']"
-41.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
-42.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
-43.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
-44.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-45.Select Add Points,click,,"//li[@role='option'][contains(.,'Add Points')]"
-46.Enter Points, type, 30, "//input[@placeholder='Enter Points']"
-47.Click Submit, click, , "//button[normalize-space()='Submit']"
-48.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-49.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
-50.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
-51.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
-52.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-53.Select Deduct Points,click,,"//li[@role='option'][contains(.,'Deduct Points')]"
-54.Enter Points, type, 10, "//input[@placeholder='Enter Points']"
-55.Click Submit, click, , "//button[normalize-space()='Submit']"
-56.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-57. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-58. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-59.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
-60. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-61.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-62.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
-63.Click Disable  Icon,click,,"//i[@title='Block']"
-64.Click Disable  User  Yes,click,,"//button[normalize-space()='Yes']"
-65.Disable Reason,type,Client Complaints,"//textarea[@id='swal2-textarea']"
-66.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-67.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-68. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-69. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-70.Click  Blocked Customers,click,,"//span[normalize-space()='Blocked Customers']"
-71.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-72.Scroll Grid, tab, 10, "//input[@aria-label='Customer Name Filter Input']"
-73.Click Enable  Icon,click,,"//i[@title='Status']"
-74.Click Enable  Yes,click,,"//button[normalize-space()='Yes']"
-75. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-76. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-77.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
-78. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-79.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-80.wait,1000,,</t>
   </si>
   <si>
     <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
@@ -3095,6 +3013,89 @@
 176.Click  Submit,click,,"//button[normalize-space()='Submit']"
 177.Verify Sucess, verify, , "//div[@aria-label='Info']"
 178.wait,2000,,</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard  Icon,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
+2. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+3.Click  Add Customers,click,,"//span[normalize-space()='Add Customers']"
+4. Verify Add Customer Heading,verify,,"//div[normalize-space()='Add Customer']"
+5.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "//label[contains(., 'Customer Full Name')]/following::input[1]"
+6.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "//input[@type='email']"
+7.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+8.Enter Video Call Limit, type, 60, "//label[contains(., 'User Used Video Call Limit in Minutes')]/following::input[1]"
+9.Open Gender,click,,"//span[@aria-label='select gender']"
+10.Select Male,click,,"//li[@aria-label='Male']"
+11.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "//input[@type='file' and @accept='image/*']"
+12.Click Submit, click, , "//button[normalize-space()='Submit']"
+13.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+14.Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+15.Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+16.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
+17.Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+18.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+19.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
+20.Click Edit Icon ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
+21.Click Close, click, , "//button[normalize-space()='Close']"
+22.Click Wallet Icon ,click,,"//i[@title='Wallet']"
+23.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
+24.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
+25.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+26.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
+27.Click Submit, click, , "//button[normalize-space()='Submit']"
+28.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+29.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
+30.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
+31.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+32.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
+33.Click Submit, click, , "//button[normalize-space()='Submit']"
+34.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
+35. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+36. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+37.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
+38. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+39.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+40.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
+41.Click Loyalty Points Icon,click,,"//i[@title='Loyalty Points']"
+42.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
+43.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
+44.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
+45.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+46.Select Add Points,click,,"//li[@role='option'][contains(.,'Add Points')]"
+47.Enter Points, type, 30, "//input[@placeholder='Enter Points']"
+48.Click Submit, click, , "//button[normalize-space()='Submit']"
+49.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+50.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
+51.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
+52.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
+53.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
+54.Select Deduct Points,click,,"//li[@role='option'][contains(.,'Deduct Points')]"
+55.Enter Points, type, 10, "//input[@placeholder='Enter Points']"
+56.Click Submit, click, , "//button[normalize-space()='Submit']"
+57.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+58. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+59.Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+60.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
+61. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+62.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+63.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
+64.Click Disable  Icon,click,,"//i[@title='Block']"
+65.Click Disable  User  Yes,click,,"//button[normalize-space()='Yes']"
+66.Disable Reason,type,Client Complaints,"//textarea[@id='swal2-textarea']"
+67.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
+68.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+69. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+70. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+71.Click  Blocked Customers,click,,"//span[normalize-space()='Blocked Customers']"
+72.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+73.Scroll Grid, tab, 10, "//input[@aria-label='Customer Name Filter Input']"
+74.Click Enable  Icon,click,,"//i[@title='Status']"
+75.Click Enable  Yes,click,,"//button[normalize-space()='Yes']"
+76. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+77. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+78.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
+79. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+80.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+81.wait,1000,,</t>
   </si>
 </sst>
 </file>
@@ -3511,7 +3512,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
@@ -3589,7 +3590,7 @@
         <v>31</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>32</v>
@@ -3661,13 +3662,13 @@
         <v>34</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>35</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>48</v>
@@ -3733,13 +3734,13 @@
         <v>57</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>60</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>61</v>
@@ -3805,7 +3806,7 @@
         <v>37</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>38</v>
@@ -3877,7 +3878,7 @@
         <v>43</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>59</v>
@@ -3949,13 +3950,13 @@
         <v>73</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>76</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>75</v>
@@ -4018,19 +4019,19 @@
         <v>74</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -4080,19 +4081,19 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>70</v>
@@ -4167,7 +4168,7 @@
         <v>55</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>77</v>
+        <v>107</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>44</v>
@@ -4243,7 +4244,7 @@
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>44</v>
@@ -4318,7 +4319,7 @@
         <v>26</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>40</v>
@@ -4377,13 +4378,13 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>45</v>
@@ -4449,13 +4450,13 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>46</v>
@@ -4521,13 +4522,13 @@
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>47</v>
@@ -4593,13 +4594,13 @@
         <v>63</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>66</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>65</v>
@@ -4666,13 +4667,13 @@
         <v>28</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>29</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>48</v>

</xml_diff>

<commit_message>
75th Commit : Locators.properties Implemented
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCDautomationforUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5787D5C3-CA9B-4D1F-AE52-D3930F559C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{285BFA70-3120-4069-AACA-82F972982231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -30,6 +30,9 @@
     <sheet name="SubscriptionPlanTest" sheetId="29" r:id="rId15"/>
     <sheet name="AddTransportCityAdmin" sheetId="30" r:id="rId16"/>
     <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId17"/>
+    <sheet name="SuperAdminLocator" sheetId="31" r:id="rId18"/>
+    <sheet name="AddCustomerLocator" sheetId="32" r:id="rId19"/>
+    <sheet name="AddAutoDriverLocator" sheetId="33" r:id="rId20"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -41,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="123">
   <si>
     <t>City Area</t>
   </si>
@@ -3096,6 +3099,281 @@
 79. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
 80.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
 81.wait,1000,,</t>
+  </si>
+  <si>
+    <t>Super Admin Locator</t>
+  </si>
+  <si>
+    <t>Verify successful authentication of the Super Admin role using valid credentials and Dashboard access validation using Locators</t>
+  </si>
+  <si>
+    <t>1. Enter  Email , type , super_admin@gmail.com, "admin.login.email"
+2. Enter Password,type,R1mep@321, "admin.login.password"
+3. Click Login,click,,"admin.login.submit_btn"
+4. Verify Dashboard,verify,,"admin.dashboard.statistics_header"</t>
+  </si>
+  <si>
+    <t>Customer Locator</t>
+  </si>
+  <si>
+    <t>Validate the end-to-end creation of a Customer Using Locator</t>
+  </si>
+  <si>
+    <t>1.Click Dashboard  Icon,click,,"admin.menu.dashboard"
+2. Click Customer  Icon,click,,"admin.menu.customer_icon"
+3.Click  Add Customers,click,,"admin.menu.add_customers"
+4. Verify Add Customer Heading,verify,,"admin.customer.add_heading"
+5.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "admin.customer.input_name"
+6.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "admin.customer.input_email"
+7.Enter Contact Number, type, {randomPhone}&gt;&gt;userPhone,"admin.customer.input_phone"
+8.Enter Video Call Limit, type, 60, "admin.customer.input_video_limit"
+9.Open Gender,click,,"admin.customer.dropdown_gender"
+10.Select Male,click,,"admin.customer.select_gender_male"
+11.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "admin.customer.upload_profile_img"
+12.Click Submit, click, , "admin.customer.submit_btn"
+13.Verify Added Succesfully, verify, , "admin.customer.toast_info"
+14. Click Customer  Icon,click,,"admin.menu.customer_icon"
+15. Click Customer  Icon,click,,"admin.menu.customer_icon"
+16.Click  Verified Customers,click,,"admin.menu.verified_customers"
+17. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading "
+18.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SuperAdminLocator</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
+    </r>
+  </si>
+  <si>
+    <t>1.Click drivers menu, click, , "admin.drivers.menu.icon"
+2.Click Add Driver menu, click, ,"admin.drivers.add_menu.link"
+3.Verify Add Driver page, verify, , "admin.drivers.add_page.header"
+4.Click Service Category Dropdown, click, , "admin.drivers.service_dropdown.select"
+5.Select Auto Ride Option, click, , "admin.drivers.autoride_option.span"
+6.Select Auto Ride Option, click, ,"admin.drivers.autoride_option.span"
+7.Wait for Auto Ride Checkbox, wait_until_visible, , "admin.drivers.autoride.checkbox"
+8.Click Auto Ride Checkbox, click, , "admin.drivers.autoride.checkbox"
+9.Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "admin.drivers.fullname.input"
+10.Enter Email, type, autodriver_{timestamp}@gmail.com &gt;&gt; autoEmail, "admin.drivers.email.input"
+11.Enter Contact Number, type, {randomPhone} &gt;&gt; autoPhone, "admin.drivers.phone.input"
+12.Click Whatsapp Checkbox, click, , "admin.drivers.whatsapp.checkbox"
+13.Enter Whatsapp Number, type, {autoPhone}, "admin.drivers.whatsapp_phone.input"
+14.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "admin.drivers.profile_image.file"
+15.Click Select Source Dropdown, click, ,"admin.drivers.source_dropdown.select"
+16.Select From Instagram Option, click, , "admin.drivers.instagram_option.span"
+17.Select Male Gender, click, ," admin.drivers.male_gender.div"
+18.Click Vehicle Type Dropdown, click, ,"admin.drivers.vehicle_dropdown.select"
+19.Select Pink Auto Option, click, ," admin.drivers.pink_auto_option.span"
+20.Enter Model Year, type, 2013, "admin.drivers.modelyear.input"
+21.Enter Plate No, type, KL-01-AB-1234,"admin.drivers.plateno.input"
+22.Enter Model Name, type, petrol, "admin.drivers.modelname.input"
+23.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "admin.drivers.vehicle_image.file"
+24.Enter Bank Name, type, HDFC Bank, "admin.drivers.bankname.input"
+25.Enter Bank Location, type, Chennai, "admin.drivers.banklocation.input"
+26.Enter Account Number, type, 50100123456789, "admin.drivers.accountno.input"
+27.Enter Account Holder Name, type, {autoName}, "admin.drivers.accountholder.input"
+28.Enter Payment Email Address, type, {autoEmail}, "admin.drivers.paymentemail.input"
+29.Enter IFSC Code, type, HDFC0001234, "admin.drivers.ifsc.input"
+30.Click Submit Button, click, , "admin.drivers.submit.button"
+31.Verify Driver Added Successfully, verify, , "admin.drivers.success_toast.div"
+32.Wait for Toast to Hide, wait, 1000, 
+33.Click drivers menu to refresh, click, , "admin.drivers.menu.icon"
+34.Click drivers menu to refresh, click, , "admin.drivers.menu.icon"
+35.Click Pending Documents Menu, click, , "admin.drivers.pending_docs.link"
+36.Filter Pending Docs by Name, type, {autoName}, "admin.drivers.name_filter.input"
+37.Click Dashboard Home Icon, click, , "admin.drivers.dashboard.icon"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+RunSheet:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> SuperAdminLocator
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>SA_TS_17</t>
+  </si>
+  <si>
+    <t>TC_CA_17_super_admin_locator</t>
+  </si>
+  <si>
+    <t>SA_TS_18</t>
+  </si>
+  <si>
+    <t>TC_CA_18_add_customer_Locator</t>
+  </si>
+  <si>
+    <t>SA_TS_19</t>
+  </si>
+  <si>
+    <t>TC_CA_19_add_verify_auto_driver</t>
   </si>
 </sst>
 </file>
@@ -4113,6 +4391,158 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04702C86-94CB-44FD-BDE6-8B1CDCE6BE04}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="26.6640625" customWidth="1"/>
+    <col min="5" max="5" width="53.21875" customWidth="1"/>
+    <col min="6" max="6" width="36.88671875" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{404CB2B3-8656-4A2D-BE0C-F25ED6C3A957}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="31.6640625" customWidth="1"/>
+    <col min="5" max="5" width="53.21875" customWidth="1"/>
+    <col min="6" max="6" width="29" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46ECEE02-404F-4AF1-8311-95653C3B218B}">
   <dimension ref="A1:H3"/>
@@ -4183,6 +4613,78 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0770089-1671-4723-B7EE-933745EC2F72}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="30.88671875" customWidth="1"/>
+    <col min="4" max="4" width="35.5546875" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>